<commit_message>
data: verified full-source CIRP refresh 2026-10-07-1902Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="189">
   <si>
     <t>Priority</t>
   </si>
@@ -1103,7 +1103,7 @@
         <v>46300.7588564394</v>
       </c>
       <c r="P2" s="2">
-        <v>46302.26843221064</v>
+        <v>46302.79192097764</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1147,7 +1147,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P3" s="2">
-        <v>46302.26843222459</v>
+        <v>46302.79192099054</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>27</v>
@@ -1197,7 +1197,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P4" s="2">
-        <v>46302.26842387108</v>
+        <v>46302.79191047805</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>23</v>
@@ -1241,7 +1241,7 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P5" s="2">
-        <v>46302.26842383233</v>
+        <v>46302.79191043837</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1288,7 +1288,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P6" s="2">
-        <v>46302.26842384538</v>
+        <v>46302.7919104524</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>23</v>
@@ -1335,7 +1335,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P7" s="2">
-        <v>46302.26842380712</v>
+        <v>46302.79191041266</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>23</v>
@@ -1382,7 +1382,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P8" s="2">
-        <v>46302.26842375574</v>
+        <v>46302.79191036006</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>23</v>
@@ -1432,7 +1432,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P9" s="2">
-        <v>46302.26842376858</v>
+        <v>46302.79191037345</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>23</v>
@@ -1482,7 +1482,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P10" s="2">
-        <v>46302.26842378132</v>
+        <v>46302.79191038655</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>23</v>
@@ -1529,7 +1529,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P11" s="2">
-        <v>46302.26842374232</v>
+        <v>46302.79191034697</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>23</v>
@@ -1579,7 +1579,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P12" s="2">
-        <v>46302.2684236893</v>
+        <v>46302.79191029487</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1623,7 +1623,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P13" s="2">
-        <v>46302.26842371625</v>
+        <v>46302.79191032116</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>27</v>
@@ -1670,7 +1670,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P14" s="2">
-        <v>46302.26842364718</v>
+        <v>46302.79191025375</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>23</v>
@@ -1717,7 +1717,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P15" s="2">
-        <v>46302.26842366141</v>
+        <v>46302.79191026733</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>27</v>
@@ -1761,7 +1761,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P16" s="2">
-        <v>46302.26842361677</v>
+        <v>46302.79191022492</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>23</v>
@@ -1808,7 +1808,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P17" s="2">
-        <v>46302.26842367557</v>
+        <v>46302.79191028092</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>23</v>
@@ -1858,7 +1858,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P18" s="2">
-        <v>46302.26841531677</v>
+        <v>46302.79189773565</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -1902,7 +1902,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P19" s="2">
-        <v>46302.26841530317</v>
+        <v>46302.79189772235</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>27</v>
@@ -1946,7 +1946,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P20" s="2">
-        <v>46302.2684152897</v>
+        <v>46302.79189770951</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>27</v>
@@ -1993,7 +1993,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P21">
-        <v>46302.26841527641</v>
+        <v>46302.79189769677</v>
       </c>
       <c r="Q21" t="s">
         <v>23</v>
@@ -2040,7 +2040,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P22">
-        <v>46302.26841524903</v>
+        <v>46302.79189767046</v>
       </c>
       <c r="Q22" t="s">
         <v>23</v>
@@ -2084,7 +2084,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P23">
-        <v>46302.26841520685</v>
+        <v>46302.79189763116</v>
       </c>
       <c r="Q23" t="s">
         <v>23</v>
@@ -2131,7 +2131,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P24">
-        <v>46302.26841522126</v>
+        <v>46302.79189764443</v>
       </c>
       <c r="Q24" t="s">
         <v>23</v>
@@ -2178,7 +2178,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P25">
-        <v>46302.26841523509</v>
+        <v>46302.79189765739</v>
       </c>
       <c r="Q25" t="s">
         <v>23</v>
@@ -2225,7 +2225,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P26">
-        <v>46302.2684151932</v>
+        <v>46302.79189761808</v>
       </c>
       <c r="Q26" t="s">
         <v>23</v>
@@ -2272,7 +2272,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P27">
-        <v>46302.26841513602</v>
+        <v>46302.79189759048</v>
       </c>
       <c r="Q27" t="s">
         <v>23</v>
@@ -2316,7 +2316,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P28">
-        <v>46302.26841514941</v>
+        <v>46302.79189760437</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>27</v>
@@ -2360,7 +2360,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P29">
-        <v>46302.26841512165</v>
+        <v>46302.79189757702</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2404,7 +2404,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P30">
-        <v>46302.26841510729</v>
+        <v>46302.79189756404</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>27</v>
@@ -2451,7 +2451,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P31">
-        <v>46302.26841507771</v>
+        <v>46302.79189753801</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>27</v>
@@ -2495,7 +2495,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P32">
-        <v>46302.26841503391</v>
+        <v>46302.79189752453</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>27</v>
@@ -2542,7 +2542,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P33">
-        <v>46302.26841501555</v>
+        <v>46302.79189751096</v>
       </c>
       <c r="Q33" t="s">
         <v>23</v>
@@ -2586,7 +2586,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P34">
-        <v>46302.2684148914</v>
+        <v>46302.79189749651</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>27</v>
@@ -2635,7 +2635,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P35" s="6">
-        <v>46302.26843226571</v>
+        <v>46302.79192102975</v>
       </c>
       <c r="Q35" s="6" t="s">
         <v>23</v>
@@ -2682,7 +2682,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P36" s="6">
-        <v>46302.26843231679</v>
+        <v>46302.79192108147</v>
       </c>
       <c r="Q36" s="6" t="s">
         <v>23</v>
@@ -2731,7 +2731,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P37" s="6">
-        <v>46302.26843229142</v>
+        <v>46302.79192105515</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>23</v>
@@ -2780,7 +2780,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P38" s="6">
-        <v>46302.2684323297</v>
+        <v>46302.79192109437</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>27</v>
@@ -2829,7 +2829,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P39" s="6">
-        <v>46302.26843234283</v>
+        <v>46302.79192110736</v>
       </c>
       <c r="Q39" s="6" t="s">
         <v>23</v>
@@ -2876,7 +2876,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P40" s="6">
-        <v>46302.26843236869</v>
+        <v>46302.79192113371</v>
       </c>
       <c r="Q40" s="5" t="s">
         <v>27</v>
@@ -2925,7 +2925,7 @@
         <v>46300.75886472998</v>
       </c>
       <c r="P41" s="6">
-        <v>46302.26844080219</v>
+        <v>46302.79193306002</v>
       </c>
       <c r="Q41" s="6" t="s">
         <v>23</v>
@@ -2974,7 +2974,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P42" s="6">
-        <v>46302.26843238134</v>
+        <v>46302.79192114654</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>23</v>
@@ -3021,7 +3021,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P43" s="6">
-        <v>46302.26843244523</v>
+        <v>46302.79192121145</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>27</v>
@@ -3072,7 +3072,7 @@
         <v>46300.75886484625</v>
       </c>
       <c r="P44" s="6">
-        <v>46302.26843240711</v>
+        <v>46302.79192117266</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>23</v>
@@ -3121,7 +3121,7 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P45" s="6">
-        <v>46302.26844081699</v>
+        <v>46302.79193307317</v>
       </c>
       <c r="Q45" s="6" t="s">
         <v>23</v>
@@ -3170,7 +3170,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P46" s="6">
-        <v>46302.2684408316</v>
+        <v>46302.79193308652</v>
       </c>
       <c r="Q46" s="5" t="s">
         <v>27</v>
@@ -3217,7 +3217,7 @@
         <v>46300.75887301003</v>
       </c>
       <c r="P47" s="6">
-        <v>46302.26844087261</v>
+        <v>46302.79193312495</v>
       </c>
       <c r="Q47" s="5" t="s">
         <v>27</v>
@@ -3264,7 +3264,7 @@
         <v>46300.75887304553</v>
       </c>
       <c r="P48" s="6">
-        <v>46302.26844088648</v>
+        <v>46302.79193313776</v>
       </c>
       <c r="Q48" s="6" t="s">
         <v>23</v>
@@ -3311,7 +3311,7 @@
         <v>46300.75887306096</v>
       </c>
       <c r="P49" s="6">
-        <v>46302.26844089953</v>
+        <v>46302.79193315036</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>23</v>
@@ -3360,7 +3360,7 @@
         <v>46300.75887309557</v>
       </c>
       <c r="P50" s="6">
-        <v>46302.26844093824</v>
+        <v>46302.79193318906</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>23</v>
@@ -3407,7 +3407,7 @@
         <v>46300.75887314334</v>
       </c>
       <c r="P51" s="6">
-        <v>46302.26844096425</v>
+        <v>46302.7919332146</v>
       </c>
       <c r="Q51" s="5" t="s">
         <v>27</v>
@@ -3456,7 +3456,7 @@
         <v>46300.75887316054</v>
       </c>
       <c r="P52" s="6">
-        <v>46302.26844097774</v>
+        <v>46302.79193322792</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>23</v>
@@ -3505,7 +3505,7 @@
         <v>46300.75887317812</v>
       </c>
       <c r="P53" s="6">
-        <v>46302.26844100373</v>
+        <v>46302.79193325419</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>27</v>
@@ -3554,7 +3554,7 @@
         <v>46300.75887319581</v>
       </c>
       <c r="P54" s="6">
-        <v>46302.26844099083</v>
+        <v>46302.79193324078</v>
       </c>
       <c r="Q54" s="5" t="s">
         <v>27</v>
@@ -3601,7 +3601,7 @@
         <v>46300.75887321083</v>
       </c>
       <c r="P55" s="6">
-        <v>46302.26844095104</v>
+        <v>46302.79193320179</v>
       </c>
       <c r="Q55" s="5" t="s">
         <v>27</v>
@@ -3834,7 +3834,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P2" s="2">
-        <v>46302.26843222459</v>
+        <v>46302.79192099054</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>27</v>
@@ -3878,7 +3878,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P3" s="2">
-        <v>46302.26842371625</v>
+        <v>46302.79191032116</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>27</v>
@@ -3925,7 +3925,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P4" s="2">
-        <v>46302.26842366141</v>
+        <v>46302.79191026733</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>27</v>
@@ -3969,7 +3969,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P5" s="2">
-        <v>46302.26841530317</v>
+        <v>46302.79189772235</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>27</v>
@@ -4013,7 +4013,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P6" s="2">
-        <v>46302.2684152897</v>
+        <v>46302.79189770951</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>27</v>
@@ -4057,7 +4057,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P7">
-        <v>46302.26841514941</v>
+        <v>46302.79189760437</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>27</v>
@@ -4101,7 +4101,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P8">
-        <v>46302.26841510729</v>
+        <v>46302.79189756404</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>27</v>
@@ -4148,7 +4148,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P9">
-        <v>46302.26841507771</v>
+        <v>46302.79189753801</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>27</v>
@@ -4192,7 +4192,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P10">
-        <v>46302.26841503391</v>
+        <v>46302.79189752453</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>27</v>
@@ -4236,7 +4236,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P11">
-        <v>46302.2684148914</v>
+        <v>46302.79189749651</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>27</v>
@@ -4285,7 +4285,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P12" s="6">
-        <v>46302.2684323297</v>
+        <v>46302.79192109437</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>27</v>
@@ -4332,7 +4332,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P13" s="6">
-        <v>46302.26843236869</v>
+        <v>46302.79192113371</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>27</v>
@@ -4379,7 +4379,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P14" s="6">
-        <v>46302.26843244523</v>
+        <v>46302.79192121145</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>27</v>
@@ -4428,7 +4428,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P15" s="6">
-        <v>46302.2684408316</v>
+        <v>46302.79193308652</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>27</v>
@@ -4475,7 +4475,7 @@
         <v>46300.75887301003</v>
       </c>
       <c r="P16" s="6">
-        <v>46302.26844087261</v>
+        <v>46302.79193312495</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>27</v>
@@ -4522,7 +4522,7 @@
         <v>46300.75887314334</v>
       </c>
       <c r="P17" s="6">
-        <v>46302.26844096425</v>
+        <v>46302.7919332146</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>27</v>
@@ -4571,7 +4571,7 @@
         <v>46300.75887317812</v>
       </c>
       <c r="P18" s="6">
-        <v>46302.26844100373</v>
+        <v>46302.79193325419</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>27</v>
@@ -4620,7 +4620,7 @@
         <v>46300.75887319581</v>
       </c>
       <c r="P19" s="6">
-        <v>46302.26844099083</v>
+        <v>46302.79193324078</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>27</v>
@@ -4667,7 +4667,7 @@
         <v>46300.75887321083</v>
       </c>
       <c r="P20" s="6">
-        <v>46302.26844095104</v>
+        <v>46302.79193320179</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>27</v>
@@ -4721,7 +4721,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4769,10 +4769,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B2">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C2" t="s">
         <v>188</v>
@@ -4784,16 +4784,16 @@
         <v>3820</v>
       </c>
       <c r="F2">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H2">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -4804,45 +4804,45 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B3">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C3" t="s">
         <v>188</v>
       </c>
       <c r="D3">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E3">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G3">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H3">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B4">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C4" t="s">
         <v>188</v>
@@ -4854,13 +4854,13 @@
         <v>160</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G4">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -4869,15 +4869,15 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B5">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C5" t="s">
         <v>188</v>
@@ -4889,21 +4889,56 @@
         <v>160</v>
       </c>
       <c r="F5">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H5">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B6">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+      <c r="E6">
+        <v>160</v>
+      </c>
+      <c r="F6">
+        <v>157</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <v>132</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-08-0914Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -12,15 +12,15 @@
     <sheet name="Runs" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-Day Working List'!$A$1:$Q$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Review'!$A$1:$Q$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-Day Working List'!$A$1:$Q$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Review'!$A$1:$Q$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="177">
   <si>
     <t>Priority</t>
   </si>
@@ -79,327 +79,327 @@
     <t>Open</t>
   </si>
   <si>
+    <t>TRUWEIGHT WELLNESS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Pharma / Healthcare</t>
+  </si>
+  <si>
+    <t>Healthcare</t>
+  </si>
+  <si>
+    <t>Chakrala Sannidhi</t>
+  </si>
+  <si>
+    <t>_</t>
+  </si>
+  <si>
+    <t>Auto-classified</t>
+  </si>
+  <si>
+    <t>ALVI TECH SERVICES PVT LTD</t>
+  </si>
+  <si>
+    <t>IT / Technology</t>
+  </si>
+  <si>
+    <t>Neha Jain Nemani</t>
+  </si>
+  <si>
+    <t>Shree Shiddhanath Cotex Private Limited</t>
+  </si>
+  <si>
+    <t>Textiles</t>
+  </si>
+  <si>
+    <t>Akhil Ahuja</t>
+  </si>
+  <si>
+    <t>The FORM G is published for the second time as per the approval by the CoC Members.</t>
+  </si>
+  <si>
+    <t>INFO-DRIVE SOFTWARE LIMITED</t>
+  </si>
+  <si>
+    <t>Sumeet Surendra Chimbalkar</t>
+  </si>
+  <si>
+    <t>The CIRP of the Corporate Debtor (“CD”) has been reinstated pursuant to the order passed by the Hon’ble NCLAT. Further, considering that 360 days of the CIRP period had already elapsed as on the date of appointment of the undersigned (Co</t>
+  </si>
+  <si>
+    <t>REAL TECH CONSTRUCTIONS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Realty / Construction</t>
+  </si>
+  <si>
+    <t>Construction / EPC</t>
+  </si>
+  <si>
+    <t>Manindra Kumar Tiwari</t>
+  </si>
+  <si>
+    <t>A.P.J. LABORATORIES LIMITED</t>
+  </si>
+  <si>
+    <t>Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>pooja damir miglani</t>
+  </si>
+  <si>
+    <t>No Fixed Assets are available, except one disputed and contiguous piece of land at Village Ambwala, Nwada Road Tehsil Paonta Sahib, Distt Sirmaur, Himachal Pradesh, India, 173025</t>
+  </si>
+  <si>
+    <t>ALLFLEX PLASTIC LLP</t>
+  </si>
+  <si>
+    <t>Chemicals</t>
+  </si>
+  <si>
+    <t>Plastics / Polymers</t>
+  </si>
+  <si>
+    <t>Mr. Hansraj Jaria</t>
+  </si>
+  <si>
+    <t>At present, the Corporate Debtor is not operational and not a going concern. Revenue from Operation for the financial year ended 31.03.2025 is ?44,98,79,958.90</t>
+  </si>
+  <si>
+    <t>LOG 9 MATERIALS SCIENTIFIC PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Power / Energy</t>
+  </si>
+  <si>
+    <t>Mrs. Neeraja Kartik</t>
+  </si>
+  <si>
+    <t>250 MWh battery production capacity and 50 MWh cell production capacity</t>
+  </si>
+  <si>
+    <t>TECHNOFAB ENGINEERING LIMITED</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Rahul Jindal</t>
+  </si>
+  <si>
+    <t>The Form G has been published on 27.09.2026 in newspapers all over India.</t>
+  </si>
+  <si>
+    <t>STC VENTURES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Other / Unclear</t>
+  </si>
+  <si>
+    <t>PURUSOTTAM BEHERA</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>VIGNESHWARA DEVELOPERS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Real Estate</t>
+  </si>
+  <si>
+    <t>Ms. Ritu Rastogi</t>
+  </si>
+  <si>
+    <t>EXTOL INDUSTRIES LIMITED</t>
+  </si>
+  <si>
+    <t>Ms. Teena Saraswat Pandey</t>
+  </si>
+  <si>
+    <t>unit closed, no employees / no workmen at CIRP commencement date</t>
+  </si>
+  <si>
+    <t>SURYA FOUNDRY PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Steel / Metals</t>
+  </si>
+  <si>
+    <t>Mr. Reetesh Kumar Agarwal</t>
+  </si>
+  <si>
+    <t>XYRON TECHNOLOGIES LIMITED</t>
+  </si>
+  <si>
+    <t>unit closed As Per Information available no employees / No workmen at the commencement of CIRP Process</t>
+  </si>
+  <si>
+    <t>VAS INFRASTRUCTURE LIMITED (CN)</t>
+  </si>
+  <si>
+    <t>Infrastructure</t>
+  </si>
+  <si>
+    <t>Infrastructure / EPC</t>
+  </si>
+  <si>
+    <t>Mr. Bimal Kumar Agarwal</t>
+  </si>
+  <si>
+    <t>The Form G has been published on 28.09.2026.</t>
+  </si>
+  <si>
+    <t>TV VISION LIMITED</t>
+  </si>
+  <si>
+    <t>ALOK KUMAR MURARKA</t>
+  </si>
+  <si>
+    <t>INDO PACIFIC PROJECTS LIMITED</t>
+  </si>
+  <si>
+    <t>Mrs. Megha Agrawal</t>
+  </si>
+  <si>
+    <t>BHUBANESHWARI SEAFOOD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Agriculture / Food</t>
+  </si>
+  <si>
+    <t>Tripti Agarwal</t>
+  </si>
+  <si>
+    <t>As per the latest available audited financial statement the Turnover in financial year 2022-2023 was Rs. 91.98 crore</t>
+  </si>
+  <si>
+    <t>GOODWILL IRON &amp; STEEL TRADERS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>MANISH AGARWALLA</t>
+  </si>
+  <si>
+    <t>Fixed assets location are taken as per the latest audited balance sheet &amp; address mention as D3/1401 NOIDA Extension .No documents and details are received from the Suspended Board of Directors. Section 19(2) application filed with the Hon'ble NC</t>
+  </si>
+  <si>
+    <t>COMET GRANITO PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Cement / Building Materials</t>
+  </si>
+  <si>
+    <t>Anil Kashi Drolia</t>
+  </si>
+  <si>
+    <t>VAASUDEVA MILK FOODS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ATKURU SAI PRASAD</t>
+  </si>
+  <si>
+    <t>Form-G Issued</t>
+  </si>
+  <si>
+    <t>M/s Margdarshak Financial Services Limited</t>
+  </si>
+  <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
+    <t>Rakesh Kumar Jindal</t>
+  </si>
+  <si>
+    <t>Form G was published for the third time with the approval of the CoC and the NCLT.</t>
+  </si>
+  <si>
+    <t>IN2IT TECHNOLOGIES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ishant jain</t>
+  </si>
+  <si>
+    <t>Re-issuance of Form G: Form G was re-issued on 17.09.2026, with 03.10.2026 as the last date for submission of EOI. Pursuant to the directions of the CoC, an Addendum to Form G was issued, revising and extending the stipulated timelines accordingly.</t>
+  </si>
+  <si>
+    <t>KM TOLL ROAD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Roads / Toll Roads</t>
+  </si>
+  <si>
+    <t>Roads / Highways</t>
+  </si>
+  <si>
+    <t>Mr. Ashish Saoji</t>
+  </si>
+  <si>
+    <t>ORGANIC WORLD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Prakul Thadi</t>
+  </si>
+  <si>
+    <t>SUN GRANITE EXPORT LIMITED</t>
+  </si>
+  <si>
+    <t>Raghunath Bhandari</t>
+  </si>
+  <si>
+    <t>SHRENIK LIMITED</t>
+  </si>
+  <si>
+    <t>RAHUL SHAH</t>
+  </si>
+  <si>
+    <t>OMKARA VIJAYALAKSHMI STRIPS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>A fresh Form-G is issued upon taking approval from the CoC on 6th October 2026. The last day for submission of EOI is 21st October 2026.</t>
+  </si>
+  <si>
+    <t>G &amp; L PROFILE AND EQUIPMENTS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Manish Kumar Bhagat</t>
+  </si>
+  <si>
+    <t>SOCRUS PHARMACEUTICALS LIMITED</t>
+  </si>
+  <si>
+    <t>kuldeep tank</t>
+  </si>
+  <si>
+    <t>PRATHAM-HEERA SALES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Mahesh Goverdhan Bagla</t>
+  </si>
+  <si>
+    <t>Recently closed</t>
+  </si>
+  <si>
+    <t>Closed recently</t>
+  </si>
+  <si>
     <t>SHIVANGI AGRO INDIA PRIVATE LIMITED</t>
   </si>
   <si>
-    <t>Agriculture / Food</t>
-  </si>
-  <si>
     <t>Mr. Manoj Sehgal</t>
   </si>
   <si>
     <t>The Corporate Debtor is Not Operational for last 2 years. Form G published on 22.09.2026 in Financial Express (English, Lucknow Edition) &amp; Jansatta (Hindi, Lucknow Edition)</t>
   </si>
   <si>
-    <t>Auto-classified</t>
-  </si>
-  <si>
     <t>SNEH EXPORTS PRIVATE LIMITED</t>
   </si>
   <si>
-    <t>Other / Unclear</t>
-  </si>
-  <si>
     <t>Garima diggiwal</t>
   </si>
   <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>TRUWEIGHT WELLNESS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Pharma / Healthcare</t>
-  </si>
-  <si>
-    <t>Healthcare</t>
-  </si>
-  <si>
-    <t>Chakrala Sannidhi</t>
-  </si>
-  <si>
-    <t>_</t>
-  </si>
-  <si>
-    <t>ALVI TECH SERVICES PVT LTD</t>
-  </si>
-  <si>
-    <t>IT / Technology</t>
-  </si>
-  <si>
-    <t>Neha Jain Nemani</t>
-  </si>
-  <si>
-    <t>Shree Shiddhanath Cotex Private Limited</t>
-  </si>
-  <si>
-    <t>Textiles</t>
-  </si>
-  <si>
-    <t>Akhil Ahuja</t>
-  </si>
-  <si>
-    <t>The FORM G is published for the second time as per the approval by the CoC Members.</t>
-  </si>
-  <si>
-    <t>INFO-DRIVE SOFTWARE LIMITED</t>
-  </si>
-  <si>
-    <t>Sumeet Surendra Chimbalkar</t>
-  </si>
-  <si>
-    <t>The CIRP of the Corporate Debtor (“CD”) has been reinstated pursuant to the order passed by the Hon’ble NCLAT. Further, considering that 360 days of the CIRP period had already elapsed as on the date of appointment of the undersigned (Co</t>
-  </si>
-  <si>
-    <t>REAL TECH CONSTRUCTIONS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Realty / Construction</t>
-  </si>
-  <si>
-    <t>Construction / EPC</t>
-  </si>
-  <si>
-    <t>Manindra Kumar Tiwari</t>
-  </si>
-  <si>
-    <t>A.P.J. LABORATORIES LIMITED</t>
-  </si>
-  <si>
-    <t>Pharmaceuticals</t>
-  </si>
-  <si>
-    <t>pooja damir miglani</t>
-  </si>
-  <si>
-    <t>No Fixed Assets are available, except one disputed and contiguous piece of land at Village Ambwala, Nwada Road Tehsil Paonta Sahib, Distt Sirmaur, Himachal Pradesh, India, 173025</t>
-  </si>
-  <si>
-    <t>ALLFLEX PLASTIC LLP</t>
-  </si>
-  <si>
-    <t>Chemicals</t>
-  </si>
-  <si>
-    <t>Plastics / Polymers</t>
-  </si>
-  <si>
-    <t>Mr. Hansraj Jaria</t>
-  </si>
-  <si>
-    <t>At present, the Corporate Debtor is not operational and not a going concern. Revenue from Operation for the financial year ended 31.03.2025 is ?44,98,79,958.90</t>
-  </si>
-  <si>
-    <t>LOG 9 MATERIALS SCIENTIFIC PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Power / Energy</t>
-  </si>
-  <si>
-    <t>Mrs. Neeraja Kartik</t>
-  </si>
-  <si>
-    <t>250 MWh battery production capacity and 50 MWh cell production capacity</t>
-  </si>
-  <si>
-    <t>TECHNOFAB ENGINEERING LIMITED</t>
-  </si>
-  <si>
-    <t>Manufacturing</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Rahul Jindal</t>
-  </si>
-  <si>
-    <t>The Form G has been published on 27.09.2026 in newspapers all over India.</t>
-  </si>
-  <si>
-    <t>STC VENTURES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>PURUSOTTAM BEHERA</t>
-  </si>
-  <si>
-    <t>VIGNESHWARA DEVELOPERS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Real Estate</t>
-  </si>
-  <si>
-    <t>Ms. Ritu Rastogi</t>
-  </si>
-  <si>
-    <t>EXTOL INDUSTRIES LIMITED</t>
-  </si>
-  <si>
-    <t>Ms. Teena Saraswat Pandey</t>
-  </si>
-  <si>
-    <t>unit closed, no employees / no workmen at CIRP commencement date</t>
-  </si>
-  <si>
-    <t>SURYA FOUNDRY PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Steel / Metals</t>
-  </si>
-  <si>
-    <t>Mr. Reetesh Kumar Agarwal</t>
-  </si>
-  <si>
-    <t>XYRON TECHNOLOGIES LIMITED</t>
-  </si>
-  <si>
-    <t>unit closed As Per Information available no employees / No workmen at the commencement of CIRP Process</t>
-  </si>
-  <si>
-    <t>VAS INFRASTRUCTURE LIMITED (CN)</t>
-  </si>
-  <si>
-    <t>Infrastructure</t>
-  </si>
-  <si>
-    <t>Infrastructure / EPC</t>
-  </si>
-  <si>
-    <t>Mr. Bimal Kumar Agarwal</t>
-  </si>
-  <si>
-    <t>The Form G has been published on 28.09.2026.</t>
-  </si>
-  <si>
-    <t>TV VISION LIMITED</t>
-  </si>
-  <si>
-    <t>ALOK KUMAR MURARKA</t>
-  </si>
-  <si>
-    <t>INDO PACIFIC PROJECTS LIMITED</t>
-  </si>
-  <si>
-    <t>Mrs. Megha Agrawal</t>
-  </si>
-  <si>
-    <t>BHUBANESHWARI SEAFOOD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Tripti Agarwal</t>
-  </si>
-  <si>
-    <t>As per the latest available audited financial statement the Turnover in financial year 2022-2023 was Rs. 91.98 crore</t>
-  </si>
-  <si>
-    <t>GOODWILL IRON &amp; STEEL TRADERS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>MANISH AGARWALLA</t>
-  </si>
-  <si>
-    <t>Fixed assets location are taken as per the latest audited balance sheet &amp; address mention as D3/1401 NOIDA Extension .No documents and details are received from the Suspended Board of Directors. Section 19(2) application filed with the Hon'ble NC</t>
-  </si>
-  <si>
-    <t>COMET GRANITO PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Cement / Building Materials</t>
-  </si>
-  <si>
-    <t>Anil Kashi Drolia</t>
-  </si>
-  <si>
-    <t>VAASUDEVA MILK FOODS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>ATKURU SAI PRASAD</t>
-  </si>
-  <si>
-    <t>Form-G Issued</t>
-  </si>
-  <si>
-    <t>M/s Margdarshak Financial Services Limited</t>
-  </si>
-  <si>
-    <t>Financial Services</t>
-  </si>
-  <si>
-    <t>Rakesh Kumar Jindal</t>
-  </si>
-  <si>
-    <t>Form G was published for the third time with the approval of the CoC and the NCLT.</t>
-  </si>
-  <si>
-    <t>IN2IT TECHNOLOGIES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>ishant jain</t>
-  </si>
-  <si>
-    <t>Re-issuance of Form G: Form G was re-issued on 17.09.2026, with 03.10.2026 as the last date for submission of EOI. Pursuant to the directions of the CoC, an Addendum to Form G was issued, revising and extending the stipulated timelines accordingly.</t>
-  </si>
-  <si>
-    <t>KM TOLL ROAD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Roads / Toll Roads</t>
-  </si>
-  <si>
-    <t>Roads / Highways</t>
-  </si>
-  <si>
-    <t>Mr. Ashish Saoji</t>
-  </si>
-  <si>
-    <t>ORGANIC WORLD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Prakul Thadi</t>
-  </si>
-  <si>
-    <t>SUN GRANITE EXPORT LIMITED</t>
-  </si>
-  <si>
-    <t>Raghunath Bhandari</t>
-  </si>
-  <si>
-    <t>SHRENIK LIMITED</t>
-  </si>
-  <si>
-    <t>RAHUL SHAH</t>
-  </si>
-  <si>
-    <t>OMKARA VIJAYALAKSHMI STRIPS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>A fresh Form-G is issued upon taking approval from the CoC on 6th October 2026. The last day for submission of EOI is 21st October 2026.</t>
-  </si>
-  <si>
-    <t>G &amp; L PROFILE AND EQUIPMENTS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Manish Kumar Bhagat</t>
-  </si>
-  <si>
-    <t>SOCRUS PHARMACEUTICALS LIMITED</t>
-  </si>
-  <si>
-    <t>kuldeep tank</t>
-  </si>
-  <si>
-    <t>PRATHAM-HEERA SALES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Mahesh Goverdhan Bagla</t>
-  </si>
-  <si>
-    <t>Recently closed</t>
-  </si>
-  <si>
-    <t>Closed recently</t>
-  </si>
-  <si>
     <t>NOEL PHARMA (INDIA) PRIVATE LIMITED</t>
   </si>
   <si>
@@ -515,42 +515,6 @@
   </si>
   <si>
     <t>Assets of the Corporate Debtor and the Personal Guarantors are proposed to be clubbed under Sec.28A of IBC for the purpose of inviting resolution plans.</t>
-  </si>
-  <si>
-    <t>EYEMYEYE PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Suresh Kannan</t>
-  </si>
-  <si>
-    <t>FUTURE CONSUMER LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Avil Jerome Menezes</t>
-  </si>
-  <si>
-    <t>Form G was published on 06 September 2026 for inviting expression of interest in the CIRP of Future Consumer Limited. The last date for submission of expression of interest is 27 September 2026.</t>
-  </si>
-  <si>
-    <t>Bhartiya Micro Credit</t>
-  </si>
-  <si>
-    <t>Reissuance of Form G, subject to the approval of the Committee of Creditors (CoC) and the Hon’ble NCLT.</t>
-  </si>
-  <si>
-    <t>GENESIS INFRATECH PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Ajay Gupta</t>
-  </si>
-  <si>
-    <t>Published in All India editions of Business Standard (English &amp; Hindi), Jaipur edition of Indian Express (English) and Alwar edition of Mahanagar Times (Hindi) on 12.09.2026.</t>
-  </si>
-  <si>
-    <t>JAI AMBE SPARES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Gajesh Labhchand Jain</t>
   </si>
   <si>
     <t>Started</t>
@@ -991,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1075,23 +1039,26 @@
       <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="G2" s="2">
-        <v>0.92</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H2" s="3">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="I2" s="2">
         <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K2" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M2" s="4" t="s">
         <v>18</v>
@@ -1100,13 +1067,13 @@
         <v>18</v>
       </c>
       <c r="O2" s="2">
-        <v>46300.7588564394</v>
+        <v>46300.7588564207</v>
       </c>
       <c r="P2" s="2">
-        <v>46302.79192097764</v>
+        <v>46303.38329450462</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="2" customFormat="1">
@@ -1117,40 +1084,40 @@
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0.91</v>
+      </c>
+      <c r="H3" s="3">
+        <v>46304</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O3" s="2">
+        <v>46300.75885634872</v>
+      </c>
+      <c r="P3" s="2">
+        <v>46303.3832944789</v>
+      </c>
+      <c r="Q3" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="H3" s="3">
-        <v>46302</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" s="2">
-        <v>1</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O3" s="2">
-        <v>46300.75885647022</v>
-      </c>
-      <c r="P3" s="2">
-        <v>46302.79192099054</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1">
@@ -1166,27 +1133,24 @@
       <c r="E4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="G4" s="2">
         <v>0.9399999999999999</v>
       </c>
       <c r="H4" s="3">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="I4" s="2">
         <v>1</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K4" s="2">
-        <v>2</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="M4" s="4" t="s">
         <v>18</v>
       </c>
@@ -1194,13 +1158,13 @@
         <v>18</v>
       </c>
       <c r="O4" s="2">
-        <v>46300.7588564207</v>
+        <v>46300.7588563655</v>
       </c>
       <c r="P4" s="2">
-        <v>46302.79191047805</v>
+        <v>46303.38329448765</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="2" customFormat="1">
@@ -1211,26 +1175,29 @@
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G5" s="2">
         <v>0.91</v>
       </c>
       <c r="H5" s="3">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="I5" s="2">
         <v>2</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K5" s="2">
         <v>1</v>
       </c>
+      <c r="L5" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="M5" s="4" t="s">
         <v>18</v>
       </c>
@@ -1238,13 +1205,13 @@
         <v>18</v>
       </c>
       <c r="O5" s="2">
-        <v>46300.75885634872</v>
+        <v>46300.75885633306</v>
       </c>
       <c r="P5" s="2">
-        <v>46302.79191043837</v>
+        <v>46303.38329446202</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:17" s="2" customFormat="1">
@@ -1255,19 +1222,22 @@
         <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>37</v>
       </c>
       <c r="G6" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="H6" s="3">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="I6" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>38</v>
@@ -1275,9 +1245,6 @@
       <c r="K6" s="2">
         <v>1</v>
       </c>
-      <c r="L6" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="M6" s="4" t="s">
         <v>18</v>
       </c>
@@ -1285,13 +1252,13 @@
         <v>18</v>
       </c>
       <c r="O6" s="2">
-        <v>46300.7588563655</v>
+        <v>46300.75885622757</v>
       </c>
       <c r="P6" s="2">
-        <v>46302.7919104524</v>
+        <v>46303.38329442757</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:17" s="2" customFormat="1">
@@ -1302,16 +1269,19 @@
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="G7" s="2">
-        <v>0.91</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H7" s="3">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="I7" s="2">
         <v>3</v>
@@ -1332,13 +1302,13 @@
         <v>18</v>
       </c>
       <c r="O7" s="2">
-        <v>46300.75885633306</v>
+        <v>46300.75885624527</v>
       </c>
       <c r="P7" s="2">
-        <v>46302.79191041266</v>
+        <v>46303.38329443617</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:17" s="2" customFormat="1">
@@ -1358,13 +1328,13 @@
         <v>45</v>
       </c>
       <c r="G8" s="2">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="H8" s="3">
         <v>46306</v>
       </c>
       <c r="I8" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>46</v>
@@ -1372,6 +1342,9 @@
       <c r="K8" s="2">
         <v>1</v>
       </c>
+      <c r="L8" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="M8" s="4" t="s">
         <v>18</v>
       </c>
@@ -1379,13 +1352,13 @@
         <v>18</v>
       </c>
       <c r="O8" s="2">
-        <v>46300.75885622757</v>
+        <v>46300.7588562628</v>
       </c>
       <c r="P8" s="2">
-        <v>46302.79191036006</v>
+        <v>46303.38329444442</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:17" s="2" customFormat="1">
@@ -1396,13 +1369,10 @@
         <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G9" s="2">
         <v>0.9399999999999999</v>
@@ -1411,16 +1381,16 @@
         <v>46306</v>
       </c>
       <c r="I9" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="K9" s="2">
         <v>1</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -1429,13 +1399,13 @@
         <v>18</v>
       </c>
       <c r="O9" s="2">
-        <v>46300.75885624527</v>
+        <v>46300.75885627908</v>
       </c>
       <c r="P9" s="2">
-        <v>46302.79191037345</v>
+        <v>46303.38329441878</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:17" s="2" customFormat="1">
@@ -1446,31 +1416,31 @@
         <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G10" s="2">
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
       <c r="H10" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="I10" s="2">
         <v>4</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K10" s="2">
         <v>1</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="M10" s="4" t="s">
         <v>18</v>
@@ -1479,13 +1449,13 @@
         <v>18</v>
       </c>
       <c r="O10" s="2">
-        <v>46300.7588562628</v>
+        <v>46300.75884793277</v>
       </c>
       <c r="P10" s="2">
-        <v>46302.79191038655</v>
+        <v>46303.38329438417</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:17" s="2" customFormat="1">
@@ -1496,29 +1466,26 @@
         <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G11" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="H11" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="I11" s="2">
         <v>4</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K11" s="2">
         <v>1</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="M11" s="4" t="s">
         <v>18</v>
       </c>
@@ -1526,13 +1493,13 @@
         <v>18</v>
       </c>
       <c r="O11" s="2">
-        <v>46300.75885627908</v>
+        <v>46300.7588479478</v>
       </c>
       <c r="P11" s="2">
-        <v>46302.79191034697</v>
-      </c>
-      <c r="Q11" s="2" t="s">
-        <v>23</v>
+        <v>46303.38329440156</v>
+      </c>
+      <c r="Q11" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:17" s="2" customFormat="1">
@@ -1543,22 +1510,22 @@
         <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>62</v>
       </c>
       <c r="G12" s="2">
-        <v>0.88</v>
+        <v>0.93</v>
       </c>
       <c r="H12" s="3">
         <v>46307</v>
       </c>
       <c r="I12" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>63</v>
@@ -1566,9 +1533,6 @@
       <c r="K12" s="2">
         <v>1</v>
       </c>
-      <c r="L12" s="2" t="s">
-        <v>64</v>
-      </c>
       <c r="M12" s="4" t="s">
         <v>18</v>
       </c>
@@ -1576,13 +1540,13 @@
         <v>18</v>
       </c>
       <c r="O12" s="2">
-        <v>46300.75884793277</v>
+        <v>46300.75884796329</v>
       </c>
       <c r="P12" s="2">
-        <v>46302.79191029487</v>
+        <v>46303.3832943571</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:17" s="2" customFormat="1">
@@ -1593,10 +1557,10 @@
         <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G13" s="2">
         <v>0.2</v>
@@ -1605,14 +1569,17 @@
         <v>46307</v>
       </c>
       <c r="I13" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K13" s="2">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K13" s="2">
-        <v>1</v>
-      </c>
       <c r="M13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1620,13 +1587,13 @@
         <v>18</v>
       </c>
       <c r="O13" s="2">
-        <v>46300.7588479478</v>
+        <v>46300.75884799581</v>
       </c>
       <c r="P13" s="2">
-        <v>46302.79191032116</v>
+        <v>46303.38329436627</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:17" s="2" customFormat="1">
@@ -1640,19 +1607,16 @@
         <v>67</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="2" t="s">
         <v>68</v>
       </c>
       <c r="G14" s="2">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H14" s="3">
         <v>46307</v>
       </c>
       <c r="I14" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>69</v>
@@ -1667,13 +1631,13 @@
         <v>18</v>
       </c>
       <c r="O14" s="2">
-        <v>46300.75884796329</v>
+        <v>46300.75885617639</v>
       </c>
       <c r="P14" s="2">
-        <v>46302.79191025375</v>
+        <v>46303.38329433652</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:17" s="2" customFormat="1">
@@ -1687,26 +1651,26 @@
         <v>70</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G15" s="2">
-        <v>0.2</v>
+        <v>0.91</v>
       </c>
       <c r="H15" s="3">
         <v>46307</v>
       </c>
       <c r="I15" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K15" s="2">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="K15" s="2">
-        <v>1</v>
-      </c>
-      <c r="L15" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="M15" s="4" t="s">
         <v>18</v>
       </c>
@@ -1714,13 +1678,13 @@
         <v>18</v>
       </c>
       <c r="O15" s="2">
-        <v>46300.75884799581</v>
+        <v>46300.75885619673</v>
       </c>
       <c r="P15" s="2">
-        <v>46302.79191026733</v>
-      </c>
-      <c r="Q15" s="5" t="s">
-        <v>27</v>
+        <v>46303.38329437528</v>
+      </c>
+      <c r="Q15" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:17" s="2" customFormat="1">
@@ -1731,16 +1695,19 @@
         <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>74</v>
       </c>
       <c r="G16" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H16" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I16" s="2">
         <v>5</v>
@@ -1751,6 +1718,9 @@
       <c r="K16" s="2">
         <v>1</v>
       </c>
+      <c r="L16" s="2" t="s">
+        <v>76</v>
+      </c>
       <c r="M16" s="4" t="s">
         <v>18</v>
       </c>
@@ -1758,13 +1728,13 @@
         <v>18</v>
       </c>
       <c r="O16" s="2">
-        <v>46300.75885617639</v>
+        <v>46300.75884788632</v>
       </c>
       <c r="P16" s="2">
-        <v>46302.79191022492</v>
+        <v>46303.38328156831</v>
       </c>
       <c r="Q16" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:17" s="2" customFormat="1">
@@ -1775,29 +1745,26 @@
         <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G17" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H17" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I17" s="2">
         <v>5</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="K17" s="2">
         <v>1</v>
       </c>
-      <c r="L17" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="M17" s="4" t="s">
         <v>18</v>
       </c>
@@ -1805,13 +1772,13 @@
         <v>18</v>
       </c>
       <c r="O17" s="2">
-        <v>46300.75885619673</v>
+        <v>46300.75884790152</v>
       </c>
       <c r="P17" s="2">
-        <v>46302.79191028092</v>
-      </c>
-      <c r="Q17" s="2" t="s">
-        <v>23</v>
+        <v>46303.38328155963</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="2" customFormat="1">
@@ -1822,32 +1789,26 @@
         <v>18</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>80</v>
+        <v>58</v>
       </c>
       <c r="G18" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H18" s="3">
         <v>46308</v>
       </c>
       <c r="I18" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K18" s="2">
         <v>1</v>
       </c>
-      <c r="L18" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="M18" s="4" t="s">
         <v>18</v>
       </c>
@@ -1855,13 +1816,13 @@
         <v>18</v>
       </c>
       <c r="O18" s="2">
-        <v>46300.75884788632</v>
+        <v>46301.38232480602</v>
       </c>
       <c r="P18" s="2">
-        <v>46302.79189773565</v>
-      </c>
-      <c r="Q18" s="2" t="s">
-        <v>23</v>
+        <v>46303.38328155097</v>
+      </c>
+      <c r="Q18" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:17" s="2" customFormat="1">
@@ -1872,26 +1833,29 @@
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G19" s="2">
+        <v>0.92</v>
+      </c>
+      <c r="H19" s="3">
+        <v>46310</v>
+      </c>
+      <c r="I19" s="2">
+        <v>7</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G19" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="H19" s="3">
-        <v>46308</v>
-      </c>
-      <c r="I19" s="2">
-        <v>6</v>
-      </c>
-      <c r="J19" s="2" t="s">
+      <c r="K19" s="2">
+        <v>1</v>
+      </c>
+      <c r="L19" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="K19" s="2">
-        <v>1</v>
-      </c>
       <c r="M19" s="4" t="s">
         <v>18</v>
       </c>
@@ -1899,42 +1863,45 @@
         <v>18</v>
       </c>
       <c r="O19" s="2">
-        <v>46300.75884790152</v>
+        <v>46300.75884787029</v>
       </c>
       <c r="P19" s="2">
-        <v>46302.79189772235</v>
-      </c>
-      <c r="Q19" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" s="2" customFormat="1">
-      <c r="A20" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="2" t="s">
+        <v>46303.38328154255</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" t="s">
         <v>85</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0.2</v>
+      <c r="E20" t="s">
+        <v>68</v>
+      </c>
+      <c r="G20">
+        <v>0.95</v>
       </c>
       <c r="H20" s="3">
-        <v>46308</v>
-      </c>
-      <c r="I20" s="2">
-        <v>6</v>
-      </c>
-      <c r="J20" s="2" t="s">
+        <v>46312</v>
+      </c>
+      <c r="I20">
+        <v>9</v>
+      </c>
+      <c r="J20" t="s">
         <v>86</v>
       </c>
-      <c r="K20" s="2">
-        <v>1</v>
+      <c r="K20">
+        <v>1</v>
+      </c>
+      <c r="L20" t="s">
+        <v>87</v>
       </c>
       <c r="M20" s="4" t="s">
         <v>18</v>
@@ -1942,14 +1909,14 @@
       <c r="N20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O20" s="2">
-        <v>46301.38232480602</v>
-      </c>
-      <c r="P20" s="2">
-        <v>46302.79189770951</v>
-      </c>
-      <c r="Q20" s="5" t="s">
-        <v>27</v>
+      <c r="O20">
+        <v>46300.75884779022</v>
+      </c>
+      <c r="P20">
+        <v>46303.38328152523</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:17">
@@ -1960,29 +1927,26 @@
         <v>18</v>
       </c>
       <c r="C21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="G21">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="H21" s="3">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="I21">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K21">
         <v>1</v>
       </c>
-      <c r="L21" t="s">
-        <v>89</v>
-      </c>
       <c r="M21" s="4" t="s">
         <v>18</v>
       </c>
@@ -1990,13 +1954,13 @@
         <v>18</v>
       </c>
       <c r="O21">
-        <v>46300.75884787029</v>
+        <v>46300.75884780569</v>
       </c>
       <c r="P21">
-        <v>46302.79189769677</v>
+        <v>46303.38328149894</v>
       </c>
       <c r="Q21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -2007,28 +1971,28 @@
         <v>18</v>
       </c>
       <c r="C22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E22" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G22">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="H22" s="3">
         <v>46312</v>
       </c>
       <c r="I22">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J22" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="K22">
         <v>1</v>
       </c>
       <c r="L22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="M22" s="4" t="s">
         <v>18</v>
@@ -2037,13 +2001,13 @@
         <v>18</v>
       </c>
       <c r="O22">
-        <v>46300.75884779022</v>
+        <v>46300.75884782107</v>
       </c>
       <c r="P22">
-        <v>46302.79189767046</v>
+        <v>46303.38328150799</v>
       </c>
       <c r="Q22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -2054,26 +2018,29 @@
         <v>18</v>
       </c>
       <c r="C23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G23">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="H23" s="3">
         <v>46312</v>
       </c>
       <c r="I23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="K23">
         <v>1</v>
       </c>
+      <c r="L23" t="s">
+        <v>97</v>
+      </c>
       <c r="M23" s="4" t="s">
         <v>18</v>
       </c>
@@ -2081,13 +2048,13 @@
         <v>18</v>
       </c>
       <c r="O23">
-        <v>46300.75884780569</v>
+        <v>46300.75884783743</v>
       </c>
       <c r="P23">
-        <v>46302.79189763116</v>
+        <v>46303.38328151646</v>
       </c>
       <c r="Q23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -2098,28 +2065,28 @@
         <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="G24">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="H24" s="3">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="I24">
         <v>10</v>
       </c>
       <c r="J24" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="K24">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L24" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="M24" s="4" t="s">
         <v>18</v>
@@ -2128,13 +2095,13 @@
         <v>18</v>
       </c>
       <c r="O24">
-        <v>46300.75884782107</v>
+        <v>46302.26841519317</v>
       </c>
       <c r="P24">
-        <v>46302.79189764443</v>
+        <v>46303.38328149018</v>
       </c>
       <c r="Q24" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -2145,29 +2112,29 @@
         <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E25" t="s">
-        <v>100</v>
+        <v>102</v>
+      </c>
+      <c r="F25" t="s">
+        <v>103</v>
       </c>
       <c r="G25">
-        <v>0.91</v>
+        <v>0.96</v>
       </c>
       <c r="H25" s="3">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="I25">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J25" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
-      <c r="L25" t="s">
-        <v>102</v>
-      </c>
       <c r="M25" s="4" t="s">
         <v>18</v>
       </c>
@@ -2175,13 +2142,13 @@
         <v>18</v>
       </c>
       <c r="O25">
-        <v>46300.75884783743</v>
+        <v>46300.75884774033</v>
       </c>
       <c r="P25">
-        <v>46302.79189765739</v>
+        <v>46303.38328147282</v>
       </c>
       <c r="Q25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2192,28 +2159,25 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E26" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="G26">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H26" s="3">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="I26">
         <v>11</v>
       </c>
       <c r="J26" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="K26">
-        <v>3</v>
-      </c>
-      <c r="L26" t="s">
-        <v>105</v>
+        <v>1</v>
       </c>
       <c r="M26" s="4" t="s">
         <v>18</v>
@@ -2222,13 +2186,13 @@
         <v>18</v>
       </c>
       <c r="O26">
-        <v>46302.26841519317</v>
+        <v>46300.75884775587</v>
       </c>
       <c r="P26">
-        <v>46302.79189761808</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>23</v>
+        <v>46303.38328148136</v>
+      </c>
+      <c r="Q26" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -2239,25 +2203,22 @@
         <v>18</v>
       </c>
       <c r="C27" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E27" t="s">
-        <v>107</v>
-      </c>
-      <c r="F27" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="G27">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="H27" s="3">
         <v>46314</v>
       </c>
       <c r="I27">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J27" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K27">
         <v>1</v>
@@ -2269,13 +2230,13 @@
         <v>18</v>
       </c>
       <c r="O27">
-        <v>46300.75884774033</v>
+        <v>46300.7588477715</v>
       </c>
       <c r="P27">
-        <v>46302.79189759048</v>
+        <v>46303.38328146389</v>
       </c>
       <c r="Q27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -2286,22 +2247,22 @@
         <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E28" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G28">
         <v>0.2</v>
       </c>
       <c r="H28" s="3">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="I28">
         <v>12</v>
       </c>
       <c r="J28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K28">
         <v>1</v>
@@ -2313,13 +2274,13 @@
         <v>18</v>
       </c>
       <c r="O28">
-        <v>46300.75884775587</v>
+        <v>46300.75884772457</v>
       </c>
       <c r="P28">
-        <v>46302.79189760437</v>
+        <v>46303.38328145499</v>
       </c>
       <c r="Q28" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -2330,26 +2291,29 @@
         <v>18</v>
       </c>
       <c r="C29" t="s">
+        <v>111</v>
+      </c>
+      <c r="E29" t="s">
+        <v>58</v>
+      </c>
+      <c r="G29">
+        <v>0.2</v>
+      </c>
+      <c r="H29" s="3">
+        <v>46316</v>
+      </c>
+      <c r="I29">
+        <v>13</v>
+      </c>
+      <c r="J29" t="s">
+        <v>27</v>
+      </c>
+      <c r="K29">
+        <v>3</v>
+      </c>
+      <c r="L29" t="s">
         <v>112</v>
       </c>
-      <c r="E29" t="s">
-        <v>94</v>
-      </c>
-      <c r="G29">
-        <v>0.93</v>
-      </c>
-      <c r="H29" s="3">
-        <v>46314</v>
-      </c>
-      <c r="I29">
-        <v>12</v>
-      </c>
-      <c r="J29" t="s">
-        <v>113</v>
-      </c>
-      <c r="K29">
-        <v>1</v>
-      </c>
       <c r="M29" s="4" t="s">
         <v>18</v>
       </c>
@@ -2357,13 +2321,13 @@
         <v>18</v>
       </c>
       <c r="O29">
-        <v>46300.7588477715</v>
+        <v>46302.26841507768</v>
       </c>
       <c r="P29">
-        <v>46302.79189757702</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>23</v>
+        <v>46303.38328143695</v>
+      </c>
+      <c r="Q29" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2374,22 +2338,22 @@
         <v>18</v>
       </c>
       <c r="C30" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E30" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G30">
         <v>0.2</v>
       </c>
       <c r="H30" s="3">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="I30">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K30">
         <v>1</v>
@@ -2401,13 +2365,13 @@
         <v>18</v>
       </c>
       <c r="O30">
-        <v>46300.75884772457</v>
+        <v>46301.38232468421</v>
       </c>
       <c r="P30">
-        <v>46302.79189756404</v>
+        <v>46303.3832814277</v>
       </c>
       <c r="Q30" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -2418,28 +2382,28 @@
         <v>18</v>
       </c>
       <c r="C31" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E31" t="s">
-        <v>25</v>
+        <v>20</v>
+      </c>
+      <c r="F31" t="s">
+        <v>40</v>
       </c>
       <c r="G31">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H31" s="3">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="I31">
         <v>14</v>
       </c>
       <c r="J31" t="s">
-        <v>35</v>
+        <v>116</v>
       </c>
       <c r="K31">
-        <v>3</v>
-      </c>
-      <c r="L31" t="s">
-        <v>117</v>
+        <v>1</v>
       </c>
       <c r="M31" s="4" t="s">
         <v>18</v>
@@ -2448,13 +2412,13 @@
         <v>18</v>
       </c>
       <c r="O31">
-        <v>46302.26841507768</v>
+        <v>46302.26841501552</v>
       </c>
       <c r="P31">
-        <v>46302.79189753801</v>
-      </c>
-      <c r="Q31" s="5" t="s">
-        <v>27</v>
+        <v>46303.38328141814</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -2465,149 +2429,154 @@
         <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E32" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G32">
         <v>0.2</v>
       </c>
       <c r="H32" s="3">
-        <v>46317</v>
+        <v>46326</v>
       </c>
       <c r="I32">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J32" t="s">
+        <v>118</v>
+      </c>
+      <c r="K32">
+        <v>1</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N32" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O32">
+        <v>46300.75884768533</v>
+      </c>
+      <c r="P32">
+        <v>46303.38328140793</v>
+      </c>
+      <c r="Q32" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
+      <c r="A33" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="K32">
-        <v>1</v>
-      </c>
-      <c r="M32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O32">
-        <v>46301.38232468421</v>
-      </c>
-      <c r="P32">
-        <v>46302.79189752453</v>
-      </c>
-      <c r="Q32" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17">
-      <c r="A33" t="s">
-        <v>18</v>
-      </c>
-      <c r="B33" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B33" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E33" t="s">
-        <v>29</v>
-      </c>
-      <c r="F33" t="s">
-        <v>48</v>
-      </c>
-      <c r="G33">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="H33" s="3">
-        <v>46317</v>
-      </c>
-      <c r="I33">
-        <v>15</v>
-      </c>
-      <c r="J33" t="s">
+      <c r="C33" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="K33">
-        <v>1</v>
-      </c>
-      <c r="M33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O33">
-        <v>46302.26841501552</v>
-      </c>
-      <c r="P33">
-        <v>46302.79189751096</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>23</v>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6">
+        <v>0.92</v>
+      </c>
+      <c r="H33" s="6">
+        <v>46302</v>
+      </c>
+      <c r="I33" s="6">
+        <v>-1</v>
+      </c>
+      <c r="J33" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="K33" s="6">
+        <v>1</v>
+      </c>
+      <c r="L33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N33" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O33" s="6">
+        <v>46300.7588564394</v>
+      </c>
+      <c r="P33" s="6">
+        <v>46303.38330297283</v>
+      </c>
+      <c r="Q33" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:17">
-      <c r="A34" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" t="s">
-        <v>18</v>
-      </c>
-      <c r="C34" t="s">
-        <v>122</v>
-      </c>
-      <c r="E34" t="s">
-        <v>25</v>
-      </c>
-      <c r="G34">
+      <c r="A34" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6">
         <v>0.2</v>
       </c>
-      <c r="H34" s="3">
-        <v>46326</v>
-      </c>
-      <c r="I34">
-        <v>24</v>
-      </c>
-      <c r="J34" t="s">
-        <v>123</v>
-      </c>
-      <c r="K34">
-        <v>1</v>
-      </c>
-      <c r="M34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O34">
-        <v>46300.75884768533</v>
-      </c>
-      <c r="P34">
-        <v>46302.79189749651</v>
+      <c r="H34" s="6">
+        <v>46302</v>
+      </c>
+      <c r="I34" s="6">
+        <v>-1</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="K34" s="6">
+        <v>1</v>
+      </c>
+      <c r="L34" s="6"/>
+      <c r="M34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O34" s="6">
+        <v>46300.75885647022</v>
+      </c>
+      <c r="P34" s="6">
+        <v>46303.38330298233</v>
       </c>
       <c r="Q34" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:17">
       <c r="A35" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>126</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="G35" s="6">
         <v>0.9399999999999999</v>
@@ -2616,7 +2585,7 @@
         <v>46301</v>
       </c>
       <c r="I35" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="J35" s="6" t="s">
         <v>127</v>
@@ -2635,18 +2604,18 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P35" s="6">
-        <v>46302.79192102975</v>
+        <v>46303.38330300884</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="36" spans="1:17">
       <c r="A36" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>128</v>
@@ -2663,7 +2632,7 @@
         <v>46300</v>
       </c>
       <c r="I36" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="J36" s="6" t="s">
         <v>130</v>
@@ -2682,28 +2651,28 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P36" s="6">
-        <v>46302.79192108147</v>
+        <v>46303.38330304309</v>
       </c>
       <c r="Q36" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>131</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G37" s="6">
         <v>0.93</v>
@@ -2712,7 +2681,7 @@
         <v>46300</v>
       </c>
       <c r="I37" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="J37" s="6" t="s">
         <v>132</v>
@@ -2731,25 +2700,25 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P37" s="6">
-        <v>46302.79192105515</v>
+        <v>46303.3833030263</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>133</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6">
@@ -2759,10 +2728,10 @@
         <v>46299</v>
       </c>
       <c r="I38" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="K38" s="6">
         <v>1</v>
@@ -2780,28 +2749,28 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P38" s="6">
-        <v>46302.79192109437</v>
+        <v>46303.38330305153</v>
       </c>
       <c r="Q38" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>135</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G39" s="6">
         <v>0.93</v>
@@ -2810,7 +2779,7 @@
         <v>46299</v>
       </c>
       <c r="I39" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J39" s="6" t="s">
         <v>136</v>
@@ -2829,25 +2798,25 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P39" s="6">
-        <v>46302.79192110736</v>
+        <v>46303.38330306018</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>137</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6">
@@ -2857,7 +2826,7 @@
         <v>46298</v>
       </c>
       <c r="I40" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J40" s="6" t="s">
         <v>138</v>
@@ -2876,28 +2845,28 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P40" s="6">
-        <v>46302.79192113371</v>
+        <v>46303.38330307746</v>
       </c>
       <c r="Q40" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" spans="1:17">
       <c r="A41" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G41" s="6">
         <v>0.9399999999999999</v>
@@ -2906,7 +2875,7 @@
         <v>46298</v>
       </c>
       <c r="I41" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J41" s="6" t="s">
         <v>140</v>
@@ -2925,18 +2894,18 @@
         <v>46300.75886472998</v>
       </c>
       <c r="P41" s="6">
-        <v>46302.79193306002</v>
+        <v>46303.38331249326</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>141</v>
@@ -2953,7 +2922,7 @@
         <v>46298</v>
       </c>
       <c r="I42" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J42" s="6" t="s">
         <v>143</v>
@@ -2974,25 +2943,25 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P42" s="6">
-        <v>46302.79192114654</v>
+        <v>46303.38330308611</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>145</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6">
@@ -3002,7 +2971,7 @@
         <v>46298</v>
       </c>
       <c r="I43" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J43" s="6" t="s">
         <v>146</v>
@@ -3021,28 +2990,28 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P43" s="6">
-        <v>46302.79192121145</v>
+        <v>46303.38330312896</v>
       </c>
       <c r="Q43" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>147</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="G44" s="6">
         <v>0.93</v>
@@ -3051,10 +3020,10 @@
         <v>46298</v>
       </c>
       <c r="I44" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="K44" s="6">
         <v>1</v>
@@ -3072,18 +3041,18 @@
         <v>46300.75886484625</v>
       </c>
       <c r="P44" s="6">
-        <v>46302.79192117266</v>
+        <v>46303.38330310328</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:17">
       <c r="A45" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>149</v>
@@ -3100,7 +3069,7 @@
         <v>46297</v>
       </c>
       <c r="I45" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J45" s="6" t="s">
         <v>150</v>
@@ -3121,25 +3090,25 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P45" s="6">
-        <v>46302.79193307317</v>
+        <v>46303.38331250347</v>
       </c>
       <c r="Q45" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="46" spans="1:17">
       <c r="A46" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>152</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="6">
@@ -3149,7 +3118,7 @@
         <v>46296</v>
       </c>
       <c r="I46" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J46" s="6" t="s">
         <v>153</v>
@@ -3170,25 +3139,25 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P46" s="6">
-        <v>46302.79193308652</v>
+        <v>46303.3833125137</v>
       </c>
       <c r="Q46" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:17">
       <c r="A47" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>155</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6">
@@ -3198,7 +3167,7 @@
         <v>46294</v>
       </c>
       <c r="I47" s="6">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="J47" s="6" t="s">
         <v>156</v>
@@ -3217,25 +3186,25 @@
         <v>46300.75887301003</v>
       </c>
       <c r="P47" s="6">
-        <v>46302.79193312495</v>
+        <v>46303.38331254272</v>
       </c>
       <c r="Q47" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="1:17">
       <c r="A48" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>157</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6">
@@ -3245,7 +3214,7 @@
         <v>46294</v>
       </c>
       <c r="I48" s="6">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="J48" s="6" t="s">
         <v>158</v>
@@ -3264,18 +3233,18 @@
         <v>46300.75887304553</v>
       </c>
       <c r="P48" s="6">
-        <v>46302.79193313776</v>
+        <v>46303.38331255232</v>
       </c>
       <c r="Q48" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="49" spans="1:17">
       <c r="A49" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>159</v>
@@ -3292,7 +3261,7 @@
         <v>46294</v>
       </c>
       <c r="I49" s="6">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="J49" s="6" t="s">
         <v>161</v>
@@ -3311,25 +3280,25 @@
         <v>46300.75887306096</v>
       </c>
       <c r="P49" s="6">
-        <v>46302.79193315036</v>
+        <v>46303.38331256139</v>
       </c>
       <c r="Q49" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>162</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
-        <v>20</v>
+        <v>82</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6">
@@ -3339,7 +3308,7 @@
         <v>46293</v>
       </c>
       <c r="I50" s="6">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="J50" s="6" t="s">
         <v>163</v>
@@ -3360,255 +3329,14 @@
         <v>46300.75887309557</v>
       </c>
       <c r="P50" s="6">
-        <v>46302.79193318906</v>
+        <v>46303.38331258995</v>
       </c>
       <c r="Q50" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="51" spans="1:17">
-      <c r="A51" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D51" s="6"/>
-      <c r="E51" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F51" s="6"/>
-      <c r="G51" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H51" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I51" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J51" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="K51" s="6">
-        <v>1</v>
-      </c>
-      <c r="L51" s="6"/>
-      <c r="M51" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N51" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O51" s="6">
-        <v>46300.75887314334</v>
-      </c>
-      <c r="P51" s="6">
-        <v>46302.7919332146</v>
-      </c>
-      <c r="Q51" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="52" spans="1:17">
-      <c r="A52" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="D52" s="6"/>
-      <c r="E52" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="F52" s="6"/>
-      <c r="G52" s="6">
-        <v>0.87</v>
-      </c>
-      <c r="H52" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I52" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J52" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="K52" s="6">
-        <v>3</v>
-      </c>
-      <c r="L52" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="M52" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N52" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O52" s="6">
-        <v>46300.75887316054</v>
-      </c>
-      <c r="P52" s="6">
-        <v>46302.79193322792</v>
-      </c>
-      <c r="Q52" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="53" spans="1:17">
-      <c r="A53" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F53" s="6"/>
-      <c r="G53" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H53" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I53" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J53" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="K53" s="6">
-        <v>1</v>
-      </c>
-      <c r="L53" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="M53" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N53" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O53" s="6">
-        <v>46300.75887317812</v>
-      </c>
-      <c r="P53" s="6">
-        <v>46302.79193325419</v>
-      </c>
-      <c r="Q53" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="54" spans="1:17">
-      <c r="A54" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H54" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I54" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J54" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="K54" s="6">
-        <v>1</v>
-      </c>
-      <c r="L54" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="M54" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N54" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O54" s="6">
-        <v>46300.75887319581</v>
-      </c>
-      <c r="P54" s="6">
-        <v>46302.79193324078</v>
-      </c>
-      <c r="Q54" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="55" spans="1:17">
-      <c r="A55" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B55" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D55" s="6"/>
-      <c r="E55" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F55" s="6"/>
-      <c r="G55" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H55" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I55" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J55" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="K55" s="6">
-        <v>2</v>
-      </c>
-      <c r="L55" s="6"/>
-      <c r="M55" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N55" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O55" s="6">
-        <v>46300.75887321083</v>
-      </c>
-      <c r="P55" s="6">
-        <v>46302.79193320179</v>
-      </c>
-      <c r="Q55" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q55"/>
+  <autoFilter ref="A1:Q50"/>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1"/>
     <hyperlink ref="N2" r:id="rId2"/>
@@ -3708,16 +3436,6 @@
     <hyperlink ref="N49" r:id="rId96"/>
     <hyperlink ref="M50" r:id="rId97"/>
     <hyperlink ref="N50" r:id="rId98"/>
-    <hyperlink ref="M51" r:id="rId99"/>
-    <hyperlink ref="N51" r:id="rId100"/>
-    <hyperlink ref="M52" r:id="rId101"/>
-    <hyperlink ref="N52" r:id="rId102"/>
-    <hyperlink ref="M53" r:id="rId103"/>
-    <hyperlink ref="N53" r:id="rId104"/>
-    <hyperlink ref="M54" r:id="rId105"/>
-    <hyperlink ref="N54" r:id="rId106"/>
-    <hyperlink ref="M55" r:id="rId107"/>
-    <hyperlink ref="N55" r:id="rId108"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3725,7 +3443,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3804,22 +3522,22 @@
         <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G2" s="2">
         <v>0.2</v>
       </c>
       <c r="H2" s="3">
-        <v>46302</v>
+        <v>46307</v>
       </c>
       <c r="I2" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="K2" s="2">
         <v>1</v>
@@ -3831,13 +3549,13 @@
         <v>18</v>
       </c>
       <c r="O2" s="2">
-        <v>46300.75885647022</v>
+        <v>46300.7588479478</v>
       </c>
       <c r="P2" s="2">
-        <v>46302.79192099054</v>
+        <v>46303.38329440156</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="2" customFormat="1">
@@ -3848,10 +3566,10 @@
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G3" s="2">
         <v>0.2</v>
@@ -3860,14 +3578,17 @@
         <v>46307</v>
       </c>
       <c r="I3" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K3" s="2">
-        <v>1</v>
-      </c>
       <c r="M3" s="4" t="s">
         <v>18</v>
       </c>
@@ -3875,13 +3596,13 @@
         <v>18</v>
       </c>
       <c r="O3" s="2">
-        <v>46300.7588479478</v>
+        <v>46300.75884799581</v>
       </c>
       <c r="P3" s="2">
-        <v>46302.79191032116</v>
+        <v>46303.38329436627</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1">
@@ -3892,29 +3613,26 @@
         <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G4" s="2">
         <v>0.2</v>
       </c>
       <c r="H4" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I4" s="2">
         <v>5</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="K4" s="2">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="M4" s="4" t="s">
         <v>18</v>
       </c>
@@ -3922,13 +3640,13 @@
         <v>18</v>
       </c>
       <c r="O4" s="2">
-        <v>46300.75884799581</v>
+        <v>46300.75884790152</v>
       </c>
       <c r="P4" s="2">
-        <v>46302.79191026733</v>
+        <v>46303.38328155963</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="2" customFormat="1">
@@ -3939,10 +3657,10 @@
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G5" s="2">
         <v>0.2</v>
@@ -3951,10 +3669,10 @@
         <v>46308</v>
       </c>
       <c r="I5" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="K5" s="2">
         <v>1</v>
@@ -3966,41 +3684,41 @@
         <v>18</v>
       </c>
       <c r="O5" s="2">
-        <v>46300.75884790152</v>
+        <v>46301.38232480602</v>
       </c>
       <c r="P5" s="2">
-        <v>46302.79189772235</v>
+        <v>46303.38328155097</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" s="2" customFormat="1">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6">
         <v>0.2</v>
       </c>
       <c r="H6" s="3">
-        <v>46308</v>
-      </c>
-      <c r="I6" s="2">
-        <v>6</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="K6" s="2">
+        <v>46314</v>
+      </c>
+      <c r="I6">
+        <v>11</v>
+      </c>
+      <c r="J6" t="s">
+        <v>106</v>
+      </c>
+      <c r="K6">
         <v>1</v>
       </c>
       <c r="M6" s="4" t="s">
@@ -4009,14 +3727,14 @@
       <c r="N6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O6" s="2">
-        <v>46301.38232480602</v>
-      </c>
-      <c r="P6" s="2">
-        <v>46302.79189770951</v>
+      <c r="O6">
+        <v>46300.75884775587</v>
+      </c>
+      <c r="P6">
+        <v>46303.38328148136</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -4027,22 +3745,22 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G7">
         <v>0.2</v>
       </c>
       <c r="H7" s="3">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="I7">
         <v>12</v>
       </c>
       <c r="J7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -4054,13 +3772,13 @@
         <v>18</v>
       </c>
       <c r="O7">
-        <v>46300.75884775587</v>
+        <v>46300.75884772457</v>
       </c>
       <c r="P7">
-        <v>46302.79189760437</v>
+        <v>46303.38328145499</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -4071,25 +3789,28 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" s="3">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="I8">
         <v>13</v>
       </c>
       <c r="J8" t="s">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L8" t="s">
+        <v>112</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>18</v>
@@ -4098,13 +3819,13 @@
         <v>18</v>
       </c>
       <c r="O8">
-        <v>46300.75884772457</v>
+        <v>46302.26841507768</v>
       </c>
       <c r="P8">
-        <v>46302.79189756404</v>
+        <v>46303.38328143695</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -4115,28 +3836,25 @@
         <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G9">
         <v>0.2</v>
       </c>
       <c r="H9" s="3">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="I9">
         <v>14</v>
       </c>
       <c r="J9" t="s">
-        <v>35</v>
+        <v>114</v>
       </c>
       <c r="K9">
-        <v>3</v>
-      </c>
-      <c r="L9" t="s">
-        <v>117</v>
+        <v>1</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -4145,13 +3863,13 @@
         <v>18</v>
       </c>
       <c r="O9">
-        <v>46302.26841507768</v>
+        <v>46301.38232468421</v>
       </c>
       <c r="P9">
-        <v>46302.79189753801</v>
+        <v>46303.3832814277</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -4162,99 +3880,102 @@
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="G10">
         <v>0.2</v>
       </c>
       <c r="H10" s="3">
-        <v>46317</v>
+        <v>46326</v>
       </c>
       <c r="I10">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J10" t="s">
+        <v>118</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O10">
+        <v>46300.75884768533</v>
+      </c>
+      <c r="P10">
+        <v>46303.38328140793</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O10">
-        <v>46301.38232468421</v>
-      </c>
-      <c r="P10">
-        <v>46302.79189752453</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
-        <v>122</v>
-      </c>
-      <c r="E11" t="s">
-        <v>25</v>
-      </c>
-      <c r="G11">
+      <c r="B11" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6">
         <v>0.2</v>
       </c>
-      <c r="H11" s="3">
-        <v>46326</v>
-      </c>
-      <c r="I11">
-        <v>24</v>
-      </c>
-      <c r="J11" t="s">
-        <v>123</v>
-      </c>
-      <c r="K11">
-        <v>1</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O11">
-        <v>46300.75884768533</v>
-      </c>
-      <c r="P11">
-        <v>46302.79189749651</v>
+      <c r="H11" s="6">
+        <v>46302</v>
+      </c>
+      <c r="I11" s="6">
+        <v>-1</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="K11" s="6">
+        <v>1</v>
+      </c>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O11" s="6">
+        <v>46300.75885647022</v>
+      </c>
+      <c r="P11" s="6">
+        <v>46303.38330298233</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>133</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6">
@@ -4264,10 +3985,10 @@
         <v>46299</v>
       </c>
       <c r="I12" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="K12" s="6">
         <v>1</v>
@@ -4285,25 +4006,25 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P12" s="6">
-        <v>46302.79192109437</v>
+        <v>46303.38330305153</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>137</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6">
@@ -4313,7 +4034,7 @@
         <v>46298</v>
       </c>
       <c r="I13" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>138</v>
@@ -4332,25 +4053,25 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P13" s="6">
-        <v>46302.79192113371</v>
+        <v>46303.38330307746</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>145</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6">
@@ -4360,7 +4081,7 @@
         <v>46298</v>
       </c>
       <c r="I14" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>146</v>
@@ -4379,25 +4100,25 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P14" s="6">
-        <v>46302.79192121145</v>
+        <v>46303.38330312896</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>152</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6">
@@ -4407,7 +4128,7 @@
         <v>46296</v>
       </c>
       <c r="I15" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>153</v>
@@ -4428,25 +4149,25 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P15" s="6">
-        <v>46302.79193308652</v>
+        <v>46303.3833125137</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>155</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>25</v>
+        <v>58</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6">
@@ -4456,7 +4177,7 @@
         <v>46294</v>
       </c>
       <c r="I16" s="6">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>156</v>
@@ -4475,206 +4196,14 @@
         <v>46300.75887301003</v>
       </c>
       <c r="P16" s="6">
-        <v>46302.79193312495</v>
+        <v>46303.38331254272</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
-      <c r="A17" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F17" s="6"/>
-      <c r="G17" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H17" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I17" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="K17" s="6">
-        <v>1</v>
-      </c>
-      <c r="L17" s="6"/>
-      <c r="M17" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N17" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O17" s="6">
-        <v>46300.75887314334</v>
-      </c>
-      <c r="P17" s="6">
-        <v>46302.7919332146</v>
-      </c>
-      <c r="Q17" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17">
-      <c r="A18" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H18" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I18" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="K18" s="6">
-        <v>1</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O18" s="6">
-        <v>46300.75887317812</v>
-      </c>
-      <c r="P18" s="6">
-        <v>46302.79193325419</v>
-      </c>
-      <c r="Q18" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17">
-      <c r="A19" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" s="6"/>
-      <c r="G19" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H19" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I19" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="K19" s="6">
-        <v>1</v>
-      </c>
-      <c r="L19" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O19" s="6">
-        <v>46300.75887319581</v>
-      </c>
-      <c r="P19" s="6">
-        <v>46302.79193324078</v>
-      </c>
-      <c r="Q19" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17">
-      <c r="A20" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F20" s="6"/>
-      <c r="G20" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H20" s="6">
-        <v>46292</v>
-      </c>
-      <c r="I20" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="K20" s="6">
-        <v>2</v>
-      </c>
-      <c r="L20" s="6"/>
-      <c r="M20" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N20" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O20" s="6">
-        <v>46300.75887321083</v>
-      </c>
-      <c r="P20" s="6">
-        <v>46302.79193320179</v>
-      </c>
-      <c r="Q20" s="5" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q20"/>
+  <autoFilter ref="A1:Q16"/>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1"/>
     <hyperlink ref="N2" r:id="rId2"/>
@@ -4706,14 +4235,6 @@
     <hyperlink ref="N15" r:id="rId28"/>
     <hyperlink ref="M16" r:id="rId29"/>
     <hyperlink ref="N16" r:id="rId30"/>
-    <hyperlink ref="M17" r:id="rId31"/>
-    <hyperlink ref="N17" r:id="rId32"/>
-    <hyperlink ref="M18" r:id="rId33"/>
-    <hyperlink ref="N18" r:id="rId34"/>
-    <hyperlink ref="M19" r:id="rId35"/>
-    <hyperlink ref="N19" r:id="rId36"/>
-    <hyperlink ref="M20" r:id="rId37"/>
-    <hyperlink ref="N20" r:id="rId38"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4721,7 +4242,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4731,51 +4252,51 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B2">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C2" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D2">
         <v>191</v>
@@ -4787,7 +4308,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -4804,13 +4325,13 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B3">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C3" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D3">
         <v>191</v>
@@ -4819,16 +4340,16 @@
         <v>3820</v>
       </c>
       <c r="F3">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H3">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -4839,48 +4360,48 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B4">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C4" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D4">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E4">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G4">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H4">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B5">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C5" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D5">
         <v>8</v>
@@ -4889,13 +4410,13 @@
         <v>160</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -4904,18 +4425,18 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B6">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C6" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D6">
         <v>8</v>
@@ -4924,21 +4445,56 @@
         <v>160</v>
       </c>
       <c r="F6">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H6">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B7">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C7" t="s">
+        <v>176</v>
+      </c>
+      <c r="D7">
+        <v>8</v>
+      </c>
+      <c r="E7">
+        <v>160</v>
+      </c>
+      <c r="F7">
+        <v>157</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+      <c r="H7">
+        <v>132</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-08-1858Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="177">
   <si>
     <t>Priority</t>
   </si>
@@ -1070,7 +1070,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P2" s="2">
-        <v>46303.38329450462</v>
+        <v>46303.78903324551</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>24</v>
@@ -1114,7 +1114,7 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P3" s="2">
-        <v>46303.3832944789</v>
+        <v>46303.78903320204</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>24</v>
@@ -1161,7 +1161,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P4" s="2">
-        <v>46303.38329448765</v>
+        <v>46303.78903321669</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>24</v>
@@ -1208,7 +1208,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P5" s="2">
-        <v>46303.38329446202</v>
+        <v>46303.78903317315</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>24</v>
@@ -1255,7 +1255,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P6" s="2">
-        <v>46303.38329442757</v>
+        <v>46303.78903311479</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>24</v>
@@ -1305,7 +1305,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P7" s="2">
-        <v>46303.38329443617</v>
+        <v>46303.78903312911</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>24</v>
@@ -1355,7 +1355,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P8" s="2">
-        <v>46303.38329444442</v>
+        <v>46303.78903314354</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>24</v>
@@ -1402,7 +1402,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P9" s="2">
-        <v>46303.38329441878</v>
+        <v>46303.78903310001</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>24</v>
@@ -1452,7 +1452,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P10" s="2">
-        <v>46303.38329438417</v>
+        <v>46303.78903304238</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>24</v>
@@ -1496,7 +1496,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P11" s="2">
-        <v>46303.38329440156</v>
+        <v>46303.78903307128</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>60</v>
@@ -1543,7 +1543,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P12" s="2">
-        <v>46303.3832943571</v>
+        <v>46303.7890329982</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>24</v>
@@ -1590,7 +1590,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P13" s="2">
-        <v>46303.38329436627</v>
+        <v>46303.78903301315</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>60</v>
@@ -1634,7 +1634,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P14" s="2">
-        <v>46303.38329433652</v>
+        <v>46303.78903296705</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>24</v>
@@ -1681,7 +1681,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P15" s="2">
-        <v>46303.38329437528</v>
+        <v>46303.78903302801</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>24</v>
@@ -1731,7 +1731,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P16" s="2">
-        <v>46303.38328156831</v>
+        <v>46303.78902500809</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>24</v>
@@ -1775,7 +1775,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P17" s="2">
-        <v>46303.38328155963</v>
+        <v>46303.78902499317</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>60</v>
@@ -1819,7 +1819,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P18" s="2">
-        <v>46303.38328155097</v>
+        <v>46303.78902497852</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>60</v>
@@ -1866,7 +1866,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P19" s="2">
-        <v>46303.38328154255</v>
+        <v>46303.78902496338</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>24</v>
@@ -1913,7 +1913,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P20">
-        <v>46303.38328152523</v>
+        <v>46303.78902493456</v>
       </c>
       <c r="Q20" t="s">
         <v>24</v>
@@ -1957,7 +1957,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P21">
-        <v>46303.38328149894</v>
+        <v>46303.78902489004</v>
       </c>
       <c r="Q21" t="s">
         <v>24</v>
@@ -2004,7 +2004,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P22">
-        <v>46303.38328150799</v>
+        <v>46303.78902490489</v>
       </c>
       <c r="Q22" t="s">
         <v>24</v>
@@ -2051,7 +2051,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P23">
-        <v>46303.38328151646</v>
+        <v>46303.78902491984</v>
       </c>
       <c r="Q23" t="s">
         <v>24</v>
@@ -2098,7 +2098,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P24">
-        <v>46303.38328149018</v>
+        <v>46303.78902487514</v>
       </c>
       <c r="Q24" t="s">
         <v>24</v>
@@ -2145,7 +2145,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P25">
-        <v>46303.38328147282</v>
+        <v>46303.78902484559</v>
       </c>
       <c r="Q25" t="s">
         <v>24</v>
@@ -2189,7 +2189,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P26">
-        <v>46303.38328148136</v>
+        <v>46303.7890248602</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>60</v>
@@ -2233,7 +2233,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P27">
-        <v>46303.38328146389</v>
+        <v>46303.78902483075</v>
       </c>
       <c r="Q27" t="s">
         <v>24</v>
@@ -2277,7 +2277,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P28">
-        <v>46303.38328145499</v>
+        <v>46303.78902481608</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>60</v>
@@ -2324,7 +2324,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P29">
-        <v>46303.38328143695</v>
+        <v>46303.78902478614</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>60</v>
@@ -2368,7 +2368,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P30">
-        <v>46303.3832814277</v>
+        <v>46303.7890247705</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>60</v>
@@ -2415,7 +2415,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P31">
-        <v>46303.38328141814</v>
+        <v>46303.78902475473</v>
       </c>
       <c r="Q31" t="s">
         <v>24</v>
@@ -2459,7 +2459,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P32">
-        <v>46303.38328140793</v>
+        <v>46303.78902473875</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>60</v>
@@ -2508,7 +2508,7 @@
         <v>46300.7588564394</v>
       </c>
       <c r="P33" s="6">
-        <v>46303.38330297283</v>
+        <v>46303.78904116363</v>
       </c>
       <c r="Q33" s="6" t="s">
         <v>24</v>
@@ -2555,7 +2555,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P34" s="6">
-        <v>46303.38330298233</v>
+        <v>46303.78904117852</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>60</v>
@@ -2604,7 +2604,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P35" s="6">
-        <v>46303.38330300884</v>
+        <v>46303.78904122258</v>
       </c>
       <c r="Q35" s="6" t="s">
         <v>24</v>
@@ -2651,7 +2651,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P36" s="6">
-        <v>46303.38330304309</v>
+        <v>46303.7890412799</v>
       </c>
       <c r="Q36" s="6" t="s">
         <v>24</v>
@@ -2700,7 +2700,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P37" s="6">
-        <v>46303.3833030263</v>
+        <v>46303.78904125095</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>24</v>
@@ -2749,7 +2749,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P38" s="6">
-        <v>46303.38330305153</v>
+        <v>46303.78904129434</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>60</v>
@@ -2798,7 +2798,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P39" s="6">
-        <v>46303.38330306018</v>
+        <v>46303.78904130949</v>
       </c>
       <c r="Q39" s="6" t="s">
         <v>24</v>
@@ -2845,7 +2845,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P40" s="6">
-        <v>46303.38330307746</v>
+        <v>46303.7890413381</v>
       </c>
       <c r="Q40" s="5" t="s">
         <v>60</v>
@@ -2894,7 +2894,7 @@
         <v>46300.75886472998</v>
       </c>
       <c r="P41" s="6">
-        <v>46303.38331249326</v>
+        <v>46303.78904942831</v>
       </c>
       <c r="Q41" s="6" t="s">
         <v>24</v>
@@ -2943,7 +2943,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P42" s="6">
-        <v>46303.38330308611</v>
+        <v>46303.78904135231</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>24</v>
@@ -2990,7 +2990,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P43" s="6">
-        <v>46303.38330312896</v>
+        <v>46303.78904142418</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>60</v>
@@ -3041,7 +3041,7 @@
         <v>46300.75886484625</v>
       </c>
       <c r="P44" s="6">
-        <v>46303.38330310328</v>
+        <v>46303.78904138121</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>24</v>
@@ -3090,7 +3090,7 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P45" s="6">
-        <v>46303.38331250347</v>
+        <v>46303.78904944336</v>
       </c>
       <c r="Q45" s="6" t="s">
         <v>24</v>
@@ -3139,7 +3139,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P46" s="6">
-        <v>46303.3833125137</v>
+        <v>46303.78904946196</v>
       </c>
       <c r="Q46" s="5" t="s">
         <v>60</v>
@@ -3186,7 +3186,7 @@
         <v>46300.75887301003</v>
       </c>
       <c r="P47" s="6">
-        <v>46303.38331254272</v>
+        <v>46303.78904952588</v>
       </c>
       <c r="Q47" s="5" t="s">
         <v>60</v>
@@ -3233,7 +3233,7 @@
         <v>46300.75887304553</v>
       </c>
       <c r="P48" s="6">
-        <v>46303.38331255232</v>
+        <v>46303.78904954536</v>
       </c>
       <c r="Q48" s="6" t="s">
         <v>24</v>
@@ -3280,7 +3280,7 @@
         <v>46300.75887306096</v>
       </c>
       <c r="P49" s="6">
-        <v>46303.38331256139</v>
+        <v>46303.7890495669</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>24</v>
@@ -3329,7 +3329,7 @@
         <v>46300.75887309557</v>
       </c>
       <c r="P50" s="6">
-        <v>46303.38331258995</v>
+        <v>46303.78904962536</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>24</v>
@@ -3552,7 +3552,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P2" s="2">
-        <v>46303.38329440156</v>
+        <v>46303.78903307128</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>60</v>
@@ -3599,7 +3599,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P3" s="2">
-        <v>46303.38329436627</v>
+        <v>46303.78903301315</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>60</v>
@@ -3643,7 +3643,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P4" s="2">
-        <v>46303.38328155963</v>
+        <v>46303.78902499317</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>60</v>
@@ -3687,7 +3687,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P5" s="2">
-        <v>46303.38328155097</v>
+        <v>46303.78902497852</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>60</v>
@@ -3731,7 +3731,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P6">
-        <v>46303.38328148136</v>
+        <v>46303.7890248602</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>60</v>
@@ -3775,7 +3775,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P7">
-        <v>46303.38328145499</v>
+        <v>46303.78902481608</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>60</v>
@@ -3822,7 +3822,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P8">
-        <v>46303.38328143695</v>
+        <v>46303.78902478614</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>60</v>
@@ -3866,7 +3866,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P9">
-        <v>46303.3832814277</v>
+        <v>46303.7890247705</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>60</v>
@@ -3910,7 +3910,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P10">
-        <v>46303.38328140793</v>
+        <v>46303.78902473875</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>60</v>
@@ -3957,7 +3957,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P11" s="6">
-        <v>46303.38330298233</v>
+        <v>46303.78904117852</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>60</v>
@@ -4006,7 +4006,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P12" s="6">
-        <v>46303.38330305153</v>
+        <v>46303.78904129434</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>60</v>
@@ -4053,7 +4053,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P13" s="6">
-        <v>46303.38330307746</v>
+        <v>46303.7890413381</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>60</v>
@@ -4100,7 +4100,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P14" s="6">
-        <v>46303.38330312896</v>
+        <v>46303.78904142418</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>60</v>
@@ -4149,7 +4149,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P15" s="6">
-        <v>46303.3833125137</v>
+        <v>46303.78904946196</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>60</v>
@@ -4196,7 +4196,7 @@
         <v>46300.75887301003</v>
       </c>
       <c r="P16" s="6">
-        <v>46303.38331254272</v>
+        <v>46303.78904952588</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>60</v>
@@ -4242,7 +4242,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4290,10 +4290,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B2">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C2" t="s">
         <v>176</v>
@@ -4325,10 +4325,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B3">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C3" t="s">
         <v>176</v>
@@ -4343,7 +4343,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -4360,10 +4360,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B4">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C4" t="s">
         <v>176</v>
@@ -4375,16 +4375,16 @@
         <v>3820</v>
       </c>
       <c r="F4">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H4">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -4395,45 +4395,45 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B5">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C5" t="s">
         <v>176</v>
       </c>
       <c r="D5">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E5">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G5">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B6">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C6" t="s">
         <v>176</v>
@@ -4445,13 +4445,13 @@
         <v>160</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -4460,15 +4460,15 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B7">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C7" t="s">
         <v>176</v>
@@ -4480,21 +4480,56 @@
         <v>160</v>
       </c>
       <c r="F7">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H7">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B8">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C8" t="s">
+        <v>176</v>
+      </c>
+      <c r="D8">
+        <v>8</v>
+      </c>
+      <c r="E8">
+        <v>160</v>
+      </c>
+      <c r="F8">
+        <v>157</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>132</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-10-0458Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -13,14 +13,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-Day Working List'!$A$1:$Q$50</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Review'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Review'!$A$1:$Q$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="180">
   <si>
     <t>Priority</t>
   </si>
@@ -79,12 +79,348 @@
     <t>Open</t>
   </si>
   <si>
+    <t>INFO-DRIVE SOFTWARE LIMITED</t>
+  </si>
+  <si>
+    <t>IT / Technology</t>
+  </si>
+  <si>
+    <t>Sumeet Surendra Chimbalkar</t>
+  </si>
+  <si>
+    <t>The CIRP of the Corporate Debtor (“CD”) has been reinstated pursuant to the order passed by the Hon’ble NCLAT. Further, considering that 360 days of the CIRP period had already elapsed as on the date of appointment of the undersigned (Co</t>
+  </si>
+  <si>
+    <t>Not in latest IBBI listing - verify with RP</t>
+  </si>
+  <si>
+    <t>REAL TECH CONSTRUCTIONS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Realty / Construction</t>
+  </si>
+  <si>
+    <t>Construction / EPC</t>
+  </si>
+  <si>
+    <t>Manindra Kumar Tiwari</t>
+  </si>
+  <si>
+    <t>Auto-classified</t>
+  </si>
+  <si>
+    <t>A.P.J. LABORATORIES LIMITED</t>
+  </si>
+  <si>
+    <t>Pharma / Healthcare</t>
+  </si>
+  <si>
+    <t>Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>pooja damir miglani</t>
+  </si>
+  <si>
+    <t>No Fixed Assets are available, except one disputed and contiguous piece of land at Village Ambwala, Nwada Road Tehsil Paonta Sahib, Distt Sirmaur, Himachal Pradesh, India, 173025</t>
+  </si>
+  <si>
+    <t>ALLFLEX PLASTIC LLP</t>
+  </si>
+  <si>
+    <t>Chemicals</t>
+  </si>
+  <si>
+    <t>Plastics / Polymers</t>
+  </si>
+  <si>
+    <t>Mr. Hansraj Jaria</t>
+  </si>
+  <si>
+    <t>At present, the Corporate Debtor is not operational and not a going concern. Revenue from Operation for the financial year ended 31.03.2025 is ?44,98,79,958.90</t>
+  </si>
+  <si>
+    <t>LOG 9 MATERIALS SCIENTIFIC PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Power / Energy</t>
+  </si>
+  <si>
+    <t>Mrs. Neeraja Kartik</t>
+  </si>
+  <si>
+    <t>250 MWh battery production capacity and 50 MWh cell production capacity</t>
+  </si>
+  <si>
+    <t>TECHNOFAB ENGINEERING LIMITED</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Rahul Jindal</t>
+  </si>
+  <si>
+    <t>The Form G has been published on 27.09.2026 in newspapers all over India.</t>
+  </si>
+  <si>
+    <t>STC VENTURES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Other / Unclear</t>
+  </si>
+  <si>
+    <t>PURUSOTTAM BEHERA</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>VIGNESHWARA DEVELOPERS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Real Estate</t>
+  </si>
+  <si>
+    <t>Ms. Ritu Rastogi</t>
+  </si>
+  <si>
+    <t>EXTOL INDUSTRIES LIMITED</t>
+  </si>
+  <si>
+    <t>Ms. Teena Saraswat Pandey</t>
+  </si>
+  <si>
+    <t>unit closed, no employees / no workmen at CIRP commencement date</t>
+  </si>
+  <si>
+    <t>SURYA FOUNDRY PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Steel / Metals</t>
+  </si>
+  <si>
+    <t>Mr. Reetesh Kumar Agarwal</t>
+  </si>
+  <si>
+    <t>XYRON TECHNOLOGIES LIMITED</t>
+  </si>
+  <si>
+    <t>unit closed As Per Information available no employees / No workmen at the commencement of CIRP Process</t>
+  </si>
+  <si>
+    <t>N KUMAR RETAILS &amp; PROPERTIES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mrs. Megha Agrawal</t>
+  </si>
+  <si>
+    <t>(Under sub-regulation (1) of regulation 36A of the Insolvency and Bankruptcy Board of India (Insolvency Resolution Process for Corporate Persons) Regulations, 2016), this corrigendum is being issued in respect of the Form G published on 18.09.2026 invitin</t>
+  </si>
+  <si>
+    <t>VAS INFRASTRUCTURE LIMITED (CN)</t>
+  </si>
+  <si>
+    <t>Infrastructure</t>
+  </si>
+  <si>
+    <t>Infrastructure / EPC</t>
+  </si>
+  <si>
+    <t>Mr. Bimal Kumar Agarwal</t>
+  </si>
+  <si>
+    <t>The Form G has been published on 28.09.2026.</t>
+  </si>
+  <si>
+    <t>TV VISION LIMITED</t>
+  </si>
+  <si>
+    <t>ALOK KUMAR MURARKA</t>
+  </si>
+  <si>
+    <t>INDO PACIFIC PROJECTS LIMITED</t>
+  </si>
+  <si>
+    <t>BHUBANESHWARI SEAFOOD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Agriculture / Food</t>
+  </si>
+  <si>
+    <t>Tripti Agarwal</t>
+  </si>
+  <si>
+    <t>As per the latest available audited financial statement the Turnover in financial year 2022-2023 was Rs. 91.98 crore</t>
+  </si>
+  <si>
+    <t>GOODWILL IRON &amp; STEEL TRADERS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>MANISH AGARWALLA</t>
+  </si>
+  <si>
+    <t>Fixed assets location are taken as per the latest audited balance sheet &amp; address mention as D3/1401 NOIDA Extension .No documents and details are received from the Suspended Board of Directors. Section 19(2) application filed with the Hon'ble NC</t>
+  </si>
+  <si>
+    <t>COMET GRANITO PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Cement / Building Materials</t>
+  </si>
+  <si>
+    <t>Anil Kashi Drolia</t>
+  </si>
+  <si>
+    <t>VAASUDEVA MILK FOODS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ATKURU SAI PRASAD</t>
+  </si>
+  <si>
+    <t>Form-G Issued</t>
+  </si>
+  <si>
+    <t>M/s Margdarshak Financial Services Limited</t>
+  </si>
+  <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
+    <t>Rakesh Kumar Jindal</t>
+  </si>
+  <si>
+    <t>Form G was published for the third time with the approval of the CoC and the NCLT.</t>
+  </si>
+  <si>
+    <t>IN2IT TECHNOLOGIES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ishant jain</t>
+  </si>
+  <si>
+    <t>Re-issuance of Form G: Form G was re-issued on 17.09.2026, with 03.10.2026 as the last date for submission of EOI. Pursuant to the directions of the CoC, an Addendum to Form G was issued, revising and extending the stipulated timelines accordingly.</t>
+  </si>
+  <si>
+    <t>KM TOLL ROAD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Roads / Toll Roads</t>
+  </si>
+  <si>
+    <t>Roads / Highways</t>
+  </si>
+  <si>
+    <t>Mr. Ashish Saoji</t>
+  </si>
+  <si>
+    <t>ORGANIC WORLD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Prakul Thadi</t>
+  </si>
+  <si>
+    <t>SUN GRANITE EXPORT LIMITED</t>
+  </si>
+  <si>
+    <t>Raghunath Bhandari</t>
+  </si>
+  <si>
+    <t>SHRENIK LIMITED</t>
+  </si>
+  <si>
+    <t>RAHUL SHAH</t>
+  </si>
+  <si>
+    <t>OMKARA VIJAYALAKSHMI STRIPS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Neha Jain Nemani</t>
+  </si>
+  <si>
+    <t>A fresh Form-G is issued upon taking approval from the CoC on 6th October 2026. The last day for submission of EOI is 21st October 2026.</t>
+  </si>
+  <si>
+    <t>G &amp; L PROFILE AND EQUIPMENTS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Manish Kumar Bhagat</t>
+  </si>
+  <si>
+    <t>SOCRUS PHARMACEUTICALS LIMITED</t>
+  </si>
+  <si>
+    <t>kuldeep tank</t>
+  </si>
+  <si>
+    <t>Sion Panvel Tollways Private Limited</t>
+  </si>
+  <si>
+    <t>Mr. Sanjay Kumar Mishra</t>
+  </si>
+  <si>
+    <t>1. Since CD is in business of road construction, there are no major tangible assets available; 2. No employee on the rolls of CD since ICD; 3. Current Form G is pursuant to NCLT order - 29 Sept'26 and 59th CoC meeting on 06 Oct'26.</t>
+  </si>
+  <si>
+    <t>AXLE PAPER PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>Mr. Kailash Shah</t>
+  </si>
+  <si>
+    <t>The installed capacity of main Products is 150MTPD.</t>
+  </si>
+  <si>
+    <t>Raheja Developers Limited - Revanta Project</t>
+  </si>
+  <si>
+    <t>Mr. Surendra Raj Gang</t>
+  </si>
+  <si>
+    <t>The CoC in its 4th meeting has resolved to scrap the earlier EOI process pursuant to Form-G dated 03 September 2026 and publish the current invitation for EOI for submission of Resolution Plans. The details of product are available in attached document.</t>
+  </si>
+  <si>
+    <t>PRATHAM-HEERA SALES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Mahesh Goverdhan Bagla</t>
+  </si>
+  <si>
+    <t>SIMARA FOODS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Navin Khandelwal</t>
+  </si>
+  <si>
+    <t>Recently closed</t>
+  </si>
+  <si>
+    <t>Closed recently</t>
+  </si>
+  <si>
+    <t>ALVI TECH SERVICES PVT LTD</t>
+  </si>
+  <si>
+    <t>Shree Shiddhanath Cotex Private Limited</t>
+  </si>
+  <si>
+    <t>Textiles</t>
+  </si>
+  <si>
+    <t>Akhil Ahuja</t>
+  </si>
+  <si>
+    <t>The FORM G is published for the second time as per the approval by the CoC Members.</t>
+  </si>
+  <si>
     <t>TRUWEIGHT WELLNESS PRIVATE LIMITED</t>
   </si>
   <si>
-    <t>Pharma / Healthcare</t>
-  </si>
-  <si>
     <t>Healthcare</t>
   </si>
   <si>
@@ -94,297 +430,6 @@
     <t>_</t>
   </si>
   <si>
-    <t>Auto-classified</t>
-  </si>
-  <si>
-    <t>ALVI TECH SERVICES PVT LTD</t>
-  </si>
-  <si>
-    <t>IT / Technology</t>
-  </si>
-  <si>
-    <t>Neha Jain Nemani</t>
-  </si>
-  <si>
-    <t>Shree Shiddhanath Cotex Private Limited</t>
-  </si>
-  <si>
-    <t>Textiles</t>
-  </si>
-  <si>
-    <t>Akhil Ahuja</t>
-  </si>
-  <si>
-    <t>The FORM G is published for the second time as per the approval by the CoC Members.</t>
-  </si>
-  <si>
-    <t>INFO-DRIVE SOFTWARE LIMITED</t>
-  </si>
-  <si>
-    <t>Sumeet Surendra Chimbalkar</t>
-  </si>
-  <si>
-    <t>The CIRP of the Corporate Debtor (“CD”) has been reinstated pursuant to the order passed by the Hon’ble NCLAT. Further, considering that 360 days of the CIRP period had already elapsed as on the date of appointment of the undersigned (Co</t>
-  </si>
-  <si>
-    <t>REAL TECH CONSTRUCTIONS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Realty / Construction</t>
-  </si>
-  <si>
-    <t>Construction / EPC</t>
-  </si>
-  <si>
-    <t>Manindra Kumar Tiwari</t>
-  </si>
-  <si>
-    <t>A.P.J. LABORATORIES LIMITED</t>
-  </si>
-  <si>
-    <t>Pharmaceuticals</t>
-  </si>
-  <si>
-    <t>pooja damir miglani</t>
-  </si>
-  <si>
-    <t>No Fixed Assets are available, except one disputed and contiguous piece of land at Village Ambwala, Nwada Road Tehsil Paonta Sahib, Distt Sirmaur, Himachal Pradesh, India, 173025</t>
-  </si>
-  <si>
-    <t>ALLFLEX PLASTIC LLP</t>
-  </si>
-  <si>
-    <t>Chemicals</t>
-  </si>
-  <si>
-    <t>Plastics / Polymers</t>
-  </si>
-  <si>
-    <t>Mr. Hansraj Jaria</t>
-  </si>
-  <si>
-    <t>At present, the Corporate Debtor is not operational and not a going concern. Revenue from Operation for the financial year ended 31.03.2025 is ?44,98,79,958.90</t>
-  </si>
-  <si>
-    <t>LOG 9 MATERIALS SCIENTIFIC PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Power / Energy</t>
-  </si>
-  <si>
-    <t>Mrs. Neeraja Kartik</t>
-  </si>
-  <si>
-    <t>250 MWh battery production capacity and 50 MWh cell production capacity</t>
-  </si>
-  <si>
-    <t>TECHNOFAB ENGINEERING LIMITED</t>
-  </si>
-  <si>
-    <t>Manufacturing</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Rahul Jindal</t>
-  </si>
-  <si>
-    <t>The Form G has been published on 27.09.2026 in newspapers all over India.</t>
-  </si>
-  <si>
-    <t>STC VENTURES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Other / Unclear</t>
-  </si>
-  <si>
-    <t>PURUSOTTAM BEHERA</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>VIGNESHWARA DEVELOPERS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Real Estate</t>
-  </si>
-  <si>
-    <t>Ms. Ritu Rastogi</t>
-  </si>
-  <si>
-    <t>EXTOL INDUSTRIES LIMITED</t>
-  </si>
-  <si>
-    <t>Ms. Teena Saraswat Pandey</t>
-  </si>
-  <si>
-    <t>unit closed, no employees / no workmen at CIRP commencement date</t>
-  </si>
-  <si>
-    <t>SURYA FOUNDRY PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Steel / Metals</t>
-  </si>
-  <si>
-    <t>Mr. Reetesh Kumar Agarwal</t>
-  </si>
-  <si>
-    <t>XYRON TECHNOLOGIES LIMITED</t>
-  </si>
-  <si>
-    <t>unit closed As Per Information available no employees / No workmen at the commencement of CIRP Process</t>
-  </si>
-  <si>
-    <t>VAS INFRASTRUCTURE LIMITED (CN)</t>
-  </si>
-  <si>
-    <t>Infrastructure</t>
-  </si>
-  <si>
-    <t>Infrastructure / EPC</t>
-  </si>
-  <si>
-    <t>Mr. Bimal Kumar Agarwal</t>
-  </si>
-  <si>
-    <t>The Form G has been published on 28.09.2026.</t>
-  </si>
-  <si>
-    <t>TV VISION LIMITED</t>
-  </si>
-  <si>
-    <t>ALOK KUMAR MURARKA</t>
-  </si>
-  <si>
-    <t>INDO PACIFIC PROJECTS LIMITED</t>
-  </si>
-  <si>
-    <t>Mrs. Megha Agrawal</t>
-  </si>
-  <si>
-    <t>BHUBANESHWARI SEAFOOD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Agriculture / Food</t>
-  </si>
-  <si>
-    <t>Tripti Agarwal</t>
-  </si>
-  <si>
-    <t>As per the latest available audited financial statement the Turnover in financial year 2022-2023 was Rs. 91.98 crore</t>
-  </si>
-  <si>
-    <t>GOODWILL IRON &amp; STEEL TRADERS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>MANISH AGARWALLA</t>
-  </si>
-  <si>
-    <t>Fixed assets location are taken as per the latest audited balance sheet &amp; address mention as D3/1401 NOIDA Extension .No documents and details are received from the Suspended Board of Directors. Section 19(2) application filed with the Hon'ble NC</t>
-  </si>
-  <si>
-    <t>COMET GRANITO PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Cement / Building Materials</t>
-  </si>
-  <si>
-    <t>Anil Kashi Drolia</t>
-  </si>
-  <si>
-    <t>VAASUDEVA MILK FOODS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>ATKURU SAI PRASAD</t>
-  </si>
-  <si>
-    <t>Form-G Issued</t>
-  </si>
-  <si>
-    <t>M/s Margdarshak Financial Services Limited</t>
-  </si>
-  <si>
-    <t>Financial Services</t>
-  </si>
-  <si>
-    <t>Rakesh Kumar Jindal</t>
-  </si>
-  <si>
-    <t>Form G was published for the third time with the approval of the CoC and the NCLT.</t>
-  </si>
-  <si>
-    <t>IN2IT TECHNOLOGIES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>ishant jain</t>
-  </si>
-  <si>
-    <t>Re-issuance of Form G: Form G was re-issued on 17.09.2026, with 03.10.2026 as the last date for submission of EOI. Pursuant to the directions of the CoC, an Addendum to Form G was issued, revising and extending the stipulated timelines accordingly.</t>
-  </si>
-  <si>
-    <t>KM TOLL ROAD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Roads / Toll Roads</t>
-  </si>
-  <si>
-    <t>Roads / Highways</t>
-  </si>
-  <si>
-    <t>Mr. Ashish Saoji</t>
-  </si>
-  <si>
-    <t>ORGANIC WORLD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Prakul Thadi</t>
-  </si>
-  <si>
-    <t>SUN GRANITE EXPORT LIMITED</t>
-  </si>
-  <si>
-    <t>Raghunath Bhandari</t>
-  </si>
-  <si>
-    <t>SHRENIK LIMITED</t>
-  </si>
-  <si>
-    <t>RAHUL SHAH</t>
-  </si>
-  <si>
-    <t>OMKARA VIJAYALAKSHMI STRIPS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>A fresh Form-G is issued upon taking approval from the CoC on 6th October 2026. The last day for submission of EOI is 21st October 2026.</t>
-  </si>
-  <si>
-    <t>G &amp; L PROFILE AND EQUIPMENTS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Manish Kumar Bhagat</t>
-  </si>
-  <si>
-    <t>SOCRUS PHARMACEUTICALS LIMITED</t>
-  </si>
-  <si>
-    <t>kuldeep tank</t>
-  </si>
-  <si>
-    <t>PRATHAM-HEERA SALES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Mahesh Goverdhan Bagla</t>
-  </si>
-  <si>
-    <t>Recently closed</t>
-  </si>
-  <si>
-    <t>Closed recently</t>
-  </si>
-  <si>
     <t>SHIVANGI AGRO INDIA PRIVATE LIMITED</t>
   </si>
   <si>
@@ -463,12 +508,6 @@
     <t>Mr. Bhoopesh Gupta</t>
   </si>
   <si>
-    <t>N KUMAR RETAILS &amp; PROPERTIES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Company has two operational grocery marts in the name of Poonam Bazaar units in Nagpur. The grocery marts are in operational status, however the financials and custody of the assets of CD are yet to be handed over to the RP.</t>
-  </si>
-  <si>
     <t>VELEX LOGISTICS PRIVATE LIMITED</t>
   </si>
   <si>
@@ -485,36 +524,6 @@
   </si>
   <si>
     <t>The Resolution Professional has issued an invitation for expression of interest on 01 September 2026.</t>
-  </si>
-  <si>
-    <t>SHAH LAXMICHAND VERSHI MASALAWALA LLP</t>
-  </si>
-  <si>
-    <t>Mr. Dakshesh Pravinchandra Choksi</t>
-  </si>
-  <si>
-    <t>AMISHI CONSUMER TECHNOLOGIES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Amit Talwar</t>
-  </si>
-  <si>
-    <t>ISHAPE APPLIANCES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Retail / Consumer</t>
-  </si>
-  <si>
-    <t>PRABHAT JAIN</t>
-  </si>
-  <si>
-    <t>JAISUBA AGRO PRODUCTS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Rajendran Shanmugam</t>
-  </si>
-  <si>
-    <t>Assets of the Corporate Debtor and the Personal Guarantors are proposed to be clubbed under Sec.28A of IBC for the purpose of inviting resolution plans.</t>
   </si>
   <si>
     <t>Started</t>
@@ -970,7 +979,7 @@
     <col min="12" max="12" width="48.7109375" customWidth="1"/>
     <col min="13" max="14" width="12.7109375" customWidth="1"/>
     <col min="15" max="16" width="20.7109375" customWidth="1"/>
-    <col min="17" max="17" width="16.7109375" customWidth="1"/>
+    <col min="17" max="17" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -1039,41 +1048,38 @@
       <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="G2" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H2" s="3">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="I2" s="2">
         <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="K2" s="2">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="2">
-        <v>2</v>
-      </c>
-      <c r="L2" s="2" t="s">
+      <c r="M2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O2" s="2">
+        <v>46300.75885633306</v>
+      </c>
+      <c r="P2" s="2">
+        <v>46303.78903317315</v>
+      </c>
+      <c r="Q2" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O2" s="2">
-        <v>46300.7588564207</v>
-      </c>
-      <c r="P2" s="2">
-        <v>46303.78903324551</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="2" customFormat="1">
@@ -1084,16 +1090,19 @@
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>26</v>
       </c>
       <c r="G3" s="2">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="H3" s="3">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="I3" s="2">
         <v>1</v>
@@ -1111,13 +1120,13 @@
         <v>18</v>
       </c>
       <c r="O3" s="2">
-        <v>46300.75885634872</v>
+        <v>46300.75885622757</v>
       </c>
       <c r="P3" s="2">
-        <v>46303.78903320204</v>
+        <v>46305.20576110142</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1">
@@ -1128,28 +1137,31 @@
         <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="G4" s="2">
         <v>0.9399999999999999</v>
       </c>
       <c r="H4" s="3">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="I4" s="2">
         <v>1</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K4" s="2">
         <v>1</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="M4" s="4" t="s">
         <v>18</v>
@@ -1158,13 +1170,13 @@
         <v>18</v>
       </c>
       <c r="O4" s="2">
-        <v>46300.7588563655</v>
+        <v>46300.75885624527</v>
       </c>
       <c r="P4" s="2">
-        <v>46303.78903321669</v>
+        <v>46305.20576108179</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="2" customFormat="1">
@@ -1175,28 +1187,31 @@
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>26</v>
+        <v>35</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="G5" s="2">
         <v>0.91</v>
       </c>
       <c r="H5" s="3">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="I5" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="K5" s="2">
         <v>1</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>18</v>
@@ -1205,13 +1220,13 @@
         <v>18</v>
       </c>
       <c r="O5" s="2">
-        <v>46300.75885633306</v>
+        <v>46300.7588562628</v>
       </c>
       <c r="P5" s="2">
-        <v>46303.78903317315</v>
+        <v>46305.20576109179</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:17" s="2" customFormat="1">
@@ -1222,29 +1237,29 @@
         <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G6" s="2">
-        <v>0.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H6" s="3">
         <v>46306</v>
       </c>
       <c r="I6" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="K6" s="2">
         <v>1</v>
       </c>
+      <c r="L6" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="M6" s="4" t="s">
         <v>18</v>
       </c>
@@ -1252,13 +1267,13 @@
         <v>18</v>
       </c>
       <c r="O6" s="2">
-        <v>46300.75885622757</v>
+        <v>46300.75885627908</v>
       </c>
       <c r="P6" s="2">
-        <v>46303.78903311479</v>
+        <v>46305.20576111179</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:17" s="2" customFormat="1">
@@ -1269,31 +1284,31 @@
         <v>18</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="G7" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="H7" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="I7" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="K7" s="2">
         <v>1</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>18</v>
@@ -1302,13 +1317,13 @@
         <v>18</v>
       </c>
       <c r="O7" s="2">
-        <v>46300.75885624527</v>
+        <v>46300.75884793277</v>
       </c>
       <c r="P7" s="2">
-        <v>46303.78903312911</v>
+        <v>46305.20576101432</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:17" s="2" customFormat="1">
@@ -1319,32 +1334,26 @@
         <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G8" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H8" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="I8" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="K8" s="2">
         <v>1</v>
       </c>
-      <c r="L8" s="2" t="s">
-        <v>47</v>
-      </c>
       <c r="M8" s="4" t="s">
         <v>18</v>
       </c>
@@ -1352,13 +1361,13 @@
         <v>18</v>
       </c>
       <c r="O8" s="2">
-        <v>46300.7588562628</v>
+        <v>46300.7588479478</v>
       </c>
       <c r="P8" s="2">
-        <v>46303.78903314354</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>24</v>
+        <v>46305.20576103318</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:17" s="2" customFormat="1">
@@ -1369,29 +1378,29 @@
         <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>49</v>
+        <v>25</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="G9" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="H9" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="I9" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="K9" s="2">
         <v>1</v>
       </c>
-      <c r="L9" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
       </c>
@@ -1399,13 +1408,13 @@
         <v>18</v>
       </c>
       <c r="O9" s="2">
-        <v>46300.75885627908</v>
+        <v>46300.75884796329</v>
       </c>
       <c r="P9" s="2">
-        <v>46303.78903310001</v>
+        <v>46305.20576097554</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:17" s="2" customFormat="1">
@@ -1416,31 +1425,28 @@
         <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G10" s="2">
-        <v>0.88</v>
+        <v>0.2</v>
       </c>
       <c r="H10" s="3">
         <v>46307</v>
       </c>
       <c r="I10" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="K10" s="2">
         <v>1</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M10" s="4" t="s">
         <v>18</v>
@@ -1449,13 +1455,13 @@
         <v>18</v>
       </c>
       <c r="O10" s="2">
-        <v>46300.75884793277</v>
+        <v>46300.75884799581</v>
       </c>
       <c r="P10" s="2">
-        <v>46303.78903304238</v>
-      </c>
-      <c r="Q10" s="2" t="s">
-        <v>24</v>
+        <v>46305.20576098546</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:17" s="2" customFormat="1">
@@ -1466,22 +1472,22 @@
         <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G11" s="2">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H11" s="3">
         <v>46307</v>
       </c>
       <c r="I11" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K11" s="2">
         <v>1</v>
@@ -1493,13 +1499,13 @@
         <v>18</v>
       </c>
       <c r="O11" s="2">
-        <v>46300.7588479478</v>
+        <v>46300.75885617639</v>
       </c>
       <c r="P11" s="2">
-        <v>46303.78903307128</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>60</v>
+        <v>46305.205761005</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:17" s="2" customFormat="1">
@@ -1513,26 +1519,26 @@
         <v>61</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="G12" s="2">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="H12" s="3">
         <v>46307</v>
       </c>
       <c r="I12" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K12" s="2">
         <v>1</v>
       </c>
+      <c r="L12" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="M12" s="4" t="s">
         <v>18</v>
       </c>
@@ -1540,13 +1546,13 @@
         <v>18</v>
       </c>
       <c r="O12" s="2">
-        <v>46300.75884796329</v>
+        <v>46300.75885619673</v>
       </c>
       <c r="P12" s="2">
-        <v>46303.7890329982</v>
+        <v>46305.20576099515</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:17" s="2" customFormat="1">
@@ -1557,29 +1563,32 @@
         <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>58</v>
+        <v>25</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="G13" s="2">
-        <v>0.2</v>
+        <v>0.93</v>
       </c>
       <c r="H13" s="3">
         <v>46307</v>
       </c>
       <c r="I13" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K13" s="2">
+        <v>2</v>
+      </c>
+      <c r="L13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K13" s="2">
-        <v>1</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="M13" s="4" t="s">
         <v>18</v>
       </c>
@@ -1587,13 +1596,13 @@
         <v>18</v>
       </c>
       <c r="O13" s="2">
-        <v>46300.75884799581</v>
+        <v>46305.20576106136</v>
       </c>
       <c r="P13" s="2">
-        <v>46303.78903301315</v>
-      </c>
-      <c r="Q13" s="5" t="s">
-        <v>60</v>
+        <v>46305.20576106139</v>
+      </c>
+      <c r="Q13" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:17" s="2" customFormat="1">
@@ -1604,19 +1613,22 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>68</v>
       </c>
       <c r="G14" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H14" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I14" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>69</v>
@@ -1624,6 +1636,9 @@
       <c r="K14" s="2">
         <v>1</v>
       </c>
+      <c r="L14" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="M14" s="4" t="s">
         <v>18</v>
       </c>
@@ -1631,13 +1646,13 @@
         <v>18</v>
       </c>
       <c r="O14" s="2">
-        <v>46300.75885617639</v>
+        <v>46300.75884788632</v>
       </c>
       <c r="P14" s="2">
-        <v>46303.78903296705</v>
+        <v>46305.20576095542</v>
       </c>
       <c r="Q14" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:17" s="2" customFormat="1">
@@ -1648,29 +1663,26 @@
         <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="G15" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H15" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I15" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="K15" s="2">
         <v>1</v>
       </c>
-      <c r="L15" s="2" t="s">
-        <v>71</v>
-      </c>
       <c r="M15" s="4" t="s">
         <v>18</v>
       </c>
@@ -1678,13 +1690,13 @@
         <v>18</v>
       </c>
       <c r="O15" s="2">
-        <v>46300.75885619673</v>
+        <v>46300.75884790152</v>
       </c>
       <c r="P15" s="2">
-        <v>46303.78903302801</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>24</v>
+        <v>46305.20576094543</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:17" s="2" customFormat="1">
@@ -1695,32 +1707,26 @@
         <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="G16" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H16" s="3">
         <v>46308</v>
       </c>
       <c r="I16" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="K16" s="2">
         <v>1</v>
       </c>
-      <c r="L16" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="M16" s="4" t="s">
         <v>18</v>
       </c>
@@ -1728,13 +1734,13 @@
         <v>18</v>
       </c>
       <c r="O16" s="2">
-        <v>46300.75884788632</v>
+        <v>46301.38232480602</v>
       </c>
       <c r="P16" s="2">
-        <v>46303.78902500809</v>
-      </c>
-      <c r="Q16" s="2" t="s">
-        <v>24</v>
+        <v>46305.20576093486</v>
+      </c>
+      <c r="Q16" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="17" spans="1:17" s="2" customFormat="1">
@@ -1745,26 +1751,29 @@
         <v>18</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="G17" s="2">
-        <v>0.2</v>
+        <v>0.92</v>
       </c>
       <c r="H17" s="3">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="I17" s="2">
         <v>5</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K17" s="2">
         <v>1</v>
       </c>
+      <c r="L17" s="2" t="s">
+        <v>77</v>
+      </c>
       <c r="M17" s="4" t="s">
         <v>18</v>
       </c>
@@ -1772,13 +1781,13 @@
         <v>18</v>
       </c>
       <c r="O17" s="2">
-        <v>46300.75884790152</v>
+        <v>46300.75884787029</v>
       </c>
       <c r="P17" s="2">
-        <v>46303.78902499317</v>
-      </c>
-      <c r="Q17" s="5" t="s">
-        <v>60</v>
+        <v>46305.20576092294</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="2" customFormat="1">
@@ -1789,26 +1798,29 @@
         <v>18</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="H18" s="3">
+        <v>46312</v>
+      </c>
+      <c r="I18" s="2">
+        <v>7</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G18" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="H18" s="3">
-        <v>46308</v>
-      </c>
-      <c r="I18" s="2">
-        <v>5</v>
-      </c>
-      <c r="J18" s="2" t="s">
+      <c r="K18" s="2">
+        <v>1</v>
+      </c>
+      <c r="L18" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="K18" s="2">
-        <v>1</v>
-      </c>
       <c r="M18" s="4" t="s">
         <v>18</v>
       </c>
@@ -1816,13 +1828,13 @@
         <v>18</v>
       </c>
       <c r="O18" s="2">
-        <v>46301.38232480602</v>
+        <v>46300.75884779022</v>
       </c>
       <c r="P18" s="2">
-        <v>46303.78902497852</v>
-      </c>
-      <c r="Q18" s="5" t="s">
-        <v>60</v>
+        <v>46305.20575279809</v>
+      </c>
+      <c r="Q18" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:17" s="2" customFormat="1">
@@ -1839,10 +1851,10 @@
         <v>82</v>
       </c>
       <c r="G19" s="2">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="H19" s="3">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="I19" s="2">
         <v>7</v>
@@ -1853,114 +1865,114 @@
       <c r="K19" s="2">
         <v>1</v>
       </c>
-      <c r="L19" s="2" t="s">
+      <c r="M19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O19" s="2">
+        <v>46300.75884780569</v>
+      </c>
+      <c r="P19" s="2">
+        <v>46305.20575282763</v>
+      </c>
+      <c r="Q19" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" s="2" customFormat="1">
+      <c r="A20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="M19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O19" s="2">
-        <v>46300.75884787029</v>
-      </c>
-      <c r="P19" s="2">
-        <v>46303.78902496338</v>
-      </c>
-      <c r="Q19" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17">
-      <c r="A20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" t="s">
-        <v>85</v>
-      </c>
-      <c r="E20" t="s">
-        <v>68</v>
-      </c>
-      <c r="G20">
-        <v>0.95</v>
+      <c r="E20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0.93</v>
       </c>
       <c r="H20" s="3">
         <v>46312</v>
       </c>
-      <c r="I20">
-        <v>9</v>
-      </c>
-      <c r="J20" t="s">
+      <c r="I20" s="2">
+        <v>7</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="K20" s="2">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="K20">
-        <v>1</v>
-      </c>
-      <c r="L20" t="s">
+      <c r="M20" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N20" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O20" s="2">
+        <v>46300.75884782107</v>
+      </c>
+      <c r="P20" s="2">
+        <v>46305.20575281785</v>
+      </c>
+      <c r="Q20" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" s="2" customFormat="1">
+      <c r="A21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="M20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N20" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O20">
-        <v>46300.75884779022</v>
-      </c>
-      <c r="P20">
-        <v>46303.78902493456</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17">
-      <c r="A21" t="s">
-        <v>18</v>
-      </c>
-      <c r="B21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="E21" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="E21" t="s">
-        <v>89</v>
-      </c>
-      <c r="G21">
-        <v>0.93</v>
+      <c r="G21" s="2">
+        <v>0.91</v>
       </c>
       <c r="H21" s="3">
         <v>46312</v>
       </c>
-      <c r="I21">
-        <v>9</v>
-      </c>
-      <c r="J21" t="s">
+      <c r="I21" s="2">
+        <v>7</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K21" s="2">
+        <v>1</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="K21">
-        <v>1</v>
-      </c>
       <c r="M21" s="4" t="s">
         <v>18</v>
       </c>
       <c r="N21" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O21">
-        <v>46300.75884780569</v>
-      </c>
-      <c r="P21">
-        <v>46303.78902489004</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>24</v>
+      <c r="O21" s="2">
+        <v>46300.75884783743</v>
+      </c>
+      <c r="P21" s="2">
+        <v>46305.20575280781</v>
+      </c>
+      <c r="Q21" s="2" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -1974,22 +1986,22 @@
         <v>91</v>
       </c>
       <c r="E22" t="s">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="G22">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="H22" s="3">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="I22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J22" t="s">
         <v>92</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L22" t="s">
         <v>93</v>
@@ -2001,13 +2013,13 @@
         <v>18</v>
       </c>
       <c r="O22">
-        <v>46300.75884782107</v>
+        <v>46302.26841519317</v>
       </c>
       <c r="P22">
-        <v>46303.78902490489</v>
+        <v>46305.20575278824</v>
       </c>
       <c r="Q22" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -2023,24 +2035,24 @@
       <c r="E23" t="s">
         <v>95</v>
       </c>
+      <c r="F23" t="s">
+        <v>96</v>
+      </c>
       <c r="G23">
-        <v>0.91</v>
+        <v>0.96</v>
       </c>
       <c r="H23" s="3">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="I23">
         <v>9</v>
       </c>
       <c r="J23" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K23">
         <v>1</v>
       </c>
-      <c r="L23" t="s">
-        <v>97</v>
-      </c>
       <c r="M23" s="4" t="s">
         <v>18</v>
       </c>
@@ -2048,13 +2060,13 @@
         <v>18</v>
       </c>
       <c r="O23">
-        <v>46300.75884783743</v>
+        <v>46300.75884774033</v>
       </c>
       <c r="P23">
-        <v>46303.78902491984</v>
+        <v>46305.20575275837</v>
       </c>
       <c r="Q23" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -2068,25 +2080,22 @@
         <v>98</v>
       </c>
       <c r="E24" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="G24">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H24" s="3">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="I24">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J24" t="s">
         <v>99</v>
       </c>
       <c r="K24">
-        <v>3</v>
-      </c>
-      <c r="L24" t="s">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="M24" s="4" t="s">
         <v>18</v>
@@ -2095,13 +2104,13 @@
         <v>18</v>
       </c>
       <c r="O24">
-        <v>46302.26841519317</v>
+        <v>46300.75884775587</v>
       </c>
       <c r="P24">
-        <v>46303.78902487514</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>24</v>
+        <v>46305.20575276836</v>
+      </c>
+      <c r="Q24" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -2112,25 +2121,22 @@
         <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E25" t="s">
-        <v>102</v>
-      </c>
-      <c r="F25" t="s">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="G25">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="H25" s="3">
         <v>46314</v>
       </c>
       <c r="I25">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="J25" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="K25">
         <v>1</v>
@@ -2142,13 +2148,13 @@
         <v>18</v>
       </c>
       <c r="O25">
-        <v>46300.75884774033</v>
+        <v>46300.7588477715</v>
       </c>
       <c r="P25">
-        <v>46303.78902484559</v>
+        <v>46305.20575277831</v>
       </c>
       <c r="Q25" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2159,22 +2165,22 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E26" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G26">
         <v>0.2</v>
       </c>
       <c r="H26" s="3">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="I26">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J26" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="K26">
         <v>1</v>
@@ -2186,13 +2192,13 @@
         <v>18</v>
       </c>
       <c r="O26">
-        <v>46300.75884775587</v>
+        <v>46300.75884772457</v>
       </c>
       <c r="P26">
-        <v>46303.7890248602</v>
+        <v>46305.20575274854</v>
       </c>
       <c r="Q26" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -2203,25 +2209,28 @@
         <v>18</v>
       </c>
       <c r="C27" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E27" t="s">
-        <v>89</v>
+        <v>49</v>
       </c>
       <c r="G27">
-        <v>0.93</v>
+        <v>0.2</v>
       </c>
       <c r="H27" s="3">
-        <v>46314</v>
+        <v>46316</v>
       </c>
       <c r="I27">
         <v>11</v>
       </c>
       <c r="J27" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L27" t="s">
+        <v>106</v>
       </c>
       <c r="M27" s="4" t="s">
         <v>18</v>
@@ -2230,13 +2239,13 @@
         <v>18</v>
       </c>
       <c r="O27">
-        <v>46300.7588477715</v>
+        <v>46302.26841507768</v>
       </c>
       <c r="P27">
-        <v>46303.78902483075</v>
-      </c>
-      <c r="Q27" t="s">
-        <v>24</v>
+        <v>46305.20575272872</v>
+      </c>
+      <c r="Q27" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -2247,22 +2256,22 @@
         <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G28">
         <v>0.2</v>
       </c>
       <c r="H28" s="3">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="I28">
         <v>12</v>
       </c>
       <c r="J28" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="K28">
         <v>1</v>
@@ -2274,13 +2283,13 @@
         <v>18</v>
       </c>
       <c r="O28">
-        <v>46300.75884772457</v>
+        <v>46301.38232468421</v>
       </c>
       <c r="P28">
-        <v>46303.78902481608</v>
+        <v>46305.20575271807</v>
       </c>
       <c r="Q28" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -2291,28 +2300,28 @@
         <v>18</v>
       </c>
       <c r="C29" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E29" t="s">
-        <v>58</v>
+        <v>30</v>
+      </c>
+      <c r="F29" t="s">
+        <v>31</v>
       </c>
       <c r="G29">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H29" s="3">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="I29">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J29" t="s">
-        <v>27</v>
+        <v>110</v>
       </c>
       <c r="K29">
-        <v>3</v>
-      </c>
-      <c r="L29" t="s">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="M29" s="4" t="s">
         <v>18</v>
@@ -2321,13 +2330,13 @@
         <v>18</v>
       </c>
       <c r="O29">
-        <v>46302.26841507768</v>
+        <v>46302.26841501552</v>
       </c>
       <c r="P29">
-        <v>46303.78902478614</v>
-      </c>
-      <c r="Q29" s="5" t="s">
-        <v>60</v>
+        <v>46305.20575270729</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2338,26 +2347,32 @@
         <v>18</v>
       </c>
       <c r="C30" t="s">
+        <v>111</v>
+      </c>
+      <c r="E30" t="s">
+        <v>95</v>
+      </c>
+      <c r="F30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G30">
+        <v>0.96</v>
+      </c>
+      <c r="H30" s="3">
+        <v>46318</v>
+      </c>
+      <c r="I30">
+        <v>13</v>
+      </c>
+      <c r="J30" t="s">
+        <v>112</v>
+      </c>
+      <c r="K30">
+        <v>1</v>
+      </c>
+      <c r="L30" t="s">
         <v>113</v>
       </c>
-      <c r="E30" t="s">
-        <v>58</v>
-      </c>
-      <c r="G30">
-        <v>0.2</v>
-      </c>
-      <c r="H30" s="3">
-        <v>46317</v>
-      </c>
-      <c r="I30">
-        <v>14</v>
-      </c>
-      <c r="J30" t="s">
-        <v>114</v>
-      </c>
-      <c r="K30">
-        <v>1</v>
-      </c>
       <c r="M30" s="4" t="s">
         <v>18</v>
       </c>
@@ -2365,13 +2380,13 @@
         <v>18</v>
       </c>
       <c r="O30">
-        <v>46301.38232468421</v>
+        <v>46305.20575267453</v>
       </c>
       <c r="P30">
-        <v>46303.7890247705</v>
-      </c>
-      <c r="Q30" s="5" t="s">
-        <v>60</v>
+        <v>46305.20575267455</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -2382,22 +2397,19 @@
         <v>18</v>
       </c>
       <c r="C31" t="s">
+        <v>114</v>
+      </c>
+      <c r="E31" t="s">
         <v>115</v>
-      </c>
-      <c r="E31" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" t="s">
-        <v>40</v>
       </c>
       <c r="G31">
         <v>0.9399999999999999</v>
       </c>
       <c r="H31" s="3">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="I31">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J31" t="s">
         <v>116</v>
@@ -2405,6 +2417,9 @@
       <c r="K31">
         <v>1</v>
       </c>
+      <c r="L31" t="s">
+        <v>117</v>
+      </c>
       <c r="M31" s="4" t="s">
         <v>18</v>
       </c>
@@ -2412,13 +2427,13 @@
         <v>18</v>
       </c>
       <c r="O31">
-        <v>46302.26841501552</v>
+        <v>46305.20575269723</v>
       </c>
       <c r="P31">
-        <v>46303.78902475473</v>
+        <v>46305.20575269724</v>
       </c>
       <c r="Q31" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -2429,169 +2444,165 @@
         <v>18</v>
       </c>
       <c r="C32" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E32" t="s">
-        <v>58</v>
+        <v>25</v>
+      </c>
+      <c r="F32" t="s">
+        <v>53</v>
       </c>
       <c r="G32">
+        <v>0.93</v>
+      </c>
+      <c r="H32" s="3">
+        <v>46319</v>
+      </c>
+      <c r="I32">
+        <v>14</v>
+      </c>
+      <c r="J32" t="s">
+        <v>119</v>
+      </c>
+      <c r="K32">
+        <v>2</v>
+      </c>
+      <c r="L32" t="s">
+        <v>120</v>
+      </c>
+      <c r="M32" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N32" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O32">
+        <v>46305.20575263901</v>
+      </c>
+      <c r="P32">
+        <v>46305.20575263904</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17">
+      <c r="A33" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" t="s">
+        <v>18</v>
+      </c>
+      <c r="C33" t="s">
+        <v>121</v>
+      </c>
+      <c r="E33" t="s">
+        <v>49</v>
+      </c>
+      <c r="G33">
         <v>0.2</v>
       </c>
-      <c r="H32" s="3">
+      <c r="H33" s="3">
         <v>46326</v>
       </c>
-      <c r="I32">
-        <v>23</v>
-      </c>
-      <c r="J32" t="s">
-        <v>118</v>
-      </c>
-      <c r="K32">
-        <v>1</v>
-      </c>
-      <c r="M32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O32">
+      <c r="I33">
+        <v>21</v>
+      </c>
+      <c r="J33" t="s">
+        <v>122</v>
+      </c>
+      <c r="K33">
+        <v>1</v>
+      </c>
+      <c r="M33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O33">
         <v>46300.75884768533</v>
       </c>
-      <c r="P32">
-        <v>46303.78902473875</v>
-      </c>
-      <c r="Q32" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17">
-      <c r="A33" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6">
+      <c r="P33">
+        <v>46305.20575261097</v>
+      </c>
+      <c r="Q33" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
+      <c r="A34" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" t="s">
+        <v>123</v>
+      </c>
+      <c r="E34" t="s">
+        <v>75</v>
+      </c>
+      <c r="G34">
         <v>0.92</v>
       </c>
-      <c r="H33" s="6">
-        <v>46302</v>
-      </c>
-      <c r="I33" s="6">
-        <v>-1</v>
-      </c>
-      <c r="J33" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="K33" s="6">
-        <v>1</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="M33" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N33" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O33" s="6">
-        <v>46300.7588564394</v>
-      </c>
-      <c r="P33" s="6">
-        <v>46303.78904116363</v>
-      </c>
-      <c r="Q33" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17">
-      <c r="A34" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C34" s="6" t="s">
+      <c r="H34" s="3">
+        <v>46332</v>
+      </c>
+      <c r="I34">
+        <v>27</v>
+      </c>
+      <c r="J34" t="s">
         <v>124</v>
       </c>
-      <c r="D34" s="6"/>
-      <c r="E34" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F34" s="6"/>
-      <c r="G34" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H34" s="6">
-        <v>46302</v>
-      </c>
-      <c r="I34" s="6">
-        <v>-1</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="K34" s="6">
-        <v>1</v>
-      </c>
-      <c r="L34" s="6"/>
-      <c r="M34" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N34" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O34" s="6">
-        <v>46300.75885647022</v>
-      </c>
-      <c r="P34" s="6">
-        <v>46303.78904117852</v>
-      </c>
-      <c r="Q34" s="5" t="s">
-        <v>60</v>
+      <c r="K34">
+        <v>4</v>
+      </c>
+      <c r="M34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N34" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O34">
+        <v>46305.20575257758</v>
+      </c>
+      <c r="P34">
+        <v>46305.2057525776</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="35" spans="1:17">
       <c r="A35" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F35" s="6" t="s">
-        <v>40</v>
-      </c>
+      <c r="F35" s="6"/>
       <c r="G35" s="6">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H35" s="6">
-        <v>46301</v>
+        <v>46304</v>
       </c>
       <c r="I35" s="6">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="K35" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L35" s="6"/>
       <c r="M35" s="6" t="s">
@@ -2601,21 +2612,21 @@
         <v>18</v>
       </c>
       <c r="O35" s="6">
-        <v>46300.75885649968</v>
+        <v>46300.75885634872</v>
       </c>
       <c r="P35" s="6">
-        <v>46303.78904122258</v>
+        <v>46305.20576919735</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:17">
       <c r="A36" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>128</v>
@@ -2626,13 +2637,13 @@
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6">
-        <v>0.92</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H36" s="6">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="I36" s="6">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="J36" s="6" t="s">
         <v>130</v>
@@ -2640,7 +2651,9 @@
       <c r="K36" s="6">
         <v>1</v>
       </c>
-      <c r="L36" s="6"/>
+      <c r="L36" s="6" t="s">
+        <v>131</v>
+      </c>
       <c r="M36" s="6" t="s">
         <v>18</v>
       </c>
@@ -2648,48 +2661,50 @@
         <v>18</v>
       </c>
       <c r="O36" s="6">
-        <v>46300.75886463693</v>
+        <v>46300.7588563655</v>
       </c>
       <c r="P36" s="6">
-        <v>46303.7890412799</v>
+        <v>46305.2057692078</v>
       </c>
       <c r="Q36" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>62</v>
+        <v>133</v>
       </c>
       <c r="G37" s="6">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H37" s="6">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="I37" s="6">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K37" s="6">
-        <v>1</v>
-      </c>
-      <c r="L37" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="L37" s="6" t="s">
+        <v>135</v>
+      </c>
       <c r="M37" s="6" t="s">
         <v>18</v>
       </c>
@@ -2697,47 +2712,47 @@
         <v>18</v>
       </c>
       <c r="O37" s="6">
-        <v>46300.75886465221</v>
+        <v>46300.7588564207</v>
       </c>
       <c r="P37" s="6">
-        <v>46303.78904125095</v>
+        <v>46305.2057692176</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6">
-        <v>0.2</v>
+        <v>0.92</v>
       </c>
       <c r="H38" s="6">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="I38" s="6">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>65</v>
+        <v>137</v>
       </c>
       <c r="K38" s="6">
         <v>1</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="M38" s="6" t="s">
         <v>18</v>
@@ -2746,43 +2761,41 @@
         <v>18</v>
       </c>
       <c r="O38" s="6">
-        <v>46300.75886466862</v>
+        <v>46300.7588564394</v>
       </c>
       <c r="P38" s="6">
-        <v>46303.78904129434</v>
-      </c>
-      <c r="Q38" s="5" t="s">
-        <v>60</v>
+        <v>46305.20576924799</v>
+      </c>
+      <c r="Q38" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>62</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="F39" s="6"/>
       <c r="G39" s="6">
-        <v>0.93</v>
+        <v>0.2</v>
       </c>
       <c r="H39" s="6">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="I39" s="6">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="K39" s="6">
         <v>1</v>
@@ -2795,44 +2808,46 @@
         <v>18</v>
       </c>
       <c r="O39" s="6">
-        <v>46300.75886468366</v>
+        <v>46300.75885647022</v>
       </c>
       <c r="P39" s="6">
-        <v>46303.78904130949</v>
-      </c>
-      <c r="Q39" s="6" t="s">
-        <v>24</v>
+        <v>46305.20576926682</v>
+      </c>
+      <c r="Q39" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F40" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>31</v>
+      </c>
       <c r="G40" s="6">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H40" s="6">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="I40" s="6">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="K40" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L40" s="6"/>
       <c r="M40" s="6" t="s">
@@ -2842,43 +2857,41 @@
         <v>18</v>
       </c>
       <c r="O40" s="6">
-        <v>46300.75886471466</v>
+        <v>46300.75885649968</v>
       </c>
       <c r="P40" s="6">
-        <v>46303.7890413381</v>
-      </c>
-      <c r="Q40" s="5" t="s">
-        <v>60</v>
+        <v>46305.20576929489</v>
+      </c>
+      <c r="Q40" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="41" spans="1:17">
       <c r="A41" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>21</v>
-      </c>
+        <v>144</v>
+      </c>
+      <c r="F41" s="6"/>
       <c r="G41" s="6">
-        <v>0.9399999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="H41" s="6">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="I41" s="6">
         <v>-5</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="K41" s="6">
         <v>1</v>
@@ -2891,48 +2904,48 @@
         <v>18</v>
       </c>
       <c r="O41" s="6">
-        <v>46300.75886472998</v>
+        <v>46300.75886463693</v>
       </c>
       <c r="P41" s="6">
-        <v>46303.78904942831</v>
+        <v>46305.20576932246</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="F42" s="6"/>
+        <v>25</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>53</v>
+      </c>
       <c r="G42" s="6">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="H42" s="6">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="I42" s="6">
         <v>-5</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="K42" s="6">
         <v>1</v>
       </c>
-      <c r="L42" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="L42" s="6"/>
       <c r="M42" s="6" t="s">
         <v>18</v>
       </c>
@@ -2940,46 +2953,48 @@
         <v>18</v>
       </c>
       <c r="O42" s="6">
-        <v>46300.75886474836</v>
+        <v>46300.75886465221</v>
       </c>
       <c r="P42" s="6">
-        <v>46303.78904135231</v>
+        <v>46305.20576930419</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6">
         <v>0.2</v>
       </c>
       <c r="H43" s="6">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="I43" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>146</v>
+        <v>56</v>
       </c>
       <c r="K43" s="6">
         <v>1</v>
       </c>
-      <c r="L43" s="6"/>
+      <c r="L43" s="6" t="s">
+        <v>149</v>
+      </c>
       <c r="M43" s="6" t="s">
         <v>18</v>
       </c>
@@ -2987,50 +3002,48 @@
         <v>18</v>
       </c>
       <c r="O43" s="6">
-        <v>46300.75886479358</v>
+        <v>46300.75886466862</v>
       </c>
       <c r="P43" s="6">
-        <v>46303.78904142418</v>
+        <v>46305.20576934127</v>
       </c>
       <c r="Q43" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="G44" s="6">
         <v>0.93</v>
       </c>
       <c r="H44" s="6">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="I44" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="K44" s="6">
         <v>1</v>
       </c>
-      <c r="L44" s="6" t="s">
-        <v>148</v>
-      </c>
+      <c r="L44" s="6"/>
       <c r="M44" s="6" t="s">
         <v>18</v>
       </c>
@@ -3038,48 +3051,46 @@
         <v>18</v>
       </c>
       <c r="O44" s="6">
-        <v>46300.75886484625</v>
+        <v>46300.75886468366</v>
       </c>
       <c r="P44" s="6">
-        <v>46303.78904138121</v>
+        <v>46305.20576933161</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="45" spans="1:17">
       <c r="A45" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6" t="s">
-        <v>142</v>
+        <v>49</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6">
-        <v>0.92</v>
+        <v>0.2</v>
       </c>
       <c r="H45" s="6">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="I45" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="K45" s="6">
         <v>1</v>
       </c>
-      <c r="L45" s="6" t="s">
-        <v>151</v>
-      </c>
+      <c r="L45" s="6"/>
       <c r="M45" s="6" t="s">
         <v>18</v>
       </c>
@@ -3087,48 +3098,48 @@
         <v>18</v>
       </c>
       <c r="O45" s="6">
-        <v>46300.75886486177</v>
+        <v>46300.75886471466</v>
       </c>
       <c r="P45" s="6">
-        <v>46303.78904944336</v>
-      </c>
-      <c r="Q45" s="6" t="s">
-        <v>24</v>
+        <v>46305.20577780272</v>
+      </c>
+      <c r="Q45" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="46" spans="1:17">
       <c r="A46" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F46" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>133</v>
+      </c>
       <c r="G46" s="6">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H46" s="6">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="I46" s="6">
         <v>-7</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K46" s="6">
         <v>1</v>
       </c>
-      <c r="L46" s="6" t="s">
-        <v>154</v>
-      </c>
+      <c r="L46" s="6"/>
       <c r="M46" s="6" t="s">
         <v>18</v>
       </c>
@@ -3136,46 +3147,48 @@
         <v>18</v>
       </c>
       <c r="O46" s="6">
-        <v>46300.75886487812</v>
+        <v>46300.75886472998</v>
       </c>
       <c r="P46" s="6">
-        <v>46303.78904946196</v>
+        <v>46303.78904942831</v>
       </c>
       <c r="Q46" s="5" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" spans="1:17">
       <c r="A47" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6" t="s">
-        <v>58</v>
+        <v>157</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="6">
-        <v>0.2</v>
+        <v>0.92</v>
       </c>
       <c r="H47" s="6">
-        <v>46294</v>
+        <v>46298</v>
       </c>
       <c r="I47" s="6">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="K47" s="6">
         <v>1</v>
       </c>
-      <c r="L47" s="6"/>
+      <c r="L47" s="6" t="s">
+        <v>159</v>
+      </c>
       <c r="M47" s="6" t="s">
         <v>18</v>
       </c>
@@ -3183,41 +3196,41 @@
         <v>18</v>
       </c>
       <c r="O47" s="6">
-        <v>46300.75887301003</v>
+        <v>46300.75886474836</v>
       </c>
       <c r="P47" s="6">
-        <v>46303.78904952588</v>
-      </c>
-      <c r="Q47" s="5" t="s">
-        <v>60</v>
+        <v>46305.20577781487</v>
+      </c>
+      <c r="Q47" s="6" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="48" spans="1:17">
       <c r="A48" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H48" s="6">
-        <v>46294</v>
+        <v>46298</v>
       </c>
       <c r="I48" s="6">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="K48" s="6">
         <v>1</v>
@@ -3230,46 +3243,48 @@
         <v>18</v>
       </c>
       <c r="O48" s="6">
-        <v>46300.75887304553</v>
+        <v>46300.75886479358</v>
       </c>
       <c r="P48" s="6">
-        <v>46303.78904954536</v>
-      </c>
-      <c r="Q48" s="6" t="s">
-        <v>24</v>
+        <v>46305.20576936999</v>
+      </c>
+      <c r="Q48" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="49" spans="1:17">
       <c r="A49" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6">
-        <v>0.87</v>
+        <v>0.92</v>
       </c>
       <c r="H49" s="6">
-        <v>46294</v>
+        <v>46297</v>
       </c>
       <c r="I49" s="6">
-        <v>-9</v>
+        <v>-8</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K49" s="6">
-        <v>2</v>
-      </c>
-      <c r="L49" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="L49" s="6" t="s">
+        <v>164</v>
+      </c>
       <c r="M49" s="6" t="s">
         <v>18</v>
       </c>
@@ -3277,47 +3292,47 @@
         <v>18</v>
       </c>
       <c r="O49" s="6">
-        <v>46300.75887306096</v>
+        <v>46300.75886486177</v>
       </c>
       <c r="P49" s="6">
-        <v>46303.7890495669</v>
+        <v>46305.20577787467</v>
       </c>
       <c r="Q49" s="6" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6">
-        <v>0.92</v>
+        <v>0.2</v>
       </c>
       <c r="H50" s="6">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="I50" s="6">
-        <v>-10</v>
+        <v>-9</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="K50" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="M50" s="6" t="s">
         <v>18</v>
@@ -3326,13 +3341,13 @@
         <v>18</v>
       </c>
       <c r="O50" s="6">
-        <v>46300.75887309557</v>
+        <v>46300.75886487812</v>
       </c>
       <c r="P50" s="6">
-        <v>46303.78904962536</v>
-      </c>
-      <c r="Q50" s="6" t="s">
-        <v>24</v>
+        <v>46305.20577788425</v>
+      </c>
+      <c r="Q50" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -3443,7 +3458,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3458,7 +3473,7 @@
     <col min="12" max="12" width="48.7109375" customWidth="1"/>
     <col min="13" max="14" width="12.7109375" customWidth="1"/>
     <col min="15" max="16" width="20.7109375" customWidth="1"/>
-    <col min="17" max="17" width="16.7109375" customWidth="1"/>
+    <col min="17" max="17" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -3522,26 +3537,29 @@
         <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="G2" s="2">
-        <v>0.2</v>
+        <v>0.91</v>
       </c>
       <c r="H2" s="3">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="I2" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>59</v>
+        <v>21</v>
       </c>
       <c r="K2" s="2">
         <v>1</v>
       </c>
+      <c r="L2" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="M2" s="4" t="s">
         <v>18</v>
       </c>
@@ -3549,13 +3567,13 @@
         <v>18</v>
       </c>
       <c r="O2" s="2">
-        <v>46300.7588479478</v>
+        <v>46300.75885633306</v>
       </c>
       <c r="P2" s="2">
-        <v>46303.78903307128</v>
+        <v>46303.78903317315</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="2" customFormat="1">
@@ -3566,10 +3584,10 @@
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G3" s="2">
         <v>0.2</v>
@@ -3578,17 +3596,14 @@
         <v>46307</v>
       </c>
       <c r="I3" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="K3" s="2">
         <v>1</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="M3" s="4" t="s">
         <v>18</v>
       </c>
@@ -3596,13 +3611,13 @@
         <v>18</v>
       </c>
       <c r="O3" s="2">
-        <v>46300.75884799581</v>
+        <v>46300.7588479478</v>
       </c>
       <c r="P3" s="2">
-        <v>46303.78903301315</v>
+        <v>46305.20576103318</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1">
@@ -3613,26 +3628,29 @@
         <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G4" s="2">
         <v>0.2</v>
       </c>
       <c r="H4" s="3">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="I4" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>78</v>
+        <v>56</v>
       </c>
       <c r="K4" s="2">
         <v>1</v>
       </c>
+      <c r="L4" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="M4" s="4" t="s">
         <v>18</v>
       </c>
@@ -3640,13 +3658,13 @@
         <v>18</v>
       </c>
       <c r="O4" s="2">
-        <v>46300.75884790152</v>
+        <v>46300.75884799581</v>
       </c>
       <c r="P4" s="2">
-        <v>46303.78902499317</v>
+        <v>46305.20576098546</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="2" customFormat="1">
@@ -3657,10 +3675,10 @@
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G5" s="2">
         <v>0.2</v>
@@ -3669,10 +3687,10 @@
         <v>46308</v>
       </c>
       <c r="I5" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="K5" s="2">
         <v>1</v>
@@ -3684,57 +3702,57 @@
         <v>18</v>
       </c>
       <c r="O5" s="2">
+        <v>46300.75884790152</v>
+      </c>
+      <c r="P5" s="2">
+        <v>46305.20576094543</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="2" customFormat="1">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="H6" s="3">
+        <v>46308</v>
+      </c>
+      <c r="I6" s="2">
+        <v>3</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="K6" s="2">
+        <v>1</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O6" s="2">
         <v>46301.38232480602</v>
       </c>
-      <c r="P5" s="2">
-        <v>46303.78902497852</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E6" t="s">
-        <v>58</v>
-      </c>
-      <c r="G6">
-        <v>0.2</v>
-      </c>
-      <c r="H6" s="3">
-        <v>46314</v>
-      </c>
-      <c r="I6">
-        <v>11</v>
-      </c>
-      <c r="J6" t="s">
-        <v>106</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O6">
-        <v>46300.75884775587</v>
-      </c>
-      <c r="P6">
-        <v>46303.7890248602</v>
+      <c r="P6" s="2">
+        <v>46305.20576093486</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -3745,22 +3763,22 @@
         <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G7">
         <v>0.2</v>
       </c>
       <c r="H7" s="3">
-        <v>46315</v>
+        <v>46314</v>
       </c>
       <c r="I7">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J7" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="K7">
         <v>1</v>
@@ -3772,13 +3790,13 @@
         <v>18</v>
       </c>
       <c r="O7">
-        <v>46300.75884772457</v>
+        <v>46300.75884775587</v>
       </c>
       <c r="P7">
-        <v>46303.78902481608</v>
+        <v>46305.20575276836</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -3789,28 +3807,25 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" s="3">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="I8">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>27</v>
+        <v>103</v>
       </c>
       <c r="K8">
-        <v>3</v>
-      </c>
-      <c r="L8" t="s">
-        <v>112</v>
+        <v>1</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>18</v>
@@ -3819,13 +3834,13 @@
         <v>18</v>
       </c>
       <c r="O8">
-        <v>46302.26841507768</v>
+        <v>46300.75884772457</v>
       </c>
       <c r="P8">
-        <v>46303.78902478614</v>
+        <v>46305.20575274854</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -3836,25 +3851,28 @@
         <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G9">
         <v>0.2</v>
       </c>
       <c r="H9" s="3">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="I9">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J9" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="K9">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L9" t="s">
+        <v>106</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -3863,13 +3881,13 @@
         <v>18</v>
       </c>
       <c r="O9">
-        <v>46301.38232468421</v>
+        <v>46302.26841507768</v>
       </c>
       <c r="P9">
-        <v>46303.7890247705</v>
+        <v>46305.20575272872</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -3880,122 +3898,117 @@
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="E10" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G10">
         <v>0.2</v>
       </c>
       <c r="H10" s="3">
+        <v>46317</v>
+      </c>
+      <c r="I10">
+        <v>12</v>
+      </c>
+      <c r="J10" t="s">
+        <v>108</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O10">
+        <v>46301.38232468421</v>
+      </c>
+      <c r="P10">
+        <v>46305.20575271807</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
+        <v>121</v>
+      </c>
+      <c r="E11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11">
+        <v>0.2</v>
+      </c>
+      <c r="H11" s="3">
         <v>46326</v>
       </c>
-      <c r="I10">
-        <v>23</v>
-      </c>
-      <c r="J10" t="s">
-        <v>118</v>
-      </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N10" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O10">
+      <c r="I11">
+        <v>21</v>
+      </c>
+      <c r="J11" t="s">
+        <v>122</v>
+      </c>
+      <c r="K11">
+        <v>1</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O11">
         <v>46300.75884768533</v>
       </c>
-      <c r="P10">
-        <v>46303.78902473875</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17">
-      <c r="A11" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="H11" s="6">
-        <v>46302</v>
-      </c>
-      <c r="I11" s="6">
-        <v>-1</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="K11" s="6">
-        <v>1</v>
-      </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O11" s="6">
-        <v>46300.75885647022</v>
-      </c>
-      <c r="P11" s="6">
-        <v>46303.78904117852</v>
+      <c r="P11">
+        <v>46305.20575261097</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6">
         <v>0.2</v>
       </c>
       <c r="H12" s="6">
-        <v>46299</v>
+        <v>46302</v>
       </c>
       <c r="I12" s="6">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>65</v>
+        <v>140</v>
       </c>
       <c r="K12" s="6">
         <v>1</v>
       </c>
-      <c r="L12" s="6" t="s">
-        <v>134</v>
-      </c>
+      <c r="L12" s="6"/>
       <c r="M12" s="6" t="s">
         <v>18</v>
       </c>
@@ -4003,46 +4016,48 @@
         <v>18</v>
       </c>
       <c r="O12" s="6">
-        <v>46300.75886466862</v>
+        <v>46300.75885647022</v>
       </c>
       <c r="P12" s="6">
-        <v>46303.78904129434</v>
+        <v>46305.20576926682</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6">
         <v>0.2</v>
       </c>
       <c r="H13" s="6">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="I13" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>138</v>
+        <v>56</v>
       </c>
       <c r="K13" s="6">
         <v>1</v>
       </c>
-      <c r="L13" s="6"/>
+      <c r="L13" s="6" t="s">
+        <v>149</v>
+      </c>
       <c r="M13" s="6" t="s">
         <v>18</v>
       </c>
@@ -4050,28 +4065,28 @@
         <v>18</v>
       </c>
       <c r="O13" s="6">
-        <v>46300.75886471466</v>
+        <v>46300.75886466862</v>
       </c>
       <c r="P13" s="6">
-        <v>46303.7890413381</v>
+        <v>46305.20576934127</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6">
@@ -4081,10 +4096,10 @@
         <v>46298</v>
       </c>
       <c r="I14" s="6">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="K14" s="6">
         <v>1</v>
@@ -4097,48 +4112,48 @@
         <v>18</v>
       </c>
       <c r="O14" s="6">
-        <v>46300.75886479358</v>
+        <v>46300.75886471466</v>
       </c>
       <c r="P14" s="6">
-        <v>46303.78904142418</v>
+        <v>46305.20577780272</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="F15" s="6"/>
+        <v>30</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>133</v>
+      </c>
       <c r="G15" s="6">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H15" s="6">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="I15" s="6">
         <v>-7</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K15" s="6">
         <v>1</v>
       </c>
-      <c r="L15" s="6" t="s">
-        <v>154</v>
-      </c>
+      <c r="L15" s="6"/>
       <c r="M15" s="6" t="s">
         <v>18</v>
       </c>
@@ -4146,41 +4161,41 @@
         <v>18</v>
       </c>
       <c r="O15" s="6">
-        <v>46300.75886487812</v>
+        <v>46300.75886472998</v>
       </c>
       <c r="P15" s="6">
-        <v>46303.78904946196</v>
+        <v>46303.78904942831</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6">
         <v>0.2</v>
       </c>
       <c r="H16" s="6">
-        <v>46294</v>
+        <v>46298</v>
       </c>
       <c r="I16" s="6">
-        <v>-9</v>
+        <v>-7</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="K16" s="6">
         <v>1</v>
@@ -4193,17 +4208,66 @@
         <v>18</v>
       </c>
       <c r="O16" s="6">
-        <v>46300.75887301003</v>
+        <v>46300.75886479358</v>
       </c>
       <c r="P16" s="6">
-        <v>46303.78904952588</v>
+        <v>46305.20576936999</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>60</v>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
+      <c r="A17" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="H17" s="6">
+        <v>46296</v>
+      </c>
+      <c r="I17" s="6">
+        <v>-9</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="K17" s="6">
+        <v>1</v>
+      </c>
+      <c r="L17" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="M17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O17" s="6">
+        <v>46300.75886487812</v>
+      </c>
+      <c r="P17" s="6">
+        <v>46305.20577788425</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:Q17"/>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1"/>
     <hyperlink ref="N2" r:id="rId2"/>
@@ -4235,6 +4299,8 @@
     <hyperlink ref="N15" r:id="rId28"/>
     <hyperlink ref="M16" r:id="rId29"/>
     <hyperlink ref="N16" r:id="rId30"/>
+    <hyperlink ref="M17" r:id="rId31"/>
+    <hyperlink ref="N17" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4242,7 +4308,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4252,86 +4318,86 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B2">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E2">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G2">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2">
         <v>0</v>
       </c>
       <c r="K2">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B3">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C3" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D3">
         <v>191</v>
@@ -4360,13 +4426,13 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B4">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D4">
         <v>191</v>
@@ -4378,7 +4444,7 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -4395,13 +4461,13 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B5">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D5">
         <v>191</v>
@@ -4410,16 +4476,16 @@
         <v>3820</v>
       </c>
       <c r="F5">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H5">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -4430,48 +4496,48 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B6">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D6">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E6">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F6">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G6">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H6">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B7">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C7" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D7">
         <v>8</v>
@@ -4480,13 +4546,13 @@
         <v>160</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -4495,18 +4561,18 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B8">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C8" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -4515,21 +4581,56 @@
         <v>160</v>
       </c>
       <c r="F8">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H8">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B9">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C9" t="s">
+        <v>179</v>
+      </c>
+      <c r="D9">
+        <v>8</v>
+      </c>
+      <c r="E9">
+        <v>160</v>
+      </c>
+      <c r="F9">
+        <v>157</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+      <c r="H9">
+        <v>132</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-10-0844Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="180">
   <si>
     <t>Priority</t>
   </si>
@@ -1123,7 +1123,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P3" s="2">
-        <v>46305.20576110142</v>
+        <v>46305.36274242896</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>28</v>
@@ -1173,7 +1173,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P4" s="2">
-        <v>46305.20576108179</v>
+        <v>46305.36274241605</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>28</v>
@@ -1223,7 +1223,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P5" s="2">
-        <v>46305.20576109179</v>
+        <v>46305.36274242261</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>28</v>
@@ -1270,7 +1270,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P6" s="2">
-        <v>46305.20576111179</v>
+        <v>46305.36274243537</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>28</v>
@@ -1320,7 +1320,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P7" s="2">
-        <v>46305.20576101432</v>
+        <v>46305.36274238358</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>28</v>
@@ -1364,7 +1364,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P8" s="2">
-        <v>46305.20576103318</v>
+        <v>46305.36274239628</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>51</v>
@@ -1411,7 +1411,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P9" s="2">
-        <v>46305.20576097554</v>
+        <v>46305.36274235664</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>28</v>
@@ -1458,7 +1458,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P10" s="2">
-        <v>46305.20576098546</v>
+        <v>46305.36274236323</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>51</v>
@@ -1502,7 +1502,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P11" s="2">
-        <v>46305.205761005</v>
+        <v>46305.36274237684</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>28</v>
@@ -1549,7 +1549,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P12" s="2">
-        <v>46305.20576099515</v>
+        <v>46305.36274237</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>28</v>
@@ -1599,7 +1599,7 @@
         <v>46305.20576106136</v>
       </c>
       <c r="P13" s="2">
-        <v>46305.20576106139</v>
+        <v>46305.36274240285</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>28</v>
@@ -1649,7 +1649,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P14" s="2">
-        <v>46305.20576095542</v>
+        <v>46305.36274234272</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>28</v>
@@ -1693,7 +1693,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P15" s="2">
-        <v>46305.20576094543</v>
+        <v>46305.36274233532</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>51</v>
@@ -1737,7 +1737,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P16" s="2">
-        <v>46305.20576093486</v>
+        <v>46305.36274232762</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>51</v>
@@ -1784,7 +1784,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P17" s="2">
-        <v>46305.20576092294</v>
+        <v>46305.36274231809</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>28</v>
@@ -1831,7 +1831,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P18" s="2">
-        <v>46305.20575279809</v>
+        <v>46305.36273430099</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>28</v>
@@ -1875,7 +1875,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P19" s="2">
-        <v>46305.20575282763</v>
+        <v>46305.36273432023</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>28</v>
@@ -1922,7 +1922,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P20" s="2">
-        <v>46305.20575281785</v>
+        <v>46305.36273431396</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>28</v>
@@ -1969,7 +1969,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P21" s="2">
-        <v>46305.20575280781</v>
+        <v>46305.36273430726</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>28</v>
@@ -2016,7 +2016,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P22">
-        <v>46305.20575278824</v>
+        <v>46305.36273429449</v>
       </c>
       <c r="Q22" t="s">
         <v>28</v>
@@ -2063,7 +2063,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P23">
-        <v>46305.20575275837</v>
+        <v>46305.36273427486</v>
       </c>
       <c r="Q23" t="s">
         <v>28</v>
@@ -2107,7 +2107,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P24">
-        <v>46305.20575276836</v>
+        <v>46305.36273428139</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>51</v>
@@ -2151,7 +2151,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P25">
-        <v>46305.20575277831</v>
+        <v>46305.36273428804</v>
       </c>
       <c r="Q25" t="s">
         <v>28</v>
@@ -2195,7 +2195,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P26">
-        <v>46305.20575274854</v>
+        <v>46305.36273426853</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>51</v>
@@ -2242,7 +2242,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P27">
-        <v>46305.20575272872</v>
+        <v>46305.36273425529</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>51</v>
@@ -2286,7 +2286,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P28">
-        <v>46305.20575271807</v>
+        <v>46305.36273424832</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>51</v>
@@ -2333,7 +2333,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P29">
-        <v>46305.20575270729</v>
+        <v>46305.36273424139</v>
       </c>
       <c r="Q29" t="s">
         <v>28</v>
@@ -2383,7 +2383,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P30">
-        <v>46305.20575267455</v>
+        <v>46305.36273422732</v>
       </c>
       <c r="Q30" t="s">
         <v>28</v>
@@ -2430,7 +2430,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P31">
-        <v>46305.20575269724</v>
+        <v>46305.36273423449</v>
       </c>
       <c r="Q31" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P32">
-        <v>46305.20575263904</v>
+        <v>46305.36273421974</v>
       </c>
       <c r="Q32" t="s">
         <v>28</v>
@@ -2524,7 +2524,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P33">
-        <v>46305.20575261097</v>
+        <v>46305.36273421196</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>51</v>
@@ -2568,7 +2568,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P34">
-        <v>46305.2057525776</v>
+        <v>46305.3627341853</v>
       </c>
       <c r="Q34" t="s">
         <v>28</v>
@@ -2615,7 +2615,7 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P35" s="6">
-        <v>46305.20576919735</v>
+        <v>46305.36275057897</v>
       </c>
       <c r="Q35" s="6" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P36" s="6">
-        <v>46305.2057692078</v>
+        <v>46305.36275058663</v>
       </c>
       <c r="Q36" s="6" t="s">
         <v>28</v>
@@ -2715,7 +2715,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P37" s="6">
-        <v>46305.2057692176</v>
+        <v>46305.36275059347</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>28</v>
@@ -2764,7 +2764,7 @@
         <v>46300.7588564394</v>
       </c>
       <c r="P38" s="6">
-        <v>46305.20576924799</v>
+        <v>46305.36275061421</v>
       </c>
       <c r="Q38" s="6" t="s">
         <v>28</v>
@@ -2811,7 +2811,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P39" s="6">
-        <v>46305.20576926682</v>
+        <v>46305.36275062726</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>51</v>
@@ -2860,7 +2860,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P40" s="6">
-        <v>46305.20576929489</v>
+        <v>46305.36275064632</v>
       </c>
       <c r="Q40" s="6" t="s">
         <v>28</v>
@@ -2907,7 +2907,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P41" s="6">
-        <v>46305.20576932246</v>
+        <v>46305.36275066455</v>
       </c>
       <c r="Q41" s="6" t="s">
         <v>28</v>
@@ -2956,7 +2956,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P42" s="6">
-        <v>46305.20576930419</v>
+        <v>46305.36275065236</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>28</v>
@@ -3005,7 +3005,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P43" s="6">
-        <v>46305.20576934127</v>
+        <v>46305.36275067714</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>51</v>
@@ -3054,7 +3054,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P44" s="6">
-        <v>46305.20576933161</v>
+        <v>46305.36275067061</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P45" s="6">
-        <v>46305.20577780272</v>
+        <v>46305.36275876115</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>51</v>
@@ -3199,7 +3199,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P47" s="6">
-        <v>46305.20577781487</v>
+        <v>46305.36275877042</v>
       </c>
       <c r="Q47" s="6" t="s">
         <v>28</v>
@@ -3246,7 +3246,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P48" s="6">
-        <v>46305.20576936999</v>
+        <v>46305.36275069558</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>51</v>
@@ -3295,7 +3295,7 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P49" s="6">
-        <v>46305.20577787467</v>
+        <v>46305.36275881311</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>28</v>
@@ -3344,7 +3344,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P50" s="6">
-        <v>46305.20577788425</v>
+        <v>46305.36275881966</v>
       </c>
       <c r="Q50" s="5" t="s">
         <v>51</v>
@@ -3614,7 +3614,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P3" s="2">
-        <v>46305.20576103318</v>
+        <v>46305.36274239628</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>51</v>
@@ -3661,7 +3661,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P4" s="2">
-        <v>46305.20576098546</v>
+        <v>46305.36274236323</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>51</v>
@@ -3705,7 +3705,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P5" s="2">
-        <v>46305.20576094543</v>
+        <v>46305.36274233532</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>51</v>
@@ -3749,7 +3749,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P6" s="2">
-        <v>46305.20576093486</v>
+        <v>46305.36274232762</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>51</v>
@@ -3793,7 +3793,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P7">
-        <v>46305.20575276836</v>
+        <v>46305.36273428139</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>51</v>
@@ -3837,7 +3837,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P8">
-        <v>46305.20575274854</v>
+        <v>46305.36273426853</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>51</v>
@@ -3884,7 +3884,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P9">
-        <v>46305.20575272872</v>
+        <v>46305.36273425529</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>51</v>
@@ -3928,7 +3928,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P10">
-        <v>46305.20575271807</v>
+        <v>46305.36273424832</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>51</v>
@@ -3972,7 +3972,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P11">
-        <v>46305.20575261097</v>
+        <v>46305.36273421196</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>51</v>
@@ -4019,7 +4019,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P12" s="6">
-        <v>46305.20576926682</v>
+        <v>46305.36275062726</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>51</v>
@@ -4068,7 +4068,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P13" s="6">
-        <v>46305.20576934127</v>
+        <v>46305.36275067714</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>51</v>
@@ -4115,7 +4115,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P14" s="6">
-        <v>46305.20577780272</v>
+        <v>46305.36275876115</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>51</v>
@@ -4211,7 +4211,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P16" s="6">
-        <v>46305.20576936999</v>
+        <v>46305.36275069558</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>51</v>
@@ -4260,7 +4260,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P17" s="6">
-        <v>46305.20577788425</v>
+        <v>46305.36275881966</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>51</v>
@@ -4308,7 +4308,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4356,10 +4356,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B2">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C2" t="s">
         <v>179</v>
@@ -4371,16 +4371,16 @@
         <v>3826</v>
       </c>
       <c r="F2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -4391,45 +4391,45 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B3">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C3" t="s">
         <v>179</v>
       </c>
       <c r="D3">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E3">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G3">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B4">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C4" t="s">
         <v>179</v>
@@ -4461,10 +4461,10 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B5">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C5" t="s">
         <v>179</v>
@@ -4479,7 +4479,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -4496,10 +4496,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B6">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C6" t="s">
         <v>179</v>
@@ -4511,16 +4511,16 @@
         <v>3820</v>
       </c>
       <c r="F6">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H6">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -4531,45 +4531,45 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B7">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C7" t="s">
         <v>179</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E7">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G7">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H7">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B8">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C8" t="s">
         <v>179</v>
@@ -4581,13 +4581,13 @@
         <v>160</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -4596,15 +4596,15 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B9">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C9" t="s">
         <v>179</v>
@@ -4616,21 +4616,56 @@
         <v>160</v>
       </c>
       <c r="F9">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H9">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B10">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C10" t="s">
+        <v>179</v>
+      </c>
+      <c r="D10">
+        <v>8</v>
+      </c>
+      <c r="E10">
+        <v>160</v>
+      </c>
+      <c r="F10">
+        <v>157</v>
+      </c>
+      <c r="G10">
+        <v>3</v>
+      </c>
+      <c r="H10">
+        <v>132</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-10-1726Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="180">
   <si>
     <t>Priority</t>
   </si>
@@ -1123,7 +1123,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P3" s="2">
-        <v>46305.36274242896</v>
+        <v>46305.72545435187</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>28</v>
@@ -1173,7 +1173,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P4" s="2">
-        <v>46305.36274241605</v>
+        <v>46305.72545433335</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>28</v>
@@ -1223,7 +1223,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P5" s="2">
-        <v>46305.36274242261</v>
+        <v>46305.72545434292</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>28</v>
@@ -1270,7 +1270,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P6" s="2">
-        <v>46305.36274243537</v>
+        <v>46305.72545436121</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>28</v>
@@ -1320,7 +1320,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P7" s="2">
-        <v>46305.36274238358</v>
+        <v>46305.72545428615</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>28</v>
@@ -1364,7 +1364,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P8" s="2">
-        <v>46305.36274239628</v>
+        <v>46305.72545430451</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>51</v>
@@ -1411,7 +1411,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P9" s="2">
-        <v>46305.36274235664</v>
+        <v>46305.7254542472</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>28</v>
@@ -1458,7 +1458,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P10" s="2">
-        <v>46305.36274236323</v>
+        <v>46305.72545425688</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>51</v>
@@ -1502,7 +1502,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P11" s="2">
-        <v>46305.36274237684</v>
+        <v>46305.72545427667</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>28</v>
@@ -1549,7 +1549,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P12" s="2">
-        <v>46305.36274237</v>
+        <v>46305.72545426671</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>28</v>
@@ -1599,7 +1599,7 @@
         <v>46305.20576106136</v>
       </c>
       <c r="P13" s="2">
-        <v>46305.36274240285</v>
+        <v>46305.72545431391</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>28</v>
@@ -1649,7 +1649,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P14" s="2">
-        <v>46305.36274234272</v>
+        <v>46305.72545422736</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>28</v>
@@ -1693,7 +1693,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P15" s="2">
-        <v>46305.36274233532</v>
+        <v>46305.72545421727</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>51</v>
@@ -1737,7 +1737,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P16" s="2">
-        <v>46305.36274232762</v>
+        <v>46305.72545420671</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>51</v>
@@ -1784,7 +1784,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P17" s="2">
-        <v>46305.36274231809</v>
+        <v>46305.72545419462</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>28</v>
@@ -1831,7 +1831,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P18" s="2">
-        <v>46305.36273430099</v>
+        <v>46305.72544558345</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>28</v>
@@ -1875,7 +1875,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P19" s="2">
-        <v>46305.36273432023</v>
+        <v>46305.72544561344</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>28</v>
@@ -1922,7 +1922,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P20" s="2">
-        <v>46305.36273431396</v>
+        <v>46305.72544560267</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>28</v>
@@ -1969,7 +1969,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P21" s="2">
-        <v>46305.36273430726</v>
+        <v>46305.72544559299</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>28</v>
@@ -2016,7 +2016,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P22">
-        <v>46305.36273429449</v>
+        <v>46305.72544557391</v>
       </c>
       <c r="Q22" t="s">
         <v>28</v>
@@ -2063,7 +2063,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P23">
-        <v>46305.36273427486</v>
+        <v>46305.72544554438</v>
       </c>
       <c r="Q23" t="s">
         <v>28</v>
@@ -2107,7 +2107,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P24">
-        <v>46305.36273428139</v>
+        <v>46305.72544555414</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>51</v>
@@ -2151,7 +2151,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P25">
-        <v>46305.36273428804</v>
+        <v>46305.72544556411</v>
       </c>
       <c r="Q25" t="s">
         <v>28</v>
@@ -2195,7 +2195,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P26">
-        <v>46305.36273426853</v>
+        <v>46305.72544553479</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>51</v>
@@ -2242,7 +2242,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P27">
-        <v>46305.36273425529</v>
+        <v>46305.7254455155</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>51</v>
@@ -2286,7 +2286,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P28">
-        <v>46305.36273424832</v>
+        <v>46305.72544550539</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>51</v>
@@ -2333,7 +2333,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P29">
-        <v>46305.36273424139</v>
+        <v>46305.7254454951</v>
       </c>
       <c r="Q29" t="s">
         <v>28</v>
@@ -2383,7 +2383,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P30">
-        <v>46305.36273422732</v>
+        <v>46305.72544547343</v>
       </c>
       <c r="Q30" t="s">
         <v>28</v>
@@ -2430,7 +2430,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P31">
-        <v>46305.36273423449</v>
+        <v>46305.72544548448</v>
       </c>
       <c r="Q31" t="s">
         <v>28</v>
@@ -2480,7 +2480,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P32">
-        <v>46305.36273421974</v>
+        <v>46305.72544546242</v>
       </c>
       <c r="Q32" t="s">
         <v>28</v>
@@ -2524,7 +2524,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P33">
-        <v>46305.36273421196</v>
+        <v>46305.72544545171</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>51</v>
@@ -2568,7 +2568,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P34">
-        <v>46305.3627341853</v>
+        <v>46305.72544541569</v>
       </c>
       <c r="Q34" t="s">
         <v>28</v>
@@ -2615,7 +2615,7 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P35" s="6">
-        <v>46305.36275057897</v>
+        <v>46305.72546245658</v>
       </c>
       <c r="Q35" s="6" t="s">
         <v>28</v>
@@ -2664,7 +2664,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P36" s="6">
-        <v>46305.36275058663</v>
+        <v>46305.72546246747</v>
       </c>
       <c r="Q36" s="6" t="s">
         <v>28</v>
@@ -2715,7 +2715,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P37" s="6">
-        <v>46305.36275059347</v>
+        <v>46305.72546247725</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>28</v>
@@ -2764,7 +2764,7 @@
         <v>46300.7588564394</v>
       </c>
       <c r="P38" s="6">
-        <v>46305.36275061421</v>
+        <v>46305.7254625063</v>
       </c>
       <c r="Q38" s="6" t="s">
         <v>28</v>
@@ -2811,7 +2811,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P39" s="6">
-        <v>46305.36275062726</v>
+        <v>46305.7254625255</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>51</v>
@@ -2860,7 +2860,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P40" s="6">
-        <v>46305.36275064632</v>
+        <v>46305.72546255367</v>
       </c>
       <c r="Q40" s="6" t="s">
         <v>28</v>
@@ -2907,7 +2907,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P41" s="6">
-        <v>46305.36275066455</v>
+        <v>46305.72546258115</v>
       </c>
       <c r="Q41" s="6" t="s">
         <v>28</v>
@@ -2956,7 +2956,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P42" s="6">
-        <v>46305.36275065236</v>
+        <v>46305.72546256285</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>28</v>
@@ -3005,7 +3005,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P43" s="6">
-        <v>46305.36275067714</v>
+        <v>46305.72546260039</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>51</v>
@@ -3054,7 +3054,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P44" s="6">
-        <v>46305.36275067061</v>
+        <v>46305.72546259048</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>28</v>
@@ -3101,7 +3101,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P45" s="6">
-        <v>46305.36275876115</v>
+        <v>46305.72547073589</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>51</v>
@@ -3199,7 +3199,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P47" s="6">
-        <v>46305.36275877042</v>
+        <v>46305.72547074813</v>
       </c>
       <c r="Q47" s="6" t="s">
         <v>28</v>
@@ -3246,7 +3246,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P48" s="6">
-        <v>46305.36275069558</v>
+        <v>46305.72546262942</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>51</v>
@@ -3295,7 +3295,7 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P49" s="6">
-        <v>46305.36275881311</v>
+        <v>46305.72547080749</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>28</v>
@@ -3344,7 +3344,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P50" s="6">
-        <v>46305.36275881966</v>
+        <v>46305.72547081784</v>
       </c>
       <c r="Q50" s="5" t="s">
         <v>51</v>
@@ -3614,7 +3614,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P3" s="2">
-        <v>46305.36274239628</v>
+        <v>46305.72545430451</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>51</v>
@@ -3661,7 +3661,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P4" s="2">
-        <v>46305.36274236323</v>
+        <v>46305.72545425688</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>51</v>
@@ -3705,7 +3705,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P5" s="2">
-        <v>46305.36274233532</v>
+        <v>46305.72545421727</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>51</v>
@@ -3749,7 +3749,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P6" s="2">
-        <v>46305.36274232762</v>
+        <v>46305.72545420671</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>51</v>
@@ -3793,7 +3793,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P7">
-        <v>46305.36273428139</v>
+        <v>46305.72544555414</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>51</v>
@@ -3837,7 +3837,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P8">
-        <v>46305.36273426853</v>
+        <v>46305.72544553479</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>51</v>
@@ -3884,7 +3884,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P9">
-        <v>46305.36273425529</v>
+        <v>46305.7254455155</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>51</v>
@@ -3928,7 +3928,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P10">
-        <v>46305.36273424832</v>
+        <v>46305.72544550539</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>51</v>
@@ -3972,7 +3972,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P11">
-        <v>46305.36273421196</v>
+        <v>46305.72544545171</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>51</v>
@@ -4019,7 +4019,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P12" s="6">
-        <v>46305.36275062726</v>
+        <v>46305.7254625255</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>51</v>
@@ -4068,7 +4068,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P13" s="6">
-        <v>46305.36275067714</v>
+        <v>46305.72546260039</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>51</v>
@@ -4115,7 +4115,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P14" s="6">
-        <v>46305.36275876115</v>
+        <v>46305.72547073589</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>51</v>
@@ -4211,7 +4211,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P16" s="6">
-        <v>46305.36275069558</v>
+        <v>46305.72546262942</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>51</v>
@@ -4260,7 +4260,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P17" s="6">
-        <v>46305.36275881966</v>
+        <v>46305.72547081784</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>51</v>
@@ -4308,7 +4308,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4356,10 +4356,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B2">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C2" t="s">
         <v>179</v>
@@ -4391,10 +4391,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B3">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C3" t="s">
         <v>179</v>
@@ -4406,16 +4406,16 @@
         <v>3826</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -4426,45 +4426,45 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B4">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C4" t="s">
         <v>179</v>
       </c>
       <c r="D4">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E4">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G4">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B5">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C5" t="s">
         <v>179</v>
@@ -4496,10 +4496,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B6">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C6" t="s">
         <v>179</v>
@@ -4514,7 +4514,7 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -4531,10 +4531,10 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B7">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C7" t="s">
         <v>179</v>
@@ -4546,16 +4546,16 @@
         <v>3820</v>
       </c>
       <c r="F7">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H7">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -4566,45 +4566,45 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B8">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C8" t="s">
         <v>179</v>
       </c>
       <c r="D8">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E8">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G8">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B9">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C9" t="s">
         <v>179</v>
@@ -4616,13 +4616,13 @@
         <v>160</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G9">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -4631,15 +4631,15 @@
         <v>0</v>
       </c>
       <c r="K9">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B10">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C10" t="s">
         <v>179</v>
@@ -4651,21 +4651,56 @@
         <v>160</v>
       </c>
       <c r="F10">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H10">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B11">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C11" t="s">
+        <v>179</v>
+      </c>
+      <c r="D11">
+        <v>8</v>
+      </c>
+      <c r="E11">
+        <v>160</v>
+      </c>
+      <c r="F11">
+        <v>157</v>
+      </c>
+      <c r="G11">
+        <v>3</v>
+      </c>
+      <c r="H11">
+        <v>132</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-11-1050Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="180">
   <si>
     <t>Priority</t>
   </si>
@@ -79,12 +79,321 @@
     <t>Open</t>
   </si>
   <si>
+    <t>REAL TECH CONSTRUCTIONS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Realty / Construction</t>
+  </si>
+  <si>
+    <t>Construction / EPC</t>
+  </si>
+  <si>
+    <t>Manindra Kumar Tiwari</t>
+  </si>
+  <si>
+    <t>Auto-classified</t>
+  </si>
+  <si>
+    <t>A.P.J. LABORATORIES LIMITED</t>
+  </si>
+  <si>
+    <t>Pharma / Healthcare</t>
+  </si>
+  <si>
+    <t>Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>pooja damir miglani</t>
+  </si>
+  <si>
+    <t>No Fixed Assets are available, except one disputed and contiguous piece of land at Village Ambwala, Nwada Road Tehsil Paonta Sahib, Distt Sirmaur, Himachal Pradesh, India, 173025</t>
+  </si>
+  <si>
+    <t>ALLFLEX PLASTIC LLP</t>
+  </si>
+  <si>
+    <t>Chemicals</t>
+  </si>
+  <si>
+    <t>Plastics / Polymers</t>
+  </si>
+  <si>
+    <t>Mr. Hansraj Jaria</t>
+  </si>
+  <si>
+    <t>At present, the Corporate Debtor is not operational and not a going concern. Revenue from Operation for the financial year ended 31.03.2025 is ?44,98,79,958.90</t>
+  </si>
+  <si>
+    <t>LOG 9 MATERIALS SCIENTIFIC PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Power / Energy</t>
+  </si>
+  <si>
+    <t>Mrs. Neeraja Kartik</t>
+  </si>
+  <si>
+    <t>250 MWh battery production capacity and 50 MWh cell production capacity</t>
+  </si>
+  <si>
+    <t>TECHNOFAB ENGINEERING LIMITED</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>Engineering</t>
+  </si>
+  <si>
+    <t>Rahul Jindal</t>
+  </si>
+  <si>
+    <t>The Form G has been published on 27.09.2026 in newspapers all over India.</t>
+  </si>
+  <si>
+    <t>STC VENTURES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Other / Unclear</t>
+  </si>
+  <si>
+    <t>PURUSOTTAM BEHERA</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>VIGNESHWARA DEVELOPERS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Real Estate</t>
+  </si>
+  <si>
+    <t>Ms. Ritu Rastogi</t>
+  </si>
+  <si>
+    <t>EXTOL INDUSTRIES LIMITED</t>
+  </si>
+  <si>
+    <t>Ms. Teena Saraswat Pandey</t>
+  </si>
+  <si>
+    <t>unit closed, no employees / no workmen at CIRP commencement date</t>
+  </si>
+  <si>
+    <t>SURYA FOUNDRY PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Steel / Metals</t>
+  </si>
+  <si>
+    <t>Mr. Reetesh Kumar Agarwal</t>
+  </si>
+  <si>
+    <t>XYRON TECHNOLOGIES LIMITED</t>
+  </si>
+  <si>
+    <t>IT / Technology</t>
+  </si>
+  <si>
+    <t>unit closed As Per Information available no employees / No workmen at the commencement of CIRP Process</t>
+  </si>
+  <si>
+    <t>N KUMAR RETAILS &amp; PROPERTIES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mrs. Megha Agrawal</t>
+  </si>
+  <si>
+    <t>(Under sub-regulation (1) of regulation 36A of the Insolvency and Bankruptcy Board of India (Insolvency Resolution Process for Corporate Persons) Regulations, 2016), this corrigendum is being issued in respect of the Form G published on 18.09.2026 invitin</t>
+  </si>
+  <si>
+    <t>VAS INFRASTRUCTURE LIMITED (CN)</t>
+  </si>
+  <si>
+    <t>Infrastructure</t>
+  </si>
+  <si>
+    <t>Infrastructure / EPC</t>
+  </si>
+  <si>
+    <t>Mr. Bimal Kumar Agarwal</t>
+  </si>
+  <si>
+    <t>The Form G has been published on 28.09.2026.</t>
+  </si>
+  <si>
+    <t>TV VISION LIMITED</t>
+  </si>
+  <si>
+    <t>ALOK KUMAR MURARKA</t>
+  </si>
+  <si>
+    <t>INDO PACIFIC PROJECTS LIMITED</t>
+  </si>
+  <si>
+    <t>BHUBANESHWARI SEAFOOD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Agriculture / Food</t>
+  </si>
+  <si>
+    <t>Tripti Agarwal</t>
+  </si>
+  <si>
+    <t>As per the latest available audited financial statement the Turnover in financial year 2022-2023 was Rs. 91.98 crore</t>
+  </si>
+  <si>
+    <t>GOODWILL IRON &amp; STEEL TRADERS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>MANISH AGARWALLA</t>
+  </si>
+  <si>
+    <t>Fixed assets location are taken as per the latest audited balance sheet &amp; address mention as D3/1401 NOIDA Extension .No documents and details are received from the Suspended Board of Directors. Section 19(2) application filed with the Hon'ble NC</t>
+  </si>
+  <si>
+    <t>COMET GRANITO PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Cement / Building Materials</t>
+  </si>
+  <si>
+    <t>Anil Kashi Drolia</t>
+  </si>
+  <si>
+    <t>VAASUDEVA MILK FOODS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ATKURU SAI PRASAD</t>
+  </si>
+  <si>
+    <t>Form-G Issued</t>
+  </si>
+  <si>
+    <t>M/s Margdarshak Financial Services Limited</t>
+  </si>
+  <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
+    <t>Rakesh Kumar Jindal</t>
+  </si>
+  <si>
+    <t>Form G was published for the third time with the approval of the CoC and the NCLT.</t>
+  </si>
+  <si>
+    <t>IN2IT TECHNOLOGIES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ishant jain</t>
+  </si>
+  <si>
+    <t>Re-issuance of Form G: Form G was re-issued on 17.09.2026, with 03.10.2026 as the last date for submission of EOI. Pursuant to the directions of the CoC, an Addendum to Form G was issued, revising and extending the stipulated timelines accordingly.</t>
+  </si>
+  <si>
+    <t>KM TOLL ROAD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Roads / Toll Roads</t>
+  </si>
+  <si>
+    <t>Roads / Highways</t>
+  </si>
+  <si>
+    <t>Mr. Ashish Saoji</t>
+  </si>
+  <si>
+    <t>ORGANIC WORLD PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Prakul Thadi</t>
+  </si>
+  <si>
+    <t>SUN GRANITE EXPORT LIMITED</t>
+  </si>
+  <si>
+    <t>Raghunath Bhandari</t>
+  </si>
+  <si>
+    <t>SHRENIK LIMITED</t>
+  </si>
+  <si>
+    <t>RAHUL SHAH</t>
+  </si>
+  <si>
+    <t>OMKARA VIJAYALAKSHMI STRIPS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Neha Jain Nemani</t>
+  </si>
+  <si>
+    <t>A fresh Form-G is issued upon taking approval from the CoC on 6th October 2026. The last day for submission of EOI is 21st October 2026.</t>
+  </si>
+  <si>
+    <t>G &amp; L PROFILE AND EQUIPMENTS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Manish Kumar Bhagat</t>
+  </si>
+  <si>
+    <t>SOCRUS PHARMACEUTICALS LIMITED</t>
+  </si>
+  <si>
+    <t>kuldeep tank</t>
+  </si>
+  <si>
+    <t>Sion Panvel Tollways Private Limited</t>
+  </si>
+  <si>
+    <t>Mr. Sanjay Kumar Mishra</t>
+  </si>
+  <si>
+    <t>1. Since CD is in business of road construction, there are no major tangible assets available; 2. No employee on the rolls of CD since ICD; 3. Current Form G is pursuant to NCLT order - 29 Sept'26 and 59th CoC meeting on 06 Oct'26.</t>
+  </si>
+  <si>
+    <t>AXLE PAPER PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>Mr. Kailash Shah</t>
+  </si>
+  <si>
+    <t>The installed capacity of main Products is 150MTPD.</t>
+  </si>
+  <si>
+    <t>Raheja Developers Limited - Revanta Project</t>
+  </si>
+  <si>
+    <t>Mr. Surendra Raj Gang</t>
+  </si>
+  <si>
+    <t>The CoC in its 4th meeting has resolved to scrap the earlier EOI process pursuant to Form-G dated 03 September 2026 and publish the current invitation for EOI for submission of Resolution Plans. The details of product are available in attached document.</t>
+  </si>
+  <si>
+    <t>PRATHAM-HEERA SALES PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Mahesh Goverdhan Bagla</t>
+  </si>
+  <si>
+    <t>SIMARA FOODS PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>Mr. Navin Khandelwal</t>
+  </si>
+  <si>
+    <t>Recently closed</t>
+  </si>
+  <si>
+    <t>Closed recently</t>
+  </si>
+  <si>
     <t>INFO-DRIVE SOFTWARE LIMITED</t>
   </si>
   <si>
-    <t>IT / Technology</t>
-  </si>
-  <si>
     <t>Sumeet Surendra Chimbalkar</t>
   </si>
   <si>
@@ -92,315 +401,6 @@
   </si>
   <si>
     <t>Not in latest IBBI listing - verify with RP</t>
-  </si>
-  <si>
-    <t>REAL TECH CONSTRUCTIONS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Realty / Construction</t>
-  </si>
-  <si>
-    <t>Construction / EPC</t>
-  </si>
-  <si>
-    <t>Manindra Kumar Tiwari</t>
-  </si>
-  <si>
-    <t>Auto-classified</t>
-  </si>
-  <si>
-    <t>A.P.J. LABORATORIES LIMITED</t>
-  </si>
-  <si>
-    <t>Pharma / Healthcare</t>
-  </si>
-  <si>
-    <t>Pharmaceuticals</t>
-  </si>
-  <si>
-    <t>pooja damir miglani</t>
-  </si>
-  <si>
-    <t>No Fixed Assets are available, except one disputed and contiguous piece of land at Village Ambwala, Nwada Road Tehsil Paonta Sahib, Distt Sirmaur, Himachal Pradesh, India, 173025</t>
-  </si>
-  <si>
-    <t>ALLFLEX PLASTIC LLP</t>
-  </si>
-  <si>
-    <t>Chemicals</t>
-  </si>
-  <si>
-    <t>Plastics / Polymers</t>
-  </si>
-  <si>
-    <t>Mr. Hansraj Jaria</t>
-  </si>
-  <si>
-    <t>At present, the Corporate Debtor is not operational and not a going concern. Revenue from Operation for the financial year ended 31.03.2025 is ?44,98,79,958.90</t>
-  </si>
-  <si>
-    <t>LOG 9 MATERIALS SCIENTIFIC PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Power / Energy</t>
-  </si>
-  <si>
-    <t>Mrs. Neeraja Kartik</t>
-  </si>
-  <si>
-    <t>250 MWh battery production capacity and 50 MWh cell production capacity</t>
-  </si>
-  <si>
-    <t>TECHNOFAB ENGINEERING LIMITED</t>
-  </si>
-  <si>
-    <t>Manufacturing</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>Rahul Jindal</t>
-  </si>
-  <si>
-    <t>The Form G has been published on 27.09.2026 in newspapers all over India.</t>
-  </si>
-  <si>
-    <t>STC VENTURES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Other / Unclear</t>
-  </si>
-  <si>
-    <t>PURUSOTTAM BEHERA</t>
-  </si>
-  <si>
-    <t>Review</t>
-  </si>
-  <si>
-    <t>VIGNESHWARA DEVELOPERS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Real Estate</t>
-  </si>
-  <si>
-    <t>Ms. Ritu Rastogi</t>
-  </si>
-  <si>
-    <t>EXTOL INDUSTRIES LIMITED</t>
-  </si>
-  <si>
-    <t>Ms. Teena Saraswat Pandey</t>
-  </si>
-  <si>
-    <t>unit closed, no employees / no workmen at CIRP commencement date</t>
-  </si>
-  <si>
-    <t>SURYA FOUNDRY PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Steel / Metals</t>
-  </si>
-  <si>
-    <t>Mr. Reetesh Kumar Agarwal</t>
-  </si>
-  <si>
-    <t>XYRON TECHNOLOGIES LIMITED</t>
-  </si>
-  <si>
-    <t>unit closed As Per Information available no employees / No workmen at the commencement of CIRP Process</t>
-  </si>
-  <si>
-    <t>N KUMAR RETAILS &amp; PROPERTIES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mrs. Megha Agrawal</t>
-  </si>
-  <si>
-    <t>(Under sub-regulation (1) of regulation 36A of the Insolvency and Bankruptcy Board of India (Insolvency Resolution Process for Corporate Persons) Regulations, 2016), this corrigendum is being issued in respect of the Form G published on 18.09.2026 invitin</t>
-  </si>
-  <si>
-    <t>VAS INFRASTRUCTURE LIMITED (CN)</t>
-  </si>
-  <si>
-    <t>Infrastructure</t>
-  </si>
-  <si>
-    <t>Infrastructure / EPC</t>
-  </si>
-  <si>
-    <t>Mr. Bimal Kumar Agarwal</t>
-  </si>
-  <si>
-    <t>The Form G has been published on 28.09.2026.</t>
-  </si>
-  <si>
-    <t>TV VISION LIMITED</t>
-  </si>
-  <si>
-    <t>ALOK KUMAR MURARKA</t>
-  </si>
-  <si>
-    <t>INDO PACIFIC PROJECTS LIMITED</t>
-  </si>
-  <si>
-    <t>BHUBANESHWARI SEAFOOD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Agriculture / Food</t>
-  </si>
-  <si>
-    <t>Tripti Agarwal</t>
-  </si>
-  <si>
-    <t>As per the latest available audited financial statement the Turnover in financial year 2022-2023 was Rs. 91.98 crore</t>
-  </si>
-  <si>
-    <t>GOODWILL IRON &amp; STEEL TRADERS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>MANISH AGARWALLA</t>
-  </si>
-  <si>
-    <t>Fixed assets location are taken as per the latest audited balance sheet &amp; address mention as D3/1401 NOIDA Extension .No documents and details are received from the Suspended Board of Directors. Section 19(2) application filed with the Hon'ble NC</t>
-  </si>
-  <si>
-    <t>COMET GRANITO PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Cement / Building Materials</t>
-  </si>
-  <si>
-    <t>Anil Kashi Drolia</t>
-  </si>
-  <si>
-    <t>VAASUDEVA MILK FOODS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>ATKURU SAI PRASAD</t>
-  </si>
-  <si>
-    <t>Form-G Issued</t>
-  </si>
-  <si>
-    <t>M/s Margdarshak Financial Services Limited</t>
-  </si>
-  <si>
-    <t>Financial Services</t>
-  </si>
-  <si>
-    <t>Rakesh Kumar Jindal</t>
-  </si>
-  <si>
-    <t>Form G was published for the third time with the approval of the CoC and the NCLT.</t>
-  </si>
-  <si>
-    <t>IN2IT TECHNOLOGIES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>ishant jain</t>
-  </si>
-  <si>
-    <t>Re-issuance of Form G: Form G was re-issued on 17.09.2026, with 03.10.2026 as the last date for submission of EOI. Pursuant to the directions of the CoC, an Addendum to Form G was issued, revising and extending the stipulated timelines accordingly.</t>
-  </si>
-  <si>
-    <t>KM TOLL ROAD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Roads / Toll Roads</t>
-  </si>
-  <si>
-    <t>Roads / Highways</t>
-  </si>
-  <si>
-    <t>Mr. Ashish Saoji</t>
-  </si>
-  <si>
-    <t>ORGANIC WORLD PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Prakul Thadi</t>
-  </si>
-  <si>
-    <t>SUN GRANITE EXPORT LIMITED</t>
-  </si>
-  <si>
-    <t>Raghunath Bhandari</t>
-  </si>
-  <si>
-    <t>SHRENIK LIMITED</t>
-  </si>
-  <si>
-    <t>RAHUL SHAH</t>
-  </si>
-  <si>
-    <t>OMKARA VIJAYALAKSHMI STRIPS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Neha Jain Nemani</t>
-  </si>
-  <si>
-    <t>A fresh Form-G is issued upon taking approval from the CoC on 6th October 2026. The last day for submission of EOI is 21st October 2026.</t>
-  </si>
-  <si>
-    <t>G &amp; L PROFILE AND EQUIPMENTS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Manish Kumar Bhagat</t>
-  </si>
-  <si>
-    <t>SOCRUS PHARMACEUTICALS LIMITED</t>
-  </si>
-  <si>
-    <t>kuldeep tank</t>
-  </si>
-  <si>
-    <t>Sion Panvel Tollways Private Limited</t>
-  </si>
-  <si>
-    <t>Mr. Sanjay Kumar Mishra</t>
-  </si>
-  <si>
-    <t>1. Since CD is in business of road construction, there are no major tangible assets available; 2. No employee on the rolls of CD since ICD; 3. Current Form G is pursuant to NCLT order - 29 Sept'26 and 59th CoC meeting on 06 Oct'26.</t>
-  </si>
-  <si>
-    <t>AXLE PAPER PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Paper</t>
-  </si>
-  <si>
-    <t>Mr. Kailash Shah</t>
-  </si>
-  <si>
-    <t>The installed capacity of main Products is 150MTPD.</t>
-  </si>
-  <si>
-    <t>Raheja Developers Limited - Revanta Project</t>
-  </si>
-  <si>
-    <t>Mr. Surendra Raj Gang</t>
-  </si>
-  <si>
-    <t>The CoC in its 4th meeting has resolved to scrap the earlier EOI process pursuant to Form-G dated 03 September 2026 and publish the current invitation for EOI for submission of Resolution Plans. The details of product are available in attached document.</t>
-  </si>
-  <si>
-    <t>PRATHAM-HEERA SALES PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Mahesh Goverdhan Bagla</t>
-  </si>
-  <si>
-    <t>SIMARA FOODS PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Navin Khandelwal</t>
-  </si>
-  <si>
-    <t>Recently closed</t>
-  </si>
-  <si>
-    <t>Closed recently</t>
   </si>
   <si>
     <t>ALVI TECH SERVICES PVT LTD</t>
@@ -1048,24 +1048,24 @@
       <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="F2" s="2" t="s">
+        <v>21</v>
+      </c>
       <c r="G2" s="2">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="H2" s="3">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="I2" s="2">
         <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K2" s="2">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="M2" s="4" t="s">
         <v>18</v>
       </c>
@@ -1073,12 +1073,12 @@
         <v>18</v>
       </c>
       <c r="O2" s="2">
-        <v>46300.75885633306</v>
+        <v>46300.75885622757</v>
       </c>
       <c r="P2" s="2">
-        <v>46303.78903317315</v>
-      </c>
-      <c r="Q2" s="5" t="s">
+        <v>46306.45019238699</v>
+      </c>
+      <c r="Q2" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1099,13 +1099,13 @@
         <v>26</v>
       </c>
       <c r="G3" s="2">
-        <v>0.89</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H3" s="3">
         <v>46306</v>
       </c>
       <c r="I3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>27</v>
@@ -1113,6 +1113,9 @@
       <c r="K3" s="2">
         <v>1</v>
       </c>
+      <c r="L3" s="2" t="s">
+        <v>28</v>
+      </c>
       <c r="M3" s="4" t="s">
         <v>18</v>
       </c>
@@ -1120,13 +1123,13 @@
         <v>18</v>
       </c>
       <c r="O3" s="2">
-        <v>46300.75885622757</v>
+        <v>46300.75885624527</v>
       </c>
       <c r="P3" s="2">
-        <v>46305.72545435187</v>
+        <v>46306.45019235874</v>
       </c>
       <c r="Q3" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1">
@@ -1146,13 +1149,13 @@
         <v>31</v>
       </c>
       <c r="G4" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H4" s="3">
         <v>46306</v>
       </c>
       <c r="I4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>32</v>
@@ -1170,13 +1173,13 @@
         <v>18</v>
       </c>
       <c r="O4" s="2">
-        <v>46300.75885624527</v>
+        <v>46300.7588562628</v>
       </c>
       <c r="P4" s="2">
-        <v>46305.72545433335</v>
+        <v>46306.45019237311</v>
       </c>
       <c r="Q4" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="2" customFormat="1">
@@ -1192,27 +1195,24 @@
       <c r="E5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="G5" s="2">
-        <v>0.91</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H5" s="3">
         <v>46306</v>
       </c>
       <c r="I5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K5" s="2">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="K5" s="2">
-        <v>1</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="M5" s="4" t="s">
         <v>18</v>
       </c>
@@ -1220,13 +1220,13 @@
         <v>18</v>
       </c>
       <c r="O5" s="2">
-        <v>46300.7588562628</v>
+        <v>46300.75885627908</v>
       </c>
       <c r="P5" s="2">
-        <v>46305.72545434292</v>
+        <v>46306.45019240092</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:17" s="2" customFormat="1">
@@ -1237,16 +1237,19 @@
         <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>40</v>
       </c>
       <c r="G6" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="H6" s="3">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="I6" s="2">
         <v>1</v>
@@ -1267,13 +1270,13 @@
         <v>18</v>
       </c>
       <c r="O6" s="2">
-        <v>46300.75885627908</v>
+        <v>46300.75884793277</v>
       </c>
       <c r="P6" s="2">
-        <v>46305.72545436121</v>
+        <v>46306.45019228883</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:17" s="2" customFormat="1">
@@ -1289,41 +1292,35 @@
       <c r="E7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="G7" s="2">
-        <v>0.88</v>
+        <v>0.2</v>
       </c>
       <c r="H7" s="3">
         <v>46307</v>
       </c>
       <c r="I7" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K7" s="2">
+        <v>1</v>
+      </c>
+      <c r="M7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O7" s="2">
+        <v>46300.7588479478</v>
+      </c>
+      <c r="P7" s="2">
+        <v>46306.45019231611</v>
+      </c>
+      <c r="Q7" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="K7" s="2">
-        <v>1</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O7" s="2">
-        <v>46300.75884793277</v>
-      </c>
-      <c r="P7" s="2">
-        <v>46305.72545428615</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:17" s="2" customFormat="1">
@@ -1334,22 +1331,25 @@
         <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="G8" s="2">
-        <v>0.2</v>
+        <v>0.93</v>
       </c>
       <c r="H8" s="3">
         <v>46307</v>
       </c>
       <c r="I8" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K8" s="2">
         <v>1</v>
@@ -1361,13 +1361,13 @@
         <v>18</v>
       </c>
       <c r="O8" s="2">
-        <v>46300.7588479478</v>
+        <v>46300.75884796329</v>
       </c>
       <c r="P8" s="2">
-        <v>46305.72545430451</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>51</v>
+        <v>46306.4501922311</v>
+      </c>
+      <c r="Q8" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:17" s="2" customFormat="1">
@@ -1378,29 +1378,29 @@
         <v>18</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G9" s="2">
-        <v>0.93</v>
+        <v>0.2</v>
       </c>
       <c r="H9" s="3">
         <v>46307</v>
       </c>
       <c r="I9" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K9" s="2">
         <v>1</v>
       </c>
+      <c r="L9" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
       </c>
@@ -1408,13 +1408,13 @@
         <v>18</v>
       </c>
       <c r="O9" s="2">
-        <v>46300.75884796329</v>
+        <v>46300.75884799581</v>
       </c>
       <c r="P9" s="2">
-        <v>46305.7254542472</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>28</v>
+        <v>46306.45019224514</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:17" s="2" customFormat="1">
@@ -1425,29 +1425,26 @@
         <v>18</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="G10" s="2">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H10" s="3">
         <v>46307</v>
       </c>
       <c r="I10" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K10" s="2">
         <v>1</v>
       </c>
-      <c r="L10" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="M10" s="4" t="s">
         <v>18</v>
       </c>
@@ -1455,13 +1452,13 @@
         <v>18</v>
       </c>
       <c r="O10" s="2">
-        <v>46300.75884799581</v>
+        <v>46300.75885617639</v>
       </c>
       <c r="P10" s="2">
-        <v>46305.72545425688</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>51</v>
+        <v>46306.45019227484</v>
+      </c>
+      <c r="Q10" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:17" s="2" customFormat="1">
@@ -1472,26 +1469,29 @@
         <v>18</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G11" s="2">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="H11" s="3">
         <v>46307</v>
       </c>
       <c r="I11" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="K11" s="2">
         <v>1</v>
       </c>
+      <c r="L11" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="M11" s="4" t="s">
         <v>18</v>
       </c>
@@ -1499,13 +1499,13 @@
         <v>18</v>
       </c>
       <c r="O11" s="2">
-        <v>46300.75885617639</v>
+        <v>46300.75885619673</v>
       </c>
       <c r="P11" s="2">
-        <v>46305.72545427667</v>
+        <v>46306.45019226002</v>
       </c>
       <c r="Q11" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:17" s="2" customFormat="1">
@@ -1516,28 +1516,31 @@
         <v>18</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="G12" s="2">
-        <v>0.91</v>
+        <v>0.93</v>
       </c>
       <c r="H12" s="3">
         <v>46307</v>
       </c>
       <c r="I12" s="2">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K12" s="2">
         <v>2</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="K12" s="2">
-        <v>1</v>
-      </c>
       <c r="L12" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M12" s="4" t="s">
         <v>18</v>
@@ -1546,13 +1549,13 @@
         <v>18</v>
       </c>
       <c r="O12" s="2">
-        <v>46300.75885619673</v>
+        <v>46305.20576106136</v>
       </c>
       <c r="P12" s="2">
-        <v>46305.72545426671</v>
+        <v>46306.45019233009</v>
       </c>
       <c r="Q12" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:17" s="2" customFormat="1">
@@ -1563,31 +1566,31 @@
         <v>18</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="F13" s="2" t="s">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="G13" s="2">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="H13" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I13" s="2">
         <v>2</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K13" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="M13" s="4" t="s">
         <v>18</v>
@@ -1596,13 +1599,13 @@
         <v>18</v>
       </c>
       <c r="O13" s="2">
-        <v>46305.20576106136</v>
+        <v>46300.75884788632</v>
       </c>
       <c r="P13" s="2">
-        <v>46305.72545431391</v>
+        <v>46306.45019220237</v>
       </c>
       <c r="Q13" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:17" s="2" customFormat="1">
@@ -1613,32 +1616,26 @@
         <v>18</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="G14" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H14" s="3">
         <v>46308</v>
       </c>
       <c r="I14" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K14" s="2">
         <v>1</v>
       </c>
-      <c r="L14" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="M14" s="4" t="s">
         <v>18</v>
       </c>
@@ -1646,13 +1643,13 @@
         <v>18</v>
       </c>
       <c r="O14" s="2">
-        <v>46300.75884788632</v>
+        <v>46300.75884790152</v>
       </c>
       <c r="P14" s="2">
-        <v>46305.72545422736</v>
-      </c>
-      <c r="Q14" s="2" t="s">
-        <v>28</v>
+        <v>46306.45019218787</v>
+      </c>
+      <c r="Q14" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:17" s="2" customFormat="1">
@@ -1663,10 +1660,10 @@
         <v>18</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G15" s="2">
         <v>0.2</v>
@@ -1675,10 +1672,10 @@
         <v>46308</v>
       </c>
       <c r="I15" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="K15" s="2">
         <v>1</v>
@@ -1690,13 +1687,13 @@
         <v>18</v>
       </c>
       <c r="O15" s="2">
-        <v>46300.75884790152</v>
+        <v>46301.38232480602</v>
       </c>
       <c r="P15" s="2">
-        <v>46305.72545421727</v>
+        <v>46306.45019217338</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:17" s="2" customFormat="1">
@@ -1707,26 +1704,29 @@
         <v>18</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" s="2">
+        <v>0.92</v>
+      </c>
+      <c r="H16" s="3">
+        <v>46310</v>
+      </c>
+      <c r="I16" s="2">
+        <v>4</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="K16" s="2">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G16" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="H16" s="3">
-        <v>46308</v>
-      </c>
-      <c r="I16" s="2">
-        <v>3</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K16" s="2">
-        <v>1</v>
-      </c>
       <c r="M16" s="4" t="s">
         <v>18</v>
       </c>
@@ -1734,13 +1734,13 @@
         <v>18</v>
       </c>
       <c r="O16" s="2">
-        <v>46301.38232480602</v>
+        <v>46300.75884787029</v>
       </c>
       <c r="P16" s="2">
-        <v>46305.72545420671</v>
-      </c>
-      <c r="Q16" s="5" t="s">
-        <v>51</v>
+        <v>46306.45019215749</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:17" s="2" customFormat="1">
@@ -1754,26 +1754,26 @@
         <v>74</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G17" s="2">
+        <v>0.95</v>
+      </c>
+      <c r="H17" s="3">
+        <v>46312</v>
+      </c>
+      <c r="I17" s="2">
+        <v>6</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="G17" s="2">
-        <v>0.92</v>
-      </c>
-      <c r="H17" s="3">
-        <v>46310</v>
-      </c>
-      <c r="I17" s="2">
-        <v>5</v>
-      </c>
-      <c r="J17" s="2" t="s">
+      <c r="K17" s="2">
+        <v>1</v>
+      </c>
+      <c r="L17" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K17" s="2">
-        <v>1</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="M17" s="4" t="s">
         <v>18</v>
       </c>
@@ -1781,13 +1781,13 @@
         <v>18</v>
       </c>
       <c r="O17" s="2">
-        <v>46300.75884787029</v>
+        <v>46300.75884779022</v>
       </c>
       <c r="P17" s="2">
-        <v>46305.72545419462</v>
+        <v>46306.45018428769</v>
       </c>
       <c r="Q17" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="2" customFormat="1">
@@ -1798,19 +1798,19 @@
         <v>18</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="G18" s="2">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="H18" s="3">
         <v>46312</v>
       </c>
       <c r="I18" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>79</v>
@@ -1818,9 +1818,6 @@
       <c r="K18" s="2">
         <v>1</v>
       </c>
-      <c r="L18" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="M18" s="4" t="s">
         <v>18</v>
       </c>
@@ -1828,13 +1825,13 @@
         <v>18</v>
       </c>
       <c r="O18" s="2">
-        <v>46300.75884779022</v>
+        <v>46300.75884780569</v>
       </c>
       <c r="P18" s="2">
-        <v>46305.72544558345</v>
+        <v>46306.4501843321</v>
       </c>
       <c r="Q18" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" spans="1:17" s="2" customFormat="1">
@@ -1845,10 +1842,10 @@
         <v>18</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="G19" s="2">
         <v>0.93</v>
@@ -1857,14 +1854,17 @@
         <v>46312</v>
       </c>
       <c r="I19" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K19" s="2">
         <v>1</v>
       </c>
+      <c r="L19" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="M19" s="4" t="s">
         <v>18</v>
       </c>
@@ -1872,13 +1872,13 @@
         <v>18</v>
       </c>
       <c r="O19" s="2">
-        <v>46300.75884780569</v>
+        <v>46300.75884782107</v>
       </c>
       <c r="P19" s="2">
-        <v>46305.72544561344</v>
+        <v>46306.45018431723</v>
       </c>
       <c r="Q19" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:17" s="2" customFormat="1">
@@ -1889,19 +1889,19 @@
         <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="G20" s="2">
-        <v>0.93</v>
+        <v>0.91</v>
       </c>
       <c r="H20" s="3">
         <v>46312</v>
       </c>
       <c r="I20" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>85</v>
@@ -1919,13 +1919,13 @@
         <v>18</v>
       </c>
       <c r="O20" s="2">
-        <v>46300.75884782107</v>
+        <v>46300.75884783743</v>
       </c>
       <c r="P20" s="2">
-        <v>46305.72544560267</v>
+        <v>46306.45018430228</v>
       </c>
       <c r="Q20" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" spans="1:17" s="2" customFormat="1">
@@ -1939,26 +1939,26 @@
         <v>87</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="G21" s="2">
         <v>0.91</v>
       </c>
       <c r="H21" s="3">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="I21" s="2">
         <v>7</v>
       </c>
       <c r="J21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="K21" s="2">
+        <v>3</v>
+      </c>
+      <c r="L21" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="K21" s="2">
-        <v>1</v>
-      </c>
-      <c r="L21" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="M21" s="4" t="s">
         <v>18</v>
       </c>
@@ -1966,13 +1966,13 @@
         <v>18</v>
       </c>
       <c r="O21" s="2">
-        <v>46300.75884783743</v>
+        <v>46302.26841519317</v>
       </c>
       <c r="P21" s="2">
-        <v>46305.72544559299</v>
+        <v>46306.45018427318</v>
       </c>
       <c r="Q21" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22" spans="1:17">
@@ -1983,28 +1983,28 @@
         <v>18</v>
       </c>
       <c r="C22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" t="s">
         <v>91</v>
       </c>
-      <c r="E22" t="s">
-        <v>20</v>
+      <c r="F22" t="s">
+        <v>92</v>
       </c>
       <c r="G22">
-        <v>0.91</v>
+        <v>0.96</v>
       </c>
       <c r="H22" s="3">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="I22">
         <v>8</v>
       </c>
       <c r="J22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K22">
-        <v>3</v>
-      </c>
-      <c r="L22" t="s">
-        <v>93</v>
+        <v>1</v>
       </c>
       <c r="M22" s="4" t="s">
         <v>18</v>
@@ -2013,13 +2013,13 @@
         <v>18</v>
       </c>
       <c r="O22">
-        <v>46302.26841519317</v>
+        <v>46300.75884774033</v>
       </c>
       <c r="P22">
-        <v>46305.72544557391</v>
+        <v>46306.450184229</v>
       </c>
       <c r="Q22" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:17">
@@ -2033,22 +2033,19 @@
         <v>94</v>
       </c>
       <c r="E23" t="s">
-        <v>95</v>
-      </c>
-      <c r="F23" t="s">
-        <v>96</v>
+        <v>44</v>
       </c>
       <c r="G23">
-        <v>0.96</v>
+        <v>0.2</v>
       </c>
       <c r="H23" s="3">
         <v>46314</v>
       </c>
       <c r="I23">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J23" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K23">
         <v>1</v>
@@ -2060,13 +2057,13 @@
         <v>18</v>
       </c>
       <c r="O23">
-        <v>46300.75884774033</v>
+        <v>46300.75884775587</v>
       </c>
       <c r="P23">
-        <v>46305.72544554438</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>28</v>
+        <v>46306.45018424345</v>
+      </c>
+      <c r="Q23" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:17">
@@ -2077,22 +2074,22 @@
         <v>18</v>
       </c>
       <c r="C24" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E24" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="G24">
-        <v>0.2</v>
+        <v>0.93</v>
       </c>
       <c r="H24" s="3">
         <v>46314</v>
       </c>
       <c r="I24">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J24" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="K24">
         <v>1</v>
@@ -2104,13 +2101,13 @@
         <v>18</v>
       </c>
       <c r="O24">
-        <v>46300.75884775587</v>
+        <v>46300.7588477715</v>
       </c>
       <c r="P24">
-        <v>46305.72544555414</v>
-      </c>
-      <c r="Q24" s="5" t="s">
-        <v>51</v>
+        <v>46306.45018425787</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:17">
@@ -2121,22 +2118,22 @@
         <v>18</v>
       </c>
       <c r="C25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E25" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="G25">
-        <v>0.93</v>
+        <v>0.2</v>
       </c>
       <c r="H25" s="3">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="I25">
         <v>9</v>
       </c>
       <c r="J25" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="K25">
         <v>1</v>
@@ -2148,13 +2145,13 @@
         <v>18</v>
       </c>
       <c r="O25">
-        <v>46300.7588477715</v>
+        <v>46300.75884772457</v>
       </c>
       <c r="P25">
-        <v>46305.72544556411</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>28</v>
+        <v>46306.45018421479</v>
+      </c>
+      <c r="Q25" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:17">
@@ -2165,25 +2162,28 @@
         <v>18</v>
       </c>
       <c r="C26" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E26" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G26">
         <v>0.2</v>
       </c>
       <c r="H26" s="3">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="I26">
         <v>10</v>
       </c>
       <c r="J26" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K26">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L26" t="s">
+        <v>102</v>
       </c>
       <c r="M26" s="4" t="s">
         <v>18</v>
@@ -2192,13 +2192,13 @@
         <v>18</v>
       </c>
       <c r="O26">
-        <v>46300.75884772457</v>
+        <v>46302.26841507768</v>
       </c>
       <c r="P26">
-        <v>46305.72544553479</v>
+        <v>46306.45018418654</v>
       </c>
       <c r="Q26" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" spans="1:17">
@@ -2209,28 +2209,25 @@
         <v>18</v>
       </c>
       <c r="C27" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E27" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G27">
         <v>0.2</v>
       </c>
       <c r="H27" s="3">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="I27">
         <v>11</v>
       </c>
       <c r="J27" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K27">
-        <v>3</v>
-      </c>
-      <c r="L27" t="s">
-        <v>106</v>
+        <v>1</v>
       </c>
       <c r="M27" s="4" t="s">
         <v>18</v>
@@ -2239,13 +2236,13 @@
         <v>18</v>
       </c>
       <c r="O27">
-        <v>46302.26841507768</v>
+        <v>46301.38232468421</v>
       </c>
       <c r="P27">
-        <v>46305.7254455155</v>
+        <v>46306.45018417132</v>
       </c>
       <c r="Q27" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" spans="1:17">
@@ -2256,22 +2253,25 @@
         <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E28" t="s">
-        <v>49</v>
+        <v>25</v>
+      </c>
+      <c r="F28" t="s">
+        <v>26</v>
       </c>
       <c r="G28">
-        <v>0.2</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H28" s="3">
         <v>46317</v>
       </c>
       <c r="I28">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J28" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="K28">
         <v>1</v>
@@ -2283,13 +2283,13 @@
         <v>18</v>
       </c>
       <c r="O28">
-        <v>46301.38232468421</v>
+        <v>46302.26841501552</v>
       </c>
       <c r="P28">
-        <v>46305.72544550539</v>
-      </c>
-      <c r="Q28" s="5" t="s">
-        <v>51</v>
+        <v>46306.45018415671</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:17">
@@ -2300,29 +2300,32 @@
         <v>18</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E29" t="s">
-        <v>30</v>
+        <v>91</v>
       </c>
       <c r="F29" t="s">
-        <v>31</v>
+        <v>92</v>
       </c>
       <c r="G29">
-        <v>0.9399999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="H29" s="3">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="I29">
         <v>12</v>
       </c>
       <c r="J29" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="K29">
         <v>1</v>
       </c>
+      <c r="L29" t="s">
+        <v>109</v>
+      </c>
       <c r="M29" s="4" t="s">
         <v>18</v>
       </c>
@@ -2330,13 +2333,13 @@
         <v>18</v>
       </c>
       <c r="O29">
-        <v>46302.26841501552</v>
+        <v>46305.20575267453</v>
       </c>
       <c r="P29">
-        <v>46305.7254454951</v>
+        <v>46306.45018412781</v>
       </c>
       <c r="Q29" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:17">
@@ -2347,22 +2350,19 @@
         <v>18</v>
       </c>
       <c r="C30" t="s">
+        <v>110</v>
+      </c>
+      <c r="E30" t="s">
         <v>111</v>
       </c>
-      <c r="E30" t="s">
-        <v>95</v>
-      </c>
-      <c r="F30" t="s">
-        <v>96</v>
-      </c>
       <c r="G30">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H30" s="3">
         <v>46318</v>
       </c>
       <c r="I30">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J30" t="s">
         <v>112</v>
@@ -2380,13 +2380,13 @@
         <v>18</v>
       </c>
       <c r="O30">
-        <v>46305.20575267453</v>
+        <v>46305.20575269723</v>
       </c>
       <c r="P30">
-        <v>46305.72544547343</v>
+        <v>46306.45018414222</v>
       </c>
       <c r="Q30" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:17">
@@ -2400,26 +2400,29 @@
         <v>114</v>
       </c>
       <c r="E31" t="s">
-        <v>115</v>
+        <v>20</v>
+      </c>
+      <c r="F31" t="s">
+        <v>48</v>
       </c>
       <c r="G31">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="H31" s="3">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="I31">
         <v>13</v>
       </c>
       <c r="J31" t="s">
+        <v>115</v>
+      </c>
+      <c r="K31">
+        <v>2</v>
+      </c>
+      <c r="L31" t="s">
         <v>116</v>
       </c>
-      <c r="K31">
-        <v>1</v>
-      </c>
-      <c r="L31" t="s">
-        <v>117</v>
-      </c>
       <c r="M31" s="4" t="s">
         <v>18</v>
       </c>
@@ -2427,13 +2430,13 @@
         <v>18</v>
       </c>
       <c r="O31">
-        <v>46305.20575269723</v>
+        <v>46305.20575263901</v>
       </c>
       <c r="P31">
-        <v>46305.72544548448</v>
+        <v>46306.45018411243</v>
       </c>
       <c r="Q31" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" spans="1:17">
@@ -2444,31 +2447,25 @@
         <v>18</v>
       </c>
       <c r="C32" t="s">
+        <v>117</v>
+      </c>
+      <c r="E32" t="s">
+        <v>44</v>
+      </c>
+      <c r="G32">
+        <v>0.2</v>
+      </c>
+      <c r="H32" s="3">
+        <v>46326</v>
+      </c>
+      <c r="I32">
+        <v>20</v>
+      </c>
+      <c r="J32" t="s">
         <v>118</v>
       </c>
-      <c r="E32" t="s">
-        <v>25</v>
-      </c>
-      <c r="F32" t="s">
-        <v>53</v>
-      </c>
-      <c r="G32">
-        <v>0.93</v>
-      </c>
-      <c r="H32" s="3">
-        <v>46319</v>
-      </c>
-      <c r="I32">
-        <v>14</v>
-      </c>
-      <c r="J32" t="s">
-        <v>119</v>
-      </c>
       <c r="K32">
-        <v>2</v>
-      </c>
-      <c r="L32" t="s">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="M32" s="4" t="s">
         <v>18</v>
@@ -2477,13 +2474,13 @@
         <v>18</v>
       </c>
       <c r="O32">
-        <v>46305.20575263901</v>
+        <v>46300.75884768533</v>
       </c>
       <c r="P32">
-        <v>46305.72544546242</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>28</v>
+        <v>46306.45018409734</v>
+      </c>
+      <c r="Q32" s="5" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="33" spans="1:17">
@@ -2494,99 +2491,104 @@
         <v>18</v>
       </c>
       <c r="C33" t="s">
+        <v>119</v>
+      </c>
+      <c r="E33" t="s">
+        <v>71</v>
+      </c>
+      <c r="G33">
+        <v>0.92</v>
+      </c>
+      <c r="H33" s="3">
+        <v>46332</v>
+      </c>
+      <c r="I33">
+        <v>26</v>
+      </c>
+      <c r="J33" t="s">
+        <v>120</v>
+      </c>
+      <c r="K33">
+        <v>4</v>
+      </c>
+      <c r="M33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N33" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="O33">
+        <v>46305.20575257758</v>
+      </c>
+      <c r="P33">
+        <v>46306.45018405222</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17">
+      <c r="A34" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E33" t="s">
-        <v>49</v>
-      </c>
-      <c r="G33">
-        <v>0.2</v>
-      </c>
-      <c r="H33" s="3">
-        <v>46326</v>
-      </c>
-      <c r="I33">
-        <v>21</v>
-      </c>
-      <c r="J33" t="s">
+      <c r="B34" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="K33">
-        <v>1</v>
-      </c>
-      <c r="M33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O33">
-        <v>46300.75884768533</v>
-      </c>
-      <c r="P33">
-        <v>46305.72544545171</v>
-      </c>
-      <c r="Q33" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17">
-      <c r="A34" t="s">
-        <v>18</v>
-      </c>
-      <c r="B34" t="s">
-        <v>18</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="C34" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="E34" t="s">
-        <v>75</v>
-      </c>
-      <c r="G34">
-        <v>0.92</v>
-      </c>
-      <c r="H34" s="3">
-        <v>46332</v>
-      </c>
-      <c r="I34">
-        <v>27</v>
-      </c>
-      <c r="J34" t="s">
+      <c r="D34" s="6"/>
+      <c r="E34" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6">
+        <v>0.91</v>
+      </c>
+      <c r="H34" s="6">
+        <v>46305</v>
+      </c>
+      <c r="I34" s="6">
+        <v>-1</v>
+      </c>
+      <c r="J34" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="K34">
-        <v>4</v>
-      </c>
-      <c r="M34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O34">
-        <v>46305.20575257758</v>
-      </c>
-      <c r="P34">
-        <v>46305.72544541569</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>28</v>
+      <c r="K34" s="6">
+        <v>1</v>
+      </c>
+      <c r="L34" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N34" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O34" s="6">
+        <v>46300.75885633306</v>
+      </c>
+      <c r="P34" s="6">
+        <v>46303.78903317315</v>
+      </c>
+      <c r="Q34" s="5" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="35" spans="1:17">
       <c r="A35" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>127</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6">
@@ -2596,10 +2598,10 @@
         <v>46304</v>
       </c>
       <c r="I35" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="J35" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="K35" s="6">
         <v>1</v>
@@ -2615,18 +2617,18 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P35" s="6">
-        <v>46305.72546245658</v>
+        <v>46306.45020025707</v>
       </c>
       <c r="Q35" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36" spans="1:17">
       <c r="A36" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>128</v>
@@ -2643,7 +2645,7 @@
         <v>46304</v>
       </c>
       <c r="I36" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="J36" s="6" t="s">
         <v>130</v>
@@ -2664,25 +2666,25 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P36" s="6">
-        <v>46305.72546246747</v>
+        <v>46306.4502002715</v>
       </c>
       <c r="Q36" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>133</v>
@@ -2694,7 +2696,7 @@
         <v>46303</v>
       </c>
       <c r="I37" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="J37" s="6" t="s">
         <v>134</v>
@@ -2715,25 +2717,25 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P37" s="6">
-        <v>46305.72546247725</v>
+        <v>46306.45020028572</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>136</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6">
@@ -2743,7 +2745,7 @@
         <v>46302</v>
       </c>
       <c r="I38" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J38" s="6" t="s">
         <v>137</v>
@@ -2764,25 +2766,25 @@
         <v>46300.7588564394</v>
       </c>
       <c r="P38" s="6">
-        <v>46305.7254625063</v>
+        <v>46306.45020032745</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" spans="1:17">
       <c r="A39" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6">
@@ -2792,7 +2794,7 @@
         <v>46302</v>
       </c>
       <c r="I39" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J39" s="6" t="s">
         <v>140</v>
@@ -2811,28 +2813,28 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P39" s="6">
-        <v>46305.7254625255</v>
+        <v>46306.45020035555</v>
       </c>
       <c r="Q39" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>141</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G40" s="6">
         <v>0.9399999999999999</v>
@@ -2841,7 +2843,7 @@
         <v>46301</v>
       </c>
       <c r="I40" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J40" s="6" t="s">
         <v>142</v>
@@ -2860,18 +2862,18 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P40" s="6">
-        <v>46305.72546255367</v>
+        <v>46306.45020039732</v>
       </c>
       <c r="Q40" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:17">
       <c r="A41" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>143</v>
@@ -2888,7 +2890,7 @@
         <v>46300</v>
       </c>
       <c r="I41" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J41" s="6" t="s">
         <v>145</v>
@@ -2907,28 +2909,28 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P41" s="6">
-        <v>46305.72546258115</v>
+        <v>46306.45020043853</v>
       </c>
       <c r="Q41" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>146</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G42" s="6">
         <v>0.93</v>
@@ -2937,7 +2939,7 @@
         <v>46300</v>
       </c>
       <c r="I42" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J42" s="6" t="s">
         <v>147</v>
@@ -2956,25 +2958,25 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P42" s="6">
-        <v>46305.72546256285</v>
+        <v>46306.45020041129</v>
       </c>
       <c r="Q42" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="43" spans="1:17">
       <c r="A43" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>148</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6">
@@ -2984,10 +2986,10 @@
         <v>46299</v>
       </c>
       <c r="I43" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="K43" s="6">
         <v>1</v>
@@ -3005,28 +3007,28 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P43" s="6">
-        <v>46305.72546260039</v>
+        <v>46306.45020046723</v>
       </c>
       <c r="Q43" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>150</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G44" s="6">
         <v>0.93</v>
@@ -3035,7 +3037,7 @@
         <v>46299</v>
       </c>
       <c r="I44" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J44" s="6" t="s">
         <v>151</v>
@@ -3054,25 +3056,25 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P44" s="6">
-        <v>46305.72546259048</v>
+        <v>46306.45020045295</v>
       </c>
       <c r="Q44" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45" spans="1:17">
       <c r="A45" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>152</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6">
@@ -3082,7 +3084,7 @@
         <v>46298</v>
       </c>
       <c r="I45" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J45" s="6" t="s">
         <v>153</v>
@@ -3101,25 +3103,25 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P45" s="6">
-        <v>46305.72547073589</v>
+        <v>46306.45020834605</v>
       </c>
       <c r="Q45" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:17">
       <c r="A46" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>154</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>133</v>
@@ -3131,7 +3133,7 @@
         <v>46298</v>
       </c>
       <c r="I46" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J46" s="6" t="s">
         <v>155</v>
@@ -3153,15 +3155,15 @@
         <v>46303.78904942831</v>
       </c>
       <c r="Q46" s="5" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:17">
       <c r="A47" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>156</v>
@@ -3178,7 +3180,7 @@
         <v>46298</v>
       </c>
       <c r="I47" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J47" s="6" t="s">
         <v>158</v>
@@ -3199,25 +3201,25 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P47" s="6">
-        <v>46305.72547074813</v>
+        <v>46306.4502083617</v>
       </c>
       <c r="Q47" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48" spans="1:17">
       <c r="A48" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C48" s="6" t="s">
         <v>160</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="6">
@@ -3227,7 +3229,7 @@
         <v>46298</v>
       </c>
       <c r="I48" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J48" s="6" t="s">
         <v>161</v>
@@ -3246,18 +3248,18 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P48" s="6">
-        <v>46305.72546262942</v>
+        <v>46306.45020050919</v>
       </c>
       <c r="Q48" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="49" spans="1:17">
       <c r="A49" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>162</v>
@@ -3274,7 +3276,7 @@
         <v>46297</v>
       </c>
       <c r="I49" s="6">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="J49" s="6" t="s">
         <v>163</v>
@@ -3295,25 +3297,25 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P49" s="6">
-        <v>46305.72547080749</v>
+        <v>46306.45020844889</v>
       </c>
       <c r="Q49" s="6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>165</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6">
@@ -3323,7 +3325,7 @@
         <v>46296</v>
       </c>
       <c r="I50" s="6">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="J50" s="6" t="s">
         <v>166</v>
@@ -3344,10 +3346,10 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P50" s="6">
-        <v>46305.72547081784</v>
+        <v>46306.45020846285</v>
       </c>
       <c r="Q50" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -3537,29 +3539,26 @@
         <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G2" s="2">
-        <v>0.91</v>
+        <v>0.2</v>
       </c>
       <c r="H2" s="3">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="I2" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="K2" s="2">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>22</v>
-      </c>
       <c r="M2" s="4" t="s">
         <v>18</v>
       </c>
@@ -3567,13 +3566,13 @@
         <v>18</v>
       </c>
       <c r="O2" s="2">
-        <v>46300.75885633306</v>
+        <v>46300.7588479478</v>
       </c>
       <c r="P2" s="2">
-        <v>46303.78903317315</v>
+        <v>46306.45019231611</v>
       </c>
       <c r="Q2" s="5" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:17" s="2" customFormat="1">
@@ -3584,10 +3583,10 @@
         <v>18</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G3" s="2">
         <v>0.2</v>
@@ -3596,14 +3595,17 @@
         <v>46307</v>
       </c>
       <c r="I3" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K3" s="2">
         <v>1</v>
       </c>
+      <c r="L3" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="M3" s="4" t="s">
         <v>18</v>
       </c>
@@ -3611,13 +3613,13 @@
         <v>18</v>
       </c>
       <c r="O3" s="2">
-        <v>46300.7588479478</v>
+        <v>46300.75884799581</v>
       </c>
       <c r="P3" s="2">
-        <v>46305.72545430451</v>
+        <v>46306.45019224514</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="2" customFormat="1">
@@ -3628,29 +3630,26 @@
         <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G4" s="2">
         <v>0.2</v>
       </c>
       <c r="H4" s="3">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I4" s="2">
         <v>2</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="K4" s="2">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="s">
-        <v>57</v>
-      </c>
       <c r="M4" s="4" t="s">
         <v>18</v>
       </c>
@@ -3658,13 +3657,13 @@
         <v>18</v>
       </c>
       <c r="O4" s="2">
-        <v>46300.75884799581</v>
+        <v>46300.75884790152</v>
       </c>
       <c r="P4" s="2">
-        <v>46305.72545425688</v>
+        <v>46306.45019218787</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:17" s="2" customFormat="1">
@@ -3675,10 +3674,10 @@
         <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G5" s="2">
         <v>0.2</v>
@@ -3687,10 +3686,10 @@
         <v>46308</v>
       </c>
       <c r="I5" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="K5" s="2">
         <v>1</v>
@@ -3702,41 +3701,41 @@
         <v>18</v>
       </c>
       <c r="O5" s="2">
-        <v>46300.75884790152</v>
+        <v>46301.38232480602</v>
       </c>
       <c r="P5" s="2">
-        <v>46305.72545421727</v>
+        <v>46306.45019217338</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" s="2" customFormat="1">
-      <c r="A6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G6" s="2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6">
         <v>0.2</v>
       </c>
       <c r="H6" s="3">
-        <v>46308</v>
-      </c>
-      <c r="I6" s="2">
-        <v>3</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K6" s="2">
+        <v>46314</v>
+      </c>
+      <c r="I6">
+        <v>8</v>
+      </c>
+      <c r="J6" t="s">
+        <v>95</v>
+      </c>
+      <c r="K6">
         <v>1</v>
       </c>
       <c r="M6" s="4" t="s">
@@ -3745,14 +3744,14 @@
       <c r="N6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O6" s="2">
-        <v>46301.38232480602</v>
-      </c>
-      <c r="P6" s="2">
-        <v>46305.72545420671</v>
+      <c r="O6">
+        <v>46300.75884775587</v>
+      </c>
+      <c r="P6">
+        <v>46306.45018424345</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:17">
@@ -3766,13 +3765,13 @@
         <v>98</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G7">
         <v>0.2</v>
       </c>
       <c r="H7" s="3">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="I7">
         <v>9</v>
@@ -3790,13 +3789,13 @@
         <v>18</v>
       </c>
       <c r="O7">
-        <v>46300.75884775587</v>
+        <v>46300.75884772457</v>
       </c>
       <c r="P7">
-        <v>46305.72544555414</v>
+        <v>46306.45018421479</v>
       </c>
       <c r="Q7" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:17">
@@ -3807,25 +3806,28 @@
         <v>18</v>
       </c>
       <c r="C8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E8" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G8">
         <v>0.2</v>
       </c>
       <c r="H8" s="3">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="I8">
         <v>10</v>
       </c>
       <c r="J8" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="L8" t="s">
+        <v>102</v>
       </c>
       <c r="M8" s="4" t="s">
         <v>18</v>
@@ -3834,13 +3836,13 @@
         <v>18</v>
       </c>
       <c r="O8">
-        <v>46300.75884772457</v>
+        <v>46302.26841507768</v>
       </c>
       <c r="P8">
-        <v>46305.72544553479</v>
+        <v>46306.45018418654</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:17">
@@ -3851,28 +3853,25 @@
         <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G9">
         <v>0.2</v>
       </c>
       <c r="H9" s="3">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="I9">
         <v>11</v>
       </c>
       <c r="J9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K9">
-        <v>3</v>
-      </c>
-      <c r="L9" t="s">
-        <v>106</v>
+        <v>1</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>18</v>
@@ -3881,13 +3880,13 @@
         <v>18</v>
       </c>
       <c r="O9">
-        <v>46302.26841507768</v>
+        <v>46301.38232468421</v>
       </c>
       <c r="P9">
-        <v>46305.7254455155</v>
+        <v>46306.45018417132</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:17">
@@ -3898,22 +3897,22 @@
         <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G10">
         <v>0.2</v>
       </c>
       <c r="H10" s="3">
-        <v>46317</v>
+        <v>46326</v>
       </c>
       <c r="I10">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J10" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -3925,72 +3924,77 @@
         <v>18</v>
       </c>
       <c r="O10">
-        <v>46301.38232468421</v>
+        <v>46300.75884768533</v>
       </c>
       <c r="P10">
-        <v>46305.72544550539</v>
+        <v>46306.45018409734</v>
       </c>
       <c r="Q10" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="A11" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G11">
-        <v>0.2</v>
-      </c>
-      <c r="H11" s="3">
-        <v>46326</v>
-      </c>
-      <c r="I11">
-        <v>21</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="B11" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="K11">
-        <v>1</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="O11">
-        <v>46300.75884768533</v>
-      </c>
-      <c r="P11">
-        <v>46305.72544545171</v>
+      <c r="C11" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6">
+        <v>0.91</v>
+      </c>
+      <c r="H11" s="6">
+        <v>46305</v>
+      </c>
+      <c r="I11" s="6">
+        <v>-1</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K11" s="6">
+        <v>1</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="M11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="N11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="O11" s="6">
+        <v>46300.75885633306</v>
+      </c>
+      <c r="P11" s="6">
+        <v>46303.78903317315</v>
       </c>
       <c r="Q11" s="5" t="s">
-        <v>51</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6">
@@ -4000,7 +4004,7 @@
         <v>46302</v>
       </c>
       <c r="I12" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J12" s="6" t="s">
         <v>140</v>
@@ -4019,25 +4023,25 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P12" s="6">
-        <v>46305.7254625255</v>
+        <v>46306.45020035555</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>148</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6">
@@ -4047,10 +4051,10 @@
         <v>46299</v>
       </c>
       <c r="I13" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="K13" s="6">
         <v>1</v>
@@ -4068,25 +4072,25 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P13" s="6">
-        <v>46305.72546260039</v>
+        <v>46306.45020046723</v>
       </c>
       <c r="Q13" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>152</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6">
@@ -4096,7 +4100,7 @@
         <v>46298</v>
       </c>
       <c r="I14" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J14" s="6" t="s">
         <v>153</v>
@@ -4115,25 +4119,25 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P14" s="6">
-        <v>46305.72547073589</v>
+        <v>46306.45020834605</v>
       </c>
       <c r="Q14" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>154</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F15" s="6" t="s">
         <v>133</v>
@@ -4145,7 +4149,7 @@
         <v>46298</v>
       </c>
       <c r="I15" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>155</v>
@@ -4167,22 +4171,22 @@
         <v>46303.78904942831</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>23</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>160</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6">
@@ -4192,7 +4196,7 @@
         <v>46298</v>
       </c>
       <c r="I16" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>161</v>
@@ -4211,25 +4215,25 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P16" s="6">
-        <v>46305.72546262942</v>
+        <v>46306.45020050919</v>
       </c>
       <c r="Q16" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>165</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6">
@@ -4239,7 +4243,7 @@
         <v>46296</v>
       </c>
       <c r="I17" s="6">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>166</v>
@@ -4260,10 +4264,10 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P17" s="6">
-        <v>46305.72547081784</v>
+        <v>46306.45020846285</v>
       </c>
       <c r="Q17" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -4308,7 +4312,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4356,10 +4360,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B2">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C2" t="s">
         <v>179</v>
@@ -4374,7 +4378,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -4391,10 +4395,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B3">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C3" t="s">
         <v>179</v>
@@ -4426,10 +4430,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B4">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C4" t="s">
         <v>179</v>
@@ -4441,16 +4445,16 @@
         <v>3826</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -4461,45 +4465,45 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B5">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C5" t="s">
         <v>179</v>
       </c>
       <c r="D5">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E5">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G5">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B6">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C6" t="s">
         <v>179</v>
@@ -4531,10 +4535,10 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B7">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C7" t="s">
         <v>179</v>
@@ -4549,7 +4553,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -4566,10 +4570,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B8">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C8" t="s">
         <v>179</v>
@@ -4581,16 +4585,16 @@
         <v>3820</v>
       </c>
       <c r="F8">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H8">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>0</v>
@@ -4601,45 +4605,45 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B9">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C9" t="s">
         <v>179</v>
       </c>
       <c r="D9">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E9">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F9">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G9">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B10">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C10" t="s">
         <v>179</v>
@@ -4651,13 +4655,13 @@
         <v>160</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G10">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -4666,15 +4670,15 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B11">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C11" t="s">
         <v>179</v>
@@ -4686,21 +4690,56 @@
         <v>160</v>
       </c>
       <c r="F11">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H11">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B12">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D12">
+        <v>8</v>
+      </c>
+      <c r="E12">
+        <v>160</v>
+      </c>
+      <c r="F12">
+        <v>157</v>
+      </c>
+      <c r="G12">
+        <v>3</v>
+      </c>
+      <c r="H12">
+        <v>132</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-11-1746Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="180">
   <si>
     <t>Priority</t>
   </si>
@@ -1076,7 +1076,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P2" s="2">
-        <v>46306.45019238699</v>
+        <v>46306.73889369357</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1126,7 +1126,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P3" s="2">
-        <v>46306.45019235874</v>
+        <v>46306.7388936651</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>23</v>
@@ -1176,7 +1176,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P4" s="2">
-        <v>46306.45019237311</v>
+        <v>46306.73889367961</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>23</v>
@@ -1223,7 +1223,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P5" s="2">
-        <v>46306.45019240092</v>
+        <v>46306.73889370801</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1273,7 +1273,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P6" s="2">
-        <v>46306.45019228883</v>
+        <v>46306.73889359355</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>23</v>
@@ -1317,7 +1317,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P7" s="2">
-        <v>46306.45019231611</v>
+        <v>46306.73889362151</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>46</v>
@@ -1364,7 +1364,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P8" s="2">
-        <v>46306.4501922311</v>
+        <v>46306.73889353455</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>23</v>
@@ -1411,7 +1411,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P9" s="2">
-        <v>46306.45019224514</v>
+        <v>46306.73889354909</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>46</v>
@@ -1455,7 +1455,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P10" s="2">
-        <v>46306.45019227484</v>
+        <v>46306.73889357936</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>23</v>
@@ -1502,7 +1502,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P11" s="2">
-        <v>46306.45019226002</v>
+        <v>46306.73889356442</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>23</v>
@@ -1552,7 +1552,7 @@
         <v>46305.20576106136</v>
       </c>
       <c r="P12" s="2">
-        <v>46306.45019233009</v>
+        <v>46306.73889363577</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1602,7 +1602,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P13" s="2">
-        <v>46306.45019220237</v>
+        <v>46306.7388935053</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>23</v>
@@ -1646,7 +1646,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P14" s="2">
-        <v>46306.45019218787</v>
+        <v>46306.73889349052</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>46</v>
@@ -1690,7 +1690,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P15" s="2">
-        <v>46306.45019217338</v>
+        <v>46306.73889347556</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -1737,7 +1737,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P16" s="2">
-        <v>46306.45019215749</v>
+        <v>46306.73889345909</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>23</v>
@@ -1784,7 +1784,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P17" s="2">
-        <v>46306.45018428769</v>
+        <v>46306.7388853133</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>23</v>
@@ -1828,7 +1828,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P18" s="2">
-        <v>46306.4501843321</v>
+        <v>46306.73888535729</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -1875,7 +1875,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P19" s="2">
-        <v>46306.45018431723</v>
+        <v>46306.73888534283</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>23</v>
@@ -1922,7 +1922,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P20" s="2">
-        <v>46306.45018430228</v>
+        <v>46306.73888532812</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>23</v>
@@ -1969,7 +1969,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P21" s="2">
-        <v>46306.45018427318</v>
+        <v>46306.73888529836</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>23</v>
@@ -2016,7 +2016,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P22">
-        <v>46306.450184229</v>
+        <v>46306.73888525447</v>
       </c>
       <c r="Q22" t="s">
         <v>23</v>
@@ -2060,7 +2060,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P23">
-        <v>46306.45018424345</v>
+        <v>46306.73888526922</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
@@ -2104,7 +2104,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P24">
-        <v>46306.45018425787</v>
+        <v>46306.7388852838</v>
       </c>
       <c r="Q24" t="s">
         <v>23</v>
@@ -2148,7 +2148,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P25">
-        <v>46306.45018421479</v>
+        <v>46306.73888524011</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>46</v>
@@ -2195,7 +2195,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P26">
-        <v>46306.45018418654</v>
+        <v>46306.73888521137</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>46</v>
@@ -2239,7 +2239,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P27">
-        <v>46306.45018417132</v>
+        <v>46306.73888519628</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>46</v>
@@ -2286,7 +2286,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P28">
-        <v>46306.45018415671</v>
+        <v>46306.73888518155</v>
       </c>
       <c r="Q28" t="s">
         <v>23</v>
@@ -2336,7 +2336,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P29">
-        <v>46306.45018412781</v>
+        <v>46306.73888515188</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2383,7 +2383,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P30">
-        <v>46306.45018414222</v>
+        <v>46306.73888516689</v>
       </c>
       <c r="Q30" t="s">
         <v>23</v>
@@ -2433,7 +2433,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P31">
-        <v>46306.45018411243</v>
+        <v>46306.73888513631</v>
       </c>
       <c r="Q31" t="s">
         <v>23</v>
@@ -2477,7 +2477,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P32">
-        <v>46306.45018409734</v>
+        <v>46306.73888512077</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>46</v>
@@ -2521,7 +2521,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P33">
-        <v>46306.45018405222</v>
+        <v>46306.73888507384</v>
       </c>
       <c r="Q33" t="s">
         <v>23</v>
@@ -2617,7 +2617,7 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P35" s="6">
-        <v>46306.45020025707</v>
+        <v>46306.73890189125</v>
       </c>
       <c r="Q35" s="6" t="s">
         <v>23</v>
@@ -2666,7 +2666,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P36" s="6">
-        <v>46306.4502002715</v>
+        <v>46306.7389019061</v>
       </c>
       <c r="Q36" s="6" t="s">
         <v>23</v>
@@ -2717,7 +2717,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P37" s="6">
-        <v>46306.45020028572</v>
+        <v>46306.73890192044</v>
       </c>
       <c r="Q37" s="6" t="s">
         <v>23</v>
@@ -2766,7 +2766,7 @@
         <v>46300.7588564394</v>
       </c>
       <c r="P38" s="6">
-        <v>46306.45020032745</v>
+        <v>46306.73890196386</v>
       </c>
       <c r="Q38" s="6" t="s">
         <v>23</v>
@@ -2813,7 +2813,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P39" s="6">
-        <v>46306.45020035555</v>
+        <v>46306.73890199242</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>46</v>
@@ -2862,7 +2862,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P40" s="6">
-        <v>46306.45020039732</v>
+        <v>46306.73890203507</v>
       </c>
       <c r="Q40" s="6" t="s">
         <v>23</v>
@@ -2909,7 +2909,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P41" s="6">
-        <v>46306.45020043853</v>
+        <v>46306.73890207729</v>
       </c>
       <c r="Q41" s="6" t="s">
         <v>23</v>
@@ -2958,7 +2958,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P42" s="6">
-        <v>46306.45020041129</v>
+        <v>46306.73890204917</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>23</v>
@@ -3007,7 +3007,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P43" s="6">
-        <v>46306.45020046723</v>
+        <v>46306.73890210572</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>46</v>
@@ -3056,7 +3056,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P44" s="6">
-        <v>46306.45020045295</v>
+        <v>46306.73890209116</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>23</v>
@@ -3103,7 +3103,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P45" s="6">
-        <v>46306.45020834605</v>
+        <v>46306.73891017484</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>46</v>
@@ -3201,7 +3201,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P47" s="6">
-        <v>46306.4502083617</v>
+        <v>46306.73891019166</v>
       </c>
       <c r="Q47" s="6" t="s">
         <v>23</v>
@@ -3248,7 +3248,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P48" s="6">
-        <v>46306.45020050919</v>
+        <v>46306.73890214869</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>46</v>
@@ -3297,7 +3297,7 @@
         <v>46300.75886486177</v>
       </c>
       <c r="P49" s="6">
-        <v>46306.45020844889</v>
+        <v>46306.73891028108</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>23</v>
@@ -3346,7 +3346,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P50" s="6">
-        <v>46306.45020846285</v>
+        <v>46306.7389102954</v>
       </c>
       <c r="Q50" s="5" t="s">
         <v>46</v>
@@ -3569,7 +3569,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P2" s="2">
-        <v>46306.45019231611</v>
+        <v>46306.73889362151</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>46</v>
@@ -3616,7 +3616,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P3" s="2">
-        <v>46306.45019224514</v>
+        <v>46306.73889354909</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>46</v>
@@ -3660,7 +3660,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P4" s="2">
-        <v>46306.45019218787</v>
+        <v>46306.73889349052</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>46</v>
@@ -3704,7 +3704,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P5" s="2">
-        <v>46306.45019217338</v>
+        <v>46306.73889347556</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>46</v>
@@ -3748,7 +3748,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P6">
-        <v>46306.45018424345</v>
+        <v>46306.73888526922</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>46</v>
@@ -3792,7 +3792,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P7">
-        <v>46306.45018421479</v>
+        <v>46306.73888524011</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>46</v>
@@ -3839,7 +3839,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P8">
-        <v>46306.45018418654</v>
+        <v>46306.73888521137</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
@@ -3883,7 +3883,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P9">
-        <v>46306.45018417132</v>
+        <v>46306.73888519628</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>46</v>
@@ -3927,7 +3927,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P10">
-        <v>46306.45018409734</v>
+        <v>46306.73888512077</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -4023,7 +4023,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P12" s="6">
-        <v>46306.45020035555</v>
+        <v>46306.73890199242</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>46</v>
@@ -4072,7 +4072,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P13" s="6">
-        <v>46306.45020046723</v>
+        <v>46306.73890210572</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -4119,7 +4119,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P14" s="6">
-        <v>46306.45020834605</v>
+        <v>46306.73891017484</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>46</v>
@@ -4215,7 +4215,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P16" s="6">
-        <v>46306.45020050919</v>
+        <v>46306.73890214869</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>46</v>
@@ -4264,7 +4264,7 @@
         <v>46300.75886487812</v>
       </c>
       <c r="P17" s="6">
-        <v>46306.45020846285</v>
+        <v>46306.7389102954</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -4312,7 +4312,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4360,10 +4360,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B2">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C2" t="s">
         <v>179</v>
@@ -4395,10 +4395,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B3">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C3" t="s">
         <v>179</v>
@@ -4413,7 +4413,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -4430,10 +4430,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B4">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C4" t="s">
         <v>179</v>
@@ -4465,10 +4465,10 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B5">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C5" t="s">
         <v>179</v>
@@ -4480,16 +4480,16 @@
         <v>3826</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -4500,45 +4500,45 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B6">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C6" t="s">
         <v>179</v>
       </c>
       <c r="D6">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E6">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G6">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B7">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C7" t="s">
         <v>179</v>
@@ -4570,10 +4570,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B8">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C8" t="s">
         <v>179</v>
@@ -4588,7 +4588,7 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -4605,10 +4605,10 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B9">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C9" t="s">
         <v>179</v>
@@ -4620,16 +4620,16 @@
         <v>3820</v>
       </c>
       <c r="F9">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H9">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -4640,45 +4640,45 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B10">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C10" t="s">
         <v>179</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E10">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F10">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G10">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B11">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C11" t="s">
         <v>179</v>
@@ -4690,13 +4690,13 @@
         <v>160</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G11">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -4705,15 +4705,15 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B12">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C12" t="s">
         <v>179</v>
@@ -4725,21 +4725,56 @@
         <v>160</v>
       </c>
       <c r="F12">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H12">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B13">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C13" t="s">
+        <v>179</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>160</v>
+      </c>
+      <c r="F13">
+        <v>157</v>
+      </c>
+      <c r="G13">
+        <v>3</v>
+      </c>
+      <c r="H13">
+        <v>132</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-12-2122Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="202">
   <si>
     <t>Priority</t>
   </si>
@@ -1145,7 +1145,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P2" s="2">
-        <v>46307.3955139285</v>
+        <v>46307.88905263421</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>24</v>
@@ -1189,7 +1189,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P3" s="2">
-        <v>46307.39551395869</v>
+        <v>46307.88905266359</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>28</v>
@@ -1327,7 +1327,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P6" s="2">
-        <v>46307.39551391241</v>
+        <v>46307.88905261796</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>24</v>
@@ -1374,7 +1374,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P7" s="2">
-        <v>46307.39550561333</v>
+        <v>46307.88904476112</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>24</v>
@@ -1424,7 +1424,7 @@
         <v>46305.20576106136</v>
       </c>
       <c r="P8" s="2">
-        <v>46307.3955139888</v>
+        <v>46307.88905269294</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>24</v>
@@ -1474,7 +1474,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P9" s="2">
-        <v>46307.39550553843</v>
+        <v>46307.88904468949</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>24</v>
@@ -1518,7 +1518,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P10" s="2">
-        <v>46307.39550555297</v>
+        <v>46307.88904470354</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>28</v>
@@ -1562,7 +1562,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P11" s="2">
-        <v>46307.39550552344</v>
+        <v>46307.88904467553</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>28</v>
@@ -1609,7 +1609,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P12" s="2">
-        <v>46307.39550550879</v>
+        <v>46307.8890446615</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>24</v>
@@ -1656,7 +1656,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P13" s="2">
-        <v>46307.39550543506</v>
+        <v>46307.88904458907</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>24</v>
@@ -1700,7 +1700,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P14" s="2">
-        <v>46307.39550544995</v>
+        <v>46307.88904460396</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>24</v>
@@ -1747,7 +1747,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P15" s="2">
-        <v>46307.39550546476</v>
+        <v>46307.88904461851</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>24</v>
@@ -1794,7 +1794,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P16" s="2">
-        <v>46307.39550547927</v>
+        <v>46307.88904463262</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>24</v>
@@ -1841,7 +1841,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P17" s="2">
-        <v>46307.39550542011</v>
+        <v>46307.88904457432</v>
       </c>
       <c r="Q17" s="2" t="s">
         <v>24</v>
@@ -1888,7 +1888,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P18" s="2">
-        <v>46307.39550540552</v>
+        <v>46307.88904455974</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>24</v>
@@ -1932,7 +1932,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P19" s="2">
-        <v>46307.3955053908</v>
+        <v>46307.88904454507</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>28</v>
@@ -1976,7 +1976,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P20" s="2">
-        <v>46307.39550537582</v>
+        <v>46307.88904452906</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>24</v>
@@ -2020,7 +2020,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P21">
-        <v>46307.39550536083</v>
+        <v>46307.88904451401</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>28</v>
@@ -2067,7 +2067,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P22">
-        <v>46307.39550534706</v>
+        <v>46307.88904449896</v>
       </c>
       <c r="Q22" t="s">
         <v>24</v>
@@ -2114,7 +2114,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P23">
-        <v>46307.39549715862</v>
+        <v>46307.889036688</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>28</v>
@@ -2161,7 +2161,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P24">
-        <v>46307.39549714453</v>
+        <v>46307.88903667321</v>
       </c>
       <c r="Q24" t="s">
         <v>24</v>
@@ -2205,7 +2205,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P25">
-        <v>46307.3954971128</v>
+        <v>46307.8890366583</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>28</v>
@@ -2252,7 +2252,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P26">
-        <v>46307.39549709752</v>
+        <v>46307.88903664359</v>
       </c>
       <c r="Q26" t="s">
         <v>24</v>
@@ -2302,7 +2302,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P27">
-        <v>46307.39549706617</v>
+        <v>46307.88903661463</v>
       </c>
       <c r="Q27" t="s">
         <v>24</v>
@@ -2349,7 +2349,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P28">
-        <v>46307.3954970824</v>
+        <v>46307.88903662929</v>
       </c>
       <c r="Q28" t="s">
         <v>24</v>
@@ -2399,7 +2399,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P29">
-        <v>46307.39549705025</v>
+        <v>46307.88903659968</v>
       </c>
       <c r="Q29" t="s">
         <v>24</v>
@@ -2446,7 +2446,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P30">
-        <v>46307.39549700749</v>
+        <v>46307.88903657054</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>28</v>
@@ -2490,7 +2490,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P31">
-        <v>46307.39549703622</v>
+        <v>46307.88903658502</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>28</v>
@@ -2537,7 +2537,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P32">
-        <v>46307.39549694471</v>
+        <v>46307.88903654088</v>
       </c>
       <c r="Q32" t="s">
         <v>24</v>
@@ -2581,7 +2581,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P33">
-        <v>46307.39549697418</v>
+        <v>46307.88903655546</v>
       </c>
       <c r="Q33" t="s">
         <v>24</v>
@@ -2625,7 +2625,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P34">
-        <v>46307.39549690611</v>
+        <v>46307.88903652613</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>28</v>
@@ -2672,7 +2672,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P35">
-        <v>46307.39549680644</v>
+        <v>46307.88903648117</v>
       </c>
       <c r="Q35" s="5" t="s">
         <v>28</v>
@@ -2722,7 +2722,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P36">
-        <v>46307.39549684314</v>
+        <v>46307.88903649613</v>
       </c>
       <c r="Q36" t="s">
         <v>24</v>
@@ -2769,7 +2769,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P37">
-        <v>46307.39549687666</v>
+        <v>46307.88903651119</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>28</v>
@@ -2813,7 +2813,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P38">
-        <v>46307.39549675402</v>
+        <v>46307.88903644997</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>28</v>
@@ -2857,7 +2857,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P39">
-        <v>46307.39549673259</v>
+        <v>46307.88903643428</v>
       </c>
       <c r="Q39" t="s">
         <v>24</v>
@@ -2904,7 +2904,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P40">
-        <v>46307.39549666933</v>
+        <v>46307.88903638735</v>
       </c>
       <c r="Q40" t="s">
         <v>24</v>
@@ -2948,7 +2948,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P41">
-        <v>46307.39549671813</v>
+        <v>46307.88903641787</v>
       </c>
       <c r="Q41" t="s">
         <v>24</v>
@@ -2997,7 +2997,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P42" s="6">
-        <v>46307.39551403373</v>
+        <v>46307.88905273634</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>24</v>
@@ -3048,7 +3048,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P43" s="6">
-        <v>46307.39551400379</v>
+        <v>46307.88905270749</v>
       </c>
       <c r="Q43" s="6" t="s">
         <v>24</v>
@@ -3099,7 +3099,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P44" s="6">
-        <v>46307.39551401839</v>
+        <v>46307.88905272199</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>24</v>
@@ -3148,7 +3148,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P45" s="6">
-        <v>46307.39551404792</v>
+        <v>46307.88905275082</v>
       </c>
       <c r="Q45" s="6" t="s">
         <v>24</v>
@@ -3197,7 +3197,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P46" s="6">
-        <v>46307.39551407743</v>
+        <v>46307.88905277973</v>
       </c>
       <c r="Q46" s="6" t="s">
         <v>24</v>
@@ -3244,7 +3244,7 @@
         <v>46300.75885634872</v>
       </c>
       <c r="P47" s="6">
-        <v>46307.39551410605</v>
+        <v>46307.88905280942</v>
       </c>
       <c r="Q47" s="6" t="s">
         <v>24</v>
@@ -3293,7 +3293,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P48" s="6">
-        <v>46307.39551412096</v>
+        <v>46307.88905282411</v>
       </c>
       <c r="Q48" s="6" t="s">
         <v>24</v>
@@ -3344,7 +3344,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P49" s="6">
-        <v>46307.395514164</v>
+        <v>46307.88905286766</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>24</v>
@@ -3391,7 +3391,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P50" s="6">
-        <v>46307.39551417845</v>
+        <v>46307.88905288192</v>
       </c>
       <c r="Q50" s="5" t="s">
         <v>28</v>
@@ -3440,7 +3440,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P51" s="6">
-        <v>46307.39552239229</v>
+        <v>46307.88906077829</v>
       </c>
       <c r="Q51" s="6" t="s">
         <v>24</v>
@@ -3487,7 +3487,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P52" s="6">
-        <v>46307.39552240674</v>
+        <v>46307.8890607925</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>24</v>
@@ -3536,7 +3536,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P53" s="6">
-        <v>46307.39552242085</v>
+        <v>46307.88906080725</v>
       </c>
       <c r="Q53" s="6" t="s">
         <v>24</v>
@@ -3585,7 +3585,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P54" s="6">
-        <v>46307.39552244938</v>
+        <v>46307.88906083583</v>
       </c>
       <c r="Q54" s="5" t="s">
         <v>28</v>
@@ -3634,7 +3634,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P55" s="6">
-        <v>46307.39552246492</v>
+        <v>46307.88906085039</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>24</v>
@@ -3681,7 +3681,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P56" s="6">
-        <v>46307.39552250843</v>
+        <v>46307.88906089382</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>28</v>
@@ -3730,7 +3730,7 @@
         <v>46300.75886472998</v>
       </c>
       <c r="P57" s="6">
-        <v>46307.3955225661</v>
+        <v>46307.88906095151</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>24</v>
@@ -3779,7 +3779,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P58" s="6">
-        <v>46307.39552249388</v>
+        <v>46307.88906087933</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>24</v>
@@ -3826,7 +3826,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P59" s="6">
-        <v>46307.39552247916</v>
+        <v>46307.88906086479</v>
       </c>
       <c r="Q59" s="5" t="s">
         <v>28</v>
@@ -4067,7 +4067,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P2" s="2">
-        <v>46307.39551395869</v>
+        <v>46307.88905266359</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>28</v>
@@ -4205,7 +4205,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P5" s="2">
-        <v>46307.39550555297</v>
+        <v>46307.88904470354</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>28</v>
@@ -4249,7 +4249,7 @@
         <v>46301.38232480602</v>
       </c>
       <c r="P6" s="2">
-        <v>46307.39550552344</v>
+        <v>46307.88904467553</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>28</v>
@@ -4293,7 +4293,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P7" s="2">
-        <v>46307.3955053908</v>
+        <v>46307.88904454507</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>28</v>
@@ -4337,7 +4337,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P8">
-        <v>46307.39550536083</v>
+        <v>46307.88904451401</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>28</v>
@@ -4384,7 +4384,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P9">
-        <v>46307.39549715862</v>
+        <v>46307.889036688</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>28</v>
@@ -4428,7 +4428,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P10">
-        <v>46307.3954971128</v>
+        <v>46307.8890366583</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>28</v>
@@ -4475,7 +4475,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P11">
-        <v>46307.39549700749</v>
+        <v>46307.88903657054</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>28</v>
@@ -4519,7 +4519,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P12">
-        <v>46307.39549703622</v>
+        <v>46307.88903658502</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>28</v>
@@ -4563,7 +4563,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P13">
-        <v>46307.39549690611</v>
+        <v>46307.88903652613</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>28</v>
@@ -4610,7 +4610,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P14">
-        <v>46307.39549680644</v>
+        <v>46307.88903648117</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>28</v>
@@ -4657,7 +4657,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P15">
-        <v>46307.39549687666</v>
+        <v>46307.88903651119</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>28</v>
@@ -4701,7 +4701,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P16">
-        <v>46307.39549675402</v>
+        <v>46307.88903644997</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>28</v>
@@ -4748,7 +4748,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P17" s="6">
-        <v>46307.39551417845</v>
+        <v>46307.88905288192</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>28</v>
@@ -4797,7 +4797,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P18" s="6">
-        <v>46307.39552244938</v>
+        <v>46307.88906083583</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>28</v>
@@ -4844,7 +4844,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P19" s="6">
-        <v>46307.39552250843</v>
+        <v>46307.88906089382</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>28</v>
@@ -4891,7 +4891,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P20" s="6">
-        <v>46307.39552247916</v>
+        <v>46307.88906086479</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>28</v>
@@ -4945,7 +4945,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -4993,10 +4993,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B2">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C2" t="s">
         <v>201</v>
@@ -5008,13 +5008,13 @@
         <v>3838</v>
       </c>
       <c r="F2">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -5028,10 +5028,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B3">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C3" t="s">
         <v>201</v>
@@ -5040,16 +5040,16 @@
         <v>192</v>
       </c>
       <c r="E3">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G3">
         <v>369</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -5058,15 +5058,15 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B4">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C4" t="s">
         <v>201</v>
@@ -5098,10 +5098,10 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B5">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C5" t="s">
         <v>201</v>
@@ -5116,7 +5116,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -5133,10 +5133,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B6">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C6" t="s">
         <v>201</v>
@@ -5168,10 +5168,10 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B7">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C7" t="s">
         <v>201</v>
@@ -5183,16 +5183,16 @@
         <v>3826</v>
       </c>
       <c r="F7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7">
         <v>0</v>
@@ -5203,45 +5203,45 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B8">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C8" t="s">
         <v>201</v>
       </c>
       <c r="D8">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E8">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G8">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B9">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C9" t="s">
         <v>201</v>
@@ -5273,10 +5273,10 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B10">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C10" t="s">
         <v>201</v>
@@ -5291,7 +5291,7 @@
         <v>0</v>
       </c>
       <c r="G10">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -5308,10 +5308,10 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B11">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C11" t="s">
         <v>201</v>
@@ -5323,16 +5323,16 @@
         <v>3820</v>
       </c>
       <c r="F11">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H11">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -5343,45 +5343,45 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B12">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C12" t="s">
         <v>201</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E12">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F12">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G12">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H12">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B13">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C13" t="s">
         <v>201</v>
@@ -5393,13 +5393,13 @@
         <v>160</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G13">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -5408,15 +5408,15 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B14">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C14" t="s">
         <v>201</v>
@@ -5428,21 +5428,56 @@
         <v>160</v>
       </c>
       <c r="F14">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H14">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B15">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C15" t="s">
+        <v>201</v>
+      </c>
+      <c r="D15">
+        <v>8</v>
+      </c>
+      <c r="E15">
+        <v>160</v>
+      </c>
+      <c r="F15">
+        <v>157</v>
+      </c>
+      <c r="G15">
+        <v>3</v>
+      </c>
+      <c r="H15">
+        <v>132</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-13-1926Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="826" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="213">
   <si>
     <t>Priority</t>
   </si>
@@ -1178,7 +1178,7 @@
         <v>46300.75884788632</v>
       </c>
       <c r="P2" s="2">
-        <v>46308.39987957306</v>
+        <v>46308.80860865589</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>24</v>
@@ -1222,7 +1222,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P3" s="2">
-        <v>46308.39987060975</v>
+        <v>46308.80860069162</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>28</v>
@@ -1310,7 +1310,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P5" s="2">
-        <v>46308.39987059969</v>
+        <v>46308.8086006791</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>28</v>
@@ -1357,7 +1357,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P6" s="2">
-        <v>46308.39987057789</v>
+        <v>46308.8086006663</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>24</v>
@@ -1404,7 +1404,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P7" s="2">
-        <v>46308.39987055867</v>
+        <v>46308.8086006416</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>24</v>
@@ -1448,7 +1448,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P8" s="2">
-        <v>46308.3998705492</v>
+        <v>46308.8086006291</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>24</v>
@@ -1495,7 +1495,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P9" s="2">
-        <v>46308.39987053999</v>
+        <v>46308.80860061695</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>24</v>
@@ -1542,7 +1542,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P10" s="2">
-        <v>46308.3998705304</v>
+        <v>46308.80860060442</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>24</v>
@@ -1589,7 +1589,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P11" s="2">
-        <v>46308.39987052104</v>
+        <v>46308.80860059104</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>24</v>
@@ -1636,7 +1636,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P12" s="2">
-        <v>46308.39987050221</v>
+        <v>46308.80860056587</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>24</v>
@@ -1680,7 +1680,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P13" s="2">
-        <v>46308.3998705116</v>
+        <v>46308.80860057846</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>28</v>
@@ -1724,7 +1724,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P14" s="2">
-        <v>46308.39987049278</v>
+        <v>46308.80860055199</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>24</v>
@@ -1768,7 +1768,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P15" s="2">
-        <v>46308.39987048287</v>
+        <v>46308.80860053844</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>28</v>
@@ -1815,7 +1815,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P16" s="2">
-        <v>46308.39987047307</v>
+        <v>46308.80860052589</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>24</v>
@@ -1862,7 +1862,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P17">
-        <v>46308.39987044345</v>
+        <v>46308.80860048686</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>28</v>
@@ -1909,7 +1909,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P18">
-        <v>46308.39987046314</v>
+        <v>46308.80860051262</v>
       </c>
       <c r="Q18" t="s">
         <v>24</v>
@@ -1953,7 +1953,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P19">
-        <v>46308.39987043281</v>
+        <v>46308.80860047329</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>28</v>
@@ -2000,7 +2000,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P20">
-        <v>46308.39987042029</v>
+        <v>46308.80860045793</v>
       </c>
       <c r="Q20" t="s">
         <v>24</v>
@@ -2050,7 +2050,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P21">
-        <v>46308.39986133329</v>
+        <v>46308.80859260492</v>
       </c>
       <c r="Q21" t="s">
         <v>24</v>
@@ -2097,7 +2097,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P22">
-        <v>46308.39986129606</v>
+        <v>46308.80859258032</v>
       </c>
       <c r="Q22" t="s">
         <v>24</v>
@@ -2144,7 +2144,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P23">
-        <v>46308.39986132326</v>
+        <v>46308.80859259245</v>
       </c>
       <c r="Q23" t="s">
         <v>24</v>
@@ -2194,7 +2194,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P24">
-        <v>46308.39986127555</v>
+        <v>46308.80859255515</v>
       </c>
       <c r="Q24" t="s">
         <v>24</v>
@@ -2241,7 +2241,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P25">
-        <v>46308.39986128596</v>
+        <v>46308.808592568</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>28</v>
@@ -2285,7 +2285,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P26">
-        <v>46308.39986126537</v>
+        <v>46308.8085925427</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>28</v>
@@ -2332,7 +2332,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P27">
-        <v>46308.39986125505</v>
+        <v>46308.8085925304</v>
       </c>
       <c r="Q27" t="s">
         <v>24</v>
@@ -2376,7 +2376,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P28">
-        <v>46308.39986124422</v>
+        <v>46308.80859251739</v>
       </c>
       <c r="Q28" t="s">
         <v>24</v>
@@ -2420,7 +2420,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P29">
-        <v>46308.39986123199</v>
+        <v>46308.80859250448</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>28</v>
@@ -2464,7 +2464,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P30">
-        <v>46308.3998612119</v>
+        <v>46308.80859249179</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>28</v>
@@ -2511,7 +2511,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P31">
-        <v>46308.39986118091</v>
+        <v>46308.80859245299</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>28</v>
@@ -2561,7 +2561,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P32">
-        <v>46308.39986119147</v>
+        <v>46308.80859246592</v>
       </c>
       <c r="Q32" t="s">
         <v>24</v>
@@ -2608,7 +2608,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P33">
-        <v>46308.39986120164</v>
+        <v>46308.80859247913</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>28</v>
@@ -2658,7 +2658,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P34">
-        <v>46308.39986117014</v>
+        <v>46308.80859243982</v>
       </c>
       <c r="Q34" t="s">
         <v>24</v>
@@ -2702,7 +2702,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P35">
-        <v>46308.3998611354</v>
+        <v>46308.80859242669</v>
       </c>
       <c r="Q35" s="5" t="s">
         <v>28</v>
@@ -2752,7 +2752,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P36">
-        <v>46308.39986111097</v>
+        <v>46308.80859240023</v>
       </c>
       <c r="Q36" t="s">
         <v>24</v>
@@ -2796,7 +2796,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P37">
-        <v>46308.39986101075</v>
+        <v>46308.80859238569</v>
       </c>
       <c r="Q37" t="s">
         <v>24</v>
@@ -2843,7 +2843,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P38">
-        <v>46308.39986099937</v>
+        <v>46308.80859237124</v>
       </c>
       <c r="Q38" t="s">
         <v>24</v>
@@ -2887,7 +2887,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P39">
-        <v>46308.39986097639</v>
+        <v>46308.80859234113</v>
       </c>
       <c r="Q39" t="s">
         <v>24</v>
@@ -2938,7 +2938,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P40" s="6">
-        <v>46308.3998796047</v>
+        <v>46308.80860869765</v>
       </c>
       <c r="Q40" s="6" t="s">
         <v>24</v>
@@ -2985,7 +2985,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P41" s="6">
-        <v>46308.39987963301</v>
+        <v>46308.8086087364</v>
       </c>
       <c r="Q41" s="5" t="s">
         <v>28</v>
@@ -3034,7 +3034,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P42" s="6">
-        <v>46308.39987966143</v>
+        <v>46308.8086087774</v>
       </c>
       <c r="Q42" s="6" t="s">
         <v>24</v>
@@ -3083,7 +3083,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P43" s="6">
-        <v>46308.39987962354</v>
+        <v>46308.80860872313</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>28</v>
@@ -3130,7 +3130,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P44" s="6">
-        <v>46308.39987959508</v>
+        <v>46308.80860868467</v>
       </c>
       <c r="Q44" s="6" t="s">
         <v>24</v>
@@ -3179,7 +3179,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P45" s="6">
-        <v>46308.39987958469</v>
+        <v>46308.80860867112</v>
       </c>
       <c r="Q45" s="6" t="s">
         <v>24</v>
@@ -3230,7 +3230,7 @@
         <v>46305.20576106136</v>
       </c>
       <c r="P46" s="6">
-        <v>46308.39987965173</v>
+        <v>46308.80860876467</v>
       </c>
       <c r="Q46" s="6" t="s">
         <v>24</v>
@@ -3279,7 +3279,7 @@
         <v>46300.75885622757</v>
       </c>
       <c r="P47" s="6">
-        <v>46308.39987969933</v>
+        <v>46308.80860882727</v>
       </c>
       <c r="Q47" s="6" t="s">
         <v>24</v>
@@ -3330,7 +3330,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P48" s="6">
-        <v>46308.39987968035</v>
+        <v>46308.80860880234</v>
       </c>
       <c r="Q48" s="6" t="s">
         <v>24</v>
@@ -3381,7 +3381,7 @@
         <v>46300.7588562628</v>
       </c>
       <c r="P49" s="6">
-        <v>46308.39987970874</v>
+        <v>46308.80860883948</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>24</v>
@@ -3430,7 +3430,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P50" s="6">
-        <v>46308.39987968992</v>
+        <v>46308.80860881492</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>24</v>
@@ -3479,7 +3479,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P51" s="6">
-        <v>46308.39987973654</v>
+        <v>46308.80860887733</v>
       </c>
       <c r="Q51" s="6" t="s">
         <v>24</v>
@@ -3528,7 +3528,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P52" s="6">
-        <v>46308.39987975493</v>
+        <v>46308.80860890263</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>24</v>
@@ -3579,7 +3579,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P53" s="6">
-        <v>46308.39988845142</v>
+        <v>46308.80861677252</v>
       </c>
       <c r="Q53" s="6" t="s">
         <v>24</v>
@@ -3626,7 +3626,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P54" s="6">
-        <v>46308.39988849323</v>
+        <v>46308.80861682777</v>
       </c>
       <c r="Q54" s="5" t="s">
         <v>28</v>
@@ -3675,7 +3675,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P55" s="6">
-        <v>46308.39988853089</v>
+        <v>46308.80861687777</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>24</v>
@@ -3722,7 +3722,7 @@
         <v>46300.75886463693</v>
       </c>
       <c r="P56" s="6">
-        <v>46308.39988854004</v>
+        <v>46308.80861688962</v>
       </c>
       <c r="Q56" s="6" t="s">
         <v>24</v>
@@ -3771,7 +3771,7 @@
         <v>46300.75886465221</v>
       </c>
       <c r="P57" s="6">
-        <v>46308.39988854943</v>
+        <v>46308.80861690162</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>24</v>
@@ -3820,7 +3820,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P58" s="6">
-        <v>46308.39988856782</v>
+        <v>46308.80861692582</v>
       </c>
       <c r="Q58" s="5" t="s">
         <v>28</v>
@@ -3869,7 +3869,7 @@
         <v>46300.75886468366</v>
       </c>
       <c r="P59" s="6">
-        <v>46308.39988857728</v>
+        <v>46308.80861693832</v>
       </c>
       <c r="Q59" s="6" t="s">
         <v>24</v>
@@ -3916,7 +3916,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P60" s="6">
-        <v>46308.39989750899</v>
+        <v>46308.80862494551</v>
       </c>
       <c r="Q60" s="5" t="s">
         <v>28</v>
@@ -4014,7 +4014,7 @@
         <v>46300.75886474836</v>
       </c>
       <c r="P62" s="6">
-        <v>46308.39989751922</v>
+        <v>46308.80862495991</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>24</v>
@@ -4061,7 +4061,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P63" s="6">
-        <v>46308.39988862519</v>
+        <v>46308.80861700077</v>
       </c>
       <c r="Q63" s="5" t="s">
         <v>28</v>
@@ -4310,7 +4310,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P2" s="2">
-        <v>46308.39987060975</v>
+        <v>46308.80860069162</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>28</v>
@@ -4398,7 +4398,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P4" s="2">
-        <v>46308.39987059969</v>
+        <v>46308.8086006791</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>28</v>
@@ -4442,7 +4442,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P5" s="2">
-        <v>46308.3998705116</v>
+        <v>46308.80860057846</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>28</v>
@@ -4486,7 +4486,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P6" s="2">
-        <v>46308.39987048287</v>
+        <v>46308.80860053844</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>28</v>
@@ -4533,7 +4533,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P7">
-        <v>46308.39987044345</v>
+        <v>46308.80860048686</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>28</v>
@@ -4577,7 +4577,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P8">
-        <v>46308.39987043281</v>
+        <v>46308.80860047329</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>28</v>
@@ -4624,7 +4624,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P9">
-        <v>46308.39986128596</v>
+        <v>46308.808592568</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>28</v>
@@ -4668,7 +4668,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P10">
-        <v>46308.39986126537</v>
+        <v>46308.8085925427</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>28</v>
@@ -4712,7 +4712,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P11">
-        <v>46308.39986123199</v>
+        <v>46308.80859250448</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>28</v>
@@ -4756,7 +4756,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P12">
-        <v>46308.3998612119</v>
+        <v>46308.80859249179</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>28</v>
@@ -4803,7 +4803,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P13">
-        <v>46308.39986118091</v>
+        <v>46308.80859245299</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>28</v>
@@ -4850,7 +4850,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P14">
-        <v>46308.39986120164</v>
+        <v>46308.80859247913</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>28</v>
@@ -4894,7 +4894,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P15">
-        <v>46308.3998611354</v>
+        <v>46308.80859242669</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>28</v>
@@ -4941,7 +4941,7 @@
         <v>46300.7588479478</v>
       </c>
       <c r="P16" s="6">
-        <v>46308.39987963301</v>
+        <v>46308.8086087364</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>28</v>
@@ -4990,7 +4990,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P17" s="6">
-        <v>46308.39987962354</v>
+        <v>46308.80860872313</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>28</v>
@@ -5037,7 +5037,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P18" s="6">
-        <v>46308.39988849323</v>
+        <v>46308.80861682777</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>28</v>
@@ -5086,7 +5086,7 @@
         <v>46300.75886466862</v>
       </c>
       <c r="P19" s="6">
-        <v>46308.39988856782</v>
+        <v>46308.80861692582</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>28</v>
@@ -5133,7 +5133,7 @@
         <v>46300.75886471466</v>
       </c>
       <c r="P20" s="6">
-        <v>46308.39989750899</v>
+        <v>46308.80862494551</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>28</v>
@@ -5229,7 +5229,7 @@
         <v>46300.75886479358</v>
       </c>
       <c r="P22" s="6">
-        <v>46308.39988862519</v>
+        <v>46308.80861700077</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>28</v>
@@ -5287,7 +5287,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -5335,10 +5335,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B2">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C2" t="s">
         <v>212</v>
@@ -5350,16 +5350,16 @@
         <v>3844</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -5370,45 +5370,45 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B3">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C3" t="s">
         <v>212</v>
       </c>
       <c r="D3">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E3">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G3">
         <v>381</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B4">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C4" t="s">
         <v>212</v>
@@ -5420,13 +5420,13 @@
         <v>3838</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H4">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -5440,10 +5440,10 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B5">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C5" t="s">
         <v>212</v>
@@ -5452,16 +5452,16 @@
         <v>192</v>
       </c>
       <c r="E5">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G5">
         <v>369</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -5470,15 +5470,15 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B6">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C6" t="s">
         <v>212</v>
@@ -5510,10 +5510,10 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B7">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C7" t="s">
         <v>212</v>
@@ -5528,7 +5528,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -5545,10 +5545,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B8">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C8" t="s">
         <v>212</v>
@@ -5580,10 +5580,10 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B9">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C9" t="s">
         <v>212</v>
@@ -5595,16 +5595,16 @@
         <v>3826</v>
       </c>
       <c r="F9">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -5615,45 +5615,45 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B10">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C10" t="s">
         <v>212</v>
       </c>
       <c r="D10">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E10">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G10">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B11">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C11" t="s">
         <v>212</v>
@@ -5685,10 +5685,10 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B12">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C12" t="s">
         <v>212</v>
@@ -5703,7 +5703,7 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -5720,10 +5720,10 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B13">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C13" t="s">
         <v>212</v>
@@ -5735,16 +5735,16 @@
         <v>3820</v>
       </c>
       <c r="F13">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H13">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -5755,45 +5755,45 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B14">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C14" t="s">
         <v>212</v>
       </c>
       <c r="D14">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E14">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G14">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B15">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C15" t="s">
         <v>212</v>
@@ -5805,13 +5805,13 @@
         <v>160</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G15">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -5820,15 +5820,15 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B16">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C16" t="s">
         <v>212</v>
@@ -5840,21 +5840,56 @@
         <v>160</v>
       </c>
       <c r="F16">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H16">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
       <c r="K16">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B17">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C17" t="s">
+        <v>212</v>
+      </c>
+      <c r="D17">
+        <v>8</v>
+      </c>
+      <c r="E17">
+        <v>160</v>
+      </c>
+      <c r="F17">
+        <v>157</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17">
+        <v>132</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-16-1651Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="226">
   <si>
     <t>Priority</t>
   </si>
@@ -1214,7 +1214,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P2" s="2">
-        <v>46311.30744705819</v>
+        <v>46311.70088691096</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1258,7 +1258,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P3" s="2">
-        <v>46311.30744707253</v>
+        <v>46311.70088692041</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>23</v>
@@ -1305,7 +1305,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P4" s="2">
-        <v>46311.30744704161</v>
+        <v>46311.70088690126</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>23</v>
@@ -1352,7 +1352,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P5" s="2">
-        <v>46311.30744702817</v>
+        <v>46311.70088689196</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1399,7 +1399,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P6" s="2">
-        <v>46311.3074470153</v>
+        <v>46311.70088688222</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>23</v>
@@ -1446,7 +1446,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P7" s="2">
-        <v>46311.30744697552</v>
+        <v>46311.70088685404</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>23</v>
@@ -1490,7 +1490,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P8" s="2">
-        <v>46311.30744698845</v>
+        <v>46311.70088686351</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
@@ -1534,7 +1534,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P9" s="2">
-        <v>46311.30744700151</v>
+        <v>46311.70088687293</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>23</v>
@@ -1578,7 +1578,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P10" s="2">
-        <v>46311.30744696164</v>
+        <v>46311.70088684419</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -1625,7 +1625,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P11" s="2">
-        <v>46311.30744694464</v>
+        <v>46311.70088683406</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>23</v>
@@ -1675,7 +1675,7 @@
         <v>46311.30744692709</v>
       </c>
       <c r="P12" s="2">
-        <v>46311.30744692712</v>
+        <v>46311.70088682229</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1722,7 +1722,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P13" s="2">
-        <v>46311.3074373737</v>
+        <v>46311.70087868374</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -1769,7 +1769,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P14" s="2">
-        <v>46311.30743740102</v>
+        <v>46311.7008787021</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>23</v>
@@ -1813,7 +1813,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P15" s="2">
-        <v>46311.30743734578</v>
+        <v>46311.70087866466</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -1860,7 +1860,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P16" s="2">
-        <v>46311.30743735946</v>
+        <v>46311.70087867416</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>23</v>
@@ -1904,7 +1904,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P17" s="2">
-        <v>46311.30743733215</v>
+        <v>46311.70087865533</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -1954,7 +1954,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P18" s="2">
-        <v>46311.30743726892</v>
+        <v>46311.70087862734</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -2001,7 +2001,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P19" s="2">
-        <v>46311.30743728172</v>
+        <v>46311.70087863646</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>23</v>
@@ -2048,7 +2048,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P20" s="2">
-        <v>46311.30743725552</v>
+        <v>46311.70087861818</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>23</v>
@@ -2095,7 +2095,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P21" s="2">
-        <v>46311.30743731892</v>
+        <v>46311.70087864589</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>46</v>
@@ -2145,7 +2145,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P22">
-        <v>46311.30743724266</v>
+        <v>46311.7008786087</v>
       </c>
       <c r="Q22" t="s">
         <v>23</v>
@@ -2192,7 +2192,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P23">
-        <v>46311.30743721643</v>
+        <v>46311.70087858952</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
@@ -2236,7 +2236,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P24">
-        <v>46311.30743722944</v>
+        <v>46311.70087859921</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>46</v>
@@ -2280,7 +2280,7 @@
         <v>46309.72495168629</v>
       </c>
       <c r="P25">
-        <v>46311.30743717797</v>
+        <v>46311.70087856058</v>
       </c>
       <c r="Q25" t="s">
         <v>23</v>
@@ -2324,7 +2324,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P26">
-        <v>46311.307437191</v>
+        <v>46311.70087857031</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>46</v>
@@ -2371,7 +2371,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P27">
-        <v>46311.30743720373</v>
+        <v>46311.70087857965</v>
       </c>
       <c r="Q27" t="s">
         <v>23</v>
@@ -2418,7 +2418,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P28">
-        <v>46311.30743712274</v>
+        <v>46311.7008785186</v>
       </c>
       <c r="Q28" t="s">
         <v>23</v>
@@ -2462,7 +2462,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P29">
-        <v>46311.30743713841</v>
+        <v>46311.7008785302</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2506,7 +2506,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P30">
-        <v>46311.30743715168</v>
+        <v>46311.70087854062</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>46</v>
@@ -2550,7 +2550,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P31">
-        <v>46311.30742787745</v>
+        <v>46311.70087044157</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>46</v>
@@ -2597,7 +2597,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P32">
-        <v>46311.30742785161</v>
+        <v>46311.70087042241</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>46</v>
@@ -2647,7 +2647,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P33">
-        <v>46311.30742783823</v>
+        <v>46311.70087041293</v>
       </c>
       <c r="Q33" t="s">
         <v>23</v>
@@ -2694,7 +2694,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P34">
-        <v>46311.30742782442</v>
+        <v>46311.70087040275</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>46</v>
@@ -2744,7 +2744,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P35">
-        <v>46311.30742786467</v>
+        <v>46311.70087043183</v>
       </c>
       <c r="Q35" t="s">
         <v>23</v>
@@ -2791,7 +2791,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P36">
-        <v>46311.30742780838</v>
+        <v>46311.70087039313</v>
       </c>
       <c r="Q36" s="5" t="s">
         <v>46</v>
@@ -2835,7 +2835,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P37">
-        <v>46311.30742765773</v>
+        <v>46311.700870364</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>46</v>
@@ -2879,7 +2879,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P38">
-        <v>46311.30742767097</v>
+        <v>46311.70087037373</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>46</v>
@@ -2926,7 +2926,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P39">
-        <v>46311.30742768373</v>
+        <v>46311.70087038344</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>46</v>
@@ -2976,7 +2976,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P40">
-        <v>46311.30742764476</v>
+        <v>46311.70087035413</v>
       </c>
       <c r="Q40" t="s">
         <v>23</v>
@@ -3023,7 +3023,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P41">
-        <v>46311.30742763128</v>
+        <v>46311.70087034364</v>
       </c>
       <c r="Q41" s="5" t="s">
         <v>46</v>
@@ -3070,7 +3070,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P42">
-        <v>46311.30742761814</v>
+        <v>46311.70087033371</v>
       </c>
       <c r="Q42" s="5" t="s">
         <v>46</v>
@@ -3117,7 +3117,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P43">
-        <v>46311.30742760486</v>
+        <v>46311.70087032368</v>
       </c>
       <c r="Q43" t="s">
         <v>23</v>
@@ -3167,7 +3167,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P44">
-        <v>46311.30742759143</v>
+        <v>46311.70087031323</v>
       </c>
       <c r="Q44" t="s">
         <v>23</v>
@@ -3211,7 +3211,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P45">
-        <v>46311.30742757768</v>
+        <v>46311.70087030291</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>46</v>
@@ -3261,7 +3261,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P46">
-        <v>46311.30742754995</v>
+        <v>46311.7008702819</v>
       </c>
       <c r="Q46" t="s">
         <v>23</v>
@@ -3305,7 +3305,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P47">
-        <v>46311.30742753583</v>
+        <v>46311.70087027091</v>
       </c>
       <c r="Q47" t="s">
         <v>23</v>
@@ -3352,7 +3352,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P48">
-        <v>46311.30742752137</v>
+        <v>46311.70087025949</v>
       </c>
       <c r="Q48" t="s">
         <v>23</v>
@@ -3396,7 +3396,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P49">
-        <v>46311.30742749263</v>
+        <v>46311.70087023666</v>
       </c>
       <c r="Q49" t="s">
         <v>23</v>
@@ -3445,7 +3445,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P50" s="6">
-        <v>46311.30744709933</v>
+        <v>46311.70088693928</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>23</v>
@@ -3492,7 +3492,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P51" s="6">
-        <v>46311.30744711268</v>
+        <v>46311.70088694827</v>
       </c>
       <c r="Q51" s="5" t="s">
         <v>46</v>
@@ -3539,7 +3539,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P52" s="6">
-        <v>46311.30744716735</v>
+        <v>46311.70088698581</v>
       </c>
       <c r="Q52" s="5" t="s">
         <v>46</v>
@@ -3586,7 +3586,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P53" s="6">
-        <v>46311.30744715399</v>
+        <v>46311.70088697635</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>46</v>
@@ -3637,7 +3637,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P54" s="6">
-        <v>46311.30745569724</v>
+        <v>46311.70089512802</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>23</v>
@@ -3686,7 +3686,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P55" s="6">
-        <v>46311.30745564263</v>
+        <v>46311.70089508668</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>23</v>
@@ -3735,7 +3735,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P56" s="6">
-        <v>46311.30745573662</v>
+        <v>46311.70089515702</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>46</v>
@@ -3782,7 +3782,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P57" s="6">
-        <v>46311.3074557103</v>
+        <v>46311.70089513763</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>23</v>
@@ -3831,7 +3831,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P58" s="6">
-        <v>46311.30745572347</v>
+        <v>46311.70089514742</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>23</v>
@@ -3933,7 +3933,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P60" s="6">
-        <v>46311.30745576383</v>
+        <v>46311.70089517583</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>23</v>
@@ -3982,7 +3982,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P61" s="6">
-        <v>46311.30745577747</v>
+        <v>46311.70089518549</v>
       </c>
       <c r="Q61" s="6" t="s">
         <v>23</v>
@@ -4031,7 +4031,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P62" s="6">
-        <v>46311.30745581691</v>
+        <v>46311.70089521474</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>23</v>
@@ -4080,7 +4080,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P63" s="6">
-        <v>46311.30745584252</v>
+        <v>46311.70089523357</v>
       </c>
       <c r="Q63" s="6" t="s">
         <v>23</v>
@@ -4131,7 +4131,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P64" s="6">
-        <v>46311.30745586863</v>
+        <v>46311.7008952556</v>
       </c>
       <c r="Q64" s="6" t="s">
         <v>23</v>
@@ -4178,7 +4178,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P65" s="6">
-        <v>46311.30746437659</v>
+        <v>46311.70090339411</v>
       </c>
       <c r="Q65" s="5" t="s">
         <v>46</v>
@@ -4227,7 +4227,7 @@
         <v>46300.75885649968</v>
       </c>
       <c r="P66" s="6">
-        <v>46311.3074644164</v>
+        <v>46311.70090342543</v>
       </c>
       <c r="Q66" s="6" t="s">
         <v>23</v>
@@ -4482,7 +4482,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P2" s="2">
-        <v>46311.30744698845</v>
+        <v>46311.70088686351</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>46</v>
@@ -4526,7 +4526,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P3" s="2">
-        <v>46311.30744696164</v>
+        <v>46311.70088684419</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>46</v>
@@ -4573,7 +4573,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P4" s="2">
-        <v>46311.3074373737</v>
+        <v>46311.70087868374</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>46</v>
@@ -4617,7 +4617,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P5" s="2">
-        <v>46311.30743734578</v>
+        <v>46311.70087866466</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>46</v>
@@ -4661,7 +4661,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P6" s="2">
-        <v>46311.30743733215</v>
+        <v>46311.70087865533</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>46</v>
@@ -4708,7 +4708,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P7" s="2">
-        <v>46311.30743731892</v>
+        <v>46311.70087864589</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>46</v>
@@ -4755,7 +4755,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P8">
-        <v>46311.30743721643</v>
+        <v>46311.70087858952</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
@@ -4799,7 +4799,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P9">
-        <v>46311.30743722944</v>
+        <v>46311.70087859921</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>46</v>
@@ -4843,7 +4843,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P10">
-        <v>46311.307437191</v>
+        <v>46311.70087857031</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -4887,7 +4887,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P11">
-        <v>46311.30743715168</v>
+        <v>46311.70087854062</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>46</v>
@@ -4931,7 +4931,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P12">
-        <v>46311.30742787745</v>
+        <v>46311.70087044157</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>46</v>
@@ -4978,7 +4978,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P13">
-        <v>46311.30742785161</v>
+        <v>46311.70087042241</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -5025,7 +5025,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P14">
-        <v>46311.30742782442</v>
+        <v>46311.70087040275</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>46</v>
@@ -5072,7 +5072,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P15">
-        <v>46311.30742780838</v>
+        <v>46311.70087039313</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -5116,7 +5116,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P16">
-        <v>46311.30742765773</v>
+        <v>46311.700870364</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>46</v>
@@ -5160,7 +5160,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P17">
-        <v>46311.30742767097</v>
+        <v>46311.70087037373</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -5207,7 +5207,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P18">
-        <v>46311.30742768373</v>
+        <v>46311.70087038344</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>46</v>
@@ -5254,7 +5254,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P19">
-        <v>46311.30742763128</v>
+        <v>46311.70087034364</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>46</v>
@@ -5301,7 +5301,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P20">
-        <v>46311.30742761814</v>
+        <v>46311.70087033371</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>46</v>
@@ -5345,7 +5345,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P21">
-        <v>46311.30742757768</v>
+        <v>46311.70087030291</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>46</v>
@@ -5392,7 +5392,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P22" s="6">
-        <v>46311.30744711268</v>
+        <v>46311.70088694827</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>46</v>
@@ -5439,7 +5439,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P23" s="6">
-        <v>46311.30744716735</v>
+        <v>46311.70088698581</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
@@ -5486,7 +5486,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P24" s="6">
-        <v>46311.30744715399</v>
+        <v>46311.70088697635</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>46</v>
@@ -5535,7 +5535,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P25" s="6">
-        <v>46311.30745573662</v>
+        <v>46311.70089515702</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>46</v>
@@ -5633,7 +5633,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P27" s="6">
-        <v>46311.30746437659</v>
+        <v>46311.70090339411</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>46</v>
@@ -5701,7 +5701,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -5749,10 +5749,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B2">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C2" t="s">
         <v>225</v>
@@ -5764,16 +5764,16 @@
         <v>3861</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H2">
         <v>0</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -5784,45 +5784,45 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B3">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C3" t="s">
         <v>225</v>
       </c>
       <c r="D3">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E3">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
         <v>394</v>
       </c>
       <c r="H3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3">
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B4">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C4" t="s">
         <v>225</v>
@@ -5831,33 +5831,33 @@
         <v>193</v>
       </c>
       <c r="E4">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H4">
         <v>2</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B5">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C5" t="s">
         <v>225</v>
@@ -5866,16 +5866,16 @@
         <v>193</v>
       </c>
       <c r="E5">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F5">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -5884,15 +5884,15 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B6">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C6" t="s">
         <v>225</v>
@@ -5901,33 +5901,33 @@
         <v>193</v>
       </c>
       <c r="E6">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G6">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B7">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C7" t="s">
         <v>225</v>
@@ -5942,7 +5942,7 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -5959,10 +5959,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B8">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C8" t="s">
         <v>225</v>
@@ -5974,16 +5974,16 @@
         <v>3844</v>
       </c>
       <c r="F8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>0</v>
@@ -5994,45 +5994,45 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B9">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C9" t="s">
         <v>225</v>
       </c>
       <c r="D9">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E9">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G9">
         <v>381</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B10">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C10" t="s">
         <v>225</v>
@@ -6044,13 +6044,13 @@
         <v>3838</v>
       </c>
       <c r="F10">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H10">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -6064,10 +6064,10 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B11">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C11" t="s">
         <v>225</v>
@@ -6076,16 +6076,16 @@
         <v>192</v>
       </c>
       <c r="E11">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G11">
         <v>369</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -6094,15 +6094,15 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B12">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C12" t="s">
         <v>225</v>
@@ -6134,10 +6134,10 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B13">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C13" t="s">
         <v>225</v>
@@ -6152,7 +6152,7 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -6169,10 +6169,10 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B14">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C14" t="s">
         <v>225</v>
@@ -6204,10 +6204,10 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B15">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C15" t="s">
         <v>225</v>
@@ -6219,16 +6219,16 @@
         <v>3826</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G15">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I15">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15">
         <v>0</v>
@@ -6239,45 +6239,45 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B16">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C16" t="s">
         <v>225</v>
       </c>
       <c r="D16">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E16">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G16">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J16">
         <v>0</v>
       </c>
       <c r="K16">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B17">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C17" t="s">
         <v>225</v>
@@ -6309,10 +6309,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B18">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C18" t="s">
         <v>225</v>
@@ -6327,7 +6327,7 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -6344,10 +6344,10 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B19">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C19" t="s">
         <v>225</v>
@@ -6359,16 +6359,16 @@
         <v>3820</v>
       </c>
       <c r="F19">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H19">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I19">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -6379,45 +6379,45 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B20">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C20" t="s">
         <v>225</v>
       </c>
       <c r="D20">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E20">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F20">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G20">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B21">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C21" t="s">
         <v>225</v>
@@ -6429,13 +6429,13 @@
         <v>160</v>
       </c>
       <c r="F21">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G21">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -6444,15 +6444,15 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B22">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C22" t="s">
         <v>225</v>
@@ -6464,21 +6464,56 @@
         <v>160</v>
       </c>
       <c r="F22">
-        <v>157</v>
+        <v>0</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>160</v>
       </c>
       <c r="H22">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B23">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C23" t="s">
+        <v>225</v>
+      </c>
+      <c r="D23">
+        <v>8</v>
+      </c>
+      <c r="E23">
+        <v>160</v>
+      </c>
+      <c r="F23">
+        <v>157</v>
+      </c>
+      <c r="G23">
+        <v>3</v>
+      </c>
+      <c r="H23">
+        <v>132</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-17-0710Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Runs" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-Day Working List'!$A$1:$Q$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'30-Day Working List'!$A$1:$Q$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Needs Review'!$A$1:$Q$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="915" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="224">
   <si>
     <t>Priority</t>
   </si>
@@ -656,12 +656,6 @@
   </si>
   <si>
     <t>Garima diggiwal</t>
-  </si>
-  <si>
-    <t>NOEL PHARMA (INDIA) PRIVATE LIMITED</t>
-  </si>
-  <si>
-    <t>Mr. Prem Chand Goyal</t>
   </si>
   <si>
     <t>Started</t>
@@ -1102,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q66"/>
+  <dimension ref="A1:Q65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1193,7 +1187,7 @@
         <v>46312</v>
       </c>
       <c r="I2" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>21</v>
@@ -1214,7 +1208,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P2" s="2">
-        <v>46311.70088691096</v>
+        <v>46312.29485674985</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1240,7 +1234,7 @@
         <v>46312</v>
       </c>
       <c r="I3" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>26</v>
@@ -1258,7 +1252,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P3" s="2">
-        <v>46311.70088692041</v>
+        <v>46312.29485676255</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>23</v>
@@ -1284,7 +1278,7 @@
         <v>46312</v>
       </c>
       <c r="I4" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>29</v>
@@ -1305,7 +1299,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P4" s="2">
-        <v>46311.70088690126</v>
+        <v>46312.29485673701</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>23</v>
@@ -1331,7 +1325,7 @@
         <v>46312</v>
       </c>
       <c r="I5" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>33</v>
@@ -1352,7 +1346,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P5" s="2">
-        <v>46311.70088689196</v>
+        <v>46312.29485672439</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1378,7 +1372,7 @@
         <v>46313</v>
       </c>
       <c r="I6" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>37</v>
@@ -1399,7 +1393,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P6" s="2">
-        <v>46311.70088688222</v>
+        <v>46312.29485671136</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>23</v>
@@ -1428,7 +1422,7 @@
         <v>46314</v>
       </c>
       <c r="I7" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>42</v>
@@ -1446,7 +1440,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P7" s="2">
-        <v>46311.70088685404</v>
+        <v>46312.29485667367</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>23</v>
@@ -1472,7 +1466,7 @@
         <v>46314</v>
       </c>
       <c r="I8" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>45</v>
@@ -1490,7 +1484,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P8" s="2">
-        <v>46311.70088686351</v>
+        <v>46312.29485668633</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
@@ -1516,7 +1510,7 @@
         <v>46314</v>
       </c>
       <c r="I9" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>48</v>
@@ -1534,7 +1528,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P9" s="2">
-        <v>46311.70088687293</v>
+        <v>46312.29485669876</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>23</v>
@@ -1560,7 +1554,7 @@
         <v>46315</v>
       </c>
       <c r="I10" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>50</v>
@@ -1578,7 +1572,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P10" s="2">
-        <v>46311.70088684419</v>
+        <v>46312.29485666077</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -1604,7 +1598,7 @@
         <v>46315</v>
       </c>
       <c r="I11" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>53</v>
@@ -1625,7 +1619,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P11" s="2">
-        <v>46311.70088683406</v>
+        <v>46312.29485664792</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>23</v>
@@ -1654,7 +1648,7 @@
         <v>46315</v>
       </c>
       <c r="I12" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>58</v>
@@ -1675,7 +1669,7 @@
         <v>46311.30744692709</v>
       </c>
       <c r="P12" s="2">
-        <v>46311.70088682229</v>
+        <v>46312.29485663317</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1701,7 +1695,7 @@
         <v>46316</v>
       </c>
       <c r="I13" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>61</v>
@@ -1722,7 +1716,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P13" s="2">
-        <v>46311.70087868374</v>
+        <v>46312.29484303323</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -1748,7 +1742,7 @@
         <v>46316</v>
       </c>
       <c r="I14" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14" s="2" t="s">
         <v>65</v>
@@ -1769,7 +1763,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P14" s="2">
-        <v>46311.7008787021</v>
+        <v>46312.29484306075</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>23</v>
@@ -1795,7 +1789,7 @@
         <v>46317</v>
       </c>
       <c r="I15" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>68</v>
@@ -1813,7 +1807,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P15" s="2">
-        <v>46311.70087866466</v>
+        <v>46312.29484300764</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -1842,7 +1836,7 @@
         <v>46317</v>
       </c>
       <c r="I16" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>72</v>
@@ -1860,7 +1854,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P16" s="2">
-        <v>46311.70087867416</v>
+        <v>46312.29484302051</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>23</v>
@@ -1886,7 +1880,7 @@
         <v>46317</v>
       </c>
       <c r="I17" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>74</v>
@@ -1904,7 +1898,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P17" s="2">
-        <v>46311.70087865533</v>
+        <v>46312.29484299479</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -1933,7 +1927,7 @@
         <v>46318</v>
       </c>
       <c r="I18" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J18" s="2" t="s">
         <v>76</v>
@@ -1954,7 +1948,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P18" s="2">
-        <v>46311.70087862734</v>
+        <v>46312.29484295692</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -1980,7 +1974,7 @@
         <v>46318</v>
       </c>
       <c r="I19" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>80</v>
@@ -2001,7 +1995,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P19" s="2">
-        <v>46311.70087863646</v>
+        <v>46312.29484296968</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>23</v>
@@ -2027,7 +2021,7 @@
         <v>46318</v>
       </c>
       <c r="I20" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>61</v>
@@ -2048,7 +2042,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P20" s="2">
-        <v>46311.70087861818</v>
+        <v>46312.29484294421</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>23</v>
@@ -2074,7 +2068,7 @@
         <v>46318</v>
       </c>
       <c r="I21" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>85</v>
@@ -2095,44 +2089,44 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P21" s="2">
-        <v>46311.70087864589</v>
+        <v>46312.29484298224</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
-      <c r="A22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22" t="s">
-        <v>18</v>
-      </c>
-      <c r="C22" t="s">
+    <row r="22" spans="1:17" s="2" customFormat="1">
+      <c r="A22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G22">
+      <c r="G22" s="2">
         <v>0.93</v>
       </c>
       <c r="H22" s="3">
         <v>46319</v>
       </c>
-      <c r="I22">
-        <v>8</v>
-      </c>
-      <c r="J22" t="s">
+      <c r="I22" s="2">
+        <v>7</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="2">
         <v>2</v>
       </c>
-      <c r="L22" t="s">
+      <c r="L22" s="2" t="s">
         <v>91</v>
       </c>
       <c r="M22" s="4" t="s">
@@ -2141,45 +2135,45 @@
       <c r="N22" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O22">
+      <c r="O22" s="2">
         <v>46305.20575263901</v>
       </c>
-      <c r="P22">
-        <v>46311.7008786087</v>
-      </c>
-      <c r="Q22" t="s">
+      <c r="P22" s="2">
+        <v>46312.29484293171</v>
+      </c>
+      <c r="Q22" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
-      <c r="A23" t="s">
-        <v>18</v>
-      </c>
-      <c r="B23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" t="s">
+    <row r="23" spans="1:17" s="2" customFormat="1">
+      <c r="A23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="2">
         <v>0.2</v>
       </c>
       <c r="H23" s="3">
         <v>46319</v>
       </c>
-      <c r="I23">
-        <v>8</v>
-      </c>
-      <c r="J23" t="s">
+      <c r="I23" s="2">
+        <v>7</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="2">
         <v>2</v>
       </c>
-      <c r="L23" t="s">
+      <c r="L23" s="2" t="s">
         <v>94</v>
       </c>
       <c r="M23" s="4" t="s">
@@ -2188,42 +2182,42 @@
       <c r="N23" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O23">
+      <c r="O23" s="2">
         <v>46307.39549700746</v>
       </c>
-      <c r="P23">
-        <v>46311.70087858952</v>
+      <c r="P23" s="2">
+        <v>46312.29484290504</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="24" spans="1:17">
-      <c r="A24" t="s">
-        <v>18</v>
-      </c>
-      <c r="B24" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" t="s">
+    <row r="24" spans="1:17" s="2" customFormat="1">
+      <c r="A24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G24">
+      <c r="G24" s="2">
         <v>0.2</v>
       </c>
       <c r="H24" s="3">
         <v>46319</v>
       </c>
-      <c r="I24">
-        <v>8</v>
-      </c>
-      <c r="J24" t="s">
+      <c r="I24" s="2">
+        <v>7</v>
+      </c>
+      <c r="J24" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="2">
         <v>1</v>
       </c>
       <c r="M24" s="4" t="s">
@@ -2232,42 +2226,42 @@
       <c r="N24" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O24">
+      <c r="O24" s="2">
         <v>46307.3954970362</v>
       </c>
-      <c r="P24">
-        <v>46311.70087859921</v>
+      <c r="P24" s="2">
+        <v>46312.29484291846</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="25" spans="1:17">
-      <c r="A25" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" t="s">
+    <row r="25" spans="1:17" s="2" customFormat="1">
+      <c r="A25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G25">
+      <c r="G25" s="2">
         <v>0.95</v>
       </c>
       <c r="H25" s="3">
         <v>46319</v>
       </c>
-      <c r="I25">
-        <v>8</v>
-      </c>
-      <c r="J25" t="s">
+      <c r="I25" s="2">
+        <v>7</v>
+      </c>
+      <c r="J25" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="2">
         <v>2</v>
       </c>
       <c r="M25" s="4" t="s">
@@ -2276,42 +2270,42 @@
       <c r="N25" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O25">
+      <c r="O25" s="2">
         <v>46309.72495168629</v>
       </c>
-      <c r="P25">
-        <v>46311.70087856058</v>
-      </c>
-      <c r="Q25" t="s">
+      <c r="P25" s="2">
+        <v>46312.29484286576</v>
+      </c>
+      <c r="Q25" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
-      <c r="A26" t="s">
-        <v>18</v>
-      </c>
-      <c r="B26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" t="s">
+    <row r="26" spans="1:17" s="2" customFormat="1">
+      <c r="A26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G26">
+      <c r="G26" s="2">
         <v>0.2</v>
       </c>
       <c r="H26" s="3">
         <v>46319</v>
       </c>
-      <c r="I26">
-        <v>8</v>
-      </c>
-      <c r="J26" t="s">
+      <c r="I26" s="2">
+        <v>7</v>
+      </c>
+      <c r="J26" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="2">
         <v>1</v>
       </c>
       <c r="M26" s="4" t="s">
@@ -2320,45 +2314,45 @@
       <c r="N26" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O26">
+      <c r="O26" s="2">
         <v>46309.72495171529</v>
       </c>
-      <c r="P26">
-        <v>46311.70087857031</v>
+      <c r="P26" s="2">
+        <v>46312.29484287875</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:17">
-      <c r="A27" t="s">
-        <v>18</v>
-      </c>
-      <c r="B27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" t="s">
+    <row r="27" spans="1:17" s="2" customFormat="1">
+      <c r="A27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G27">
+      <c r="G27" s="2">
         <v>0.91</v>
       </c>
       <c r="H27" s="3">
         <v>46319</v>
       </c>
-      <c r="I27">
-        <v>8</v>
-      </c>
-      <c r="J27" t="s">
+      <c r="I27" s="2">
+        <v>7</v>
+      </c>
+      <c r="J27" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="K27">
+      <c r="K27" s="2">
         <v>2</v>
       </c>
       <c r="M27" s="4" t="s">
@@ -2367,13 +2361,13 @@
       <c r="N27" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O27">
+      <c r="O27" s="2">
         <v>46310.31707038325</v>
       </c>
-      <c r="P27">
-        <v>46311.70087857965</v>
-      </c>
-      <c r="Q27" t="s">
+      <c r="P27" s="2">
+        <v>46312.29484289186</v>
+      </c>
+      <c r="Q27" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2397,7 +2391,7 @@
         <v>46320</v>
       </c>
       <c r="I28">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J28" t="s">
         <v>106</v>
@@ -2418,7 +2412,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P28">
-        <v>46311.7008785186</v>
+        <v>46312.29484281153</v>
       </c>
       <c r="Q28" t="s">
         <v>23</v>
@@ -2444,7 +2438,7 @@
         <v>46320</v>
       </c>
       <c r="I29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J29" t="s">
         <v>109</v>
@@ -2462,7 +2456,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P29">
-        <v>46311.7008785302</v>
+        <v>46312.29484282663</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2488,7 +2482,7 @@
         <v>46320</v>
       </c>
       <c r="I30">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J30" t="s">
         <v>111</v>
@@ -2506,7 +2500,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P30">
-        <v>46311.70087854062</v>
+        <v>46312.29484284001</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>46</v>
@@ -2532,7 +2526,7 @@
         <v>46321</v>
       </c>
       <c r="I31">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J31" t="s">
         <v>113</v>
@@ -2550,7 +2544,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P31">
-        <v>46311.70087044157</v>
+        <v>46312.29483166153</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>46</v>
@@ -2576,7 +2570,7 @@
         <v>46322</v>
       </c>
       <c r="I32">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J32" t="s">
         <v>115</v>
@@ -2597,7 +2591,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P32">
-        <v>46311.70087042241</v>
+        <v>46312.29483163588</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>46</v>
@@ -2626,7 +2620,7 @@
         <v>46322</v>
       </c>
       <c r="I33">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J33" t="s">
         <v>118</v>
@@ -2647,7 +2641,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P33">
-        <v>46311.70087041293</v>
+        <v>46312.294831623</v>
       </c>
       <c r="Q33" t="s">
         <v>23</v>
@@ -2673,7 +2667,7 @@
         <v>46322</v>
       </c>
       <c r="I34">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J34" t="s">
         <v>121</v>
@@ -2694,7 +2688,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P34">
-        <v>46311.70087040275</v>
+        <v>46312.29483160963</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>46</v>
@@ -2723,7 +2717,7 @@
         <v>46322</v>
       </c>
       <c r="I35">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J35" t="s">
         <v>124</v>
@@ -2744,7 +2738,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P35">
-        <v>46311.70087043183</v>
+        <v>46312.29483164889</v>
       </c>
       <c r="Q35" t="s">
         <v>23</v>
@@ -2770,7 +2764,7 @@
         <v>46322</v>
       </c>
       <c r="I36">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J36" t="s">
         <v>127</v>
@@ -2791,7 +2785,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P36">
-        <v>46311.70087039313</v>
+        <v>46312.29483159653</v>
       </c>
       <c r="Q36" s="5" t="s">
         <v>46</v>
@@ -2817,7 +2811,7 @@
         <v>46323</v>
       </c>
       <c r="I37">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J37" t="s">
         <v>130</v>
@@ -2835,7 +2829,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P37">
-        <v>46311.700870364</v>
+        <v>46312.29483155741</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>46</v>
@@ -2861,7 +2855,7 @@
         <v>46323</v>
       </c>
       <c r="I38">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J38" t="s">
         <v>132</v>
@@ -2879,7 +2873,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P38">
-        <v>46311.70087037373</v>
+        <v>46312.2948315709</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>46</v>
@@ -2905,7 +2899,7 @@
         <v>46323</v>
       </c>
       <c r="I39">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J39" t="s">
         <v>134</v>
@@ -2926,7 +2920,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P39">
-        <v>46311.70087038344</v>
+        <v>46312.29483158379</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>46</v>
@@ -2955,7 +2949,7 @@
         <v>46323</v>
       </c>
       <c r="I40">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J40" t="s">
         <v>139</v>
@@ -2976,7 +2970,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P40">
-        <v>46311.70087035413</v>
+        <v>46312.29483154425</v>
       </c>
       <c r="Q40" t="s">
         <v>23</v>
@@ -3002,7 +2996,7 @@
         <v>46323</v>
       </c>
       <c r="I41">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J41" t="s">
         <v>142</v>
@@ -3023,7 +3017,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P41">
-        <v>46311.70087034364</v>
+        <v>46312.29483153038</v>
       </c>
       <c r="Q41" s="5" t="s">
         <v>46</v>
@@ -3049,7 +3043,7 @@
         <v>46324</v>
       </c>
       <c r="I42">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J42" t="s">
         <v>145</v>
@@ -3070,7 +3064,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P42">
-        <v>46311.70087033371</v>
+        <v>46312.29483151647</v>
       </c>
       <c r="Q42" s="5" t="s">
         <v>46</v>
@@ -3096,7 +3090,7 @@
         <v>46324</v>
       </c>
       <c r="I43">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J43" t="s">
         <v>148</v>
@@ -3117,7 +3111,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P43">
-        <v>46311.70087032368</v>
+        <v>46312.29483150326</v>
       </c>
       <c r="Q43" t="s">
         <v>23</v>
@@ -3146,7 +3140,7 @@
         <v>46325</v>
       </c>
       <c r="I44">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J44" t="s">
         <v>152</v>
@@ -3167,7 +3161,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P44">
-        <v>46311.70087031323</v>
+        <v>46312.29483148939</v>
       </c>
       <c r="Q44" t="s">
         <v>23</v>
@@ -3193,7 +3187,7 @@
         <v>46326</v>
       </c>
       <c r="I45">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J45" t="s">
         <v>155</v>
@@ -3211,7 +3205,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P45">
-        <v>46311.70087030291</v>
+        <v>46312.29483147463</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>46</v>
@@ -3240,7 +3234,7 @@
         <v>46328</v>
       </c>
       <c r="I46">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J46" t="s">
         <v>157</v>
@@ -3261,7 +3255,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P46">
-        <v>46311.7008702819</v>
+        <v>46312.29483144655</v>
       </c>
       <c r="Q46" t="s">
         <v>23</v>
@@ -3287,7 +3281,7 @@
         <v>46332</v>
       </c>
       <c r="I47">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J47" t="s">
         <v>160</v>
@@ -3305,7 +3299,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P47">
-        <v>46311.70087027091</v>
+        <v>46312.29483143263</v>
       </c>
       <c r="Q47" t="s">
         <v>23</v>
@@ -3331,7 +3325,7 @@
         <v>46333</v>
       </c>
       <c r="I48">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J48" t="s">
         <v>96</v>
@@ -3352,7 +3346,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P48">
-        <v>46311.70087025949</v>
+        <v>46312.29483141792</v>
       </c>
       <c r="Q48" t="s">
         <v>23</v>
@@ -3378,7 +3372,7 @@
         <v>46333</v>
       </c>
       <c r="I49">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J49" t="s">
         <v>164</v>
@@ -3396,7 +3390,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P49">
-        <v>46311.70087023666</v>
+        <v>46312.29483138782</v>
       </c>
       <c r="Q49" t="s">
         <v>23</v>
@@ -3424,7 +3418,7 @@
         <v>46310</v>
       </c>
       <c r="I50" s="6">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="J50" s="6" t="s">
         <v>168</v>
@@ -3445,7 +3439,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P50" s="6">
-        <v>46311.70088693928</v>
+        <v>46312.29485678871</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>23</v>
@@ -3473,7 +3467,7 @@
         <v>46309</v>
       </c>
       <c r="I51" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="J51" s="6" t="s">
         <v>171</v>
@@ -3492,7 +3486,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P51" s="6">
-        <v>46311.70088694827</v>
+        <v>46312.29485680167</v>
       </c>
       <c r="Q51" s="5" t="s">
         <v>46</v>
@@ -3520,7 +3514,7 @@
         <v>46308</v>
       </c>
       <c r="I52" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J52" s="6" t="s">
         <v>173</v>
@@ -3539,7 +3533,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P52" s="6">
-        <v>46311.70088698581</v>
+        <v>46312.29485685294</v>
       </c>
       <c r="Q52" s="5" t="s">
         <v>46</v>
@@ -3567,7 +3561,7 @@
         <v>46308</v>
       </c>
       <c r="I53" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J53" s="6" t="s">
         <v>175</v>
@@ -3586,7 +3580,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P53" s="6">
-        <v>46311.70088697635</v>
+        <v>46312.29485684038</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>46</v>
@@ -3616,7 +3610,7 @@
         <v>46307</v>
       </c>
       <c r="I54" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J54" s="6" t="s">
         <v>179</v>
@@ -3637,7 +3631,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P54" s="6">
-        <v>46311.70089512802</v>
+        <v>46312.29486540094</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>23</v>
@@ -3667,7 +3661,7 @@
         <v>46307</v>
       </c>
       <c r="I55" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J55" s="6" t="s">
         <v>182</v>
@@ -3686,7 +3680,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P55" s="6">
-        <v>46311.70089508668</v>
+        <v>46312.2948653477</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>23</v>
@@ -3714,7 +3708,7 @@
         <v>46307</v>
       </c>
       <c r="I56" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J56" s="6" t="s">
         <v>184</v>
@@ -3735,7 +3729,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P56" s="6">
-        <v>46311.70089515702</v>
+        <v>46312.29486543904</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>46</v>
@@ -3763,7 +3757,7 @@
         <v>46307</v>
       </c>
       <c r="I57" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J57" s="6" t="s">
         <v>187</v>
@@ -3782,7 +3776,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P57" s="6">
-        <v>46311.70089513763</v>
+        <v>46312.29486541387</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>23</v>
@@ -3810,7 +3804,7 @@
         <v>46307</v>
       </c>
       <c r="I58" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J58" s="6" t="s">
         <v>184</v>
@@ -3831,7 +3825,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P58" s="6">
-        <v>46311.70089514742</v>
+        <v>46312.29486542654</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>23</v>
@@ -3861,7 +3855,7 @@
         <v>46307</v>
       </c>
       <c r="I59" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J59" s="6" t="s">
         <v>85</v>
@@ -3912,7 +3906,7 @@
         <v>46306</v>
       </c>
       <c r="I60" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J60" s="6" t="s">
         <v>194</v>
@@ -3933,7 +3927,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P60" s="6">
-        <v>46311.70089517583</v>
+        <v>46312.29486546413</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>23</v>
@@ -3961,7 +3955,7 @@
         <v>46306</v>
       </c>
       <c r="I61" s="6">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="J61" s="6" t="s">
         <v>197</v>
@@ -3982,7 +3976,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P61" s="6">
-        <v>46311.70089518549</v>
+        <v>46312.29486547723</v>
       </c>
       <c r="Q61" s="6" t="s">
         <v>23</v>
@@ -4010,7 +4004,7 @@
         <v>46305</v>
       </c>
       <c r="I62" s="6">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="J62" s="6" t="s">
         <v>200</v>
@@ -4031,7 +4025,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P62" s="6">
-        <v>46311.70089521474</v>
+        <v>46312.29486551596</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>23</v>
@@ -4059,7 +4053,7 @@
         <v>46304</v>
       </c>
       <c r="I63" s="6">
-        <v>-7</v>
+        <v>-8</v>
       </c>
       <c r="J63" s="6" t="s">
         <v>204</v>
@@ -4080,7 +4074,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P63" s="6">
-        <v>46311.70089523357</v>
+        <v>46312.29486554277</v>
       </c>
       <c r="Q63" s="6" t="s">
         <v>23</v>
@@ -4110,7 +4104,7 @@
         <v>46303</v>
       </c>
       <c r="I64" s="6">
-        <v>-8</v>
+        <v>-9</v>
       </c>
       <c r="J64" s="6" t="s">
         <v>208</v>
@@ -4131,7 +4125,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P64" s="6">
-        <v>46311.7008952556</v>
+        <v>46312.29486556918</v>
       </c>
       <c r="Q64" s="6" t="s">
         <v>23</v>
@@ -4159,7 +4153,7 @@
         <v>46302</v>
       </c>
       <c r="I65" s="6">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="J65" s="6" t="s">
         <v>211</v>
@@ -4178,63 +4172,14 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P65" s="6">
-        <v>46311.70090339411</v>
+        <v>46312.29487409964</v>
       </c>
       <c r="Q65" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="66" spans="1:17">
-      <c r="A66" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="B66" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="D66" s="6"/>
-      <c r="E66" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="G66" s="6">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="H66" s="6">
-        <v>46301</v>
-      </c>
-      <c r="I66" s="6">
-        <v>-10</v>
-      </c>
-      <c r="J66" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="K66" s="6">
-        <v>2</v>
-      </c>
-      <c r="L66" s="6"/>
-      <c r="M66" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="O66" s="6">
-        <v>46300.75885649968</v>
-      </c>
-      <c r="P66" s="6">
-        <v>46311.70090342543</v>
-      </c>
-      <c r="Q66" s="6" t="s">
-        <v>23</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:Q66"/>
+  <autoFilter ref="A1:Q65"/>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1"/>
     <hyperlink ref="N2" r:id="rId2"/>
@@ -4364,8 +4309,6 @@
     <hyperlink ref="N64" r:id="rId126"/>
     <hyperlink ref="M65" r:id="rId127"/>
     <hyperlink ref="N65" r:id="rId128"/>
-    <hyperlink ref="M66" r:id="rId129"/>
-    <hyperlink ref="N66" r:id="rId130"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4464,7 +4407,7 @@
         <v>46314</v>
       </c>
       <c r="I2" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>45</v>
@@ -4482,7 +4425,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P2" s="2">
-        <v>46311.70088686351</v>
+        <v>46312.29485668633</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>46</v>
@@ -4508,7 +4451,7 @@
         <v>46315</v>
       </c>
       <c r="I3" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>50</v>
@@ -4526,7 +4469,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P3" s="2">
-        <v>46311.70088684419</v>
+        <v>46312.29485666077</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>46</v>
@@ -4552,7 +4495,7 @@
         <v>46316</v>
       </c>
       <c r="I4" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>61</v>
@@ -4573,7 +4516,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P4" s="2">
-        <v>46311.70087868374</v>
+        <v>46312.29484303323</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>46</v>
@@ -4599,7 +4542,7 @@
         <v>46317</v>
       </c>
       <c r="I5" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>68</v>
@@ -4617,7 +4560,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P5" s="2">
-        <v>46311.70087866466</v>
+        <v>46312.29484300764</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>46</v>
@@ -4643,7 +4586,7 @@
         <v>46317</v>
       </c>
       <c r="I6" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>74</v>
@@ -4661,7 +4604,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P6" s="2">
-        <v>46311.70087865533</v>
+        <v>46312.29484299479</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>46</v>
@@ -4687,7 +4630,7 @@
         <v>46318</v>
       </c>
       <c r="I7" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>85</v>
@@ -4708,41 +4651,41 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P7" s="2">
-        <v>46311.70087864589</v>
+        <v>46312.29484298224</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" t="s">
+    <row r="8" spans="1:17" s="2" customFormat="1">
+      <c r="A8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="2">
         <v>0.2</v>
       </c>
       <c r="H8" s="3">
         <v>46319</v>
       </c>
-      <c r="I8">
-        <v>8</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="I8" s="2">
+        <v>7</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="2">
         <v>2</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="2" t="s">
         <v>94</v>
       </c>
       <c r="M8" s="4" t="s">
@@ -4751,42 +4694,42 @@
       <c r="N8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="2">
         <v>46307.39549700746</v>
       </c>
-      <c r="P8">
-        <v>46311.70087858952</v>
+      <c r="P8" s="2">
+        <v>46312.29484290504</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
-      <c r="A9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" t="s">
+    <row r="9" spans="1:17" s="2" customFormat="1">
+      <c r="A9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="2">
         <v>0.2</v>
       </c>
       <c r="H9" s="3">
         <v>46319</v>
       </c>
-      <c r="I9">
-        <v>8</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="I9" s="2">
+        <v>7</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="2">
         <v>1</v>
       </c>
       <c r="M9" s="4" t="s">
@@ -4795,42 +4738,42 @@
       <c r="N9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="2">
         <v>46307.3954970362</v>
       </c>
-      <c r="P9">
-        <v>46311.70087859921</v>
+      <c r="P9" s="2">
+        <v>46312.29484291846</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:17">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
+    <row r="10" spans="1:17" s="2" customFormat="1">
+      <c r="A10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="2">
         <v>0.2</v>
       </c>
       <c r="H10" s="3">
         <v>46319</v>
       </c>
-      <c r="I10">
-        <v>8</v>
-      </c>
-      <c r="J10" t="s">
+      <c r="I10" s="2">
+        <v>7</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="2">
         <v>1</v>
       </c>
       <c r="M10" s="4" t="s">
@@ -4839,11 +4782,11 @@
       <c r="N10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="2">
         <v>46309.72495171529</v>
       </c>
-      <c r="P10">
-        <v>46311.70087857031</v>
+      <c r="P10" s="2">
+        <v>46312.29484287875</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -4869,7 +4812,7 @@
         <v>46320</v>
       </c>
       <c r="I11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J11" t="s">
         <v>111</v>
@@ -4887,7 +4830,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P11">
-        <v>46311.70087854062</v>
+        <v>46312.29484284001</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>46</v>
@@ -4913,7 +4856,7 @@
         <v>46321</v>
       </c>
       <c r="I12">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J12" t="s">
         <v>113</v>
@@ -4931,7 +4874,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P12">
-        <v>46311.70087044157</v>
+        <v>46312.29483166153</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>46</v>
@@ -4957,7 +4900,7 @@
         <v>46322</v>
       </c>
       <c r="I13">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J13" t="s">
         <v>115</v>
@@ -4978,7 +4921,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P13">
-        <v>46311.70087042241</v>
+        <v>46312.29483163588</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -5004,7 +4947,7 @@
         <v>46322</v>
       </c>
       <c r="I14">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
         <v>121</v>
@@ -5025,7 +4968,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P14">
-        <v>46311.70087040275</v>
+        <v>46312.29483160963</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>46</v>
@@ -5051,7 +4994,7 @@
         <v>46322</v>
       </c>
       <c r="I15">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J15" t="s">
         <v>127</v>
@@ -5072,7 +5015,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P15">
-        <v>46311.70087039313</v>
+        <v>46312.29483159653</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -5098,7 +5041,7 @@
         <v>46323</v>
       </c>
       <c r="I16">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J16" t="s">
         <v>130</v>
@@ -5116,7 +5059,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P16">
-        <v>46311.700870364</v>
+        <v>46312.29483155741</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>46</v>
@@ -5142,7 +5085,7 @@
         <v>46323</v>
       </c>
       <c r="I17">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J17" t="s">
         <v>132</v>
@@ -5160,7 +5103,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P17">
-        <v>46311.70087037373</v>
+        <v>46312.2948315709</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -5186,7 +5129,7 @@
         <v>46323</v>
       </c>
       <c r="I18">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J18" t="s">
         <v>134</v>
@@ -5207,7 +5150,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P18">
-        <v>46311.70087038344</v>
+        <v>46312.29483158379</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>46</v>
@@ -5233,7 +5176,7 @@
         <v>46323</v>
       </c>
       <c r="I19">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J19" t="s">
         <v>142</v>
@@ -5254,7 +5197,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P19">
-        <v>46311.70087034364</v>
+        <v>46312.29483153038</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>46</v>
@@ -5280,7 +5223,7 @@
         <v>46324</v>
       </c>
       <c r="I20">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J20" t="s">
         <v>145</v>
@@ -5301,7 +5244,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P20">
-        <v>46311.70087033371</v>
+        <v>46312.29483151647</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>46</v>
@@ -5327,7 +5270,7 @@
         <v>46326</v>
       </c>
       <c r="I21">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J21" t="s">
         <v>155</v>
@@ -5345,7 +5288,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P21">
-        <v>46311.70087030291</v>
+        <v>46312.29483147463</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>46</v>
@@ -5373,7 +5316,7 @@
         <v>46309</v>
       </c>
       <c r="I22" s="6">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="J22" s="6" t="s">
         <v>171</v>
@@ -5392,7 +5335,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P22" s="6">
-        <v>46311.70088694827</v>
+        <v>46312.29485680167</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>46</v>
@@ -5420,7 +5363,7 @@
         <v>46308</v>
       </c>
       <c r="I23" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J23" s="6" t="s">
         <v>173</v>
@@ -5439,7 +5382,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P23" s="6">
-        <v>46311.70088698581</v>
+        <v>46312.29485685294</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
@@ -5467,7 +5410,7 @@
         <v>46308</v>
       </c>
       <c r="I24" s="6">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="J24" s="6" t="s">
         <v>175</v>
@@ -5486,7 +5429,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P24" s="6">
-        <v>46311.70088697635</v>
+        <v>46312.29485684038</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>46</v>
@@ -5514,7 +5457,7 @@
         <v>46307</v>
       </c>
       <c r="I25" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J25" s="6" t="s">
         <v>184</v>
@@ -5535,7 +5478,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P25" s="6">
-        <v>46311.70089515702</v>
+        <v>46312.29486543904</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>46</v>
@@ -5565,7 +5508,7 @@
         <v>46307</v>
       </c>
       <c r="I26" s="6">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="J26" s="6" t="s">
         <v>85</v>
@@ -5614,7 +5557,7 @@
         <v>46302</v>
       </c>
       <c r="I27" s="6">
-        <v>-9</v>
+        <v>-10</v>
       </c>
       <c r="J27" s="6" t="s">
         <v>211</v>
@@ -5633,7 +5576,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P27" s="6">
-        <v>46311.70090339411</v>
+        <v>46312.29487409964</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>46</v>
@@ -5701,7 +5644,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -5711,51 +5654,51 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>222</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B2">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D2">
         <v>194</v>
@@ -5767,7 +5710,7 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -5784,13 +5727,13 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B3">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C3" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D3">
         <v>194</v>
@@ -5799,16 +5742,16 @@
         <v>3861</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -5819,98 +5762,98 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B4">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D4">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E4">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G4">
         <v>394</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B5">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C5" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D5">
         <v>193</v>
       </c>
       <c r="E5">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H5">
         <v>2</v>
       </c>
       <c r="I5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B6">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C6" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D6">
         <v>193</v>
       </c>
       <c r="E6">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F6">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G6">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -5919,53 +5862,53 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B7">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C7" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D7">
         <v>193</v>
       </c>
       <c r="E7">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G7">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B8">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D8">
         <v>193</v>
@@ -5977,7 +5920,7 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -5994,13 +5937,13 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B9">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C9" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D9">
         <v>193</v>
@@ -6009,16 +5952,16 @@
         <v>3844</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -6029,48 +5972,48 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B10">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D10">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E10">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>381</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B11">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C11" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D11">
         <v>192</v>
@@ -6079,13 +6022,13 @@
         <v>3838</v>
       </c>
       <c r="F11">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H11">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -6099,28 +6042,28 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B12">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C12" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D12">
         <v>192</v>
       </c>
       <c r="E12">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G12">
         <v>369</v>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -6129,18 +6072,18 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B13">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C13" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D13">
         <v>192</v>
@@ -6169,13 +6112,13 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B14">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C14" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D14">
         <v>192</v>
@@ -6187,7 +6130,7 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -6204,13 +6147,13 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B15">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C15" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D15">
         <v>192</v>
@@ -6239,13 +6182,13 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B16">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C16" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D16">
         <v>192</v>
@@ -6254,16 +6197,16 @@
         <v>3826</v>
       </c>
       <c r="F16">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -6274,48 +6217,48 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B17">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C17" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D17">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E17">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G17">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B18">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C18" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D18">
         <v>191</v>
@@ -6344,13 +6287,13 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B19">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C19" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D19">
         <v>191</v>
@@ -6362,7 +6305,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -6379,13 +6322,13 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B20">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C20" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D20">
         <v>191</v>
@@ -6394,16 +6337,16 @@
         <v>3820</v>
       </c>
       <c r="F20">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H20">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -6414,48 +6357,48 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B21">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C21" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D21">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E21">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F21">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G21">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H21">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B22">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C22" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D22">
         <v>8</v>
@@ -6464,13 +6407,13 @@
         <v>160</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G22">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -6479,18 +6422,18 @@
         <v>0</v>
       </c>
       <c r="K22">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B23">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C23" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D23">
         <v>8</v>
@@ -6499,21 +6442,56 @@
         <v>160</v>
       </c>
       <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>160</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11">
+      <c r="A24">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B24">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C24" t="s">
+        <v>223</v>
+      </c>
+      <c r="D24">
+        <v>8</v>
+      </c>
+      <c r="E24">
+        <v>160</v>
+      </c>
+      <c r="F24">
         <v>157</v>
       </c>
-      <c r="G23">
+      <c r="G24">
         <v>3</v>
       </c>
-      <c r="H23">
+      <c r="H24">
         <v>132</v>
       </c>
-      <c r="I23">
-        <v>1</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-17-1548Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="224">
   <si>
     <t>Priority</t>
   </si>
@@ -1208,7 +1208,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P2" s="2">
-        <v>46312.29485674985</v>
+        <v>46312.65711586995</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1252,7 +1252,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P3" s="2">
-        <v>46312.29485676255</v>
+        <v>46312.65711588449</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>23</v>
@@ -1299,7 +1299,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P4" s="2">
-        <v>46312.29485673701</v>
+        <v>46312.65711585592</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>23</v>
@@ -1346,7 +1346,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P5" s="2">
-        <v>46312.29485672439</v>
+        <v>46312.65711584162</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1393,7 +1393,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P6" s="2">
-        <v>46312.29485671136</v>
+        <v>46312.65711582667</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>23</v>
@@ -1440,7 +1440,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P7" s="2">
-        <v>46312.29485667367</v>
+        <v>46312.65711578376</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>23</v>
@@ -1484,7 +1484,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P8" s="2">
-        <v>46312.29485668633</v>
+        <v>46312.65711579815</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
@@ -1528,7 +1528,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P9" s="2">
-        <v>46312.29485669876</v>
+        <v>46312.6571158125</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>23</v>
@@ -1572,7 +1572,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P10" s="2">
-        <v>46312.29485666077</v>
+        <v>46312.65711576909</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -1619,7 +1619,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P11" s="2">
-        <v>46312.29485664792</v>
+        <v>46312.65711575456</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>23</v>
@@ -1669,7 +1669,7 @@
         <v>46311.30744692709</v>
       </c>
       <c r="P12" s="2">
-        <v>46312.29485663317</v>
+        <v>46312.65711573853</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1716,7 +1716,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P13" s="2">
-        <v>46312.29484303323</v>
+        <v>46312.65710777805</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -1763,7 +1763,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P14" s="2">
-        <v>46312.29484306075</v>
+        <v>46312.65710780673</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>23</v>
@@ -1807,7 +1807,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P15" s="2">
-        <v>46312.29484300764</v>
+        <v>46312.65710774902</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -1854,7 +1854,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P16" s="2">
-        <v>46312.29484302051</v>
+        <v>46312.65710776359</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>23</v>
@@ -1898,7 +1898,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P17" s="2">
-        <v>46312.29484299479</v>
+        <v>46312.65710773495</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -1948,7 +1948,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P18" s="2">
-        <v>46312.29484295692</v>
+        <v>46312.65710769239</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -1995,7 +1995,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P19" s="2">
-        <v>46312.29484296968</v>
+        <v>46312.65710770644</v>
       </c>
       <c r="Q19" s="2" t="s">
         <v>23</v>
@@ -2042,7 +2042,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P20" s="2">
-        <v>46312.29484294421</v>
+        <v>46312.65710767791</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>23</v>
@@ -2089,7 +2089,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P21" s="2">
-        <v>46312.29484298224</v>
+        <v>46312.65710772065</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>46</v>
@@ -2139,7 +2139,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P22" s="2">
-        <v>46312.29484293171</v>
+        <v>46312.65710766351</v>
       </c>
       <c r="Q22" s="2" t="s">
         <v>23</v>
@@ -2186,7 +2186,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P23" s="2">
-        <v>46312.29484290504</v>
+        <v>46312.65710763459</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
@@ -2230,7 +2230,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P24" s="2">
-        <v>46312.29484291846</v>
+        <v>46312.65710764895</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>46</v>
@@ -2274,7 +2274,7 @@
         <v>46309.72495168629</v>
       </c>
       <c r="P25" s="2">
-        <v>46312.29484286576</v>
+        <v>46312.65710759105</v>
       </c>
       <c r="Q25" s="2" t="s">
         <v>23</v>
@@ -2318,7 +2318,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P26" s="2">
-        <v>46312.29484287875</v>
+        <v>46312.65710760548</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>46</v>
@@ -2365,7 +2365,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P27" s="2">
-        <v>46312.29484289186</v>
+        <v>46312.65710761982</v>
       </c>
       <c r="Q27" s="2" t="s">
         <v>23</v>
@@ -2412,7 +2412,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P28">
-        <v>46312.29484281153</v>
+        <v>46312.65710753087</v>
       </c>
       <c r="Q28" t="s">
         <v>23</v>
@@ -2456,7 +2456,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P29">
-        <v>46312.29484282663</v>
+        <v>46312.65710754672</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2500,7 +2500,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P30">
-        <v>46312.29484284001</v>
+        <v>46312.65710756149</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>46</v>
@@ -2544,7 +2544,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P31">
-        <v>46312.29483166153</v>
+        <v>46312.65709963298</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>46</v>
@@ -2591,7 +2591,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P32">
-        <v>46312.29483163588</v>
+        <v>46312.65709960293</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>46</v>
@@ -2641,7 +2641,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P33">
-        <v>46312.294831623</v>
+        <v>46312.65709958807</v>
       </c>
       <c r="Q33" t="s">
         <v>23</v>
@@ -2688,7 +2688,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P34">
-        <v>46312.29483160963</v>
+        <v>46312.65709957341</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>46</v>
@@ -2738,7 +2738,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P35">
-        <v>46312.29483164889</v>
+        <v>46312.65709961824</v>
       </c>
       <c r="Q35" t="s">
         <v>23</v>
@@ -2785,7 +2785,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P36">
-        <v>46312.29483159653</v>
+        <v>46312.65709955859</v>
       </c>
       <c r="Q36" s="5" t="s">
         <v>46</v>
@@ -2829,7 +2829,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P37">
-        <v>46312.29483155741</v>
+        <v>46312.65709951358</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>46</v>
@@ -2873,7 +2873,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P38">
-        <v>46312.2948315709</v>
+        <v>46312.65709952823</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>46</v>
@@ -2920,7 +2920,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P39">
-        <v>46312.29483158379</v>
+        <v>46312.6570995425</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>46</v>
@@ -2970,7 +2970,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P40">
-        <v>46312.29483154425</v>
+        <v>46312.65709949912</v>
       </c>
       <c r="Q40" t="s">
         <v>23</v>
@@ -3017,7 +3017,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P41">
-        <v>46312.29483153038</v>
+        <v>46312.65709948403</v>
       </c>
       <c r="Q41" s="5" t="s">
         <v>46</v>
@@ -3064,7 +3064,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P42">
-        <v>46312.29483151647</v>
+        <v>46312.65709946943</v>
       </c>
       <c r="Q42" s="5" t="s">
         <v>46</v>
@@ -3111,7 +3111,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P43">
-        <v>46312.29483150326</v>
+        <v>46312.65709945454</v>
       </c>
       <c r="Q43" t="s">
         <v>23</v>
@@ -3161,7 +3161,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P44">
-        <v>46312.29483148939</v>
+        <v>46312.65709943903</v>
       </c>
       <c r="Q44" t="s">
         <v>23</v>
@@ -3205,7 +3205,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P45">
-        <v>46312.29483147463</v>
+        <v>46312.65709942421</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>46</v>
@@ -3255,7 +3255,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P46">
-        <v>46312.29483144655</v>
+        <v>46312.65709939371</v>
       </c>
       <c r="Q46" t="s">
         <v>23</v>
@@ -3299,7 +3299,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P47">
-        <v>46312.29483143263</v>
+        <v>46312.65709937788</v>
       </c>
       <c r="Q47" t="s">
         <v>23</v>
@@ -3346,7 +3346,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P48">
-        <v>46312.29483141792</v>
+        <v>46312.65709936203</v>
       </c>
       <c r="Q48" t="s">
         <v>23</v>
@@ -3390,7 +3390,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P49">
-        <v>46312.29483138782</v>
+        <v>46312.65709933193</v>
       </c>
       <c r="Q49" t="s">
         <v>23</v>
@@ -3439,7 +3439,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P50" s="6">
-        <v>46312.29485678871</v>
+        <v>46312.65711591329</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>23</v>
@@ -3486,7 +3486,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P51" s="6">
-        <v>46312.29485680167</v>
+        <v>46312.65711592732</v>
       </c>
       <c r="Q51" s="5" t="s">
         <v>46</v>
@@ -3533,7 +3533,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P52" s="6">
-        <v>46312.29485685294</v>
+        <v>46312.65711598445</v>
       </c>
       <c r="Q52" s="5" t="s">
         <v>46</v>
@@ -3580,7 +3580,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P53" s="6">
-        <v>46312.29485684038</v>
+        <v>46312.65711597015</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>46</v>
@@ -3631,7 +3631,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P54" s="6">
-        <v>46312.29486540094</v>
+        <v>46312.65712399615</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>23</v>
@@ -3680,7 +3680,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P55" s="6">
-        <v>46312.2948653477</v>
+        <v>46312.65712393675</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>23</v>
@@ -3729,7 +3729,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P56" s="6">
-        <v>46312.29486543904</v>
+        <v>46312.65712403938</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>46</v>
@@ -3776,7 +3776,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P57" s="6">
-        <v>46312.29486541387</v>
+        <v>46312.6571240104</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>23</v>
@@ -3825,7 +3825,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P58" s="6">
-        <v>46312.29486542654</v>
+        <v>46312.65712402533</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>23</v>
@@ -3927,7 +3927,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P60" s="6">
-        <v>46312.29486546413</v>
+        <v>46312.65712406745</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>23</v>
@@ -3976,7 +3976,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P61" s="6">
-        <v>46312.29486547723</v>
+        <v>46312.65712408235</v>
       </c>
       <c r="Q61" s="6" t="s">
         <v>23</v>
@@ -4025,7 +4025,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P62" s="6">
-        <v>46312.29486551596</v>
+        <v>46312.65712412516</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>23</v>
@@ -4074,7 +4074,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P63" s="6">
-        <v>46312.29486554277</v>
+        <v>46312.6571241546</v>
       </c>
       <c r="Q63" s="6" t="s">
         <v>23</v>
@@ -4125,7 +4125,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P64" s="6">
-        <v>46312.29486556918</v>
+        <v>46312.65712418339</v>
       </c>
       <c r="Q64" s="6" t="s">
         <v>23</v>
@@ -4172,7 +4172,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P65" s="6">
-        <v>46312.29487409964</v>
+        <v>46312.65713212876</v>
       </c>
       <c r="Q65" s="5" t="s">
         <v>46</v>
@@ -4425,7 +4425,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P2" s="2">
-        <v>46312.29485668633</v>
+        <v>46312.65711579815</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>46</v>
@@ -4469,7 +4469,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P3" s="2">
-        <v>46312.29485666077</v>
+        <v>46312.65711576909</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>46</v>
@@ -4516,7 +4516,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P4" s="2">
-        <v>46312.29484303323</v>
+        <v>46312.65710777805</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>46</v>
@@ -4560,7 +4560,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P5" s="2">
-        <v>46312.29484300764</v>
+        <v>46312.65710774902</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>46</v>
@@ -4604,7 +4604,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P6" s="2">
-        <v>46312.29484299479</v>
+        <v>46312.65710773495</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>46</v>
@@ -4651,7 +4651,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P7" s="2">
-        <v>46312.29484298224</v>
+        <v>46312.65710772065</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>46</v>
@@ -4698,7 +4698,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P8" s="2">
-        <v>46312.29484290504</v>
+        <v>46312.65710763459</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>46</v>
@@ -4742,7 +4742,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P9" s="2">
-        <v>46312.29484291846</v>
+        <v>46312.65710764895</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>46</v>
@@ -4786,7 +4786,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P10" s="2">
-        <v>46312.29484287875</v>
+        <v>46312.65710760548</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>46</v>
@@ -4830,7 +4830,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P11">
-        <v>46312.29484284001</v>
+        <v>46312.65710756149</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>46</v>
@@ -4874,7 +4874,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P12">
-        <v>46312.29483166153</v>
+        <v>46312.65709963298</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>46</v>
@@ -4921,7 +4921,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P13">
-        <v>46312.29483163588</v>
+        <v>46312.65709960293</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>46</v>
@@ -4968,7 +4968,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P14">
-        <v>46312.29483160963</v>
+        <v>46312.65709957341</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>46</v>
@@ -5015,7 +5015,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P15">
-        <v>46312.29483159653</v>
+        <v>46312.65709955859</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>46</v>
@@ -5059,7 +5059,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P16">
-        <v>46312.29483155741</v>
+        <v>46312.65709951358</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>46</v>
@@ -5103,7 +5103,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P17">
-        <v>46312.2948315709</v>
+        <v>46312.65709952823</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>46</v>
@@ -5150,7 +5150,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P18">
-        <v>46312.29483158379</v>
+        <v>46312.6570995425</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>46</v>
@@ -5197,7 +5197,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P19">
-        <v>46312.29483153038</v>
+        <v>46312.65709948403</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>46</v>
@@ -5244,7 +5244,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P20">
-        <v>46312.29483151647</v>
+        <v>46312.65709946943</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>46</v>
@@ -5288,7 +5288,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P21">
-        <v>46312.29483147463</v>
+        <v>46312.65709942421</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>46</v>
@@ -5335,7 +5335,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P22" s="6">
-        <v>46312.29485680167</v>
+        <v>46312.65711592732</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>46</v>
@@ -5382,7 +5382,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P23" s="6">
-        <v>46312.29485685294</v>
+        <v>46312.65711598445</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>46</v>
@@ -5429,7 +5429,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P24" s="6">
-        <v>46312.29485684038</v>
+        <v>46312.65711597015</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>46</v>
@@ -5478,7 +5478,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P25" s="6">
-        <v>46312.29486543904</v>
+        <v>46312.65712403938</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>46</v>
@@ -5576,7 +5576,7 @@
         <v>46300.75885647022</v>
       </c>
       <c r="P27" s="6">
-        <v>46312.29487409964</v>
+        <v>46312.65713212876</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>46</v>
@@ -5644,7 +5644,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -5692,10 +5692,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46312.29481460934</v>
+        <v>46312.65708521284</v>
       </c>
       <c r="B2">
-        <v>46312.29886374016</v>
+        <v>46312.65865222656</v>
       </c>
       <c r="C2" t="s">
         <v>223</v>
@@ -5727,10 +5727,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B3">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C3" t="s">
         <v>223</v>
@@ -5745,7 +5745,7 @@
         <v>0</v>
       </c>
       <c r="G3">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -5762,10 +5762,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B4">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C4" t="s">
         <v>223</v>
@@ -5777,16 +5777,16 @@
         <v>3861</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G4">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -5797,45 +5797,45 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B5">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C5" t="s">
         <v>223</v>
       </c>
       <c r="D5">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E5">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
         <v>394</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B6">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C6" t="s">
         <v>223</v>
@@ -5844,33 +5844,33 @@
         <v>193</v>
       </c>
       <c r="E6">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H6">
         <v>2</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B7">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C7" t="s">
         <v>223</v>
@@ -5879,16 +5879,16 @@
         <v>193</v>
       </c>
       <c r="E7">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F7">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G7">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H7">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -5897,15 +5897,15 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B8">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C8" t="s">
         <v>223</v>
@@ -5914,33 +5914,33 @@
         <v>193</v>
       </c>
       <c r="E8">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G8">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B9">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C9" t="s">
         <v>223</v>
@@ -5955,7 +5955,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -5972,10 +5972,10 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B10">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C10" t="s">
         <v>223</v>
@@ -5987,16 +5987,16 @@
         <v>3844</v>
       </c>
       <c r="F10">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -6007,45 +6007,45 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B11">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C11" t="s">
         <v>223</v>
       </c>
       <c r="D11">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E11">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G11">
         <v>381</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B12">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C12" t="s">
         <v>223</v>
@@ -6057,13 +6057,13 @@
         <v>3838</v>
       </c>
       <c r="F12">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H12">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I12">
         <v>0</v>
@@ -6077,10 +6077,10 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B13">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C13" t="s">
         <v>223</v>
@@ -6089,16 +6089,16 @@
         <v>192</v>
       </c>
       <c r="E13">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G13">
         <v>369</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -6107,15 +6107,15 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B14">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C14" t="s">
         <v>223</v>
@@ -6147,10 +6147,10 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B15">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C15" t="s">
         <v>223</v>
@@ -6165,7 +6165,7 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -6182,10 +6182,10 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B16">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C16" t="s">
         <v>223</v>
@@ -6217,10 +6217,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B17">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C17" t="s">
         <v>223</v>
@@ -6232,16 +6232,16 @@
         <v>3826</v>
       </c>
       <c r="F17">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -6252,45 +6252,45 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B18">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C18" t="s">
         <v>223</v>
       </c>
       <c r="D18">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E18">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G18">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B19">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C19" t="s">
         <v>223</v>
@@ -6322,10 +6322,10 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B20">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C20" t="s">
         <v>223</v>
@@ -6340,7 +6340,7 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -6357,10 +6357,10 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B21">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C21" t="s">
         <v>223</v>
@@ -6372,16 +6372,16 @@
         <v>3820</v>
       </c>
       <c r="F21">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G21">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H21">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J21">
         <v>0</v>
@@ -6392,45 +6392,45 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B22">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C22" t="s">
         <v>223</v>
       </c>
       <c r="D22">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E22">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F22">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G22">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H22">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B23">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C23" t="s">
         <v>223</v>
@@ -6442,13 +6442,13 @@
         <v>160</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G23">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -6457,15 +6457,15 @@
         <v>0</v>
       </c>
       <c r="K23">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B24">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C24" t="s">
         <v>223</v>
@@ -6477,21 +6477,56 @@
         <v>160</v>
       </c>
       <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>160</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B25">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C25" t="s">
+        <v>223</v>
+      </c>
+      <c r="D25">
+        <v>8</v>
+      </c>
+      <c r="E25">
+        <v>160</v>
+      </c>
+      <c r="F25">
         <v>157</v>
       </c>
-      <c r="G24">
+      <c r="G25">
         <v>3</v>
       </c>
-      <c r="H24">
+      <c r="H25">
         <v>132</v>
       </c>
-      <c r="I24">
-        <v>1</v>
-      </c>
-      <c r="J24">
-        <v>0</v>
-      </c>
-      <c r="K24">
+      <c r="I25">
+        <v>1</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-18-1604Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="222">
   <si>
     <t>Priority</t>
   </si>
@@ -1202,7 +1202,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P2" s="2">
-        <v>46313.30532584916</v>
+        <v>46313.66772332653</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1249,7 +1249,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P3" s="2">
-        <v>46313.30532580941</v>
+        <v>46313.66772328764</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>23</v>
@@ -1293,7 +1293,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P4" s="2">
-        <v>46313.30532582265</v>
+        <v>46313.66772330055</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>31</v>
@@ -1337,7 +1337,7 @@
         <v>46300.7588477715</v>
       </c>
       <c r="P5" s="2">
-        <v>46313.30532583613</v>
+        <v>46313.66772331384</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1381,7 +1381,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P6" s="2">
-        <v>46313.30532579589</v>
+        <v>46313.66772327427</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>31</v>
@@ -1428,7 +1428,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P7" s="2">
-        <v>46313.30532578268</v>
+        <v>46313.66772326059</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>23</v>
@@ -1478,7 +1478,7 @@
         <v>46311.30744692709</v>
       </c>
       <c r="P8" s="2">
-        <v>46313.30532576742</v>
+        <v>46313.6677232455</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>23</v>
@@ -1525,7 +1525,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P9" s="2">
-        <v>46313.30531728507</v>
+        <v>46313.6677142169</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>31</v>
@@ -1572,7 +1572,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P10" s="2">
-        <v>46313.30531731113</v>
+        <v>46313.66771424172</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>23</v>
@@ -1616,7 +1616,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P11" s="2">
-        <v>46313.30531725841</v>
+        <v>46313.66771419167</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>31</v>
@@ -1663,7 +1663,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P12" s="2">
-        <v>46313.30531727153</v>
+        <v>46313.66771420432</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1707,7 +1707,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P13" s="2">
-        <v>46313.30531724413</v>
+        <v>46313.66771417948</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>31</v>
@@ -1757,7 +1757,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P14" s="2">
-        <v>46313.30531720298</v>
+        <v>46313.66771414227</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>23</v>
@@ -1804,7 +1804,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P15" s="2">
-        <v>46313.3053172166</v>
+        <v>46313.66771415442</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>23</v>
@@ -1851,7 +1851,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P16" s="2">
-        <v>46313.30531718949</v>
+        <v>46313.66771412977</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>23</v>
@@ -1898,7 +1898,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P17" s="2">
-        <v>46313.30531722958</v>
+        <v>46313.66771416669</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>31</v>
@@ -1948,7 +1948,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P18" s="2">
-        <v>46313.30531717594</v>
+        <v>46313.66771411694</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -1995,7 +1995,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P19" s="2">
-        <v>46313.30531714948</v>
+        <v>46313.66771409143</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>31</v>
@@ -2039,7 +2039,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P20" s="2">
-        <v>46313.30531716249</v>
+        <v>46313.66771410416</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>31</v>
@@ -2083,7 +2083,7 @@
         <v>46309.72495168629</v>
       </c>
       <c r="P21" s="2">
-        <v>46313.30531711045</v>
+        <v>46313.66771405283</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>23</v>
@@ -2127,7 +2127,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P22" s="2">
-        <v>46313.30531712321</v>
+        <v>46313.66771406602</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>31</v>
@@ -2174,7 +2174,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P23" s="2">
-        <v>46313.30531713596</v>
+        <v>46313.66771407861</v>
       </c>
       <c r="Q23" s="2" t="s">
         <v>23</v>
@@ -2221,7 +2221,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P24" s="2">
-        <v>46313.30531705452</v>
+        <v>46313.66771399752</v>
       </c>
       <c r="Q24" s="2" t="s">
         <v>23</v>
@@ -2265,7 +2265,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P25" s="2">
-        <v>46313.30531706983</v>
+        <v>46313.66771401245</v>
       </c>
       <c r="Q25" s="2" t="s">
         <v>23</v>
@@ -2309,7 +2309,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P26" s="2">
-        <v>46313.3053170835</v>
+        <v>46313.66771402624</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>31</v>
@@ -2353,7 +2353,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P27">
-        <v>46313.30530860629</v>
+        <v>46313.66770577192</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>31</v>
@@ -2400,7 +2400,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P28">
-        <v>46313.30530857794</v>
+        <v>46313.66770574598</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>31</v>
@@ -2450,7 +2450,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P29">
-        <v>46313.3053085645</v>
+        <v>46313.66770573297</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2497,7 +2497,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P30">
-        <v>46313.30530854941</v>
+        <v>46313.66770571972</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>31</v>
@@ -2547,7 +2547,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P31">
-        <v>46313.30530859238</v>
+        <v>46313.66770575889</v>
       </c>
       <c r="Q31" t="s">
         <v>23</v>
@@ -2594,7 +2594,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P32">
-        <v>46313.30530853521</v>
+        <v>46313.66770570714</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>31</v>
@@ -2638,7 +2638,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P33">
-        <v>46313.30530849531</v>
+        <v>46313.6677056671</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>31</v>
@@ -2682,7 +2682,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P34">
-        <v>46313.30530850866</v>
+        <v>46313.66770568074</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>31</v>
@@ -2729,7 +2729,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P35">
-        <v>46313.30530852199</v>
+        <v>46313.66770569394</v>
       </c>
       <c r="Q35" s="5" t="s">
         <v>31</v>
@@ -2779,7 +2779,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P36">
-        <v>46313.30530848172</v>
+        <v>46313.66770565418</v>
       </c>
       <c r="Q36" t="s">
         <v>23</v>
@@ -2826,7 +2826,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P37">
-        <v>46313.3053084683</v>
+        <v>46313.66770564076</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>31</v>
@@ -2873,7 +2873,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P38">
-        <v>46313.3053084546</v>
+        <v>46313.66770562722</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>31</v>
@@ -2920,7 +2920,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P39">
-        <v>46313.30530844122</v>
+        <v>46313.66770561394</v>
       </c>
       <c r="Q39" t="s">
         <v>23</v>
@@ -2970,7 +2970,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P40">
-        <v>46313.30530842762</v>
+        <v>46313.66770560007</v>
       </c>
       <c r="Q40" t="s">
         <v>23</v>
@@ -3014,7 +3014,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P41">
-        <v>46313.30530841411</v>
+        <v>46313.66770558676</v>
       </c>
       <c r="Q41" s="5" t="s">
         <v>31</v>
@@ -3064,7 +3064,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P42">
-        <v>46313.30530838588</v>
+        <v>46313.66770555852</v>
       </c>
       <c r="Q42" t="s">
         <v>23</v>
@@ -3108,7 +3108,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P43">
-        <v>46313.30530837171</v>
+        <v>46313.66770554411</v>
       </c>
       <c r="Q43" t="s">
         <v>23</v>
@@ -3155,7 +3155,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P44">
-        <v>46313.3053083565</v>
+        <v>46313.66770552914</v>
       </c>
       <c r="Q44" t="s">
         <v>23</v>
@@ -3199,7 +3199,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P45">
-        <v>46313.30530832517</v>
+        <v>46313.66770549942</v>
       </c>
       <c r="Q45" t="s">
         <v>23</v>
@@ -3248,7 +3248,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P46" s="6">
-        <v>46313.30532588915</v>
+        <v>46313.66772336456</v>
       </c>
       <c r="Q46" s="6" t="s">
         <v>23</v>
@@ -3295,7 +3295,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P47" s="6">
-        <v>46313.30532590194</v>
+        <v>46313.6677233767</v>
       </c>
       <c r="Q47" s="6" t="s">
         <v>23</v>
@@ -3344,7 +3344,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P48" s="6">
-        <v>46313.30532587588</v>
+        <v>46313.66772335224</v>
       </c>
       <c r="Q48" s="6" t="s">
         <v>23</v>
@@ -3393,7 +3393,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P49" s="6">
-        <v>46313.30532586262</v>
+        <v>46313.66772333956</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>23</v>
@@ -3442,7 +3442,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P50" s="6">
-        <v>46313.30532592876</v>
+        <v>46313.66772340168</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>23</v>
@@ -3489,7 +3489,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P51" s="6">
-        <v>46313.30532594294</v>
+        <v>46313.6677234138</v>
       </c>
       <c r="Q51" s="5" t="s">
         <v>31</v>
@@ -3536,7 +3536,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P52" s="6">
-        <v>46313.30532599742</v>
+        <v>46313.66772346423</v>
       </c>
       <c r="Q52" s="5" t="s">
         <v>31</v>
@@ -3583,7 +3583,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P53" s="6">
-        <v>46313.30532598343</v>
+        <v>46313.66772345122</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>31</v>
@@ -3634,7 +3634,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P54" s="6">
-        <v>46313.30533904954</v>
+        <v>46313.66773176777</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>23</v>
@@ -3683,7 +3683,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P55" s="6">
-        <v>46313.30533899343</v>
+        <v>46313.66773171356</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>23</v>
@@ -3732,7 +3732,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P56" s="6">
-        <v>46313.3053390893</v>
+        <v>46313.66773180514</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>31</v>
@@ -3779,7 +3779,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P57" s="6">
-        <v>46313.30533906279</v>
+        <v>46313.66773178015</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>23</v>
@@ -3828,7 +3828,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P58" s="6">
-        <v>46313.30533907594</v>
+        <v>46313.66773179277</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>23</v>
@@ -3930,7 +3930,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P60" s="6">
-        <v>46313.30533911665</v>
+        <v>46313.66773183009</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>23</v>
@@ -3979,7 +3979,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P61" s="6">
-        <v>46313.30533913011</v>
+        <v>46313.66773184277</v>
       </c>
       <c r="Q61" s="6" t="s">
         <v>23</v>
@@ -4028,7 +4028,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P62" s="6">
-        <v>46313.30533917051</v>
+        <v>46313.66773188084</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>23</v>
@@ -4077,7 +4077,7 @@
         <v>46300.7588563655</v>
       </c>
       <c r="P63" s="6">
-        <v>46313.30533919778</v>
+        <v>46313.66773190629</v>
       </c>
       <c r="Q63" s="6" t="s">
         <v>23</v>
@@ -4128,7 +4128,7 @@
         <v>46300.7588564207</v>
       </c>
       <c r="P64" s="6">
-        <v>46313.30533922432</v>
+        <v>46313.66773193169</v>
       </c>
       <c r="Q64" s="6" t="s">
         <v>23</v>
@@ -4379,7 +4379,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P2" s="2">
-        <v>46313.30532582265</v>
+        <v>46313.66772330055</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>31</v>
@@ -4423,7 +4423,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P3" s="2">
-        <v>46313.30532579589</v>
+        <v>46313.66772327427</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>31</v>
@@ -4470,7 +4470,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P4" s="2">
-        <v>46313.30531728507</v>
+        <v>46313.6677142169</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>31</v>
@@ -4514,7 +4514,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P5" s="2">
-        <v>46313.30531725841</v>
+        <v>46313.66771419167</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>31</v>
@@ -4558,7 +4558,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P6" s="2">
-        <v>46313.30531724413</v>
+        <v>46313.66771417948</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>31</v>
@@ -4605,7 +4605,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P7" s="2">
-        <v>46313.30531722958</v>
+        <v>46313.66771416669</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>31</v>
@@ -4652,7 +4652,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P8" s="2">
-        <v>46313.30531714948</v>
+        <v>46313.66771409143</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>31</v>
@@ -4696,7 +4696,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P9" s="2">
-        <v>46313.30531716249</v>
+        <v>46313.66771410416</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>31</v>
@@ -4740,7 +4740,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P10" s="2">
-        <v>46313.30531712321</v>
+        <v>46313.66771406602</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>31</v>
@@ -4784,7 +4784,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P11" s="2">
-        <v>46313.3053170835</v>
+        <v>46313.66771402624</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>31</v>
@@ -4828,7 +4828,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P12">
-        <v>46313.30530860629</v>
+        <v>46313.66770577192</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>31</v>
@@ -4875,7 +4875,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P13">
-        <v>46313.30530857794</v>
+        <v>46313.66770574598</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>31</v>
@@ -4922,7 +4922,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P14">
-        <v>46313.30530854941</v>
+        <v>46313.66770571972</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>31</v>
@@ -4969,7 +4969,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P15">
-        <v>46313.30530853521</v>
+        <v>46313.66770570714</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>31</v>
@@ -5013,7 +5013,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P16">
-        <v>46313.30530849531</v>
+        <v>46313.6677056671</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>31</v>
@@ -5057,7 +5057,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P17">
-        <v>46313.30530850866</v>
+        <v>46313.66770568074</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>31</v>
@@ -5104,7 +5104,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P18">
-        <v>46313.30530852199</v>
+        <v>46313.66770569394</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>31</v>
@@ -5151,7 +5151,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P19">
-        <v>46313.3053084683</v>
+        <v>46313.66770564076</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>31</v>
@@ -5198,7 +5198,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P20">
-        <v>46313.3053084546</v>
+        <v>46313.66770562722</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>31</v>
@@ -5242,7 +5242,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P21">
-        <v>46313.30530841411</v>
+        <v>46313.66770558676</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>31</v>
@@ -5289,7 +5289,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P22" s="6">
-        <v>46313.30532594294</v>
+        <v>46313.6677234138</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>31</v>
@@ -5336,7 +5336,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P23" s="6">
-        <v>46313.30532599742</v>
+        <v>46313.66772346423</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>31</v>
@@ -5383,7 +5383,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P24" s="6">
-        <v>46313.30532598343</v>
+        <v>46313.66772345122</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>31</v>
@@ -5432,7 +5432,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P25" s="6">
-        <v>46313.3053390893</v>
+        <v>46313.66773180514</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>31</v>
@@ -5549,7 +5549,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -5597,10 +5597,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46313.30528009156</v>
+        <v>46313.66768650556</v>
       </c>
       <c r="B2">
-        <v>46313.3091804056</v>
+        <v>46313.66945401487</v>
       </c>
       <c r="C2" t="s">
         <v>221</v>
@@ -5632,10 +5632,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46312.65708521284</v>
+        <v>46313.30528009156</v>
       </c>
       <c r="B3">
-        <v>46312.65865222656</v>
+        <v>46313.3091804056</v>
       </c>
       <c r="C3" t="s">
         <v>221</v>
@@ -5667,10 +5667,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46312.29481460934</v>
+        <v>46312.65708521284</v>
       </c>
       <c r="B4">
-        <v>46312.29886374016</v>
+        <v>46312.65865222656</v>
       </c>
       <c r="C4" t="s">
         <v>221</v>
@@ -5702,10 +5702,10 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B5">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C5" t="s">
         <v>221</v>
@@ -5720,7 +5720,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -5737,10 +5737,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B6">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C6" t="s">
         <v>221</v>
@@ -5752,16 +5752,16 @@
         <v>3861</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -5772,45 +5772,45 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B7">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C7" t="s">
         <v>221</v>
       </c>
       <c r="D7">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E7">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7">
         <v>394</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7">
         <v>0</v>
       </c>
       <c r="K7">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B8">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C8" t="s">
         <v>221</v>
@@ -5819,33 +5819,33 @@
         <v>193</v>
       </c>
       <c r="E8">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H8">
         <v>2</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8">
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B9">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C9" t="s">
         <v>221</v>
@@ -5854,16 +5854,16 @@
         <v>193</v>
       </c>
       <c r="E9">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F9">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G9">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H9">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I9">
         <v>1</v>
@@ -5872,15 +5872,15 @@
         <v>0</v>
       </c>
       <c r="K9">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B10">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C10" t="s">
         <v>221</v>
@@ -5889,33 +5889,33 @@
         <v>193</v>
       </c>
       <c r="E10">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G10">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10">
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B11">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C11" t="s">
         <v>221</v>
@@ -5930,7 +5930,7 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -5947,10 +5947,10 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B12">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C12" t="s">
         <v>221</v>
@@ -5962,16 +5962,16 @@
         <v>3844</v>
       </c>
       <c r="F12">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H12">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -5982,45 +5982,45 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B13">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C13" t="s">
         <v>221</v>
       </c>
       <c r="D13">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E13">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G13">
         <v>381</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B14">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C14" t="s">
         <v>221</v>
@@ -6032,13 +6032,13 @@
         <v>3838</v>
       </c>
       <c r="F14">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H14">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -6052,10 +6052,10 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B15">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C15" t="s">
         <v>221</v>
@@ -6064,16 +6064,16 @@
         <v>192</v>
       </c>
       <c r="E15">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G15">
         <v>369</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -6082,15 +6082,15 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B16">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C16" t="s">
         <v>221</v>
@@ -6122,10 +6122,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B17">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C17" t="s">
         <v>221</v>
@@ -6140,7 +6140,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -6157,10 +6157,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B18">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C18" t="s">
         <v>221</v>
@@ -6192,10 +6192,10 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B19">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C19" t="s">
         <v>221</v>
@@ -6207,16 +6207,16 @@
         <v>3826</v>
       </c>
       <c r="F19">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G19">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J19">
         <v>0</v>
@@ -6227,45 +6227,45 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B20">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C20" t="s">
         <v>221</v>
       </c>
       <c r="D20">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E20">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G20">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B21">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C21" t="s">
         <v>221</v>
@@ -6297,10 +6297,10 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B22">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C22" t="s">
         <v>221</v>
@@ -6315,7 +6315,7 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -6332,10 +6332,10 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B23">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C23" t="s">
         <v>221</v>
@@ -6347,16 +6347,16 @@
         <v>3820</v>
       </c>
       <c r="F23">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H23">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -6367,45 +6367,45 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B24">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C24" t="s">
         <v>221</v>
       </c>
       <c r="D24">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E24">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F24">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G24">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H24">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B25">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C25" t="s">
         <v>221</v>
@@ -6417,13 +6417,13 @@
         <v>160</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G25">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -6432,15 +6432,15 @@
         <v>0</v>
       </c>
       <c r="K25">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B26">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C26" t="s">
         <v>221</v>
@@ -6452,21 +6452,56 @@
         <v>160</v>
       </c>
       <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>160</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B27">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C27" t="s">
+        <v>221</v>
+      </c>
+      <c r="D27">
+        <v>8</v>
+      </c>
+      <c r="E27">
+        <v>160</v>
+      </c>
+      <c r="F27">
         <v>157</v>
       </c>
-      <c r="G26">
+      <c r="G27">
         <v>3</v>
       </c>
-      <c r="H26">
+      <c r="H27">
         <v>132</v>
       </c>
-      <c r="I26">
-        <v>1</v>
-      </c>
-      <c r="J26">
-        <v>0</v>
-      </c>
-      <c r="K26">
+      <c r="I27">
+        <v>1</v>
+      </c>
+      <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-20-1725Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1048" uniqueCount="242">
   <si>
     <t>Priority</t>
   </si>
@@ -1259,7 +1259,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P2" s="2">
-        <v>46315.32478204358</v>
+        <v>46315.72473460915</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>22</v>
@@ -1306,7 +1306,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P3" s="2">
-        <v>46315.32478203406</v>
+        <v>46315.72473460237</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>27</v>
@@ -1356,7 +1356,7 @@
         <v>46311.30744692709</v>
       </c>
       <c r="P4" s="2">
-        <v>46315.3247820244</v>
+        <v>46315.72473459573</v>
       </c>
       <c r="Q4" s="2" t="s">
         <v>27</v>
@@ -1403,7 +1403,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P5" s="2">
-        <v>46315.32478205338</v>
+        <v>46315.7247346163</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>22</v>
@@ -1450,7 +1450,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P6" s="2">
-        <v>46315.32478199558</v>
+        <v>46315.72473457522</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>22</v>
@@ -1497,7 +1497,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P7" s="2">
-        <v>46315.32478201466</v>
+        <v>46315.72473458862</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>27</v>
@@ -1541,7 +1541,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P8" s="2">
-        <v>46315.32478197602</v>
+        <v>46315.72473456129</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>22</v>
@@ -1588,7 +1588,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P9" s="2">
-        <v>46315.32478198586</v>
+        <v>46315.7247345682</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>27</v>
@@ -1632,7 +1632,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P10" s="2">
-        <v>46315.32478196619</v>
+        <v>46315.72473455409</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>22</v>
@@ -1682,7 +1682,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P11" s="2">
-        <v>46315.32478194736</v>
+        <v>46315.72473454012</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>27</v>
@@ -1729,7 +1729,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P12" s="2">
-        <v>46315.32478195665</v>
+        <v>46315.72473454728</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>27</v>
@@ -1776,7 +1776,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P13" s="2">
-        <v>46315.32478192714</v>
+        <v>46315.7247345249</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>27</v>
@@ -1823,7 +1823,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P14" s="2">
-        <v>46315.32478193731</v>
+        <v>46315.7247345326</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>22</v>
@@ -1873,7 +1873,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P15" s="2">
-        <v>46315.3247819168</v>
+        <v>46315.72473451625</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>27</v>
@@ -1920,7 +1920,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P16" s="2">
-        <v>46315.32478189487</v>
+        <v>46315.72473449912</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>22</v>
@@ -1964,7 +1964,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P17" s="2">
-        <v>46315.32478190657</v>
+        <v>46315.72473450827</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>22</v>
@@ -2099,7 +2099,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P20" s="2">
-        <v>46315.32477360639</v>
+        <v>46315.72472657061</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>27</v>
@@ -2146,7 +2146,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P21" s="2">
-        <v>46315.32477355783</v>
+        <v>46315.72472653515</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>27</v>
@@ -2190,7 +2190,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P22" s="2">
-        <v>46315.32477356735</v>
+        <v>46315.72472654199</v>
       </c>
       <c r="Q22" s="2" t="s">
         <v>27</v>
@@ -2234,7 +2234,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P23" s="2">
-        <v>46315.32477357671</v>
+        <v>46315.72472654899</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>22</v>
@@ -2281,7 +2281,7 @@
         <v>46314.33169674601</v>
       </c>
       <c r="P24" s="2">
-        <v>46315.32477359596</v>
+        <v>46315.72472656357</v>
       </c>
       <c r="Q24" s="2" t="s">
         <v>27</v>
@@ -2325,7 +2325,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P25" s="2">
-        <v>46315.32477354836</v>
+        <v>46315.72472652839</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>22</v>
@@ -2372,7 +2372,7 @@
         <v>46314.78238309515</v>
       </c>
       <c r="P26" s="2">
-        <v>46315.32477353862</v>
+        <v>46315.72472652127</v>
       </c>
       <c r="Q26" s="2" t="s">
         <v>27</v>
@@ -2419,7 +2419,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P27" s="2">
-        <v>46315.32477351849</v>
+        <v>46315.7247265066</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>22</v>
@@ -2469,7 +2469,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P28" s="2">
-        <v>46315.32477350852</v>
+        <v>46315.72472649911</v>
       </c>
       <c r="Q28" s="2" t="s">
         <v>27</v>
@@ -2516,7 +2516,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P29" s="2">
-        <v>46315.32477349844</v>
+        <v>46315.72472649151</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>22</v>
@@ -2566,7 +2566,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P30" s="2">
-        <v>46315.32477352854</v>
+        <v>46315.72472651398</v>
       </c>
       <c r="Q30" s="2" t="s">
         <v>27</v>
@@ -2613,7 +2613,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P31" s="2">
-        <v>46315.32477348828</v>
+        <v>46315.72472648304</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>22</v>
@@ -2657,7 +2657,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P32">
-        <v>46315.32477345787</v>
+        <v>46315.72472645972</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>22</v>
@@ -2701,7 +2701,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P33">
-        <v>46315.32477346843</v>
+        <v>46315.7247264679</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>22</v>
@@ -2748,7 +2748,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P34">
-        <v>46315.32477347844</v>
+        <v>46315.72472647548</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>22</v>
@@ -2798,7 +2798,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P35">
-        <v>46315.32477344586</v>
+        <v>46315.72472645014</v>
       </c>
       <c r="Q35" t="s">
         <v>27</v>
@@ -2892,7 +2892,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P37">
-        <v>46315.32476352833</v>
+        <v>46315.72471826433</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>22</v>
@@ -2939,7 +2939,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P38">
-        <v>46315.32476351815</v>
+        <v>46315.72471825714</v>
       </c>
       <c r="Q38" t="s">
         <v>27</v>
@@ -2989,7 +2989,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P39">
-        <v>46315.32476350772</v>
+        <v>46315.72471824988</v>
       </c>
       <c r="Q39" t="s">
         <v>27</v>
@@ -3033,7 +3033,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P40">
-        <v>46315.32476346933</v>
+        <v>46315.72471822131</v>
       </c>
       <c r="Q40" s="5" t="s">
         <v>22</v>
@@ -3077,7 +3077,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P41">
-        <v>46315.32476349834</v>
+        <v>46315.72471824281</v>
       </c>
       <c r="Q41" s="5" t="s">
         <v>22</v>
@@ -3121,7 +3121,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P42">
-        <v>46315.32476348878</v>
+        <v>46315.7247182357</v>
       </c>
       <c r="Q42" s="5" t="s">
         <v>22</v>
@@ -3165,7 +3165,7 @@
         <v>46314.33168865994</v>
       </c>
       <c r="P43">
-        <v>46315.32476345929</v>
+        <v>46315.72471821371</v>
       </c>
       <c r="Q43" t="s">
         <v>27</v>
@@ -3215,7 +3215,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P44">
-        <v>46315.32476344939</v>
+        <v>46315.72471820593</v>
       </c>
       <c r="Q44" t="s">
         <v>27</v>
@@ -3259,7 +3259,7 @@
         <v>46314.78237020577</v>
       </c>
       <c r="P45">
-        <v>46315.3247634396</v>
+        <v>46315.72471819708</v>
       </c>
       <c r="Q45" t="s">
         <v>27</v>
@@ -3303,7 +3303,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P46">
-        <v>46315.32476342953</v>
+        <v>46315.72471818957</v>
       </c>
       <c r="Q46" s="5" t="s">
         <v>22</v>
@@ -3347,7 +3347,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P47">
-        <v>46315.32476341919</v>
+        <v>46315.72471818211</v>
       </c>
       <c r="Q47" s="5" t="s">
         <v>22</v>
@@ -3391,7 +3391,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P48">
-        <v>46315.32476340861</v>
+        <v>46315.72471817457</v>
       </c>
       <c r="Q48" t="s">
         <v>27</v>
@@ -3438,7 +3438,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P49">
-        <v>46315.32476338734</v>
+        <v>46315.72471815905</v>
       </c>
       <c r="Q49" t="s">
         <v>27</v>
@@ -3482,7 +3482,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P50">
-        <v>46315.32476339814</v>
+        <v>46315.72471816689</v>
       </c>
       <c r="Q50" t="s">
         <v>27</v>
@@ -3526,7 +3526,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P51">
-        <v>46315.3247633656</v>
+        <v>46315.72471814244</v>
       </c>
       <c r="Q51" s="5" t="s">
         <v>22</v>
@@ -3573,7 +3573,7 @@
         <v>46314.78237008413</v>
       </c>
       <c r="P52">
-        <v>46315.32476337639</v>
+        <v>46315.72471815073</v>
       </c>
       <c r="Q52" t="s">
         <v>27</v>
@@ -3617,7 +3617,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P53">
-        <v>46315.32476335378</v>
+        <v>46315.72471813348</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>22</v>
@@ -3667,7 +3667,7 @@
         <v>46314.78236997747</v>
       </c>
       <c r="P54">
-        <v>46315.32476333033</v>
+        <v>46315.72471811428</v>
       </c>
       <c r="Q54" t="s">
         <v>27</v>
@@ -3716,7 +3716,7 @@
         <v>46300.75884774033</v>
       </c>
       <c r="P55" s="6">
-        <v>46315.32478206314</v>
+        <v>46315.72473462328</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>27</v>
@@ -3763,7 +3763,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P56" s="6">
-        <v>46315.32478207248</v>
+        <v>46315.72473463017</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>22</v>
@@ -3812,7 +3812,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P57" s="6">
-        <v>46315.32479014729</v>
+        <v>46315.72474256394</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>27</v>
@@ -3861,7 +3861,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P58" s="6">
-        <v>46315.32479015972</v>
+        <v>46315.72474257381</v>
       </c>
       <c r="Q58" s="6" t="s">
         <v>27</v>
@@ -3908,7 +3908,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P59" s="6">
-        <v>46315.32479017045</v>
+        <v>46315.7247425824</v>
       </c>
       <c r="Q59" s="6" t="s">
         <v>27</v>
@@ -3957,7 +3957,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P60" s="6">
-        <v>46315.32479018066</v>
+        <v>46315.72474259041</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>27</v>
@@ -4006,7 +4006,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P61" s="6">
-        <v>46315.32479019045</v>
+        <v>46315.72474259797</v>
       </c>
       <c r="Q61" s="6" t="s">
         <v>27</v>
@@ -4055,7 +4055,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P62" s="6">
-        <v>46315.32479020972</v>
+        <v>46315.72474261288</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>27</v>
@@ -4102,7 +4102,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P63" s="6">
-        <v>46315.32479021895</v>
+        <v>46315.72474262045</v>
       </c>
       <c r="Q63" s="5" t="s">
         <v>22</v>
@@ -4149,7 +4149,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P64" s="6">
-        <v>46315.32479025755</v>
+        <v>46315.72474264888</v>
       </c>
       <c r="Q64" s="5" t="s">
         <v>22</v>
@@ -4196,7 +4196,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P65" s="6">
-        <v>46315.32479022881</v>
+        <v>46315.72474262786</v>
       </c>
       <c r="Q65" s="5" t="s">
         <v>22</v>
@@ -4247,7 +4247,7 @@
         <v>46300.75884793277</v>
       </c>
       <c r="P66" s="6">
-        <v>46315.32479032435</v>
+        <v>46315.7247426968</v>
       </c>
       <c r="Q66" s="6" t="s">
         <v>27</v>
@@ -4296,7 +4296,7 @@
         <v>46300.75884796329</v>
       </c>
       <c r="P67" s="6">
-        <v>46315.32479031511</v>
+        <v>46315.72474269001</v>
       </c>
       <c r="Q67" s="6" t="s">
         <v>27</v>
@@ -4345,7 +4345,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P68" s="6">
-        <v>46315.32479029585</v>
+        <v>46315.72474267632</v>
       </c>
       <c r="Q68" s="5" t="s">
         <v>22</v>
@@ -4392,7 +4392,7 @@
         <v>46300.75885617639</v>
       </c>
       <c r="P69" s="6">
-        <v>46315.3247903339</v>
+        <v>46315.72474270329</v>
       </c>
       <c r="Q69" s="6" t="s">
         <v>27</v>
@@ -4441,7 +4441,7 @@
         <v>46300.75885619673</v>
       </c>
       <c r="P70" s="6">
-        <v>46315.32479030552</v>
+        <v>46315.7247426833</v>
       </c>
       <c r="Q70" s="6" t="s">
         <v>27</v>
@@ -4492,7 +4492,7 @@
         <v>46305.20576106136</v>
       </c>
       <c r="P71" s="6">
-        <v>46315.32480097551</v>
+        <v>46315.72475242602</v>
       </c>
       <c r="Q71" s="6" t="s">
         <v>27</v>
@@ -4543,7 +4543,7 @@
         <v>46300.75885624527</v>
       </c>
       <c r="P72" s="6">
-        <v>46315.32480098611</v>
+        <v>46315.72475243433</v>
       </c>
       <c r="Q72" s="6" t="s">
         <v>27</v>
@@ -4592,7 +4592,7 @@
         <v>46300.75885627908</v>
       </c>
       <c r="P73" s="6">
-        <v>46315.32480101725</v>
+        <v>46315.72475245793</v>
       </c>
       <c r="Q73" s="6" t="s">
         <v>27</v>
@@ -4641,7 +4641,7 @@
         <v>46300.75885633306</v>
       </c>
       <c r="P74" s="6">
-        <v>46315.32480103798</v>
+        <v>46315.72475247212</v>
       </c>
       <c r="Q74" s="6" t="s">
         <v>27</v>
@@ -4912,7 +4912,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P2" s="2">
-        <v>46315.32478204358</v>
+        <v>46315.72473460915</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>22</v>
@@ -4959,7 +4959,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P3" s="2">
-        <v>46315.32478205338</v>
+        <v>46315.7247346163</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>22</v>
@@ -5006,7 +5006,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P4" s="2">
-        <v>46315.32478199558</v>
+        <v>46315.72473457522</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>22</v>
@@ -5050,7 +5050,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P5" s="2">
-        <v>46315.32478197602</v>
+        <v>46315.72473456129</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>22</v>
@@ -5094,7 +5094,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P6" s="2">
-        <v>46315.32478196619</v>
+        <v>46315.72473455409</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>22</v>
@@ -5141,7 +5141,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P7" s="2">
-        <v>46315.32478193731</v>
+        <v>46315.7247345326</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>22</v>
@@ -5188,7 +5188,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P8" s="2">
-        <v>46315.32478189487</v>
+        <v>46315.72473449912</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>22</v>
@@ -5232,7 +5232,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P9" s="2">
-        <v>46315.32478190657</v>
+        <v>46315.72473450827</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>22</v>
@@ -5364,7 +5364,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P12" s="2">
-        <v>46315.32477357671</v>
+        <v>46315.72472654899</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>22</v>
@@ -5408,7 +5408,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P13" s="2">
-        <v>46315.32477354836</v>
+        <v>46315.72472652839</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>22</v>
@@ -5455,7 +5455,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P14" s="2">
-        <v>46315.32477351849</v>
+        <v>46315.7247265066</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>22</v>
@@ -5502,7 +5502,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P15" s="2">
-        <v>46315.32477349844</v>
+        <v>46315.72472649151</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>22</v>
@@ -5549,7 +5549,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P16" s="2">
-        <v>46315.32477348828</v>
+        <v>46315.72472648304</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>22</v>
@@ -5593,7 +5593,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P17">
-        <v>46315.32477345787</v>
+        <v>46315.72472645972</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>22</v>
@@ -5637,7 +5637,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P18">
-        <v>46315.32477346843</v>
+        <v>46315.7247264679</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>22</v>
@@ -5684,7 +5684,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P19">
-        <v>46315.32477347844</v>
+        <v>46315.72472647548</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>22</v>
@@ -5778,7 +5778,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P21">
-        <v>46315.32476352833</v>
+        <v>46315.72471826433</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>22</v>
@@ -5822,7 +5822,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P22">
-        <v>46315.32476346933</v>
+        <v>46315.72471822131</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>22</v>
@@ -5866,7 +5866,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P23">
-        <v>46315.32476349834</v>
+        <v>46315.72471824281</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>22</v>
@@ -5910,7 +5910,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P24">
-        <v>46315.32476348878</v>
+        <v>46315.7247182357</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>22</v>
@@ -5954,7 +5954,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P25">
-        <v>46315.32476342953</v>
+        <v>46315.72471818957</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>22</v>
@@ -5998,7 +5998,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P26">
-        <v>46315.32476341919</v>
+        <v>46315.72471818211</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>22</v>
@@ -6042,7 +6042,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P27">
-        <v>46315.3247633656</v>
+        <v>46315.72471814244</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>22</v>
@@ -6086,7 +6086,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P28">
-        <v>46315.32476335378</v>
+        <v>46315.72471813348</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>22</v>
@@ -6133,7 +6133,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P29" s="6">
-        <v>46315.32478207248</v>
+        <v>46315.72473463017</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>22</v>
@@ -6180,7 +6180,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P30" s="6">
-        <v>46315.32479021895</v>
+        <v>46315.72474262045</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>22</v>
@@ -6227,7 +6227,7 @@
         <v>46300.75884790152</v>
       </c>
       <c r="P31" s="6">
-        <v>46315.32479025755</v>
+        <v>46315.72474264888</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>22</v>
@@ -6274,7 +6274,7 @@
         <v>46310.71708389919</v>
       </c>
       <c r="P32" s="6">
-        <v>46315.32479022881</v>
+        <v>46315.72474262786</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>22</v>
@@ -6323,7 +6323,7 @@
         <v>46300.75884799581</v>
       </c>
       <c r="P33" s="6">
-        <v>46315.32479029585</v>
+        <v>46315.72474267632</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>22</v>
@@ -6403,7 +6403,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -6451,10 +6451,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46315.32474515907</v>
+        <v>46315.72470289427</v>
       </c>
       <c r="B2">
-        <v>46315.32820895511</v>
+        <v>46315.72632052699</v>
       </c>
       <c r="C2" t="s">
         <v>241</v>
@@ -6486,10 +6486,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46314.78235376754</v>
+        <v>46315.32474515907</v>
       </c>
       <c r="B3">
-        <v>46314.78404047032</v>
+        <v>46315.32820895511</v>
       </c>
       <c r="C3" t="s">
         <v>241</v>
@@ -6501,16 +6501,16 @@
         <v>3875</v>
       </c>
       <c r="F3">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G3">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="H3">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -6521,10 +6521,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46314.33167013015</v>
+        <v>46314.78235376754</v>
       </c>
       <c r="B4">
-        <v>46314.33543636992</v>
+        <v>46314.78404047032</v>
       </c>
       <c r="C4" t="s">
         <v>241</v>
@@ -6533,33 +6533,33 @@
         <v>194</v>
       </c>
       <c r="E4">
-        <v>3867</v>
+        <v>3875</v>
       </c>
       <c r="F4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G4">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4">
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3867</v>
+        <v>3875</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46313.66768650556</v>
+        <v>46314.33167013015</v>
       </c>
       <c r="B5">
-        <v>46313.66945401487</v>
+        <v>46314.33543636992</v>
       </c>
       <c r="C5" t="s">
         <v>241</v>
@@ -6568,16 +6568,16 @@
         <v>194</v>
       </c>
       <c r="E5">
-        <v>3861</v>
+        <v>3867</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G5">
         <v>393</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -6586,15 +6586,15 @@
         <v>0</v>
       </c>
       <c r="K5">
-        <v>3861</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46313.30528009156</v>
+        <v>46313.66768650556</v>
       </c>
       <c r="B6">
-        <v>46313.3091804056</v>
+        <v>46313.66945401487</v>
       </c>
       <c r="C6" t="s">
         <v>241</v>
@@ -6626,10 +6626,10 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46312.65708521284</v>
+        <v>46313.30528009156</v>
       </c>
       <c r="B7">
-        <v>46312.65865222656</v>
+        <v>46313.3091804056</v>
       </c>
       <c r="C7" t="s">
         <v>241</v>
@@ -6661,10 +6661,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46312.29481460934</v>
+        <v>46312.65708521284</v>
       </c>
       <c r="B8">
-        <v>46312.29886374016</v>
+        <v>46312.65865222656</v>
       </c>
       <c r="C8" t="s">
         <v>241</v>
@@ -6696,10 +6696,10 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B9">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C9" t="s">
         <v>241</v>
@@ -6714,7 +6714,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -6731,10 +6731,10 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B10">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C10" t="s">
         <v>241</v>
@@ -6746,16 +6746,16 @@
         <v>3861</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J10">
         <v>0</v>
@@ -6766,45 +6766,45 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B11">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C11" t="s">
         <v>241</v>
       </c>
       <c r="D11">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E11">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11">
         <v>394</v>
       </c>
       <c r="H11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B12">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C12" t="s">
         <v>241</v>
@@ -6813,33 +6813,33 @@
         <v>193</v>
       </c>
       <c r="E12">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H12">
         <v>2</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B13">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C13" t="s">
         <v>241</v>
@@ -6848,16 +6848,16 @@
         <v>193</v>
       </c>
       <c r="E13">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F13">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G13">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H13">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -6866,15 +6866,15 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B14">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C14" t="s">
         <v>241</v>
@@ -6883,33 +6883,33 @@
         <v>193</v>
       </c>
       <c r="E14">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G14">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B15">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C15" t="s">
         <v>241</v>
@@ -6924,7 +6924,7 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -6941,10 +6941,10 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B16">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C16" t="s">
         <v>241</v>
@@ -6956,16 +6956,16 @@
         <v>3844</v>
       </c>
       <c r="F16">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G16">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -6976,45 +6976,45 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B17">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C17" t="s">
         <v>241</v>
       </c>
       <c r="D17">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E17">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G17">
         <v>381</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17">
         <v>0</v>
       </c>
       <c r="K17">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B18">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C18" t="s">
         <v>241</v>
@@ -7026,13 +7026,13 @@
         <v>3838</v>
       </c>
       <c r="F18">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H18">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -7046,10 +7046,10 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B19">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C19" t="s">
         <v>241</v>
@@ -7058,16 +7058,16 @@
         <v>192</v>
       </c>
       <c r="E19">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G19">
         <v>369</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -7076,15 +7076,15 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B20">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C20" t="s">
         <v>241</v>
@@ -7116,10 +7116,10 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B21">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C21" t="s">
         <v>241</v>
@@ -7134,7 +7134,7 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -7151,10 +7151,10 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B22">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C22" t="s">
         <v>241</v>
@@ -7186,10 +7186,10 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B23">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C23" t="s">
         <v>241</v>
@@ -7201,16 +7201,16 @@
         <v>3826</v>
       </c>
       <c r="F23">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G23">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H23">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J23">
         <v>0</v>
@@ -7221,45 +7221,45 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B24">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C24" t="s">
         <v>241</v>
       </c>
       <c r="D24">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E24">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G24">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B25">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C25" t="s">
         <v>241</v>
@@ -7291,10 +7291,10 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B26">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C26" t="s">
         <v>241</v>
@@ -7309,7 +7309,7 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -7326,10 +7326,10 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B27">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C27" t="s">
         <v>241</v>
@@ -7341,16 +7341,16 @@
         <v>3820</v>
       </c>
       <c r="F27">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H27">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I27">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J27">
         <v>0</v>
@@ -7361,45 +7361,45 @@
     </row>
     <row r="28" spans="1:11">
       <c r="A28">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B28">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C28" t="s">
         <v>241</v>
       </c>
       <c r="D28">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E28">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F28">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G28">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H28">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B29">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C29" t="s">
         <v>241</v>
@@ -7411,13 +7411,13 @@
         <v>160</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G29">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -7426,15 +7426,15 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B30">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C30" t="s">
         <v>241</v>
@@ -7446,21 +7446,56 @@
         <v>160</v>
       </c>
       <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>160</v>
+      </c>
+      <c r="H30">
+        <v>0</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11">
+      <c r="A31">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B31">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C31" t="s">
+        <v>241</v>
+      </c>
+      <c r="D31">
+        <v>8</v>
+      </c>
+      <c r="E31">
+        <v>160</v>
+      </c>
+      <c r="F31">
         <v>157</v>
       </c>
-      <c r="G30">
+      <c r="G31">
         <v>3</v>
       </c>
-      <c r="H30">
+      <c r="H31">
         <v>132</v>
       </c>
-      <c r="I30">
-        <v>1</v>
-      </c>
-      <c r="J30">
-        <v>0</v>
-      </c>
-      <c r="K30">
+      <c r="I31">
+        <v>1</v>
+      </c>
+      <c r="J31">
+        <v>0</v>
+      </c>
+      <c r="K31">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-24-1610Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1031" uniqueCount="233">
   <si>
     <t>Priority</t>
   </si>
@@ -1238,7 +1238,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P2" s="2">
-        <v>46319.31124307877</v>
+        <v>46319.6720323364</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>24</v>
@@ -1285,7 +1285,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P3" s="2">
-        <v>46319.31124312037</v>
+        <v>46319.67203239504</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>29</v>
@@ -1329,7 +1329,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P4" s="2">
-        <v>46319.3112431103</v>
+        <v>46319.67203238071</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>29</v>
@@ -1373,7 +1373,7 @@
         <v>46309.72495168629</v>
       </c>
       <c r="P5" s="2">
-        <v>46319.31124308932</v>
+        <v>46319.67203235119</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>24</v>
@@ -1417,7 +1417,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P6" s="2">
-        <v>46319.31124306845</v>
+        <v>46319.67203232172</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>29</v>
@@ -1464,7 +1464,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P7" s="2">
-        <v>46319.31124305852</v>
+        <v>46319.6720323073</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>24</v>
@@ -1511,7 +1511,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P8" s="2">
-        <v>46319.31124303818</v>
+        <v>46319.67203227813</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>24</v>
@@ -1555,7 +1555,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P9" s="2">
-        <v>46319.31124304838</v>
+        <v>46319.67203229253</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>24</v>
@@ -1599,7 +1599,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P10" s="2">
-        <v>46319.31124302751</v>
+        <v>46319.6720322632</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>29</v>
@@ -1646,7 +1646,7 @@
         <v>46314.33169674601</v>
       </c>
       <c r="P11" s="2">
-        <v>46319.31124301718</v>
+        <v>46319.67203224816</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>24</v>
@@ -1690,7 +1690,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P12" s="2">
-        <v>46319.31124299391</v>
+        <v>46319.67203221709</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>29</v>
@@ -1737,7 +1737,7 @@
         <v>46314.78238309515</v>
       </c>
       <c r="P13" s="2">
-        <v>46319.31123518888</v>
+        <v>46319.67202416656</v>
       </c>
       <c r="Q13" s="2" t="s">
         <v>24</v>
@@ -1787,7 +1787,7 @@
         <v>46316.72656555651</v>
       </c>
       <c r="P14" s="2">
-        <v>46319.31123519874</v>
+        <v>46319.67202418121</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>24</v>
@@ -1834,7 +1834,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P15" s="2">
-        <v>46319.31123515825</v>
+        <v>46319.67202412229</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>29</v>
@@ -1884,7 +1884,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P16" s="2">
-        <v>46319.31123514791</v>
+        <v>46319.67202410727</v>
       </c>
       <c r="Q16" s="2" t="s">
         <v>24</v>
@@ -1931,7 +1931,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P17" s="2">
-        <v>46319.3112351377</v>
+        <v>46319.67202409279</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>29</v>
@@ -1981,7 +1981,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P18" s="2">
-        <v>46319.31123516827</v>
+        <v>46319.67202413744</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>24</v>
@@ -2028,7 +2028,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P19" s="2">
-        <v>46319.3112351789</v>
+        <v>46319.6720241523</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>29</v>
@@ -2078,7 +2078,7 @@
         <v>46318.72197647238</v>
       </c>
       <c r="P20" s="2">
-        <v>46319.31123512736</v>
+        <v>46319.67202407819</v>
       </c>
       <c r="Q20" s="2" t="s">
         <v>24</v>
@@ -2122,7 +2122,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P21" s="2">
-        <v>46319.31123511731</v>
+        <v>46319.67202406382</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>29</v>
@@ -2166,7 +2166,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P22" s="2">
-        <v>46319.31123510764</v>
+        <v>46319.67202404972</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>29</v>
@@ -2213,7 +2213,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P23" s="2">
-        <v>46319.31123509742</v>
+        <v>46319.67202403478</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>29</v>
@@ -2263,7 +2263,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P24" s="2">
-        <v>46319.31123508725</v>
+        <v>46319.67202402036</v>
       </c>
       <c r="Q24" s="2" t="s">
         <v>24</v>
@@ -2310,7 +2310,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P25" s="2">
-        <v>46319.31123507673</v>
+        <v>46319.67202400527</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>29</v>
@@ -2357,7 +2357,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P26" s="2">
-        <v>46319.31123506638</v>
+        <v>46319.67202399077</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>29</v>
@@ -2404,7 +2404,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P27" s="2">
-        <v>46319.31123505588</v>
+        <v>46319.67202397493</v>
       </c>
       <c r="Q27" s="2" t="s">
         <v>24</v>
@@ -2454,7 +2454,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P28" s="2">
-        <v>46319.31123504513</v>
+        <v>46319.6720239597</v>
       </c>
       <c r="Q28" s="2" t="s">
         <v>24</v>
@@ -2498,7 +2498,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P29" s="2">
-        <v>46319.31123503462</v>
+        <v>46319.67202394507</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>29</v>
@@ -2542,7 +2542,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P30" s="2">
-        <v>46319.31123500071</v>
+        <v>46319.67202389851</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>29</v>
@@ -2586,7 +2586,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P31" s="2">
-        <v>46319.31123501338</v>
+        <v>46319.67202391473</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>29</v>
@@ -2674,7 +2674,7 @@
         <v>46314.33168865994</v>
       </c>
       <c r="P33">
-        <v>46319.31122718789</v>
+        <v>46319.67201587754</v>
       </c>
       <c r="Q33" t="s">
         <v>24</v>
@@ -2724,7 +2724,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P34">
-        <v>46319.31122714668</v>
+        <v>46319.67201581824</v>
       </c>
       <c r="Q34" t="s">
         <v>24</v>
@@ -2768,7 +2768,7 @@
         <v>46314.78237020577</v>
       </c>
       <c r="P35">
-        <v>46319.31122716745</v>
+        <v>46319.67201584783</v>
       </c>
       <c r="Q35" t="s">
         <v>24</v>
@@ -2818,7 +2818,7 @@
         <v>46316.72655645811</v>
       </c>
       <c r="P36">
-        <v>46319.31122715756</v>
+        <v>46319.67201583322</v>
       </c>
       <c r="Q36" t="s">
         <v>24</v>
@@ -2865,7 +2865,7 @@
         <v>46316.72655650476</v>
       </c>
       <c r="P37">
-        <v>46319.31122717782</v>
+        <v>46319.67201586255</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>29</v>
@@ -2912,7 +2912,7 @@
         <v>46316.72655654202</v>
       </c>
       <c r="P38">
-        <v>46319.31122712474</v>
+        <v>46319.67201578798</v>
       </c>
       <c r="Q38" s="5" t="s">
         <v>29</v>
@@ -2956,7 +2956,7 @@
         <v>46317.72506061158</v>
       </c>
       <c r="P39">
-        <v>46319.31122713599</v>
+        <v>46319.67201580332</v>
       </c>
       <c r="Q39" s="5" t="s">
         <v>29</v>
@@ -3000,7 +3000,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P40">
-        <v>46319.31122711344</v>
+        <v>46319.67201577258</v>
       </c>
       <c r="Q40" s="5" t="s">
         <v>29</v>
@@ -3044,7 +3044,7 @@
         <v>46317.32462326912</v>
       </c>
       <c r="P41">
-        <v>46319.31122710262</v>
+        <v>46319.6720157571</v>
       </c>
       <c r="Q41" t="s">
         <v>24</v>
@@ -3094,7 +3094,7 @@
         <v>46316.72655637826</v>
       </c>
       <c r="P42">
-        <v>46319.31122709193</v>
+        <v>46319.67201574158</v>
       </c>
       <c r="Q42" t="s">
         <v>24</v>
@@ -3138,7 +3138,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P43">
-        <v>46319.31122708121</v>
+        <v>46319.6720157262</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>29</v>
@@ -3188,7 +3188,7 @@
         <v>46318.72196821687</v>
       </c>
       <c r="P44">
-        <v>46319.3112270712</v>
+        <v>46319.67201571072</v>
       </c>
       <c r="Q44" t="s">
         <v>24</v>
@@ -3232,7 +3232,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P45">
-        <v>46319.3112270615</v>
+        <v>46319.67201569511</v>
       </c>
       <c r="Q45" t="s">
         <v>24</v>
@@ -3279,7 +3279,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P46">
-        <v>46319.31122704193</v>
+        <v>46319.67201566448</v>
       </c>
       <c r="Q46" t="s">
         <v>24</v>
@@ -3323,7 +3323,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P47">
-        <v>46319.31122705174</v>
+        <v>46319.67201567992</v>
       </c>
       <c r="Q47" t="s">
         <v>24</v>
@@ -3367,7 +3367,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P48">
-        <v>46319.3112270315</v>
+        <v>46319.67201564834</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>29</v>
@@ -3414,7 +3414,7 @@
         <v>46314.78237008413</v>
       </c>
       <c r="P49">
-        <v>46319.31122702015</v>
+        <v>46319.6720156327</v>
       </c>
       <c r="Q49" t="s">
         <v>24</v>
@@ -3458,7 +3458,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P50">
-        <v>46319.3112270085</v>
+        <v>46319.67201561624</v>
       </c>
       <c r="Q50" s="5" t="s">
         <v>29</v>
@@ -3508,7 +3508,7 @@
         <v>46314.78236997747</v>
       </c>
       <c r="P51">
-        <v>46319.31122698387</v>
+        <v>46319.67201558428</v>
       </c>
       <c r="Q51" t="s">
         <v>24</v>
@@ -3559,7 +3559,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P52" s="6">
-        <v>46319.31124315045</v>
+        <v>46319.67203243825</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>24</v>
@@ -3608,7 +3608,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P53" s="6">
-        <v>46319.31124314042</v>
+        <v>46319.67203242406</v>
       </c>
       <c r="Q53" s="6" t="s">
         <v>24</v>
@@ -3657,7 +3657,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P54" s="6">
-        <v>46319.31124313032</v>
+        <v>46319.67203240913</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>24</v>
@@ -3706,7 +3706,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P55" s="6">
-        <v>46319.31124316031</v>
+        <v>46319.67203245271</v>
       </c>
       <c r="Q55" s="5" t="s">
         <v>29</v>
@@ -3753,7 +3753,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P56" s="6">
-        <v>46319.31124318061</v>
+        <v>46319.67203248162</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>29</v>
@@ -3802,7 +3802,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P57" s="6">
-        <v>46319.31124319069</v>
+        <v>46319.67203249614</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>24</v>
@@ -3849,7 +3849,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P58" s="6">
-        <v>46319.31124317043</v>
+        <v>46319.67203246716</v>
       </c>
       <c r="Q58" s="5" t="s">
         <v>29</v>
@@ -3898,7 +3898,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P59" s="6">
-        <v>46319.31125106096</v>
+        <v>46319.67204108166</v>
       </c>
       <c r="Q59" s="5" t="s">
         <v>29</v>
@@ -3947,7 +3947,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P60" s="6">
-        <v>46319.31125104808</v>
+        <v>46319.6720410651</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>24</v>
@@ -3994,7 +3994,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P61" s="6">
-        <v>46319.31125111277</v>
+        <v>46319.67204115519</v>
       </c>
       <c r="Q61" s="5" t="s">
         <v>29</v>
@@ -4043,7 +4043,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P62" s="6">
-        <v>46319.31125108213</v>
+        <v>46319.6720411113</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>24</v>
@@ -4092,7 +4092,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P63" s="6">
-        <v>46319.31125109221</v>
+        <v>46319.67204112567</v>
       </c>
       <c r="Q63" s="5" t="s">
         <v>29</v>
@@ -4139,7 +4139,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P64" s="6">
-        <v>46319.31125114338</v>
+        <v>46319.6720411994</v>
       </c>
       <c r="Q64" s="5" t="s">
         <v>29</v>
@@ -4188,7 +4188,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P65" s="6">
-        <v>46319.31125115341</v>
+        <v>46319.67204121367</v>
       </c>
       <c r="Q65" s="6" t="s">
         <v>24</v>
@@ -4237,7 +4237,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P66" s="6">
-        <v>46319.31125117404</v>
+        <v>46319.67204124287</v>
       </c>
       <c r="Q66" s="6" t="s">
         <v>24</v>
@@ -4284,7 +4284,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P67" s="6">
-        <v>46319.3112511936</v>
+        <v>46319.67204127228</v>
       </c>
       <c r="Q67" s="6" t="s">
         <v>24</v>
@@ -4333,7 +4333,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P68" s="6">
-        <v>46319.31125118386</v>
+        <v>46319.67204125795</v>
       </c>
       <c r="Q68" s="6" t="s">
         <v>24</v>
@@ -4382,7 +4382,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P69" s="6">
-        <v>46319.31125116362</v>
+        <v>46319.67204122802</v>
       </c>
       <c r="Q69" s="6" t="s">
         <v>24</v>
@@ -4431,7 +4431,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P70" s="6">
-        <v>46319.31125121377</v>
+        <v>46319.67204130143</v>
       </c>
       <c r="Q70" s="6" t="s">
         <v>24</v>
@@ -4478,7 +4478,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P71" s="6">
-        <v>46319.31125122361</v>
+        <v>46319.67204131561</v>
       </c>
       <c r="Q71" s="5" t="s">
         <v>29</v>
@@ -4746,7 +4746,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P2" s="2">
-        <v>46319.31124312037</v>
+        <v>46319.67203239504</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>29</v>
@@ -4790,7 +4790,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P3" s="2">
-        <v>46319.3112431103</v>
+        <v>46319.67203238071</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>29</v>
@@ -4834,7 +4834,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P4" s="2">
-        <v>46319.31124306845</v>
+        <v>46319.67203232172</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>29</v>
@@ -4878,7 +4878,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P5" s="2">
-        <v>46319.31124302751</v>
+        <v>46319.6720322632</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>29</v>
@@ -4922,7 +4922,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P6" s="2">
-        <v>46319.31124299391</v>
+        <v>46319.67203221709</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>29</v>
@@ -4969,7 +4969,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P7" s="2">
-        <v>46319.31123515825</v>
+        <v>46319.67202412229</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>29</v>
@@ -5016,7 +5016,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P8" s="2">
-        <v>46319.3112351377</v>
+        <v>46319.67202409279</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>29</v>
@@ -5063,7 +5063,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P9" s="2">
-        <v>46319.3112351789</v>
+        <v>46319.6720241523</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>29</v>
@@ -5107,7 +5107,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P10" s="2">
-        <v>46319.31123511731</v>
+        <v>46319.67202406382</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>29</v>
@@ -5151,7 +5151,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P11" s="2">
-        <v>46319.31123510764</v>
+        <v>46319.67202404972</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>29</v>
@@ -5198,7 +5198,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P12" s="2">
-        <v>46319.31123509742</v>
+        <v>46319.67202403478</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>29</v>
@@ -5245,7 +5245,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P13" s="2">
-        <v>46319.31123507673</v>
+        <v>46319.67202400527</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>29</v>
@@ -5292,7 +5292,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P14" s="2">
-        <v>46319.31123506638</v>
+        <v>46319.67202399077</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>29</v>
@@ -5336,7 +5336,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P15" s="2">
-        <v>46319.31123503462</v>
+        <v>46319.67202394507</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>29</v>
@@ -5380,7 +5380,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P16" s="2">
-        <v>46319.31123500071</v>
+        <v>46319.67202389851</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>29</v>
@@ -5424,7 +5424,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P17" s="2">
-        <v>46319.31123501338</v>
+        <v>46319.67202391473</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>29</v>
@@ -5515,7 +5515,7 @@
         <v>46316.72655650476</v>
       </c>
       <c r="P19">
-        <v>46319.31122717782</v>
+        <v>46319.67201586255</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>29</v>
@@ -5562,7 +5562,7 @@
         <v>46316.72655654202</v>
       </c>
       <c r="P20">
-        <v>46319.31122712474</v>
+        <v>46319.67201578798</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>29</v>
@@ -5606,7 +5606,7 @@
         <v>46317.72506061158</v>
       </c>
       <c r="P21">
-        <v>46319.31122713599</v>
+        <v>46319.67201580332</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>29</v>
@@ -5650,7 +5650,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P22">
-        <v>46319.31122711344</v>
+        <v>46319.67201577258</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>29</v>
@@ -5694,7 +5694,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P23">
-        <v>46319.31122708121</v>
+        <v>46319.6720157262</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>29</v>
@@ -5738,7 +5738,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P24">
-        <v>46319.3112270315</v>
+        <v>46319.67201564834</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>29</v>
@@ -5782,7 +5782,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P25">
-        <v>46319.3112270085</v>
+        <v>46319.67201561624</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>29</v>
@@ -5831,7 +5831,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P26" s="6">
-        <v>46319.31124316031</v>
+        <v>46319.67203245271</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>29</v>
@@ -5878,7 +5878,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P27" s="6">
-        <v>46319.31124318061</v>
+        <v>46319.67203248162</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>29</v>
@@ -5925,7 +5925,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P28" s="6">
-        <v>46319.31124317043</v>
+        <v>46319.67203246716</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>29</v>
@@ -5974,7 +5974,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P29" s="6">
-        <v>46319.31125106096</v>
+        <v>46319.67204108166</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>29</v>
@@ -6021,7 +6021,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P30" s="6">
-        <v>46319.31125111277</v>
+        <v>46319.67204115519</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>29</v>
@@ -6070,7 +6070,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P31" s="6">
-        <v>46319.31125109221</v>
+        <v>46319.67204112567</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>29</v>
@@ -6117,7 +6117,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P32" s="6">
-        <v>46319.31125114338</v>
+        <v>46319.6720411994</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>29</v>
@@ -6164,7 +6164,7 @@
         <v>46308.39987059968</v>
       </c>
       <c r="P33" s="6">
-        <v>46319.31125122361</v>
+        <v>46319.67204131561</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>29</v>
@@ -6244,7 +6244,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -6292,10 +6292,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46319.31121266444</v>
+        <v>46319.67200058671</v>
       </c>
       <c r="B2">
-        <v>46319.31353464982</v>
+        <v>46319.6736326805</v>
       </c>
       <c r="C2" t="s">
         <v>232</v>
@@ -6327,10 +6327,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46318.72195433634</v>
+        <v>46319.31121266444</v>
       </c>
       <c r="B3">
-        <v>46318.72353879309</v>
+        <v>46319.31353464982</v>
       </c>
       <c r="C3" t="s">
         <v>232</v>
@@ -6342,7 +6342,7 @@
         <v>3885</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G3">
         <v>406</v>
@@ -6362,10 +6362,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46318.32371957044</v>
+        <v>46318.72195433634</v>
       </c>
       <c r="B4">
-        <v>46318.32702615024</v>
+        <v>46318.72353879309</v>
       </c>
       <c r="C4" t="s">
         <v>232</v>
@@ -6374,10 +6374,10 @@
         <v>195</v>
       </c>
       <c r="E4">
-        <v>3883</v>
+        <v>3885</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4">
         <v>406</v>
@@ -6392,15 +6392,15 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3883</v>
+        <v>3885</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46317.72504084905</v>
+        <v>46318.32371957044</v>
       </c>
       <c r="B5">
-        <v>46317.72671046003</v>
+        <v>46318.32702615024</v>
       </c>
       <c r="C5" t="s">
         <v>232</v>
@@ -6412,13 +6412,13 @@
         <v>3883</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -6432,10 +6432,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46317.32460656222</v>
+        <v>46317.72504084905</v>
       </c>
       <c r="B6">
-        <v>46317.32634152405</v>
+        <v>46317.72671046003</v>
       </c>
       <c r="C6" t="s">
         <v>232</v>
@@ -6444,13 +6444,13 @@
         <v>195</v>
       </c>
       <c r="E6">
-        <v>3882</v>
+        <v>3883</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -6462,33 +6462,33 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3882</v>
+        <v>3883</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46316.72653559106</v>
+        <v>46317.32460656222</v>
       </c>
       <c r="B7">
-        <v>46316.72825635534</v>
+        <v>46317.32634152405</v>
       </c>
       <c r="C7" t="s">
         <v>232</v>
       </c>
       <c r="D7">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E7">
-        <v>3880</v>
+        <v>3882</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G7">
         <v>405</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -6497,15 +6497,15 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>3880</v>
+        <v>3882</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46316.32743514836</v>
+        <v>46316.72653559106</v>
       </c>
       <c r="B8">
-        <v>46316.33233177644</v>
+        <v>46316.72825635534</v>
       </c>
       <c r="C8" t="s">
         <v>232</v>
@@ -6514,16 +6514,16 @@
         <v>194</v>
       </c>
       <c r="E8">
-        <v>3875</v>
+        <v>3880</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G8">
         <v>405</v>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I8">
         <v>0</v>
@@ -6532,15 +6532,15 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3875</v>
+        <v>3880</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46315.72470289427</v>
+        <v>46316.32743514836</v>
       </c>
       <c r="B9">
-        <v>46315.72632052699</v>
+        <v>46316.33233177644</v>
       </c>
       <c r="C9" t="s">
         <v>232</v>
@@ -6555,7 +6555,7 @@
         <v>0</v>
       </c>
       <c r="G9">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -6572,10 +6572,10 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46315.32474515907</v>
+        <v>46315.72470289427</v>
       </c>
       <c r="B10">
-        <v>46315.32820895511</v>
+        <v>46315.72632052699</v>
       </c>
       <c r="C10" t="s">
         <v>232</v>
@@ -6607,10 +6607,10 @@
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46314.78235376754</v>
+        <v>46315.32474515907</v>
       </c>
       <c r="B11">
-        <v>46314.78404047032</v>
+        <v>46315.32820895511</v>
       </c>
       <c r="C11" t="s">
         <v>232</v>
@@ -6622,16 +6622,16 @@
         <v>3875</v>
       </c>
       <c r="F11">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="H11">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -6642,10 +6642,10 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46314.33167013015</v>
+        <v>46314.78235376754</v>
       </c>
       <c r="B12">
-        <v>46314.33543636992</v>
+        <v>46314.78404047032</v>
       </c>
       <c r="C12" t="s">
         <v>232</v>
@@ -6654,33 +6654,33 @@
         <v>194</v>
       </c>
       <c r="E12">
-        <v>3867</v>
+        <v>3875</v>
       </c>
       <c r="F12">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G12">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="H12">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>3867</v>
+        <v>3875</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46313.66768650556</v>
+        <v>46314.33167013015</v>
       </c>
       <c r="B13">
-        <v>46313.66945401487</v>
+        <v>46314.33543636992</v>
       </c>
       <c r="C13" t="s">
         <v>232</v>
@@ -6689,16 +6689,16 @@
         <v>194</v>
       </c>
       <c r="E13">
-        <v>3861</v>
+        <v>3867</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G13">
         <v>393</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -6707,15 +6707,15 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>3861</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46313.30528009156</v>
+        <v>46313.66768650556</v>
       </c>
       <c r="B14">
-        <v>46313.3091804056</v>
+        <v>46313.66945401487</v>
       </c>
       <c r="C14" t="s">
         <v>232</v>
@@ -6747,10 +6747,10 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46312.65708521284</v>
+        <v>46313.30528009156</v>
       </c>
       <c r="B15">
-        <v>46312.65865222656</v>
+        <v>46313.3091804056</v>
       </c>
       <c r="C15" t="s">
         <v>232</v>
@@ -6782,10 +6782,10 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46312.29481460934</v>
+        <v>46312.65708521284</v>
       </c>
       <c r="B16">
-        <v>46312.29886374016</v>
+        <v>46312.65865222656</v>
       </c>
       <c r="C16" t="s">
         <v>232</v>
@@ -6817,10 +6817,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B17">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C17" t="s">
         <v>232</v>
@@ -6835,7 +6835,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H17">
         <v>0</v>
@@ -6852,10 +6852,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B18">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C18" t="s">
         <v>232</v>
@@ -6867,16 +6867,16 @@
         <v>3861</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G18">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H18">
         <v>0</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18">
         <v>0</v>
@@ -6887,45 +6887,45 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B19">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C19" t="s">
         <v>232</v>
       </c>
       <c r="D19">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E19">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19">
         <v>394</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
       <c r="K19">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B20">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C20" t="s">
         <v>232</v>
@@ -6934,33 +6934,33 @@
         <v>193</v>
       </c>
       <c r="E20">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H20">
         <v>2</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B21">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C21" t="s">
         <v>232</v>
@@ -6969,16 +6969,16 @@
         <v>193</v>
       </c>
       <c r="E21">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F21">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G21">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H21">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -6987,15 +6987,15 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B22">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C22" t="s">
         <v>232</v>
@@ -7004,33 +7004,33 @@
         <v>193</v>
       </c>
       <c r="E22">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G22">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B23">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C23" t="s">
         <v>232</v>
@@ -7045,7 +7045,7 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -7062,10 +7062,10 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B24">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C24" t="s">
         <v>232</v>
@@ -7077,16 +7077,16 @@
         <v>3844</v>
       </c>
       <c r="F24">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -7097,45 +7097,45 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B25">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C25" t="s">
         <v>232</v>
       </c>
       <c r="D25">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E25">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G25">
         <v>381</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B26">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C26" t="s">
         <v>232</v>
@@ -7147,13 +7147,13 @@
         <v>3838</v>
       </c>
       <c r="F26">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H26">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -7167,10 +7167,10 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B27">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C27" t="s">
         <v>232</v>
@@ -7179,16 +7179,16 @@
         <v>192</v>
       </c>
       <c r="E27">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G27">
         <v>369</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -7197,15 +7197,15 @@
         <v>0</v>
       </c>
       <c r="K27">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B28">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C28" t="s">
         <v>232</v>
@@ -7237,10 +7237,10 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B29">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C29" t="s">
         <v>232</v>
@@ -7255,7 +7255,7 @@
         <v>0</v>
       </c>
       <c r="G29">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -7272,10 +7272,10 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B30">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C30" t="s">
         <v>232</v>
@@ -7307,10 +7307,10 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B31">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C31" t="s">
         <v>232</v>
@@ -7322,16 +7322,16 @@
         <v>3826</v>
       </c>
       <c r="F31">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G31">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J31">
         <v>0</v>
@@ -7342,45 +7342,45 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B32">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C32" t="s">
         <v>232</v>
       </c>
       <c r="D32">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E32">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F32">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G32">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32">
         <v>0</v>
       </c>
       <c r="K32">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="33" spans="1:11">
       <c r="A33">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B33">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C33" t="s">
         <v>232</v>
@@ -7412,10 +7412,10 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B34">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C34" t="s">
         <v>232</v>
@@ -7430,7 +7430,7 @@
         <v>0</v>
       </c>
       <c r="G34">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H34">
         <v>0</v>
@@ -7447,10 +7447,10 @@
     </row>
     <row r="35" spans="1:11">
       <c r="A35">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B35">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C35" t="s">
         <v>232</v>
@@ -7462,16 +7462,16 @@
         <v>3820</v>
       </c>
       <c r="F35">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G35">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H35">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I35">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J35">
         <v>0</v>
@@ -7482,45 +7482,45 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B36">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C36" t="s">
         <v>232</v>
       </c>
       <c r="D36">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E36">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F36">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G36">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H36">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J36">
         <v>0</v>
       </c>
       <c r="K36">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B37">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C37" t="s">
         <v>232</v>
@@ -7532,13 +7532,13 @@
         <v>160</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G37">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -7547,15 +7547,15 @@
         <v>0</v>
       </c>
       <c r="K37">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="38" spans="1:11">
       <c r="A38">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B38">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C38" t="s">
         <v>232</v>
@@ -7567,21 +7567,56 @@
         <v>160</v>
       </c>
       <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38">
+        <v>160</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11">
+      <c r="A39">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B39">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C39" t="s">
+        <v>232</v>
+      </c>
+      <c r="D39">
+        <v>8</v>
+      </c>
+      <c r="E39">
+        <v>160</v>
+      </c>
+      <c r="F39">
         <v>157</v>
       </c>
-      <c r="G38">
+      <c r="G39">
         <v>3</v>
       </c>
-      <c r="H38">
+      <c r="H39">
         <v>132</v>
       </c>
-      <c r="I38">
-        <v>1</v>
-      </c>
-      <c r="J38">
-        <v>0</v>
-      </c>
-      <c r="K38">
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-25-1640Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="231">
   <si>
     <t>Priority</t>
   </si>
@@ -1229,7 +1229,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P2" s="2">
-        <v>46320.32085588058</v>
+        <v>46320.6929425636</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>23</v>
@@ -1273,7 +1273,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P3" s="2">
-        <v>46320.32085589516</v>
+        <v>46320.692942578</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>23</v>
@@ -1317,7 +1317,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P4" s="2">
-        <v>46320.32085586598</v>
+        <v>46320.6929425487</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>30</v>
@@ -1364,7 +1364,7 @@
         <v>46314.33169674601</v>
       </c>
       <c r="P5" s="2">
-        <v>46320.32085585117</v>
+        <v>46320.69294253403</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>23</v>
@@ -1408,7 +1408,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P6" s="2">
-        <v>46320.32085581985</v>
+        <v>46320.69294250303</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>30</v>
@@ -1455,7 +1455,7 @@
         <v>46314.78238309515</v>
       </c>
       <c r="P7" s="2">
-        <v>46320.32084753965</v>
+        <v>46320.69293422026</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>23</v>
@@ -1505,7 +1505,7 @@
         <v>46316.72656555651</v>
       </c>
       <c r="P8" s="2">
-        <v>46320.32084755447</v>
+        <v>46320.69293423482</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>23</v>
@@ -1552,7 +1552,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P9" s="2">
-        <v>46320.32084749614</v>
+        <v>46320.69293417776</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>30</v>
@@ -1602,7 +1602,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P10" s="2">
-        <v>46320.32084748147</v>
+        <v>46320.69293416294</v>
       </c>
       <c r="Q10" s="2" t="s">
         <v>23</v>
@@ -1649,7 +1649,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P11" s="2">
-        <v>46320.32084746652</v>
+        <v>46320.69293414867</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>30</v>
@@ -1699,7 +1699,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P12" s="2">
-        <v>46320.3208475104</v>
+        <v>46320.69293419189</v>
       </c>
       <c r="Q12" s="2" t="s">
         <v>23</v>
@@ -1746,7 +1746,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P13" s="2">
-        <v>46320.32084752488</v>
+        <v>46320.69293420629</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>30</v>
@@ -1796,7 +1796,7 @@
         <v>46318.72197647238</v>
       </c>
       <c r="P14" s="2">
-        <v>46320.32084745196</v>
+        <v>46320.69293413446</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>23</v>
@@ -1840,7 +1840,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P15" s="2">
-        <v>46320.32084743775</v>
+        <v>46320.69293412055</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>30</v>
@@ -1884,7 +1884,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P16" s="2">
-        <v>46320.32084742378</v>
+        <v>46320.69293410664</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>30</v>
@@ -1931,7 +1931,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P17" s="2">
-        <v>46320.32084740869</v>
+        <v>46320.69293409197</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>30</v>
@@ -1981,7 +1981,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P18" s="2">
-        <v>46320.32084739432</v>
+        <v>46320.69293407778</v>
       </c>
       <c r="Q18" s="2" t="s">
         <v>23</v>
@@ -2028,7 +2028,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P19" s="2">
-        <v>46320.32084737946</v>
+        <v>46320.69293406293</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>30</v>
@@ -2075,7 +2075,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P20" s="2">
-        <v>46320.32084736499</v>
+        <v>46320.69293404857</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>30</v>
@@ -2122,7 +2122,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P21" s="2">
-        <v>46320.32084734984</v>
+        <v>46320.69293403376</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>23</v>
@@ -2172,7 +2172,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P22" s="2">
-        <v>46320.32084733485</v>
+        <v>46320.69293401903</v>
       </c>
       <c r="Q22" s="2" t="s">
         <v>23</v>
@@ -2216,7 +2216,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P23" s="2">
-        <v>46320.3208473202</v>
+        <v>46320.69293400446</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>30</v>
@@ -2260,7 +2260,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P24" s="2">
-        <v>46320.32084727324</v>
+        <v>46320.69293395866</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>30</v>
@@ -2304,7 +2304,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P25" s="2">
-        <v>46320.32084728919</v>
+        <v>46320.69293397453</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>30</v>
@@ -2392,7 +2392,7 @@
         <v>46314.33168865994</v>
       </c>
       <c r="P27" s="2">
-        <v>46320.32083894681</v>
+        <v>46320.69292548197</v>
       </c>
       <c r="Q27" s="2" t="s">
         <v>23</v>
@@ -2442,7 +2442,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P28">
-        <v>46320.32083888754</v>
+        <v>46320.69292542169</v>
       </c>
       <c r="Q28" t="s">
         <v>23</v>
@@ -2486,7 +2486,7 @@
         <v>46314.78237020577</v>
       </c>
       <c r="P29">
-        <v>46320.32083891718</v>
+        <v>46320.69292545304</v>
       </c>
       <c r="Q29" t="s">
         <v>23</v>
@@ -2536,7 +2536,7 @@
         <v>46316.72655645811</v>
       </c>
       <c r="P30">
-        <v>46320.32083890243</v>
+        <v>46320.69292543724</v>
       </c>
       <c r="Q30" t="s">
         <v>23</v>
@@ -2583,7 +2583,7 @@
         <v>46316.72655650476</v>
       </c>
       <c r="P31">
-        <v>46320.3208389317</v>
+        <v>46320.69292546777</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>30</v>
@@ -2630,7 +2630,7 @@
         <v>46316.72655654202</v>
       </c>
       <c r="P32">
-        <v>46320.32083885691</v>
+        <v>46320.69292539194</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>30</v>
@@ -2674,7 +2674,7 @@
         <v>46317.72506061158</v>
       </c>
       <c r="P33">
-        <v>46320.32083887186</v>
+        <v>46320.69292540668</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>30</v>
@@ -2718,7 +2718,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P34">
-        <v>46320.32083884165</v>
+        <v>46320.69292537658</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>30</v>
@@ -2762,7 +2762,7 @@
         <v>46317.32462326912</v>
       </c>
       <c r="P35">
-        <v>46320.32083882676</v>
+        <v>46320.6929253605</v>
       </c>
       <c r="Q35" t="s">
         <v>23</v>
@@ -2812,7 +2812,7 @@
         <v>46316.72655637826</v>
       </c>
       <c r="P36">
-        <v>46320.32083881187</v>
+        <v>46320.69292534533</v>
       </c>
       <c r="Q36" t="s">
         <v>23</v>
@@ -2856,7 +2856,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P37">
-        <v>46320.3208387964</v>
+        <v>46320.69292532978</v>
       </c>
       <c r="Q37" s="5" t="s">
         <v>30</v>
@@ -2906,7 +2906,7 @@
         <v>46318.72196821687</v>
       </c>
       <c r="P38">
-        <v>46320.3208387815</v>
+        <v>46320.6929253148</v>
       </c>
       <c r="Q38" t="s">
         <v>23</v>
@@ -2950,7 +2950,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P39">
-        <v>46320.32083876541</v>
+        <v>46320.69292529984</v>
       </c>
       <c r="Q39" t="s">
         <v>23</v>
@@ -2997,7 +2997,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P40">
-        <v>46320.32083873428</v>
+        <v>46320.69292526841</v>
       </c>
       <c r="Q40" t="s">
         <v>23</v>
@@ -3041,7 +3041,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P41">
-        <v>46320.32083874943</v>
+        <v>46320.69292528417</v>
       </c>
       <c r="Q41" t="s">
         <v>23</v>
@@ -3085,7 +3085,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P42">
-        <v>46320.32083871875</v>
+        <v>46320.6929252531</v>
       </c>
       <c r="Q42" s="5" t="s">
         <v>30</v>
@@ -3132,7 +3132,7 @@
         <v>46314.78237008413</v>
       </c>
       <c r="P43">
-        <v>46320.32083870213</v>
+        <v>46320.69292523749</v>
       </c>
       <c r="Q43" t="s">
         <v>23</v>
@@ -3176,7 +3176,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P44">
-        <v>46320.32083868645</v>
+        <v>46320.69292522156</v>
       </c>
       <c r="Q44" s="5" t="s">
         <v>30</v>
@@ -3226,7 +3226,7 @@
         <v>46314.78236997747</v>
       </c>
       <c r="P45">
-        <v>46320.32083865559</v>
+        <v>46320.69292519092</v>
       </c>
       <c r="Q45" t="s">
         <v>23</v>
@@ -3277,7 +3277,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P46" s="6">
-        <v>46320.32085593873</v>
+        <v>46320.69294262146</v>
       </c>
       <c r="Q46" s="6" t="s">
         <v>23</v>
@@ -3326,7 +3326,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P47" s="6">
-        <v>46320.32085599675</v>
+        <v>46320.69294268152</v>
       </c>
       <c r="Q47" s="5" t="s">
         <v>30</v>
@@ -3373,7 +3373,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P48" s="6">
-        <v>46320.32085598254</v>
+        <v>46320.69294266718</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>30</v>
@@ -3420,7 +3420,7 @@
         <v>46309.72495168629</v>
       </c>
       <c r="P49" s="6">
-        <v>46320.32085595385</v>
+        <v>46320.69294263656</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>23</v>
@@ -3467,7 +3467,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P50" s="6">
-        <v>46320.32085592383</v>
+        <v>46320.6929426069</v>
       </c>
       <c r="Q50" s="5" t="s">
         <v>30</v>
@@ -3516,7 +3516,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P51" s="6">
-        <v>46320.32085590947</v>
+        <v>46320.6929425923</v>
       </c>
       <c r="Q51" s="6" t="s">
         <v>23</v>
@@ -3567,7 +3567,7 @@
         <v>46305.20575267453</v>
       </c>
       <c r="P52" s="6">
-        <v>46320.32085603944</v>
+        <v>46320.69294272408</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>23</v>
@@ -3616,7 +3616,7 @@
         <v>46305.20575269723</v>
       </c>
       <c r="P53" s="6">
-        <v>46320.3208560252</v>
+        <v>46320.69294271015</v>
       </c>
       <c r="Q53" s="6" t="s">
         <v>23</v>
@@ -3665,7 +3665,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P54" s="6">
-        <v>46320.32085601115</v>
+        <v>46320.69294269622</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>23</v>
@@ -3714,7 +3714,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P55" s="6">
-        <v>46320.32085605386</v>
+        <v>46320.69294273822</v>
       </c>
       <c r="Q55" s="5" t="s">
         <v>30</v>
@@ -3761,7 +3761,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P56" s="6">
-        <v>46320.32085608264</v>
+        <v>46320.69294276673</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>30</v>
@@ -3810,7 +3810,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P57" s="6">
-        <v>46320.32085609702</v>
+        <v>46320.69294278146</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>23</v>
@@ -3857,7 +3857,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P58" s="6">
-        <v>46320.32085606855</v>
+        <v>46320.69294275272</v>
       </c>
       <c r="Q58" s="5" t="s">
         <v>30</v>
@@ -3906,7 +3906,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P59" s="6">
-        <v>46320.32086435916</v>
+        <v>46320.69295145541</v>
       </c>
       <c r="Q59" s="5" t="s">
         <v>30</v>
@@ -3955,7 +3955,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P60" s="6">
-        <v>46320.32086434212</v>
+        <v>46320.69295143897</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>23</v>
@@ -4002,7 +4002,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P61" s="6">
-        <v>46320.32086443242</v>
+        <v>46320.69295152815</v>
       </c>
       <c r="Q61" s="5" t="s">
         <v>30</v>
@@ -4051,7 +4051,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P62" s="6">
-        <v>46320.32086438912</v>
+        <v>46320.69295148482</v>
       </c>
       <c r="Q62" s="6" t="s">
         <v>23</v>
@@ -4100,7 +4100,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P63" s="6">
-        <v>46320.32086440336</v>
+        <v>46320.69295149899</v>
       </c>
       <c r="Q63" s="5" t="s">
         <v>30</v>
@@ -4147,7 +4147,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P64" s="6">
-        <v>46320.32086447579</v>
+        <v>46320.69295157161</v>
       </c>
       <c r="Q64" s="5" t="s">
         <v>30</v>
@@ -4196,7 +4196,7 @@
         <v>46302.26841519317</v>
       </c>
       <c r="P65" s="6">
-        <v>46320.32086449</v>
+        <v>46320.6929515858</v>
       </c>
       <c r="Q65" s="6" t="s">
         <v>23</v>
@@ -4245,7 +4245,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P66" s="6">
-        <v>46320.32086451913</v>
+        <v>46320.69295161423</v>
       </c>
       <c r="Q66" s="6" t="s">
         <v>23</v>
@@ -4292,7 +4292,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P67" s="6">
-        <v>46320.32086454726</v>
+        <v>46320.69295164223</v>
       </c>
       <c r="Q67" s="6" t="s">
         <v>23</v>
@@ -4341,7 +4341,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P68" s="6">
-        <v>46320.3208645331</v>
+        <v>46320.692951628</v>
       </c>
       <c r="Q68" s="6" t="s">
         <v>23</v>
@@ -4390,7 +4390,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P69" s="6">
-        <v>46320.32086450433</v>
+        <v>46320.69295159983</v>
       </c>
       <c r="Q69" s="6" t="s">
         <v>23</v>
@@ -4439,7 +4439,7 @@
         <v>46300.75884787029</v>
       </c>
       <c r="P70" s="6">
-        <v>46320.32086457592</v>
+        <v>46320.69295167056</v>
       </c>
       <c r="Q70" s="6" t="s">
         <v>23</v>
@@ -4702,7 +4702,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P2" s="2">
-        <v>46320.32085586598</v>
+        <v>46320.6929425487</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>30</v>
@@ -4746,7 +4746,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P3" s="2">
-        <v>46320.32085581985</v>
+        <v>46320.69294250303</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>30</v>
@@ -4793,7 +4793,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P4" s="2">
-        <v>46320.32084749614</v>
+        <v>46320.69293417776</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>30</v>
@@ -4840,7 +4840,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P5" s="2">
-        <v>46320.32084746652</v>
+        <v>46320.69293414867</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>30</v>
@@ -4887,7 +4887,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P6" s="2">
-        <v>46320.32084752488</v>
+        <v>46320.69293420629</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>30</v>
@@ -4931,7 +4931,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P7" s="2">
-        <v>46320.32084743775</v>
+        <v>46320.69293412055</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>30</v>
@@ -4975,7 +4975,7 @@
         <v>46309.72494259723</v>
       </c>
       <c r="P8" s="2">
-        <v>46320.32084742378</v>
+        <v>46320.69293410664</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>30</v>
@@ -5022,7 +5022,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P9" s="2">
-        <v>46320.32084740869</v>
+        <v>46320.69293409197</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>30</v>
@@ -5069,7 +5069,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P10" s="2">
-        <v>46320.32084737946</v>
+        <v>46320.69293406293</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>30</v>
@@ -5116,7 +5116,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P11" s="2">
-        <v>46320.32084736499</v>
+        <v>46320.69293404857</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>30</v>
@@ -5160,7 +5160,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P12" s="2">
-        <v>46320.3208473202</v>
+        <v>46320.69293400446</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>30</v>
@@ -5204,7 +5204,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P13" s="2">
-        <v>46320.32084727324</v>
+        <v>46320.69293395866</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>30</v>
@@ -5248,7 +5248,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P14" s="2">
-        <v>46320.32084728919</v>
+        <v>46320.69293397453</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>30</v>
@@ -5339,7 +5339,7 @@
         <v>46316.72655650476</v>
       </c>
       <c r="P16">
-        <v>46320.3208389317</v>
+        <v>46320.69292546777</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>30</v>
@@ -5386,7 +5386,7 @@
         <v>46316.72655654202</v>
       </c>
       <c r="P17">
-        <v>46320.32083885691</v>
+        <v>46320.69292539194</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>30</v>
@@ -5430,7 +5430,7 @@
         <v>46317.72506061158</v>
       </c>
       <c r="P18">
-        <v>46320.32083887186</v>
+        <v>46320.69292540668</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>30</v>
@@ -5474,7 +5474,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P19">
-        <v>46320.32083884165</v>
+        <v>46320.69292537658</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>30</v>
@@ -5518,7 +5518,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P20">
-        <v>46320.3208387964</v>
+        <v>46320.69292532978</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>30</v>
@@ -5562,7 +5562,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P21">
-        <v>46320.32083871875</v>
+        <v>46320.6929252531</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>30</v>
@@ -5606,7 +5606,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P22">
-        <v>46320.32083868645</v>
+        <v>46320.69292522156</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>30</v>
@@ -5655,7 +5655,7 @@
         <v>46307.39549700746</v>
       </c>
       <c r="P23" s="6">
-        <v>46320.32085599675</v>
+        <v>46320.69294268152</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>30</v>
@@ -5702,7 +5702,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P24" s="6">
-        <v>46320.32085598254</v>
+        <v>46320.69294266718</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>30</v>
@@ -5749,7 +5749,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P25" s="6">
-        <v>46320.32085592383</v>
+        <v>46320.6929426069</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>30</v>
@@ -5798,7 +5798,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P26" s="6">
-        <v>46320.32085605386</v>
+        <v>46320.69294273822</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>30</v>
@@ -5845,7 +5845,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P27" s="6">
-        <v>46320.32085608264</v>
+        <v>46320.69294276673</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>30</v>
@@ -5892,7 +5892,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P28" s="6">
-        <v>46320.32085606855</v>
+        <v>46320.69294275272</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>30</v>
@@ -5941,7 +5941,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P29" s="6">
-        <v>46320.32086435916</v>
+        <v>46320.69295145541</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>30</v>
@@ -5988,7 +5988,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P30" s="6">
-        <v>46320.32086443242</v>
+        <v>46320.69295152815</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>30</v>
@@ -6037,7 +6037,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P31" s="6">
-        <v>46320.32086440336</v>
+        <v>46320.69295149899</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>30</v>
@@ -6084,7 +6084,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P32" s="6">
-        <v>46320.32086447579</v>
+        <v>46320.69295157161</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>30</v>
@@ -6162,7 +6162,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -6210,10 +6210,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46320.32081964578</v>
+        <v>46320.69290182104</v>
       </c>
       <c r="B2">
-        <v>46320.32393692334</v>
+        <v>46320.69482767315</v>
       </c>
       <c r="C2" t="s">
         <v>230</v>
@@ -6245,10 +6245,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46319.67200058671</v>
+        <v>46320.32081964578</v>
       </c>
       <c r="B3">
-        <v>46319.6736326805</v>
+        <v>46320.32393692334</v>
       </c>
       <c r="C3" t="s">
         <v>230</v>
@@ -6280,10 +6280,10 @@
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46319.31121266444</v>
+        <v>46319.67200058671</v>
       </c>
       <c r="B4">
-        <v>46319.31353464982</v>
+        <v>46319.6736326805</v>
       </c>
       <c r="C4" t="s">
         <v>230</v>
@@ -6315,10 +6315,10 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46318.72195433634</v>
+        <v>46319.31121266444</v>
       </c>
       <c r="B5">
-        <v>46318.72353879309</v>
+        <v>46319.31353464982</v>
       </c>
       <c r="C5" t="s">
         <v>230</v>
@@ -6330,7 +6330,7 @@
         <v>3885</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5">
         <v>406</v>
@@ -6350,10 +6350,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46318.32371957044</v>
+        <v>46318.72195433634</v>
       </c>
       <c r="B6">
-        <v>46318.32702615024</v>
+        <v>46318.72353879309</v>
       </c>
       <c r="C6" t="s">
         <v>230</v>
@@ -6362,10 +6362,10 @@
         <v>195</v>
       </c>
       <c r="E6">
-        <v>3883</v>
+        <v>3885</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>406</v>
@@ -6380,15 +6380,15 @@
         <v>0</v>
       </c>
       <c r="K6">
-        <v>3883</v>
+        <v>3885</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46317.72504084905</v>
+        <v>46318.32371957044</v>
       </c>
       <c r="B7">
-        <v>46317.72671046003</v>
+        <v>46318.32702615024</v>
       </c>
       <c r="C7" t="s">
         <v>230</v>
@@ -6400,13 +6400,13 @@
         <v>3883</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -6420,10 +6420,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46317.32460656222</v>
+        <v>46317.72504084905</v>
       </c>
       <c r="B8">
-        <v>46317.32634152405</v>
+        <v>46317.72671046003</v>
       </c>
       <c r="C8" t="s">
         <v>230</v>
@@ -6432,13 +6432,13 @@
         <v>195</v>
       </c>
       <c r="E8">
-        <v>3882</v>
+        <v>3883</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -6450,33 +6450,33 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>3882</v>
+        <v>3883</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46316.72653559106</v>
+        <v>46317.32460656222</v>
       </c>
       <c r="B9">
-        <v>46316.72825635534</v>
+        <v>46317.32634152405</v>
       </c>
       <c r="C9" t="s">
         <v>230</v>
       </c>
       <c r="D9">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E9">
-        <v>3880</v>
+        <v>3882</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G9">
         <v>405</v>
       </c>
       <c r="H9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I9">
         <v>0</v>
@@ -6485,15 +6485,15 @@
         <v>0</v>
       </c>
       <c r="K9">
-        <v>3880</v>
+        <v>3882</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46316.32743514836</v>
+        <v>46316.72653559106</v>
       </c>
       <c r="B10">
-        <v>46316.33233177644</v>
+        <v>46316.72825635534</v>
       </c>
       <c r="C10" t="s">
         <v>230</v>
@@ -6502,16 +6502,16 @@
         <v>194</v>
       </c>
       <c r="E10">
-        <v>3875</v>
+        <v>3880</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>405</v>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -6520,15 +6520,15 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3875</v>
+        <v>3880</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46315.72470289427</v>
+        <v>46316.32743514836</v>
       </c>
       <c r="B11">
-        <v>46315.72632052699</v>
+        <v>46316.33233177644</v>
       </c>
       <c r="C11" t="s">
         <v>230</v>
@@ -6543,7 +6543,7 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -6560,10 +6560,10 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46315.32474515907</v>
+        <v>46315.72470289427</v>
       </c>
       <c r="B12">
-        <v>46315.32820895511</v>
+        <v>46315.72632052699</v>
       </c>
       <c r="C12" t="s">
         <v>230</v>
@@ -6595,10 +6595,10 @@
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46314.78235376754</v>
+        <v>46315.32474515907</v>
       </c>
       <c r="B13">
-        <v>46314.78404047032</v>
+        <v>46315.32820895511</v>
       </c>
       <c r="C13" t="s">
         <v>230</v>
@@ -6610,16 +6610,16 @@
         <v>3875</v>
       </c>
       <c r="F13">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="H13">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J13">
         <v>0</v>
@@ -6630,10 +6630,10 @@
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46314.33167013015</v>
+        <v>46314.78235376754</v>
       </c>
       <c r="B14">
-        <v>46314.33543636992</v>
+        <v>46314.78404047032</v>
       </c>
       <c r="C14" t="s">
         <v>230</v>
@@ -6642,33 +6642,33 @@
         <v>194</v>
       </c>
       <c r="E14">
-        <v>3867</v>
+        <v>3875</v>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G14">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14">
         <v>0</v>
       </c>
       <c r="K14">
-        <v>3867</v>
+        <v>3875</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46313.66768650556</v>
+        <v>46314.33167013015</v>
       </c>
       <c r="B15">
-        <v>46313.66945401487</v>
+        <v>46314.33543636992</v>
       </c>
       <c r="C15" t="s">
         <v>230</v>
@@ -6677,16 +6677,16 @@
         <v>194</v>
       </c>
       <c r="E15">
-        <v>3861</v>
+        <v>3867</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G15">
         <v>393</v>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I15">
         <v>0</v>
@@ -6695,15 +6695,15 @@
         <v>0</v>
       </c>
       <c r="K15">
-        <v>3861</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46313.30528009156</v>
+        <v>46313.66768650556</v>
       </c>
       <c r="B16">
-        <v>46313.3091804056</v>
+        <v>46313.66945401487</v>
       </c>
       <c r="C16" t="s">
         <v>230</v>
@@ -6735,10 +6735,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46312.65708521284</v>
+        <v>46313.30528009156</v>
       </c>
       <c r="B17">
-        <v>46312.65865222656</v>
+        <v>46313.3091804056</v>
       </c>
       <c r="C17" t="s">
         <v>230</v>
@@ -6770,10 +6770,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46312.29481460934</v>
+        <v>46312.65708521284</v>
       </c>
       <c r="B18">
-        <v>46312.29886374016</v>
+        <v>46312.65865222656</v>
       </c>
       <c r="C18" t="s">
         <v>230</v>
@@ -6805,10 +6805,10 @@
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B19">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C19" t="s">
         <v>230</v>
@@ -6823,7 +6823,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -6840,10 +6840,10 @@
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B20">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C20" t="s">
         <v>230</v>
@@ -6855,16 +6855,16 @@
         <v>3861</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J20">
         <v>0</v>
@@ -6875,45 +6875,45 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B21">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C21" t="s">
         <v>230</v>
       </c>
       <c r="D21">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E21">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G21">
         <v>394</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B22">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C22" t="s">
         <v>230</v>
@@ -6922,33 +6922,33 @@
         <v>193</v>
       </c>
       <c r="E22">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G22">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H22">
         <v>2</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B23">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C23" t="s">
         <v>230</v>
@@ -6957,16 +6957,16 @@
         <v>193</v>
       </c>
       <c r="E23">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F23">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G23">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H23">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I23">
         <v>1</v>
@@ -6975,15 +6975,15 @@
         <v>0</v>
       </c>
       <c r="K23">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B24">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C24" t="s">
         <v>230</v>
@@ -6992,33 +6992,33 @@
         <v>193</v>
       </c>
       <c r="E24">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G24">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24">
         <v>0</v>
       </c>
       <c r="K24">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="25" spans="1:11">
       <c r="A25">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B25">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C25" t="s">
         <v>230</v>
@@ -7033,7 +7033,7 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H25">
         <v>0</v>
@@ -7050,10 +7050,10 @@
     </row>
     <row r="26" spans="1:11">
       <c r="A26">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B26">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C26" t="s">
         <v>230</v>
@@ -7065,16 +7065,16 @@
         <v>3844</v>
       </c>
       <c r="F26">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G26">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26">
         <v>0</v>
@@ -7085,45 +7085,45 @@
     </row>
     <row r="27" spans="1:11">
       <c r="A27">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B27">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C27" t="s">
         <v>230</v>
       </c>
       <c r="D27">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E27">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G27">
         <v>381</v>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
       <c r="K27">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B28">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C28" t="s">
         <v>230</v>
@@ -7135,13 +7135,13 @@
         <v>3838</v>
       </c>
       <c r="F28">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G28">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H28">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -7155,10 +7155,10 @@
     </row>
     <row r="29" spans="1:11">
       <c r="A29">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B29">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C29" t="s">
         <v>230</v>
@@ -7167,16 +7167,16 @@
         <v>192</v>
       </c>
       <c r="E29">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G29">
         <v>369</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I29">
         <v>0</v>
@@ -7185,15 +7185,15 @@
         <v>0</v>
       </c>
       <c r="K29">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="30" spans="1:11">
       <c r="A30">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B30">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C30" t="s">
         <v>230</v>
@@ -7225,10 +7225,10 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B31">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C31" t="s">
         <v>230</v>
@@ -7243,7 +7243,7 @@
         <v>0</v>
       </c>
       <c r="G31">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -7260,10 +7260,10 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B32">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C32" t="s">
         <v>230</v>
@@ -7295,10 +7295,10 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B33">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C33" t="s">
         <v>230</v>
@@ -7310,16 +7310,16 @@
         <v>3826</v>
       </c>
       <c r="F33">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G33">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33">
         <v>0</v>
@@ -7330,45 +7330,45 @@
     </row>
     <row r="34" spans="1:11">
       <c r="A34">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B34">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C34" t="s">
         <v>230</v>
       </c>
       <c r="D34">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E34">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G34">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34">
         <v>0</v>
       </c>
       <c r="K34">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="35" spans="1:11">
       <c r="A35">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B35">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C35" t="s">
         <v>230</v>
@@ -7400,10 +7400,10 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B36">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C36" t="s">
         <v>230</v>
@@ -7418,7 +7418,7 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -7435,10 +7435,10 @@
     </row>
     <row r="37" spans="1:11">
       <c r="A37">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B37">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C37" t="s">
         <v>230</v>
@@ -7450,16 +7450,16 @@
         <v>3820</v>
       </c>
       <c r="F37">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H37">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I37">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J37">
         <v>0</v>
@@ -7470,45 +7470,45 @@
     </row>
     <row r="38" spans="1:11">
       <c r="A38">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B38">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C38" t="s">
         <v>230</v>
       </c>
       <c r="D38">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E38">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F38">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G38">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J38">
         <v>0</v>
       </c>
       <c r="K38">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B39">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C39" t="s">
         <v>230</v>
@@ -7520,13 +7520,13 @@
         <v>160</v>
       </c>
       <c r="F39">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G39">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -7535,15 +7535,15 @@
         <v>0</v>
       </c>
       <c r="K39">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="40" spans="1:11">
       <c r="A40">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B40">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C40" t="s">
         <v>230</v>
@@ -7555,21 +7555,56 @@
         <v>160</v>
       </c>
       <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40">
+        <v>160</v>
+      </c>
+      <c r="H40">
+        <v>0</v>
+      </c>
+      <c r="I40">
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <v>0</v>
+      </c>
+      <c r="K40">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B41">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C41" t="s">
+        <v>230</v>
+      </c>
+      <c r="D41">
+        <v>8</v>
+      </c>
+      <c r="E41">
+        <v>160</v>
+      </c>
+      <c r="F41">
         <v>157</v>
       </c>
-      <c r="G40">
+      <c r="G41">
         <v>3</v>
       </c>
-      <c r="H40">
+      <c r="H41">
         <v>132</v>
       </c>
-      <c r="I40">
-        <v>1</v>
-      </c>
-      <c r="J40">
-        <v>0</v>
-      </c>
-      <c r="K40">
+      <c r="I41">
+        <v>1</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
         <v>3814</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: verified full-source CIRP refresh 2026-10-27-1811Z
</commit_message>
<xml_diff>
--- a/docs/cirp-eoi-monitor.xlsx
+++ b/docs/cirp-eoi-monitor.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1098" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="240">
   <si>
     <t>Priority</t>
   </si>
@@ -1256,7 +1256,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P2" s="2">
-        <v>46322.33712158864</v>
+        <v>46322.75576081187</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>23</v>
@@ -1306,7 +1306,7 @@
         <v>46307.39549684311</v>
       </c>
       <c r="P3" s="2">
-        <v>46322.33712157336</v>
+        <v>46322.75576079699</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>29</v>
@@ -1353,7 +1353,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P4" s="2">
-        <v>46322.33712162068</v>
+        <v>46322.75576084184</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>23</v>
@@ -1403,7 +1403,7 @@
         <v>46308.39986117012</v>
       </c>
       <c r="P5" s="2">
-        <v>46322.33712160422</v>
+        <v>46322.75576082633</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>29</v>
@@ -1450,7 +1450,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P6" s="2">
-        <v>46322.33712155752</v>
+        <v>46322.75576078182</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>23</v>
@@ -1500,7 +1500,7 @@
         <v>46318.72197647238</v>
       </c>
       <c r="P7" s="2">
-        <v>46322.3371216357</v>
+        <v>46322.75576085648</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>29</v>
@@ -1544,7 +1544,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P8" s="2">
-        <v>46322.33712152159</v>
+        <v>46322.75576074986</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>23</v>
@@ -1635,7 +1635,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P10" s="2">
-        <v>46322.3371132651</v>
+        <v>46322.75575236943</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>23</v>
@@ -1685,7 +1685,7 @@
         <v>46310.31706138982</v>
       </c>
       <c r="P11" s="2">
-        <v>46322.33711327983</v>
+        <v>46322.75575238423</v>
       </c>
       <c r="Q11" s="2" t="s">
         <v>29</v>
@@ -1732,7 +1732,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P12" s="2">
-        <v>46322.33712154124</v>
+        <v>46322.75576076626</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>23</v>
@@ -1779,7 +1779,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P13" s="2">
-        <v>46322.33711325082</v>
+        <v>46322.75575235485</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>23</v>
@@ -1826,7 +1826,7 @@
         <v>46310.31706133292</v>
       </c>
       <c r="P14" s="2">
-        <v>46322.33711323598</v>
+        <v>46322.75575234003</v>
       </c>
       <c r="Q14" s="2" t="s">
         <v>29</v>
@@ -1876,7 +1876,7 @@
         <v>46309.72494249383</v>
       </c>
       <c r="P15" s="2">
-        <v>46322.33711322111</v>
+        <v>46322.75575232491</v>
       </c>
       <c r="Q15" s="2" t="s">
         <v>29</v>
@@ -1920,7 +1920,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P16" s="2">
-        <v>46322.33711313302</v>
+        <v>46322.75575223567</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>23</v>
@@ -1964,7 +1964,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P17" s="2">
-        <v>46322.3371131629</v>
+        <v>46322.75575226529</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>23</v>
@@ -2008,7 +2008,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P18" s="2">
-        <v>46322.33711317724</v>
+        <v>46322.75575227962</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>23</v>
@@ -2052,7 +2052,7 @@
         <v>46317.32462342</v>
       </c>
       <c r="P19" s="2">
-        <v>46322.33711314818</v>
+        <v>46322.75575225037</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>23</v>
@@ -2099,7 +2099,7 @@
         <v>46321.78119819488</v>
       </c>
       <c r="P20" s="2">
-        <v>46322.33711319194</v>
+        <v>46322.75575229495</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>23</v>
@@ -2143,7 +2143,7 @@
         <v>46314.33168865994</v>
       </c>
       <c r="P21" s="2">
-        <v>46322.33711311797</v>
+        <v>46322.75575222072</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>29</v>
@@ -2193,7 +2193,7 @@
         <v>46308.39986111095</v>
       </c>
       <c r="P22" s="2">
-        <v>46322.33711296376</v>
+        <v>46322.755752112</v>
       </c>
       <c r="Q22" s="2" t="s">
         <v>29</v>
@@ -2237,7 +2237,7 @@
         <v>46314.78237020577</v>
       </c>
       <c r="P23" s="2">
-        <v>46322.33711298033</v>
+        <v>46322.75575212925</v>
       </c>
       <c r="Q23" s="2" t="s">
         <v>29</v>
@@ -2334,7 +2334,7 @@
         <v>46316.72655650476</v>
       </c>
       <c r="P25" s="2">
-        <v>46322.33711299603</v>
+        <v>46322.75575214464</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>23</v>
@@ -2381,7 +2381,7 @@
         <v>46316.72655654202</v>
       </c>
       <c r="P26" s="2">
-        <v>46322.33711301215</v>
+        <v>46322.75575216</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>23</v>
@@ -2425,7 +2425,7 @@
         <v>46317.72506061158</v>
       </c>
       <c r="P27" s="2">
-        <v>46322.33711302684</v>
+        <v>46322.75575217516</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>23</v>
@@ -2472,7 +2472,7 @@
         <v>46322.33711306576</v>
       </c>
       <c r="P28" s="2">
-        <v>46322.33711306579</v>
+        <v>46322.75575219038</v>
       </c>
       <c r="Q28" s="2" t="s">
         <v>29</v>
@@ -2522,7 +2522,7 @@
         <v>46322.33711310413</v>
       </c>
       <c r="P29" s="2">
-        <v>46322.33711310416</v>
+        <v>46322.75575220548</v>
       </c>
       <c r="Q29" s="2" t="s">
         <v>29</v>
@@ -2566,7 +2566,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P30" s="2">
-        <v>46322.33709433489</v>
+        <v>46322.75574370971</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>23</v>
@@ -2610,7 +2610,7 @@
         <v>46317.32462326912</v>
       </c>
       <c r="P31" s="2">
-        <v>46322.33709431971</v>
+        <v>46322.75574369454</v>
       </c>
       <c r="Q31" s="2" t="s">
         <v>29</v>
@@ -2660,7 +2660,7 @@
         <v>46316.72655637826</v>
       </c>
       <c r="P32">
-        <v>46322.33709430446</v>
+        <v>46322.75574367941</v>
       </c>
       <c r="Q32" t="s">
         <v>29</v>
@@ -2704,7 +2704,7 @@
         <v>46322.33709429001</v>
       </c>
       <c r="P33">
-        <v>46322.33709429002</v>
+        <v>46322.75574366422</v>
       </c>
       <c r="Q33" t="s">
         <v>29</v>
@@ -2748,7 +2748,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P34">
-        <v>46322.33709421431</v>
+        <v>46322.75574363404</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>23</v>
@@ -2798,7 +2798,7 @@
         <v>46318.72196821687</v>
       </c>
       <c r="P35">
-        <v>46322.33709419827</v>
+        <v>46322.75574361828</v>
       </c>
       <c r="Q35" t="s">
         <v>29</v>
@@ -2842,7 +2842,7 @@
         <v>46305.20575257758</v>
       </c>
       <c r="P36">
-        <v>46322.33709418272</v>
+        <v>46322.75574360317</v>
       </c>
       <c r="Q36" t="s">
         <v>29</v>
@@ -2889,7 +2889,7 @@
         <v>46307.39549666931</v>
       </c>
       <c r="P37">
-        <v>46322.33709409014</v>
+        <v>46322.75574351154</v>
       </c>
       <c r="Q37" t="s">
         <v>29</v>
@@ -2933,7 +2933,7 @@
         <v>46307.39549671811</v>
       </c>
       <c r="P38">
-        <v>46322.33709410558</v>
+        <v>46322.75574352728</v>
       </c>
       <c r="Q38" t="s">
         <v>29</v>
@@ -2983,7 +2983,7 @@
         <v>46321.78118945728</v>
       </c>
       <c r="P39">
-        <v>46322.33709415259</v>
+        <v>46322.75574357322</v>
       </c>
       <c r="Q39" t="s">
         <v>29</v>
@@ -3030,7 +3030,7 @@
         <v>46321.78118948529</v>
       </c>
       <c r="P40">
-        <v>46322.33709416768</v>
+        <v>46322.75574358809</v>
       </c>
       <c r="Q40" s="5" t="s">
         <v>23</v>
@@ -3074,7 +3074,7 @@
         <v>46321.78118951154</v>
       </c>
       <c r="P41">
-        <v>46322.33709413683</v>
+        <v>46322.75574355766</v>
       </c>
       <c r="Q41" t="s">
         <v>29</v>
@@ -3121,7 +3121,7 @@
         <v>46321.78118953448</v>
       </c>
       <c r="P42">
-        <v>46322.33709412182</v>
+        <v>46322.75574354275</v>
       </c>
       <c r="Q42" s="5" t="s">
         <v>23</v>
@@ -3165,7 +3165,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P43">
-        <v>46322.33709405849</v>
+        <v>46322.75574347987</v>
       </c>
       <c r="Q43" s="5" t="s">
         <v>23</v>
@@ -3212,7 +3212,7 @@
         <v>46314.78237008413</v>
       </c>
       <c r="P44">
-        <v>46322.33709407449</v>
+        <v>46322.75574349572</v>
       </c>
       <c r="Q44" t="s">
         <v>29</v>
@@ -3259,7 +3259,7 @@
         <v>46322.33709404008</v>
       </c>
       <c r="P45">
-        <v>46322.33709404011</v>
+        <v>46322.75574346405</v>
       </c>
       <c r="Q45" s="5" t="s">
         <v>23</v>
@@ -3303,7 +3303,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P46">
-        <v>46322.3370938954</v>
+        <v>46322.75574344768</v>
       </c>
       <c r="Q46" s="5" t="s">
         <v>23</v>
@@ -3353,7 +3353,7 @@
         <v>46314.78236997747</v>
       </c>
       <c r="P47">
-        <v>46322.33709386474</v>
+        <v>46322.75574341475</v>
       </c>
       <c r="Q47" t="s">
         <v>29</v>
@@ -3400,7 +3400,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P48" s="6">
-        <v>46322.33712166532</v>
+        <v>46322.75576088589</v>
       </c>
       <c r="Q48" s="5" t="s">
         <v>23</v>
@@ -3449,7 +3449,7 @@
         <v>46314.78238309515</v>
       </c>
       <c r="P49" s="6">
-        <v>46322.33712165045</v>
+        <v>46322.75576087122</v>
       </c>
       <c r="Q49" s="6" t="s">
         <v>29</v>
@@ -3500,7 +3500,7 @@
         <v>46316.72656555651</v>
       </c>
       <c r="P50" s="6">
-        <v>46322.33712167979</v>
+        <v>46322.75576090072</v>
       </c>
       <c r="Q50" s="6" t="s">
         <v>29</v>
@@ -3549,7 +3549,7 @@
         <v>46307.3954969447</v>
       </c>
       <c r="P51" s="6">
-        <v>46322.33712172463</v>
+        <v>46322.75576094435</v>
       </c>
       <c r="Q51" s="6" t="s">
         <v>29</v>
@@ -3596,7 +3596,7 @@
         <v>46307.39549697415</v>
       </c>
       <c r="P52" s="6">
-        <v>46322.33712175374</v>
+        <v>46322.75576097339</v>
       </c>
       <c r="Q52" s="6" t="s">
         <v>29</v>
@@ -3643,7 +3643,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P53" s="6">
-        <v>46322.33712173929</v>
+        <v>46322.75576095919</v>
       </c>
       <c r="Q53" s="5" t="s">
         <v>23</v>
@@ -3692,7 +3692,7 @@
         <v>46314.33169674601</v>
       </c>
       <c r="P54" s="6">
-        <v>46322.33712169448</v>
+        <v>46322.75576091508</v>
       </c>
       <c r="Q54" s="6" t="s">
         <v>29</v>
@@ -3743,7 +3743,7 @@
         <v>46305.20575263901</v>
       </c>
       <c r="P55" s="6">
-        <v>46322.33712180416</v>
+        <v>46322.75576101762</v>
       </c>
       <c r="Q55" s="6" t="s">
         <v>29</v>
@@ -3790,7 +3790,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P56" s="6">
-        <v>46322.33712181933</v>
+        <v>46322.75576103213</v>
       </c>
       <c r="Q56" s="5" t="s">
         <v>23</v>
@@ -3837,7 +3837,7 @@
         <v>46309.72495168629</v>
       </c>
       <c r="P57" s="6">
-        <v>46322.33713004381</v>
+        <v>46322.7557694499</v>
       </c>
       <c r="Q57" s="6" t="s">
         <v>29</v>
@@ -3884,7 +3884,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P58" s="6">
-        <v>46322.33713006006</v>
+        <v>46322.7557694655</v>
       </c>
       <c r="Q58" s="5" t="s">
         <v>23</v>
@@ -3933,7 +3933,7 @@
         <v>46310.31707038325</v>
       </c>
       <c r="P59" s="6">
-        <v>46322.33712177046</v>
+        <v>46322.75576098805</v>
       </c>
       <c r="Q59" s="6" t="s">
         <v>29</v>
@@ -3982,7 +3982,7 @@
         <v>46308.39986132324</v>
       </c>
       <c r="P60" s="6">
-        <v>46322.3371300755</v>
+        <v>46322.75576947999</v>
       </c>
       <c r="Q60" s="6" t="s">
         <v>29</v>
@@ -4031,7 +4031,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P61" s="6">
-        <v>46322.33713010699</v>
+        <v>46322.75576951126</v>
       </c>
       <c r="Q61" s="5" t="s">
         <v>23</v>
@@ -4078,7 +4078,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P62" s="6">
-        <v>46322.33713013773</v>
+        <v>46322.75576954072</v>
       </c>
       <c r="Q62" s="5" t="s">
         <v>23</v>
@@ -4127,7 +4127,7 @@
         <v>46302.26841501552</v>
       </c>
       <c r="P63" s="6">
-        <v>46322.33713015265</v>
+        <v>46322.7557695557</v>
       </c>
       <c r="Q63" s="6" t="s">
         <v>29</v>
@@ -4174,7 +4174,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P64" s="6">
-        <v>46322.33713016736</v>
+        <v>46322.75576957061</v>
       </c>
       <c r="Q64" s="5" t="s">
         <v>23</v>
@@ -4223,7 +4223,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P65" s="6">
-        <v>46322.33713021239</v>
+        <v>46322.75576961404</v>
       </c>
       <c r="Q65" s="5" t="s">
         <v>23</v>
@@ -4272,7 +4272,7 @@
         <v>46307.39549714451</v>
       </c>
       <c r="P66" s="6">
-        <v>46322.33713018164</v>
+        <v>46322.75576958477</v>
       </c>
       <c r="Q66" s="6" t="s">
         <v>29</v>
@@ -4319,7 +4319,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P67" s="6">
-        <v>46322.33713027163</v>
+        <v>46322.75576967155</v>
       </c>
       <c r="Q67" s="5" t="s">
         <v>23</v>
@@ -4368,7 +4368,7 @@
         <v>46307.39550534703</v>
       </c>
       <c r="P68" s="6">
-        <v>46322.33713024201</v>
+        <v>46322.75576964267</v>
       </c>
       <c r="Q68" s="6" t="s">
         <v>29</v>
@@ -4417,7 +4417,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P69" s="6">
-        <v>46322.33713025663</v>
+        <v>46322.755769657</v>
       </c>
       <c r="Q69" s="5" t="s">
         <v>23</v>
@@ -4464,7 +4464,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P70" s="6">
-        <v>46322.33713028709</v>
+        <v>46322.75576968751</v>
       </c>
       <c r="Q70" s="5" t="s">
         <v>23</v>
@@ -4513,7 +4513,7 @@
         <v>46300.75884779022</v>
       </c>
       <c r="P71" s="6">
-        <v>46322.33713868664</v>
+        <v>46322.75577815934</v>
       </c>
       <c r="Q71" s="6" t="s">
         <v>29</v>
@@ -4560,7 +4560,7 @@
         <v>46300.75884780569</v>
       </c>
       <c r="P72" s="6">
-        <v>46322.33713870335</v>
+        <v>46322.75577817467</v>
       </c>
       <c r="Q72" s="6" t="s">
         <v>29</v>
@@ -4609,7 +4609,7 @@
         <v>46300.75884782107</v>
       </c>
       <c r="P73" s="6">
-        <v>46322.33713871896</v>
+        <v>46322.7557781904</v>
       </c>
       <c r="Q73" s="6" t="s">
         <v>29</v>
@@ -4658,7 +4658,7 @@
         <v>46300.75884783743</v>
       </c>
       <c r="P74" s="6">
-        <v>46322.337138734</v>
+        <v>46322.75577820546</v>
       </c>
       <c r="Q74" s="6" t="s">
         <v>29</v>
@@ -4932,7 +4932,7 @@
         <v>46307.39549680641</v>
       </c>
       <c r="P2" s="2">
-        <v>46322.33712158864</v>
+        <v>46322.75576081187</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>23</v>
@@ -4979,7 +4979,7 @@
         <v>46307.39549687663</v>
       </c>
       <c r="P3" s="2">
-        <v>46322.33712162068</v>
+        <v>46322.75576084184</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>23</v>
@@ -5026,7 +5026,7 @@
         <v>46311.30742780836</v>
       </c>
       <c r="P4" s="2">
-        <v>46322.33712155752</v>
+        <v>46322.75576078182</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>23</v>
@@ -5070,7 +5070,7 @@
         <v>46309.72494256633</v>
       </c>
       <c r="P5" s="2">
-        <v>46322.33712152159</v>
+        <v>46322.75576074986</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>23</v>
@@ -5161,7 +5161,7 @@
         <v>46309.72494262765</v>
       </c>
       <c r="P7" s="2">
-        <v>46322.3371132651</v>
+        <v>46322.75575236943</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>23</v>
@@ -5208,7 +5208,7 @@
         <v>46310.71706723773</v>
       </c>
       <c r="P8" s="2">
-        <v>46322.33712154124</v>
+        <v>46322.75576076626</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>23</v>
@@ -5255,7 +5255,7 @@
         <v>46309.72494253634</v>
       </c>
       <c r="P9" s="2">
-        <v>46322.33711325082</v>
+        <v>46322.75575235485</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>23</v>
@@ -5299,7 +5299,7 @@
         <v>46300.75884768533</v>
       </c>
       <c r="P10" s="2">
-        <v>46322.33711313302</v>
+        <v>46322.75575223567</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>23</v>
@@ -5343,7 +5343,7 @@
         <v>46314.3316886879</v>
       </c>
       <c r="P11" s="2">
-        <v>46322.3371131629</v>
+        <v>46322.75575226529</v>
       </c>
       <c r="Q11" s="5" t="s">
         <v>23</v>
@@ -5387,7 +5387,7 @@
         <v>46314.78237029647</v>
       </c>
       <c r="P12" s="2">
-        <v>46322.33711317724</v>
+        <v>46322.75575227962</v>
       </c>
       <c r="Q12" s="5" t="s">
         <v>23</v>
@@ -5431,7 +5431,7 @@
         <v>46317.32462342</v>
       </c>
       <c r="P13" s="2">
-        <v>46322.33711314818</v>
+        <v>46322.75575225037</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>23</v>
@@ -5478,7 +5478,7 @@
         <v>46321.78119819488</v>
       </c>
       <c r="P14" s="2">
-        <v>46322.33711319194</v>
+        <v>46322.75575229495</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>23</v>
@@ -5575,7 +5575,7 @@
         <v>46316.72655650476</v>
       </c>
       <c r="P16" s="2">
-        <v>46322.33711299603</v>
+        <v>46322.75575214464</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>23</v>
@@ -5622,7 +5622,7 @@
         <v>46316.72655654202</v>
       </c>
       <c r="P17" s="2">
-        <v>46322.33711301215</v>
+        <v>46322.75575216</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>23</v>
@@ -5666,7 +5666,7 @@
         <v>46317.72506061158</v>
       </c>
       <c r="P18" s="2">
-        <v>46322.33711302684</v>
+        <v>46322.75575217516</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>23</v>
@@ -5710,7 +5710,7 @@
         <v>46314.33168861312</v>
       </c>
       <c r="P19" s="2">
-        <v>46322.33709433489</v>
+        <v>46322.75574370971</v>
       </c>
       <c r="Q19" s="5" t="s">
         <v>23</v>
@@ -5754,7 +5754,7 @@
         <v>46314.33168857944</v>
       </c>
       <c r="P20">
-        <v>46322.33709421431</v>
+        <v>46322.75574363404</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>23</v>
@@ -5801,7 +5801,7 @@
         <v>46321.78118948529</v>
       </c>
       <c r="P21">
-        <v>46322.33709416768</v>
+        <v>46322.75574358809</v>
       </c>
       <c r="Q21" s="5" t="s">
         <v>23</v>
@@ -5848,7 +5848,7 @@
         <v>46321.78118953448</v>
       </c>
       <c r="P22">
-        <v>46322.33709412182</v>
+        <v>46322.75574354275</v>
       </c>
       <c r="Q22" s="5" t="s">
         <v>23</v>
@@ -5892,7 +5892,7 @@
         <v>46314.78237005197</v>
       </c>
       <c r="P23">
-        <v>46322.33709405849</v>
+        <v>46322.75574347987</v>
       </c>
       <c r="Q23" s="5" t="s">
         <v>23</v>
@@ -5939,7 +5939,7 @@
         <v>46322.33709404008</v>
       </c>
       <c r="P24">
-        <v>46322.33709404011</v>
+        <v>46322.75574346405</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>23</v>
@@ -5983,7 +5983,7 @@
         <v>46314.78237001975</v>
       </c>
       <c r="P25">
-        <v>46322.3370938954</v>
+        <v>46322.75574344768</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>23</v>
@@ -6030,7 +6030,7 @@
         <v>46307.39549690609</v>
       </c>
       <c r="P26" s="6">
-        <v>46322.33712166532</v>
+        <v>46322.75576088589</v>
       </c>
       <c r="Q26" s="5" t="s">
         <v>23</v>
@@ -6077,7 +6077,7 @@
         <v>46308.39986123197</v>
       </c>
       <c r="P27" s="6">
-        <v>46322.33712173929</v>
+        <v>46322.75576095919</v>
       </c>
       <c r="Q27" s="5" t="s">
         <v>23</v>
@@ -6124,7 +6124,7 @@
         <v>46307.3954970362</v>
       </c>
       <c r="P28" s="6">
-        <v>46322.33712181933</v>
+        <v>46322.75576103213</v>
       </c>
       <c r="Q28" s="5" t="s">
         <v>23</v>
@@ -6171,7 +6171,7 @@
         <v>46309.72495171529</v>
       </c>
       <c r="P29" s="6">
-        <v>46322.33713006006</v>
+        <v>46322.7557694655</v>
       </c>
       <c r="Q29" s="5" t="s">
         <v>23</v>
@@ -6220,7 +6220,7 @@
         <v>46311.30743731892</v>
       </c>
       <c r="P30" s="6">
-        <v>46322.33713010699</v>
+        <v>46322.75576951126</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>23</v>
@@ -6267,7 +6267,7 @@
         <v>46301.38232468421</v>
       </c>
       <c r="P31" s="6">
-        <v>46322.33713013773</v>
+        <v>46322.75576954072</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>23</v>
@@ -6314,7 +6314,7 @@
         <v>46309.72495178872</v>
       </c>
       <c r="P32" s="6">
-        <v>46322.33713016736</v>
+        <v>46322.75576957061</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>23</v>
@@ -6363,7 +6363,7 @@
         <v>46302.26841507768</v>
       </c>
       <c r="P33" s="6">
-        <v>46322.33713021239</v>
+        <v>46322.75576961404</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>23</v>
@@ -6410,7 +6410,7 @@
         <v>46300.75884772457</v>
       </c>
       <c r="P34" s="6">
-        <v>46322.33713027163</v>
+        <v>46322.75576967155</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>23</v>
@@ -6459,7 +6459,7 @@
         <v>46314.78239219591</v>
       </c>
       <c r="P35" s="6">
-        <v>46322.33713025663</v>
+        <v>46322.755769657</v>
       </c>
       <c r="Q35" s="5" t="s">
         <v>23</v>
@@ -6506,7 +6506,7 @@
         <v>46300.75884775587</v>
       </c>
       <c r="P36" s="6">
-        <v>46322.33713028709</v>
+        <v>46322.75576968751</v>
       </c>
       <c r="Q36" s="5" t="s">
         <v>23</v>
@@ -6592,7 +6592,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="20.7109375" customWidth="1"/>
@@ -6640,10 +6640,10 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2">
-        <v>46322.33707509178</v>
+        <v>46322.75572704514</v>
       </c>
       <c r="B2">
-        <v>46322.34166988715</v>
+        <v>46322.7576227476</v>
       </c>
       <c r="C2" t="s">
         <v>239</v>
@@ -6655,13 +6655,13 @@
         <v>3896</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G2">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -6675,10 +6675,10 @@
     </row>
     <row r="3" spans="1:12">
       <c r="A3">
-        <v>46321.78117365606</v>
+        <v>46322.33707509178</v>
       </c>
       <c r="B3">
-        <v>46321.78282221615</v>
+        <v>46322.34166988715</v>
       </c>
       <c r="C3" t="s">
         <v>239</v>
@@ -6687,16 +6687,16 @@
         <v>195</v>
       </c>
       <c r="E3">
-        <v>3891</v>
+        <v>3896</v>
       </c>
       <c r="F3">
         <v>5</v>
       </c>
       <c r="G3">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -6705,15 +6705,15 @@
         <v>0</v>
       </c>
       <c r="K3">
-        <v>3891</v>
+        <v>3896</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4">
-        <v>46321.33147967936</v>
+        <v>46321.78117365606</v>
       </c>
       <c r="B4">
-        <v>46321.33464941346</v>
+        <v>46321.78282221615</v>
       </c>
       <c r="C4" t="s">
         <v>239</v>
@@ -6722,16 +6722,16 @@
         <v>195</v>
       </c>
       <c r="E4">
-        <v>3885</v>
+        <v>3891</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G4">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -6740,15 +6740,15 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>3885</v>
+        <v>3891</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5">
-        <v>46320.69290182104</v>
+        <v>46321.33147967936</v>
       </c>
       <c r="B5">
-        <v>46320.69482767315</v>
+        <v>46321.33464941346</v>
       </c>
       <c r="C5" t="s">
         <v>239</v>
@@ -6763,7 +6763,7 @@
         <v>0</v>
       </c>
       <c r="G5">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -6780,10 +6780,10 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6">
-        <v>46320.32081964578</v>
+        <v>46320.69290182104</v>
       </c>
       <c r="B6">
-        <v>46320.32393692334</v>
+        <v>46320.69482767315</v>
       </c>
       <c r="C6" t="s">
         <v>239</v>
@@ -6815,10 +6815,10 @@
     </row>
     <row r="7" spans="1:12">
       <c r="A7">
-        <v>46319.67200058671</v>
+        <v>46320.32081964578</v>
       </c>
       <c r="B7">
-        <v>46319.6736326805</v>
+        <v>46320.32393692334</v>
       </c>
       <c r="C7" t="s">
         <v>239</v>
@@ -6850,10 +6850,10 @@
     </row>
     <row r="8" spans="1:12">
       <c r="A8">
-        <v>46319.31121266444</v>
+        <v>46319.67200058671</v>
       </c>
       <c r="B8">
-        <v>46319.31353464982</v>
+        <v>46319.6736326805</v>
       </c>
       <c r="C8" t="s">
         <v>239</v>
@@ -6885,10 +6885,10 @@
     </row>
     <row r="9" spans="1:12">
       <c r="A9">
-        <v>46318.72195433634</v>
+        <v>46319.31121266444</v>
       </c>
       <c r="B9">
-        <v>46318.72353879309</v>
+        <v>46319.31353464982</v>
       </c>
       <c r="C9" t="s">
         <v>239</v>
@@ -6900,7 +6900,7 @@
         <v>3885</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G9">
         <v>406</v>
@@ -6920,10 +6920,10 @@
     </row>
     <row r="10" spans="1:12">
       <c r="A10">
-        <v>46318.32371957044</v>
+        <v>46318.72195433634</v>
       </c>
       <c r="B10">
-        <v>46318.32702615024</v>
+        <v>46318.72353879309</v>
       </c>
       <c r="C10" t="s">
         <v>239</v>
@@ -6932,10 +6932,10 @@
         <v>195</v>
       </c>
       <c r="E10">
-        <v>3883</v>
+        <v>3885</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10">
         <v>406</v>
@@ -6950,15 +6950,15 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>3883</v>
+        <v>3885</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11">
-        <v>46317.72504084905</v>
+        <v>46318.32371957044</v>
       </c>
       <c r="B11">
-        <v>46317.72671046003</v>
+        <v>46318.32702615024</v>
       </c>
       <c r="C11" t="s">
         <v>239</v>
@@ -6970,13 +6970,13 @@
         <v>3883</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -6990,10 +6990,10 @@
     </row>
     <row r="12" spans="1:12">
       <c r="A12">
-        <v>46317.32460656222</v>
+        <v>46317.72504084905</v>
       </c>
       <c r="B12">
-        <v>46317.32634152405</v>
+        <v>46317.72671046003</v>
       </c>
       <c r="C12" t="s">
         <v>239</v>
@@ -7002,13 +7002,13 @@
         <v>195</v>
       </c>
       <c r="E12">
-        <v>3882</v>
+        <v>3883</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -7020,33 +7020,33 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>3882</v>
+        <v>3883</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13">
-        <v>46316.72653559106</v>
+        <v>46317.32460656222</v>
       </c>
       <c r="B13">
-        <v>46316.72825635534</v>
+        <v>46317.32634152405</v>
       </c>
       <c r="C13" t="s">
         <v>239</v>
       </c>
       <c r="D13">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E13">
-        <v>3880</v>
+        <v>3882</v>
       </c>
       <c r="F13">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G13">
         <v>405</v>
       </c>
       <c r="H13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I13">
         <v>0</v>
@@ -7055,15 +7055,15 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>3880</v>
+        <v>3882</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14">
-        <v>46316.32743514836</v>
+        <v>46316.72653559106</v>
       </c>
       <c r="B14">
-        <v>46316.33233177644</v>
+        <v>46316.72825635534</v>
       </c>
       <c r="C14" t="s">
         <v>239</v>
@@ -7072,16 +7072,16 @@
         <v>194</v>
       </c>
       <c r="E14">
-        <v>3875</v>
+        <v>3880</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G14">
         <v>405</v>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -7090,15 +7090,15 @@
         <v>0</v>
       </c>
       <c r="K14">
-        <v>3875</v>
+        <v>3880</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15">
-        <v>46315.72470289427</v>
+        <v>46316.32743514836</v>
       </c>
       <c r="B15">
-        <v>46315.72632052699</v>
+        <v>46316.33233177644</v>
       </c>
       <c r="C15" t="s">
         <v>239</v>
@@ -7113,7 +7113,7 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="H15">
         <v>0</v>
@@ -7130,10 +7130,10 @@
     </row>
     <row r="16" spans="1:12">
       <c r="A16">
-        <v>46315.32474515907</v>
+        <v>46315.72470289427</v>
       </c>
       <c r="B16">
-        <v>46315.32820895511</v>
+        <v>46315.72632052699</v>
       </c>
       <c r="C16" t="s">
         <v>239</v>
@@ -7165,10 +7165,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17">
-        <v>46314.78235376754</v>
+        <v>46315.32474515907</v>
       </c>
       <c r="B17">
-        <v>46314.78404047032</v>
+        <v>46315.32820895511</v>
       </c>
       <c r="C17" t="s">
         <v>239</v>
@@ -7180,16 +7180,16 @@
         <v>3875</v>
       </c>
       <c r="F17">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G17">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="H17">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -7200,10 +7200,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18">
-        <v>46314.33167013015</v>
+        <v>46314.78235376754</v>
       </c>
       <c r="B18">
-        <v>46314.33543636992</v>
+        <v>46314.78404047032</v>
       </c>
       <c r="C18" t="s">
         <v>239</v>
@@ -7212,33 +7212,33 @@
         <v>194</v>
       </c>
       <c r="E18">
-        <v>3867</v>
+        <v>3875</v>
       </c>
       <c r="F18">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G18">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="H18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18">
         <v>0</v>
       </c>
       <c r="K18">
-        <v>3867</v>
+        <v>3875</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19">
-        <v>46313.66768650556</v>
+        <v>46314.33167013015</v>
       </c>
       <c r="B19">
-        <v>46313.66945401487</v>
+        <v>46314.33543636992</v>
       </c>
       <c r="C19" t="s">
         <v>239</v>
@@ -7247,16 +7247,16 @@
         <v>194</v>
       </c>
       <c r="E19">
-        <v>3861</v>
+        <v>3867</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G19">
         <v>393</v>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I19">
         <v>0</v>
@@ -7265,15 +7265,15 @@
         <v>0</v>
       </c>
       <c r="K19">
-        <v>3861</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="20" spans="1:11">
       <c r="A20">
-        <v>46313.30528009156</v>
+        <v>46313.66768650556</v>
       </c>
       <c r="B20">
-        <v>46313.3091804056</v>
+        <v>46313.66945401487</v>
       </c>
       <c r="C20" t="s">
         <v>239</v>
@@ -7305,10 +7305,10 @@
     </row>
     <row r="21" spans="1:11">
       <c r="A21">
-        <v>46312.65708521284</v>
+        <v>46313.30528009156</v>
       </c>
       <c r="B21">
-        <v>46312.65865222656</v>
+        <v>46313.3091804056</v>
       </c>
       <c r="C21" t="s">
         <v>239</v>
@@ -7340,10 +7340,10 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22">
-        <v>46312.29481460934</v>
+        <v>46312.65708521284</v>
       </c>
       <c r="B22">
-        <v>46312.29886374016</v>
+        <v>46312.65865222656</v>
       </c>
       <c r="C22" t="s">
         <v>239</v>
@@ -7375,10 +7375,10 @@
     </row>
     <row r="23" spans="1:11">
       <c r="A23">
-        <v>46311.70085467582</v>
+        <v>46312.29481460934</v>
       </c>
       <c r="B23">
-        <v>46311.70249357724</v>
+        <v>46312.29886374016</v>
       </c>
       <c r="C23" t="s">
         <v>239</v>
@@ -7393,7 +7393,7 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -7410,10 +7410,10 @@
     </row>
     <row r="24" spans="1:11">
       <c r="A24">
-        <v>46311.3074085582</v>
+        <v>46311.70085467582</v>
       </c>
       <c r="B24">
-        <v>46311.31082826155</v>
+        <v>46311.70249357724</v>
       </c>
       <c r="C24" t="s">
         <v>239</v>
@@ -7425,16 +7425,16 @@
         <v>3861</v>
       </c>
       <c r="F24">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="H24">
         <v>0</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J24">
         <v>0</v>
@@ -7445,45 +7445,45 @@
     </row>
     <row r="25" spans="1:11">
       <c r="A25">
-        <v>46310.71705220221</v>
+        <v>46311.3074085582</v>
       </c>
       <c r="B25">
-        <v>46310.71871343154</v>
+        <v>46311.31082826155</v>
       </c>
       <c r="C25" t="s">
         <v>239</v>
       </c>
       <c r="D25">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E25">
-        <v>3858</v>
+        <v>3861</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25">
         <v>394</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25">
         <v>0</v>
       </c>
       <c r="K25">
-        <v>3858</v>
+        <v>3861</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26">
-        <v>46310.31704895089</v>
+        <v>46310.71705220221</v>
       </c>
       <c r="B26">
-        <v>46310.31885341345</v>
+        <v>46310.71871343154</v>
       </c>
       <c r="C26" t="s">
         <v>239</v>
@@ -7492,33 +7492,33 @@
         <v>193</v>
       </c>
       <c r="E26">
-        <v>3856</v>
+        <v>3858</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="H26">
         <v>2</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26">
         <v>0</v>
       </c>
       <c r="K26">
-        <v>3856</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="27" spans="1:11">
       <c r="A27">
-        <v>46309.72492152842</v>
+        <v>46310.31704895089</v>
       </c>
       <c r="B27">
-        <v>46309.72666770707</v>
+        <v>46310.31885341345</v>
       </c>
       <c r="C27" t="s">
         <v>239</v>
@@ -7527,16 +7527,16 @@
         <v>193</v>
       </c>
       <c r="E27">
-        <v>3854</v>
+        <v>3856</v>
       </c>
       <c r="F27">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="G27">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="H27">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I27">
         <v>1</v>
@@ -7545,15 +7545,15 @@
         <v>0</v>
       </c>
       <c r="K27">
-        <v>3854</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="28" spans="1:11">
       <c r="A28">
-        <v>46309.32656703098</v>
+        <v>46309.72492152842</v>
       </c>
       <c r="B28">
-        <v>46309.3297855199</v>
+        <v>46309.72666770707</v>
       </c>
       <c r="C28" t="s">
         <v>239</v>
@@ -7562,33 +7562,33 @@
         <v>193</v>
       </c>
       <c r="E28">
-        <v>3844</v>
+        <v>3854</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G28">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28">
         <v>0</v>
       </c>
       <c r="K28">
-        <v>3844</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29">
-        <v>46308.80857426515</v>
+        <v>46309.32656703098</v>
       </c>
       <c r="B29">
-        <v>46308.81014075634</v>
+        <v>46309.3297855199</v>
       </c>
       <c r="C29" t="s">
         <v>239</v>
@@ -7603,7 +7603,7 @@
         <v>0</v>
       </c>
       <c r="G29">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -7620,10 +7620,10 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30">
-        <v>46308.39983395509</v>
+        <v>46308.80857426515</v>
       </c>
       <c r="B30">
-        <v>46308.40210717713</v>
+        <v>46308.81014075634</v>
       </c>
       <c r="C30" t="s">
         <v>239</v>
@@ -7635,16 +7635,16 @@
         <v>3844</v>
       </c>
       <c r="F30">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G30">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="H30">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30">
         <v>0</v>
@@ -7655,45 +7655,45 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31">
-        <v>46307.88901948844</v>
+        <v>46308.39983395509</v>
       </c>
       <c r="B31">
-        <v>46307.89058348727</v>
+        <v>46308.40210717713</v>
       </c>
       <c r="C31" t="s">
         <v>239</v>
       </c>
       <c r="D31">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E31">
-        <v>3838</v>
+        <v>3844</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G31">
         <v>381</v>
       </c>
       <c r="H31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J31">
         <v>0</v>
       </c>
       <c r="K31">
-        <v>3838</v>
+        <v>3844</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32">
-        <v>46307.39547700758</v>
+        <v>46307.88901948844</v>
       </c>
       <c r="B32">
-        <v>46307.40588718568</v>
+        <v>46307.89058348727</v>
       </c>
       <c r="C32" t="s">
         <v>239</v>
@@ -7705,13 +7705,13 @@
         <v>3838</v>
       </c>
       <c r="F32">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="G32">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="H32">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I32">
         <v>0</v>
@@ -7725,10 +7725,10 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33">
-        <v>46306.73887016933</v>
+        <v>46307.39547700758</v>
       </c>
       <c r="B33">
-        <v>46306.74049537522</v>
+        <v>46307.40588718568</v>
       </c>
       <c r="C33" t="s">
         <v>239</v>
@@ -7737,16 +7737,16 @@
         <v>192</v>
       </c>
       <c r="E33">
-        <v>3826</v>
+        <v>3838</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G33">
         <v>369</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I33">
         <v>0</v>
@@ -7755,15 +7755,15 @@
         <v>0</v>
       </c>
       <c r="K33">
-        <v>3826</v>
+        <v>3838</v>
       </c>
     </row>
     <row r="34" spans="1:11">
       <c r="A34">
-        <v>46306.45016971852</v>
+        <v>46306.73887016933</v>
       </c>
       <c r="B34">
-        <v>46306.45174895023</v>
+        <v>46306.74049537522</v>
       </c>
       <c r="C34" t="s">
         <v>239</v>
@@ -7795,10 +7795,10 @@
     </row>
     <row r="35" spans="1:11">
       <c r="A35">
-        <v>46305.7254269891</v>
+        <v>46306.45016971852</v>
       </c>
       <c r="B35">
-        <v>46305.72703482325</v>
+        <v>46306.45174895023</v>
       </c>
       <c r="C35" t="s">
         <v>239</v>
@@ -7813,7 +7813,7 @@
         <v>0</v>
       </c>
       <c r="G35">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="H35">
         <v>0</v>
@@ -7830,10 +7830,10 @@
     </row>
     <row r="36" spans="1:11">
       <c r="A36">
-        <v>46305.36271514557</v>
+        <v>46305.7254269891</v>
       </c>
       <c r="B36">
-        <v>46305.36432437652</v>
+        <v>46305.72703482325</v>
       </c>
       <c r="C36" t="s">
         <v>239</v>
@@ -7865,10 +7865,10 @@
     </row>
     <row r="37" spans="1:11">
       <c r="A37">
-        <v>46305.20573401557</v>
+        <v>46305.36271514557</v>
       </c>
       <c r="B37">
-        <v>46305.20740965955</v>
+        <v>46305.36432437652</v>
       </c>
       <c r="C37" t="s">
         <v>239</v>
@@ -7880,16 +7880,16 @@
         <v>3826</v>
       </c>
       <c r="F37">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="H37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37">
         <v>0</v>
@@ -7900,45 +7900,45 @@
     </row>
     <row r="38" spans="1:11">
       <c r="A38">
-        <v>46303.78900727724</v>
+        <v>46305.20573401557</v>
       </c>
       <c r="B38">
-        <v>46303.79055355475</v>
+        <v>46305.20740965955</v>
       </c>
       <c r="C38" t="s">
         <v>239</v>
       </c>
       <c r="D38">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E38">
-        <v>3820</v>
+        <v>3826</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G38">
-        <v>373</v>
+        <v>365</v>
       </c>
       <c r="H38">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I38">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38">
         <v>0</v>
       </c>
       <c r="K38">
-        <v>3820</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="39" spans="1:11">
       <c r="A39">
-        <v>46303.38326038567</v>
+        <v>46303.78900727724</v>
       </c>
       <c r="B39">
-        <v>46303.38502199544</v>
+        <v>46303.79055355475</v>
       </c>
       <c r="C39" t="s">
         <v>239</v>
@@ -7970,10 +7970,10 @@
     </row>
     <row r="40" spans="1:11">
       <c r="A40">
-        <v>46302.79187874035</v>
+        <v>46303.38326038567</v>
       </c>
       <c r="B40">
-        <v>46302.79368556542</v>
+        <v>46303.38502199544</v>
       </c>
       <c r="C40" t="s">
         <v>239</v>
@@ -7988,7 +7988,7 @@
         <v>0</v>
       </c>
       <c r="G40">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -8005,10 +8005,10 @@
     </row>
     <row r="41" spans="1:11">
       <c r="A41">
-        <v>46302.26839808295</v>
+        <v>46302.79187874035</v>
       </c>
       <c r="B41">
-        <v>46302.2700367639</v>
+        <v>46302.79368556542</v>
       </c>
       <c r="C41" t="s">
         <v>239</v>
@@ -8020,16 +8020,16 @@
         <v>3820</v>
       </c>
       <c r="F41">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="G41">
-        <v>163</v>
+        <v>374</v>
       </c>
       <c r="H41">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="I41">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="J41">
         <v>0</v>
@@ -8040,45 +8040,45 @@
     </row>
     <row r="42" spans="1:11">
       <c r="A42">
-        <v>46301.38230919655</v>
+        <v>46302.26839808295</v>
       </c>
       <c r="B42">
-        <v>46301.3823941568</v>
+        <v>46302.2700367639</v>
       </c>
       <c r="C42" t="s">
         <v>239</v>
       </c>
       <c r="D42">
-        <v>8</v>
+        <v>191</v>
       </c>
       <c r="E42">
-        <v>160</v>
+        <v>3820</v>
       </c>
       <c r="F42">
-        <v>6</v>
+        <v>211</v>
       </c>
       <c r="G42">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="H42">
-        <v>4</v>
+        <v>124</v>
       </c>
       <c r="I42">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J42">
         <v>0</v>
       </c>
       <c r="K42">
-        <v>3817</v>
+        <v>3820</v>
       </c>
     </row>
     <row r="43" spans="1:11">
       <c r="A43">
-        <v>46300.7718278824</v>
+        <v>46301.38230919655</v>
       </c>
       <c r="B43">
-        <v>46300.77190961051</v>
+        <v>46301.3823941568</v>
       </c>
       <c r="C43" t="s">
         <v>239</v>
@@ -8090,13 +8090,13 @@
         <v>160</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G43">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="H43">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -8105,15 +8105,15 @@
         <v>0</v>
       </c>
       <c r="K43">
-        <v>3814</v>
+        <v>3817</v>
       </c>
     </row>
     <row r="44" spans="1:11">
       <c r="A44">
-        <v>46300.75883115231</v>
+        <v>46300.7718278824</v>
       </c>
       <c r="B44">
-        <v>46300.75891177973</v>
+        <v>46300.77190961051</v>
       </c>
       <c r="C44" t="s">
         <v>239</v>
@@ -8125,21 +8125,56 @@
         <v>160</v>
       </c>
       <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44">
+        <v>160</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44">
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <v>0</v>
+      </c>
+      <c r="K44">
+        <v>3814</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="A45">
+        <v>46300.75883115231</v>
+      </c>
+      <c r="B45">
+        <v>46300.75891177973</v>
+      </c>
+      <c r="C45" t="s">
+        <v>239</v>
+      </c>
+      <c r="D45">
+        <v>8</v>
+      </c>
+      <c r="E45">
+        <v>160</v>
+      </c>
+      <c r="F45">
         <v>157</v>
       </c>
-      <c r="G44">
+      <c r="G45">
         <v>3</v>
       </c>
-      <c r="H44">
+      <c r="H45">
         <v>132</v>
       </c>
-      <c r="I44">
-        <v>1</v>
-      </c>
-      <c r="J44">
-        <v>0</v>
-      </c>
-      <c r="K44">
+      <c r="I45">
+        <v>1</v>
+      </c>
+      <c r="J45">
+        <v>0</v>
+      </c>
+      <c r="K45">
         <v>3814</v>
       </c>
     </row>

</xml_diff>